<commit_message>
vengeanceaiUSCMODEL7: audit fixes for NWC, SGA, CapEx, exit 16x
- Operating NWC as one % of sales (fade → 3%); ends ~$297M AR/deferred drain
- SG&A floor 15% / −75bps grind; labels SG&A and R&D
- Faster CapEx fade to 1%; primary exit 16x (25x bull sensitivity)
- Mid-year CF dates via EDATE(transaction, (t-0.5)*12)

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -459,7 +459,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -647,7 +647,6 @@
     <xf numFmtId="164" fontId="39" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -6140,7 +6139,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="9.08984375" customWidth="1" min="15" max="15"/>
   </cols>
@@ -6530,7 +6529,7 @@
       <c r="K17" s="97" t="n"/>
       <c r="L17" s="114" t="inlineStr">
         <is>
-          <t>Terminal value methods (MODEL3)</t>
+          <t>Terminal value methods (MODEL7)</t>
         </is>
       </c>
       <c r="M17" s="111" t="n"/>
@@ -6541,7 +6540,7 @@
       <c r="A18" s="97" t="n"/>
       <c r="B18" s="97" t="inlineStr">
         <is>
-          <t>Date (mid-year convention)</t>
+          <t>Date (mid-year via EDATE from transaction)</t>
         </is>
       </c>
       <c r="C18" s="97" t="n"/>
@@ -6550,70 +6549,71 @@
         <v/>
       </c>
       <c r="E18" s="116">
-        <f>DATE(YEAR($D$10)+E19,3,31)</f>
+        <f>EDATE($D$9,(E19-0.5)*12)</f>
         <v/>
       </c>
       <c r="F18" s="116">
-        <f>DATE(YEAR($D$10)+F19,3,31)</f>
+        <f>EDATE($D$9,(F19-0.5)*12)</f>
         <v/>
       </c>
       <c r="G18" s="116">
-        <f>DATE(YEAR($D$10)+G19,3,31)</f>
+        <f>EDATE($D$9,(G19-0.5)*12)</f>
         <v/>
       </c>
       <c r="H18" s="116">
-        <f>DATE(YEAR($D$10)+H19,3,31)</f>
+        <f>EDATE($D$9,(H19-0.5)*12)</f>
         <v/>
       </c>
       <c r="I18" s="116">
-        <f>DATE(YEAR($D$10)+I19,3,31)</f>
-        <v/>
-      </c>
-      <c r="J18" s="117">
+        <f>EDATE($D$9,(I19-0.5)*12)</f>
+        <v/>
+      </c>
+      <c r="J18" s="116">
         <f>I18</f>
         <v/>
       </c>
       <c r="K18" s="97" t="n"/>
       <c r="L18" s="97" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA (in J27) — primary</t>
+          <t>Exit EV/EBITDA @ D8 (primary 16x)</t>
         </is>
       </c>
       <c r="M18" s="109">
         <f>J27</f>
         <v/>
       </c>
-      <c r="N18" s="97">
-        <f>(I26*(1+D7))/(D6-D7)</f>
-        <v/>
+      <c r="N18" s="97" t="inlineStr">
+        <is>
+          <t>← used in XNPV</t>
+        </is>
       </c>
       <c r="O18" s="97" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="97" t="n"/>
-      <c r="B19" s="118" t="inlineStr">
+      <c r="B19" s="117" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="118" t="n"/>
+      <c r="C19" s="117" t="n"/>
       <c r="D19" s="115" t="n"/>
-      <c r="E19" s="119" t="n">
+      <c r="E19" s="118" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="120">
+      <c r="F19" s="119">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="120">
+      <c r="G19" s="119">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="120">
+      <c r="H19" s="119">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="120">
+      <c r="I19" s="119">
         <f>H19+1</f>
         <v/>
       </c>
@@ -6628,38 +6628,39 @@
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="121">
-        <f>D8*(I21+I23)</f>
-        <v/>
+      <c r="N19" s="120" t="inlineStr">
+        <is>
+          <t>← sanity check</t>
+        </is>
       </c>
       <c r="O19" s="97" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="97" t="n"/>
-      <c r="B20" s="118" t="inlineStr">
-        <is>
-          <t>Year Fraction (display only; not applied to CF)</t>
+      <c r="B20" s="117" t="inlineStr">
+        <is>
+          <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
       <c r="C20" s="97" t="n"/>
       <c r="D20" s="97" t="n"/>
-      <c r="E20" s="122">
+      <c r="E20" s="121">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="122">
+      <c r="F20" s="121">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="122">
+      <c r="G20" s="121">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="122">
+      <c r="H20" s="121">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="122">
+      <c r="I20" s="121">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
@@ -6674,7 +6675,7 @@
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="123">
+      <c r="N20" s="122">
         <f>AVERAGE(N18:N19)</f>
         <v/>
       </c>
@@ -6711,9 +6712,20 @@
       </c>
       <c r="J21" s="97" t="n"/>
       <c r="K21" s="97" t="n"/>
-      <c r="L21" s="97" t="n"/>
-      <c r="M21" s="97" t="n"/>
-      <c r="N21" s="97" t="n"/>
+      <c r="L21" s="97" t="inlineStr">
+        <is>
+          <t>Bull case TV @ 25x (sensitivity only)</t>
+        </is>
+      </c>
+      <c r="M21" s="109">
+        <f>($I$21+$I$23)*25.0</f>
+        <v/>
+      </c>
+      <c r="N21" s="97" t="inlineStr">
+        <is>
+          <t>← not in base case</t>
+        </is>
+      </c>
       <c r="O21" s="97" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -6725,23 +6737,23 @@
       </c>
       <c r="C22" s="97" t="n"/>
       <c r="D22" s="97" t="n"/>
-      <c r="E22" s="124">
+      <c r="E22" s="123">
         <f>E21*$D$5</f>
         <v/>
       </c>
-      <c r="F22" s="124">
+      <c r="F22" s="123">
         <f>F21*$D$5</f>
         <v/>
       </c>
-      <c r="G22" s="124">
+      <c r="G22" s="123">
         <f>G21*$D$5</f>
         <v/>
       </c>
-      <c r="H22" s="124">
+      <c r="H22" s="123">
         <f>H21*$D$5</f>
         <v/>
       </c>
-      <c r="I22" s="124">
+      <c r="I22" s="123">
         <f>I21*$D$5</f>
         <v/>
       </c>
@@ -6761,23 +6773,23 @@
       </c>
       <c r="C23" s="97" t="n"/>
       <c r="D23" s="97" t="n"/>
-      <c r="E23" s="124">
+      <c r="E23" s="123">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="124">
+      <c r="F23" s="123">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="124">
+      <c r="G23" s="123">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="124">
+      <c r="H23" s="123">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="124">
+      <c r="I23" s="123">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
@@ -6869,23 +6881,23 @@
       </c>
       <c r="C26" s="97" t="n"/>
       <c r="D26" s="97" t="n"/>
-      <c r="E26" s="123">
+      <c r="E26" s="122">
         <f>E21-E22+E23-E24-E25</f>
         <v/>
       </c>
-      <c r="F26" s="123">
+      <c r="F26" s="122">
         <f>F21-F22+F23-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="123">
+      <c r="G26" s="122">
         <f>G21-G22+G23-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="123">
+      <c r="H26" s="122">
         <f>H21-H22+H23-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="123">
+      <c r="I26" s="122">
         <f>I21-I22+I23-I24-I25</f>
         <v/>
       </c>
@@ -6900,7 +6912,7 @@
       <c r="A27" s="97" t="n"/>
       <c r="B27" s="97" t="inlineStr">
         <is>
-          <t>(Entry)/Exit TV — Exit EV/EBITDA</t>
+          <t>(Entry)/Exit TV — Exit EV/EBITDA (primary 16x)</t>
         </is>
       </c>
       <c r="C27" s="97" t="n"/>
@@ -6931,30 +6943,30 @@
         </is>
       </c>
       <c r="C28" s="97" t="n"/>
-      <c r="D28" s="123" t="n">
+      <c r="D28" s="122" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="125">
+      <c r="E28" s="124">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="125">
+      <c r="F28" s="124">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="125">
+      <c r="G28" s="124">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="125">
+      <c r="H28" s="124">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="125">
+      <c r="I28" s="124">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="125">
+      <c r="J28" s="124">
         <f>J27+J26</f>
         <v/>
       </c>
@@ -7052,7 +7064,7 @@
       <c r="A32" s="97" t="n"/>
       <c r="B32" s="97" t="inlineStr">
         <is>
-          <t>Enterprise Value (XNPV, mid-year dates)</t>
+          <t>Enterprise Value (XNPV, mid-year EDATE dates)</t>
         </is>
       </c>
       <c r="C32" s="97" t="n"/>
@@ -7078,7 +7090,7 @@
         </is>
       </c>
       <c r="M32" s="97" t="n"/>
-      <c r="N32" s="126">
+      <c r="N32" s="125">
         <f>D37/I37-1</f>
         <v/>
       </c>
@@ -7114,7 +7126,7 @@
         </is>
       </c>
       <c r="M33" s="97" t="n"/>
-      <c r="N33" s="126">
+      <c r="N33" s="125">
         <f>XIRR(D29:J29,D18:J18)</f>
         <v/>
       </c>
@@ -7157,7 +7169,7 @@
         </is>
       </c>
       <c r="C35" s="97" t="n"/>
-      <c r="D35" s="123">
+      <c r="D35" s="122">
         <f>D32+D33-D34</f>
         <v/>
       </c>
@@ -7168,7 +7180,7 @@
         </is>
       </c>
       <c r="H35" s="97" t="n"/>
-      <c r="I35" s="123">
+      <c r="I35" s="122">
         <f>I32+I33-I34</f>
         <v/>
       </c>
@@ -7190,7 +7202,7 @@
       <c r="E36" s="97" t="n"/>
       <c r="G36" s="97" t="n"/>
       <c r="H36" s="97" t="n"/>
-      <c r="I36" s="127" t="n"/>
+      <c r="I36" s="126" t="n"/>
       <c r="J36" s="97" t="n"/>
       <c r="L36" s="97" t="inlineStr">
         <is>
@@ -7198,7 +7210,7 @@
         </is>
       </c>
       <c r="M36" s="97" t="n"/>
-      <c r="N36" s="127">
+      <c r="N36" s="126">
         <f>I37</f>
         <v/>
       </c>
@@ -7212,7 +7224,7 @@
         </is>
       </c>
       <c r="C37" s="97" t="n"/>
-      <c r="D37" s="127">
+      <c r="D37" s="126">
         <f>D35/D12</f>
         <v/>
       </c>
@@ -7223,7 +7235,7 @@
         </is>
       </c>
       <c r="H37" s="97" t="n"/>
-      <c r="I37" s="127">
+      <c r="I37" s="126">
         <f>D11</f>
         <v/>
       </c>
@@ -7234,7 +7246,7 @@
         </is>
       </c>
       <c r="M37" s="97" t="n"/>
-      <c r="N37" s="127">
+      <c r="N37" s="126">
         <f>D37-I37</f>
         <v/>
       </c>
@@ -7256,7 +7268,7 @@
         </is>
       </c>
       <c r="M38" s="97" t="n"/>
-      <c r="N38" s="127">
+      <c r="N38" s="126">
         <f>SUM(N36:N37)</f>
         <v/>
       </c>
@@ -7299,7 +7311,7 @@
         </is>
       </c>
       <c r="C41" s="111" t="n"/>
-      <c r="D41" s="128" t="n"/>
+      <c r="D41" s="127" t="n"/>
       <c r="E41" s="111" t="n"/>
       <c r="F41" s="111" t="n"/>
       <c r="G41" s="111" t="n"/>
@@ -7325,7 +7337,7 @@
       <c r="F42" s="97" t="n"/>
       <c r="G42" s="97" t="n"/>
       <c r="H42" s="97" t="n"/>
-      <c r="N42" s="129" t="inlineStr">
+      <c r="N42" s="128" t="inlineStr">
         <is>
           <t>This file is for educational purposes only. E&amp;OE</t>
         </is>
@@ -7350,7 +7362,7 @@
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="97" t="n"/>
-      <c r="B44" s="130" t="inlineStr">
+      <c r="B44" s="129" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7366,7 +7378,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="97" t="n"/>
-      <c r="B45" s="130" t="inlineStr">
+      <c r="B45" s="129" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7382,7 +7394,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="97" t="n"/>
-      <c r="B46" s="130" t="inlineStr">
+      <c r="B46" s="129" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -7417,7 +7429,7 @@
       <c r="F48" s="97" t="n"/>
       <c r="G48" s="97" t="n"/>
       <c r="H48" s="97" t="n"/>
-      <c r="N48" s="131" t="inlineStr">
+      <c r="N48" s="130" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -7433,7 +7445,7 @@
       <c r="F49" s="97" t="n"/>
       <c r="G49" s="97" t="n"/>
       <c r="H49" s="97" t="n"/>
-      <c r="N49" s="132" t="inlineStr">
+      <c r="N49" s="131" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>

</xml_diff>

<commit_message>
vengeanceaiUSCMODEL8: comps-sourced 17.5x exit + audit CF fixes
Source base exit EV/EBITDA from public peer comps (EFX/VRSK/SPGI/MCO/MSCI
median ~18.1x → 17.5x base; bull 25x; bear 12.8x Gordon). Flatten NWC to
2.5% of sales, keep SG&A floor 15%/−75bps and CapEx fade→1%, relabel SG&A/R&D,
add WACC×exit sensitivity tables, and refresh on-sheet HOW/WHY/SOURCE notes.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -82,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="16">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\(#,##0\)_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.0000_ ;\-0.0000\ "/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -94,8 +94,13 @@
     <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0.00_-;\(#,##0.00\)_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="175" formatCode="0.0"/>
+    <numFmt numFmtId="176" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="177" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="178" formatCode="#,##0.0"/>
+    <numFmt numFmtId="179" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="47">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -352,11 +357,47 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="000000FF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="8"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F4E79"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -398,8 +439,28 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00833C0C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -447,6 +508,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -459,7 +534,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -611,26 +686,41 @@
     <xf numFmtId="164" fontId="27" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="42" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="33" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="32" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="39" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="30" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -644,10 +734,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="39" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="46" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -672,6 +762,19 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="38" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="38" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1471,55 +1574,26 @@
 </chartSpace>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>1</col>
-      <colOff>714374</colOff>
-      <row>3</row>
-      <rowOff>19050</rowOff>
-    </from>
-    <to>
-      <col>4</col>
-      <colOff>661827</colOff>
-      <row>9</row>
-      <rowOff>114300</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Picture 1">
-          <a:hlinkClick r:id="rId1"/>
-        </cNvPr>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="1447799" y="762000"/>
-          <a:ext cx="3359943" cy="1581150"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>vengeanceaiUSCMODEL8</author>
+  </authors>
+  <commentList>
+    <comment ref="D8" authorId="0" shapeId="0">
+      <text>
+        <t>Exit EV/EBITDA multiple (BASE)
+HOW: Yellow POLICY input D8 = 17.5x; TV = Year-5 EBITDA × D8.
+WHY: Sourced from public peer EV/EBITDA (EFX/VRSK/SPGI/MCO/MSCI). Peer median ≈ 18.1x → base 17.5x (also ≈ 50/50 of bull 25x and bear/Gordon 12.8x). NOT FICO spot (~25–27x).
+SOURCE (peer comps): https://vcpscanner.com/valuation/fico/relative
+SOURCE (FICO spot): https://www.alphaspread.com/security/nyse/fico/relative-valuation/ratio/enterprise-value-to-ebitda</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
@@ -1573,49 +1647,6 @@
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>1</col>
-      <colOff>38101</colOff>
-      <row>131</row>
-      <rowOff>129314</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>783591</colOff>
-      <row>135</row>
-      <rowOff>144144</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Picture 3">
-          <a:hlinkClick r:id="rId1"/>
-        </cNvPr>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="647701" y="5158514"/>
-          <a:ext cx="742950" cy="813659"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
     <clientData/>
   </twoCellAnchor>
 </wsDr>
@@ -2405,7 +2436,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" scale="64"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -6125,7 +6155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:R72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.54296875" customWidth="1" min="1" max="1"/>
@@ -6139,9 +6169,10 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="9.08984375" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -6160,1488 +6191,1980 @@
       <c r="I1" s="93" t="n"/>
       <c r="J1" s="93" t="n"/>
       <c r="K1" s="94" t="n"/>
-      <c r="L1" s="94" t="n"/>
-      <c r="M1" s="94" t="n"/>
-      <c r="N1" s="94" t="n"/>
+      <c r="L1" s="95" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSCMODEL8 — Public Peer EV/EBITDA Comps</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="93" t="n"/>
-      <c r="B2" s="95" t="inlineStr">
+      <c r="B2" s="96" t="inlineStr">
         <is>
           <t>DCF Model</t>
         </is>
       </c>
-      <c r="C2" s="96" t="n"/>
-      <c r="D2" s="96" t="n"/>
-      <c r="E2" s="96" t="n"/>
+      <c r="C2" s="97" t="n"/>
+      <c r="D2" s="97" t="n"/>
+      <c r="E2" s="97" t="n"/>
       <c r="F2" s="94" t="n"/>
       <c r="G2" s="94" t="n"/>
       <c r="H2" s="93" t="n"/>
-      <c r="I2" s="95" t="n"/>
-      <c r="J2" s="96" t="n"/>
-      <c r="K2" s="96" t="n"/>
-      <c r="L2" s="96" t="n"/>
-      <c r="M2" s="94" t="n"/>
-      <c r="N2" s="94" t="n"/>
+      <c r="I2" s="96" t="n"/>
+      <c r="J2" s="97" t="n"/>
+      <c r="K2" s="97" t="n"/>
+      <c r="L2" s="98" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="M2" s="99" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="N2" s="99" t="inlineStr">
+        <is>
+          <t>EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="O2" s="98" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="97" t="n"/>
-      <c r="B3" s="98" t="n"/>
-      <c r="C3" s="97" t="n"/>
-      <c r="D3" s="99" t="n"/>
-      <c r="E3" s="100" t="n"/>
-      <c r="F3" s="100" t="n"/>
-      <c r="G3" s="100" t="n"/>
-      <c r="H3" s="100" t="n"/>
-      <c r="I3" s="100" t="n"/>
-      <c r="J3" s="97" t="n"/>
-      <c r="K3" s="97" t="n"/>
-      <c r="L3" s="97" t="n"/>
-      <c r="M3" s="97" t="n"/>
-      <c r="N3" s="97" t="n"/>
-      <c r="O3" s="97" t="n"/>
+      <c r="A3" s="100" t="n"/>
+      <c r="B3" s="101" t="n"/>
+      <c r="C3" s="100" t="n"/>
+      <c r="D3" s="102" t="n"/>
+      <c r="E3" s="103" t="n"/>
+      <c r="F3" s="103" t="n"/>
+      <c r="G3" s="103" t="n"/>
+      <c r="H3" s="103" t="n"/>
+      <c r="I3" s="103" t="n"/>
+      <c r="J3" s="100" t="n"/>
+      <c r="K3" s="100" t="n"/>
+      <c r="L3" s="104" t="inlineStr">
+        <is>
+          <t>EFX</t>
+        </is>
+      </c>
+      <c r="M3" s="104" t="inlineStr">
+        <is>
+          <t>Equifax</t>
+        </is>
+      </c>
+      <c r="N3" s="105" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="O3" s="104" t="inlineStr">
+        <is>
+          <t>VCP Scanner peer set</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="97" t="n"/>
-      <c r="B4" s="101" t="inlineStr">
+      <c r="A4" s="100" t="n"/>
+      <c r="B4" s="106" t="inlineStr">
         <is>
           <t>Assumptions</t>
         </is>
       </c>
-      <c r="C4" s="102" t="n"/>
-      <c r="D4" s="102" t="n"/>
-      <c r="E4" s="100" t="n"/>
-      <c r="F4" s="97" t="n"/>
-      <c r="G4" s="97" t="n"/>
-      <c r="H4" s="97" t="n"/>
-      <c r="I4" s="97" t="n"/>
-      <c r="J4" s="97" t="n"/>
-      <c r="K4" s="97" t="n"/>
-      <c r="L4" s="97" t="n"/>
-      <c r="M4" s="97" t="n"/>
-      <c r="N4" s="97" t="n"/>
-      <c r="O4" s="97" t="n"/>
+      <c r="C4" s="107" t="n"/>
+      <c r="D4" s="107" t="n"/>
+      <c r="E4" s="103" t="n"/>
+      <c r="F4" s="100" t="n"/>
+      <c r="G4" s="100" t="n"/>
+      <c r="H4" s="100" t="n"/>
+      <c r="I4" s="100" t="n"/>
+      <c r="J4" s="100" t="n"/>
+      <c r="K4" s="100" t="n"/>
+      <c r="L4" s="104" t="inlineStr">
+        <is>
+          <t>VRSK</t>
+        </is>
+      </c>
+      <c r="M4" s="104" t="inlineStr">
+        <is>
+          <t>Verisk Analytics</t>
+        </is>
+      </c>
+      <c r="N4" s="105" t="n">
+        <v>17.42</v>
+      </c>
+      <c r="O4" s="104" t="inlineStr">
+        <is>
+          <t>VCP Scanner peer set</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="97" t="n"/>
-      <c r="B5" s="103" t="inlineStr">
+      <c r="A5" s="100" t="n"/>
+      <c r="B5" s="108" t="inlineStr">
         <is>
           <t>Tax Rate (unlevered / on EBIT)</t>
         </is>
       </c>
-      <c r="C5" s="100" t="n"/>
-      <c r="D5" s="104" t="n">
+      <c r="C5" s="103" t="n"/>
+      <c r="D5" s="109" t="n">
         <v>0.25</v>
       </c>
-      <c r="E5" s="100" t="n"/>
-      <c r="F5" s="97" t="n"/>
-      <c r="G5" s="97" t="n"/>
-      <c r="H5" s="97" t="n"/>
-      <c r="I5" s="97" t="n"/>
-      <c r="J5" s="97" t="n"/>
-      <c r="K5" s="97" t="n"/>
-      <c r="L5" s="97" t="n"/>
-      <c r="M5" s="97" t="n"/>
-      <c r="N5" s="97" t="n"/>
-      <c r="O5" s="97" t="n"/>
+      <c r="E5" s="103" t="n"/>
+      <c r="F5" s="100" t="n"/>
+      <c r="G5" s="100" t="n"/>
+      <c r="H5" s="100" t="n"/>
+      <c r="I5" s="100" t="n"/>
+      <c r="J5" s="100" t="n"/>
+      <c r="K5" s="100" t="n"/>
+      <c r="L5" s="104" t="inlineStr">
+        <is>
+          <t>SPGI</t>
+        </is>
+      </c>
+      <c r="M5" s="104" t="inlineStr">
+        <is>
+          <t>S&amp;P Global</t>
+        </is>
+      </c>
+      <c r="N5" s="105" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="O5" s="104" t="inlineStr">
+        <is>
+          <t>VCP Scanner peer set</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="97" t="n"/>
-      <c r="B6" s="103" t="inlineStr">
+      <c r="A6" s="100" t="n"/>
+      <c r="B6" s="108" t="inlineStr">
         <is>
           <t>Discount Rate</t>
         </is>
       </c>
-      <c r="C6" s="97" t="n"/>
-      <c r="D6" s="104" t="n">
+      <c r="C6" s="100" t="n"/>
+      <c r="D6" s="109" t="n">
         <v>0.12</v>
       </c>
-      <c r="E6" s="97" t="n"/>
-      <c r="F6" s="97" t="n"/>
-      <c r="G6" s="97" t="n"/>
-      <c r="H6" s="97" t="n"/>
-      <c r="I6" s="97" t="n"/>
-      <c r="J6" s="97" t="n"/>
-      <c r="K6" s="97" t="n"/>
-      <c r="L6" s="97" t="n"/>
-      <c r="M6" s="97" t="n"/>
-      <c r="N6" s="97" t="n"/>
-      <c r="O6" s="97" t="n"/>
+      <c r="E6" s="100" t="n"/>
+      <c r="F6" s="100" t="n"/>
+      <c r="G6" s="100" t="n"/>
+      <c r="H6" s="100" t="n"/>
+      <c r="I6" s="100" t="n"/>
+      <c r="J6" s="100" t="n"/>
+      <c r="K6" s="100" t="n"/>
+      <c r="L6" s="104" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="M6" s="104" t="inlineStr">
+        <is>
+          <t>Moody's</t>
+        </is>
+      </c>
+      <c r="N6" s="105" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="O6" s="104" t="inlineStr">
+        <is>
+          <t>VCP Scanner peer set</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="97" t="n"/>
-      <c r="B7" s="97" t="inlineStr">
+      <c r="A7" s="100" t="n"/>
+      <c r="B7" s="100" t="inlineStr">
         <is>
           <t>Perpetural Growth Rate</t>
         </is>
       </c>
-      <c r="C7" s="97" t="n"/>
-      <c r="D7" s="104" t="n">
+      <c r="C7" s="100" t="n"/>
+      <c r="D7" s="109" t="n">
         <v>0.03</v>
       </c>
-      <c r="E7" s="97" t="n"/>
-      <c r="F7" s="97" t="n"/>
-      <c r="G7" s="97" t="n"/>
-      <c r="H7" s="97" t="n"/>
-      <c r="I7" s="97" t="n"/>
-      <c r="J7" s="97" t="n"/>
-      <c r="K7" s="97" t="n"/>
-      <c r="L7" s="97" t="n"/>
-      <c r="M7" s="97" t="n"/>
-      <c r="N7" s="97" t="n"/>
-      <c r="O7" s="97" t="n"/>
+      <c r="E7" s="100" t="n"/>
+      <c r="F7" s="100" t="n"/>
+      <c r="G7" s="100" t="n"/>
+      <c r="H7" s="100" t="n"/>
+      <c r="I7" s="100" t="n"/>
+      <c r="J7" s="100" t="n"/>
+      <c r="K7" s="100" t="n"/>
+      <c r="L7" s="104" t="inlineStr">
+        <is>
+          <t>MSCI</t>
+        </is>
+      </c>
+      <c r="M7" s="104" t="inlineStr">
+        <is>
+          <t>MSCI Inc.</t>
+        </is>
+      </c>
+      <c r="N7" s="105" t="n">
+        <v>23.74</v>
+      </c>
+      <c r="O7" s="104" t="inlineStr">
+        <is>
+          <t>VCP Scanner peer set</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="97" t="n"/>
-      <c r="B8" s="97" t="inlineStr">
-        <is>
-          <t>EV/EBITDA Mulltiple</t>
-        </is>
-      </c>
-      <c r="C8" s="97" t="n"/>
-      <c r="D8" s="105" t="n">
-        <v>7</v>
-      </c>
-      <c r="E8" s="97" t="n"/>
-      <c r="F8" s="97" t="n"/>
-      <c r="G8" s="97" t="n"/>
-      <c r="H8" s="97" t="n"/>
-      <c r="I8" s="97" t="n"/>
-      <c r="J8" s="97" t="n"/>
-      <c r="K8" s="97" t="n"/>
-      <c r="L8" s="97" t="n"/>
-      <c r="M8" s="97" t="n"/>
-      <c r="N8" s="97" t="n"/>
-      <c r="O8" s="97" t="n"/>
+      <c r="A8" s="100" t="n"/>
+      <c r="B8" s="100" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA (BASE 17.5x — peer comps)</t>
+        </is>
+      </c>
+      <c r="C8" s="110" t="inlineStr">
+        <is>
+          <t>BASE 17.5x ≈ peer median 18.1x (VCP Scanner). Bull 25x / Bear 12.8x.</t>
+        </is>
+      </c>
+      <c r="D8" s="111" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E8" s="100" t="n"/>
+      <c r="F8" s="112" t="inlineStr">
+        <is>
+          <t>Peer EV/EBITDA comps (click)</t>
+        </is>
+      </c>
+      <c r="G8" s="112" t="inlineStr">
+        <is>
+          <t>FICO spot EV/EBITDA (click)</t>
+        </is>
+      </c>
+      <c r="H8" s="100" t="n"/>
+      <c r="I8" s="100" t="n"/>
+      <c r="J8" s="100" t="n"/>
+      <c r="K8" s="100" t="n"/>
+      <c r="L8" s="113" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="M8" s="113" t="inlineStr">
+        <is>
+          <t>Peer set</t>
+        </is>
+      </c>
+      <c r="N8" s="114" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="O8" s="113" t="inlineStr">
+        <is>
+          <t>Sorted median (SPGI)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="97" t="n"/>
-      <c r="B9" s="97" t="inlineStr">
+      <c r="A9" s="100" t="n"/>
+      <c r="B9" s="100" t="inlineStr">
         <is>
           <t>Transaction Date</t>
         </is>
       </c>
-      <c r="C9" s="97" t="n"/>
-      <c r="D9" s="106" t="n">
+      <c r="C9" s="100" t="n"/>
+      <c r="D9" s="115" t="n">
         <v>43100</v>
       </c>
-      <c r="E9" s="97" t="n"/>
-      <c r="F9" s="97" t="n"/>
-      <c r="G9" s="97" t="n"/>
-      <c r="H9" s="97" t="n"/>
-      <c r="I9" s="97" t="n"/>
-      <c r="J9" s="97" t="n"/>
-      <c r="K9" s="97" t="n"/>
-      <c r="L9" s="97" t="n"/>
-      <c r="M9" s="97" t="n"/>
-      <c r="N9" s="97" t="n"/>
-      <c r="O9" s="97" t="n"/>
+      <c r="E9" s="100" t="n"/>
+      <c r="F9" s="100" t="n"/>
+      <c r="G9" s="100" t="n"/>
+      <c r="H9" s="100" t="n"/>
+      <c r="I9" s="100" t="n"/>
+      <c r="J9" s="100" t="n"/>
+      <c r="K9" s="100" t="n"/>
+      <c r="L9" s="116" t="inlineStr">
+        <is>
+          <t>Base exit (D8)</t>
+        </is>
+      </c>
+      <c r="M9" s="116" t="n"/>
+      <c r="N9" s="117" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="O9" s="116" t="inlineStr">
+        <is>
+          <t>Near peer median; audit 17.5x</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="97" t="n"/>
-      <c r="B10" s="97" t="inlineStr">
+      <c r="A10" s="100" t="n"/>
+      <c r="B10" s="100" t="inlineStr">
         <is>
           <t>Fiscal Year End</t>
         </is>
       </c>
-      <c r="C10" s="97" t="n"/>
-      <c r="D10" s="106" t="n">
+      <c r="C10" s="100" t="n"/>
+      <c r="D10" s="115" t="n">
         <v>43281</v>
       </c>
-      <c r="E10" s="97" t="n"/>
-      <c r="F10" s="97" t="n"/>
-      <c r="G10" s="97" t="n"/>
-      <c r="H10" s="97" t="n"/>
-      <c r="I10" s="97" t="n"/>
-      <c r="J10" s="97" t="n"/>
-      <c r="K10" s="97" t="n"/>
-      <c r="L10" s="97" t="n"/>
-      <c r="M10" s="97" t="n"/>
-      <c r="N10" s="97" t="n"/>
-      <c r="O10" s="97" t="n"/>
+      <c r="E10" s="100" t="n"/>
+      <c r="F10" s="100" t="n"/>
+      <c r="G10" s="100" t="n"/>
+      <c r="H10" s="100" t="n"/>
+      <c r="I10" s="100" t="n"/>
+      <c r="J10" s="100" t="n"/>
+      <c r="K10" s="100" t="n"/>
+      <c r="L10" s="112" t="inlineStr">
+        <is>
+          <t>Peer comps (click)</t>
+        </is>
+      </c>
+      <c r="M10" s="112" t="inlineStr">
+        <is>
+          <t>FICO spot EV/EBITDA (click)</t>
+        </is>
+      </c>
+      <c r="N10" s="100" t="n"/>
+      <c r="O10" s="100" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="97" t="n"/>
-      <c r="B11" s="97" t="inlineStr">
+      <c r="A11" s="100" t="n"/>
+      <c r="B11" s="100" t="inlineStr">
         <is>
           <t>Current Price</t>
         </is>
       </c>
-      <c r="C11" s="97" t="n"/>
-      <c r="D11" s="107" t="n">
+      <c r="C11" s="100" t="n"/>
+      <c r="D11" s="118" t="n">
         <v>25</v>
       </c>
-      <c r="E11" s="97" t="n"/>
-      <c r="F11" s="97" t="n"/>
-      <c r="G11" s="97" t="n"/>
-      <c r="H11" s="97" t="n"/>
-      <c r="I11" s="97" t="n"/>
-      <c r="J11" s="97" t="n"/>
-      <c r="K11" s="97" t="n"/>
-      <c r="L11" s="97" t="n"/>
-      <c r="M11" s="97" t="n"/>
-      <c r="N11" s="97" t="n"/>
-      <c r="O11" s="97" t="n"/>
+      <c r="E11" s="100" t="n"/>
+      <c r="F11" s="100" t="n"/>
+      <c r="G11" s="100" t="n"/>
+      <c r="H11" s="100" t="n"/>
+      <c r="I11" s="100" t="n"/>
+      <c r="J11" s="100" t="n"/>
+      <c r="K11" s="100" t="n"/>
+      <c r="L11" s="100" t="n"/>
+      <c r="M11" s="100" t="n"/>
+      <c r="N11" s="100" t="n"/>
+      <c r="O11" s="100" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="97" t="n"/>
-      <c r="B12" s="97" t="inlineStr">
+      <c r="A12" s="100" t="n"/>
+      <c r="B12" s="100" t="inlineStr">
         <is>
           <t>Shares Outstanding</t>
         </is>
       </c>
-      <c r="C12" s="97" t="n"/>
-      <c r="D12" s="108" t="n">
+      <c r="C12" s="100" t="n"/>
+      <c r="D12" s="119" t="n">
         <v>20000</v>
       </c>
-      <c r="E12" s="97" t="n"/>
-      <c r="F12" s="97" t="n"/>
-      <c r="G12" s="97" t="n"/>
-      <c r="H12" s="97" t="n"/>
-      <c r="I12" s="97" t="n"/>
-      <c r="J12" s="97" t="n"/>
-      <c r="K12" s="97" t="n"/>
-      <c r="L12" s="97" t="n"/>
-      <c r="M12" s="97" t="n"/>
-      <c r="N12" s="97" t="n"/>
-      <c r="O12" s="97" t="n"/>
+      <c r="E12" s="100" t="n"/>
+      <c r="F12" s="100" t="n"/>
+      <c r="G12" s="100" t="n"/>
+      <c r="H12" s="100" t="n"/>
+      <c r="I12" s="100" t="n"/>
+      <c r="J12" s="100" t="n"/>
+      <c r="K12" s="100" t="n"/>
+      <c r="L12" s="100" t="n"/>
+      <c r="M12" s="100" t="n"/>
+      <c r="N12" s="100" t="n"/>
+      <c r="O12" s="100" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="97" t="n"/>
-      <c r="B13" s="97" t="inlineStr">
+      <c r="A13" s="100" t="n"/>
+      <c r="B13" s="100" t="inlineStr">
         <is>
           <t>Debt</t>
         </is>
       </c>
-      <c r="C13" s="97" t="n"/>
-      <c r="D13" s="108" t="n">
+      <c r="C13" s="100" t="n"/>
+      <c r="D13" s="119" t="n">
         <v>30000</v>
       </c>
-      <c r="E13" s="97" t="n"/>
-      <c r="F13" s="97" t="n"/>
-      <c r="G13" s="97" t="n"/>
-      <c r="H13" s="97" t="n"/>
-      <c r="I13" s="97" t="n"/>
-      <c r="J13" s="97" t="n"/>
-      <c r="K13" s="97" t="n"/>
-      <c r="L13" s="97" t="n"/>
-      <c r="M13" s="97" t="n"/>
-      <c r="N13" s="97" t="n"/>
-      <c r="O13" s="97" t="n"/>
+      <c r="E13" s="100" t="n"/>
+      <c r="F13" s="100" t="n"/>
+      <c r="G13" s="100" t="n"/>
+      <c r="H13" s="100" t="n"/>
+      <c r="I13" s="100" t="n"/>
+      <c r="J13" s="100" t="n"/>
+      <c r="K13" s="100" t="n"/>
+      <c r="L13" s="100" t="n"/>
+      <c r="M13" s="100" t="n"/>
+      <c r="N13" s="100" t="n"/>
+      <c r="O13" s="100" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="97" t="n"/>
-      <c r="B14" s="97" t="inlineStr">
+      <c r="A14" s="100" t="n"/>
+      <c r="B14" s="100" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="C14" s="97" t="n"/>
-      <c r="D14" s="108" t="n">
+      <c r="C14" s="100" t="n"/>
+      <c r="D14" s="119" t="n">
         <v>239549.5203651849</v>
       </c>
-      <c r="E14" s="97" t="n"/>
-      <c r="F14" s="97" t="n"/>
-      <c r="G14" s="97" t="n"/>
-      <c r="H14" s="97" t="n"/>
-      <c r="I14" s="97" t="n"/>
-      <c r="J14" s="97" t="n"/>
-      <c r="K14" s="97" t="n"/>
-      <c r="L14" s="97" t="n"/>
-      <c r="M14" s="97" t="n"/>
-      <c r="N14" s="97" t="n"/>
-      <c r="O14" s="97" t="n"/>
+      <c r="E14" s="100" t="n"/>
+      <c r="F14" s="100" t="n"/>
+      <c r="G14" s="100" t="n"/>
+      <c r="H14" s="100" t="n"/>
+      <c r="I14" s="100" t="n"/>
+      <c r="J14" s="100" t="n"/>
+      <c r="K14" s="100" t="n"/>
+      <c r="L14" s="100" t="n"/>
+      <c r="M14" s="100" t="n"/>
+      <c r="N14" s="100" t="n"/>
+      <c r="O14" s="100" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="97" t="n"/>
-      <c r="B15" s="97" t="inlineStr">
+      <c r="A15" s="100" t="n"/>
+      <c r="B15" s="100" t="inlineStr">
         <is>
           <t>Capex (FY1 forecast, linked)</t>
         </is>
       </c>
-      <c r="C15" s="97" t="n"/>
-      <c r="D15" s="109">
+      <c r="C15" s="100" t="n"/>
+      <c r="D15" s="120">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="E15" s="97" t="n"/>
-      <c r="F15" s="97" t="n"/>
-      <c r="G15" s="97" t="n"/>
-      <c r="H15" s="97" t="n"/>
-      <c r="I15" s="97" t="n"/>
-      <c r="J15" s="97" t="n"/>
-      <c r="K15" s="97" t="n"/>
-      <c r="L15" s="97" t="n"/>
-      <c r="M15" s="97" t="n"/>
-      <c r="N15" s="97" t="n"/>
-      <c r="O15" s="97" t="n"/>
+      <c r="E15" s="100" t="n"/>
+      <c r="F15" s="100" t="n"/>
+      <c r="G15" s="100" t="n"/>
+      <c r="H15" s="100" t="n"/>
+      <c r="I15" s="100" t="n"/>
+      <c r="J15" s="100" t="n"/>
+      <c r="K15" s="100" t="n"/>
+      <c r="L15" s="100" t="n"/>
+      <c r="M15" s="100" t="n"/>
+      <c r="N15" s="100" t="n"/>
+      <c r="O15" s="100" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="97" t="n"/>
-      <c r="B16" s="97" t="n"/>
-      <c r="C16" s="97" t="n"/>
-      <c r="D16" s="106" t="n"/>
-      <c r="J16" s="97" t="n"/>
-      <c r="K16" s="97" t="n"/>
-      <c r="L16" s="97" t="n"/>
-      <c r="M16" s="97" t="n"/>
-      <c r="N16" s="97" t="n"/>
-      <c r="O16" s="97" t="n"/>
+      <c r="A16" s="100" t="n"/>
+      <c r="B16" s="100" t="n"/>
+      <c r="C16" s="100" t="n"/>
+      <c r="D16" s="115" t="n"/>
+      <c r="J16" s="100" t="n"/>
+      <c r="K16" s="100" t="n"/>
+      <c r="L16" s="100" t="n"/>
+      <c r="M16" s="100" t="n"/>
+      <c r="N16" s="100" t="n"/>
+      <c r="O16" s="100" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="97" t="n"/>
-      <c r="B17" s="110" t="inlineStr">
+      <c r="A17" s="100" t="n"/>
+      <c r="B17" s="121" t="inlineStr">
         <is>
           <t>Discounted Cash Flow</t>
         </is>
       </c>
-      <c r="C17" s="111" t="n"/>
-      <c r="D17" s="112" t="inlineStr">
+      <c r="C17" s="122" t="n"/>
+      <c r="D17" s="123" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="E17" s="113">
+      <c r="E17" s="124">
         <f>YEAR(E18)</f>
         <v/>
       </c>
-      <c r="F17" s="113">
+      <c r="F17" s="124">
         <f>YEAR(F18)</f>
         <v/>
       </c>
-      <c r="G17" s="113">
+      <c r="G17" s="124">
         <f>YEAR(G18)</f>
         <v/>
       </c>
-      <c r="H17" s="113">
+      <c r="H17" s="124">
         <f>YEAR(H18)</f>
         <v/>
       </c>
-      <c r="I17" s="113">
+      <c r="I17" s="124">
         <f>YEAR(I18)</f>
         <v/>
       </c>
-      <c r="J17" s="112" t="inlineStr">
+      <c r="J17" s="123" t="inlineStr">
         <is>
           <t>Exit</t>
         </is>
       </c>
-      <c r="K17" s="97" t="n"/>
-      <c r="L17" s="114" t="inlineStr">
-        <is>
-          <t>Terminal value methods (MODEL7)</t>
-        </is>
-      </c>
-      <c r="M17" s="111" t="n"/>
-      <c r="N17" s="111" t="n"/>
-      <c r="O17" s="97" t="n"/>
+      <c r="K17" s="100" t="n"/>
+      <c r="L17" s="125" t="inlineStr">
+        <is>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL8)</t>
+        </is>
+      </c>
+      <c r="O17" s="100" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="97" t="n"/>
-      <c r="B18" s="97" t="inlineStr">
-        <is>
-          <t>Date (mid-year via EDATE from transaction)</t>
-        </is>
-      </c>
-      <c r="C18" s="97" t="n"/>
-      <c r="D18" s="115">
-        <f>D9</f>
-        <v/>
-      </c>
-      <c r="E18" s="116">
-        <f>EDATE($D$9,(E19-0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="F18" s="116">
-        <f>EDATE($D$9,(F19-0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="G18" s="116">
-        <f>EDATE($D$9,(G19-0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="H18" s="116">
-        <f>EDATE($D$9,(H19-0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="I18" s="116">
-        <f>EDATE($D$9,(I19-0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="J18" s="116">
+      <c r="A18" s="100" t="n"/>
+      <c r="B18" s="100" t="inlineStr">
+        <is>
+          <t>Date (mid-year via EDATE; periods are 0-based)</t>
+        </is>
+      </c>
+      <c r="C18" s="100" t="n"/>
+      <c r="D18" s="126">
+        <f>$D$9</f>
+        <v/>
+      </c>
+      <c r="E18" s="126">
+        <f>EDATE($D$9,(E19+0.5)*12)</f>
+        <v/>
+      </c>
+      <c r="F18" s="126">
+        <f>EDATE($D$9,(F19+0.5)*12)</f>
+        <v/>
+      </c>
+      <c r="G18" s="126">
+        <f>EDATE($D$9,(G19+0.5)*12)</f>
+        <v/>
+      </c>
+      <c r="H18" s="126">
+        <f>EDATE($D$9,(H19+0.5)*12)</f>
+        <v/>
+      </c>
+      <c r="I18" s="126">
+        <f>EDATE($D$9,(I19+0.5)*12)</f>
+        <v/>
+      </c>
+      <c r="J18" s="126">
         <f>I18</f>
         <v/>
       </c>
-      <c r="K18" s="97" t="n"/>
-      <c r="L18" s="97" t="inlineStr">
-        <is>
-          <t>Exit EV/EBITDA @ D8 (primary 16x)</t>
-        </is>
-      </c>
-      <c r="M18" s="109">
+      <c r="K18" s="100" t="n"/>
+      <c r="L18" s="100" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA @ D8 (BASE 17.5x)</t>
+        </is>
+      </c>
+      <c r="M18" s="120">
         <f>J27</f>
         <v/>
       </c>
-      <c r="N18" s="97" t="inlineStr">
+      <c r="N18" s="100" t="inlineStr">
         <is>
           <t>← used in XNPV</t>
         </is>
       </c>
-      <c r="O18" s="97" t="n"/>
+      <c r="O18" s="100" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="97" t="n"/>
-      <c r="B19" s="117" t="inlineStr">
+      <c r="A19" s="100" t="n"/>
+      <c r="B19" s="127" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="117" t="n"/>
-      <c r="D19" s="115" t="n"/>
-      <c r="E19" s="118" t="n">
+      <c r="C19" s="127" t="n"/>
+      <c r="D19" s="128" t="n"/>
+      <c r="E19" s="129" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="119">
+      <c r="F19" s="130">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="119">
+      <c r="G19" s="130">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="119">
+      <c r="H19" s="130">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="119">
+      <c r="I19" s="130">
         <f>H19+1</f>
         <v/>
       </c>
-      <c r="J19" s="115" t="n"/>
-      <c r="K19" s="97" t="n"/>
-      <c r="L19" s="97" t="inlineStr">
-        <is>
-          <t>Gordon cross-check</t>
-        </is>
-      </c>
-      <c r="M19" s="109">
+      <c r="J19" s="128" t="n"/>
+      <c r="K19" s="100" t="n"/>
+      <c r="L19" s="100" t="inlineStr">
+        <is>
+          <t>Gordon cross-check (g=D7)</t>
+        </is>
+      </c>
+      <c r="M19" s="120">
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="120" t="inlineStr">
+      <c r="N19" s="131" t="inlineStr">
         <is>
           <t>← sanity check</t>
         </is>
       </c>
-      <c r="O19" s="97" t="n"/>
+      <c r="O19" s="100" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="97" t="n"/>
-      <c r="B20" s="117" t="inlineStr">
+      <c r="A20" s="100" t="n"/>
+      <c r="B20" s="127" t="inlineStr">
         <is>
           <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
-      <c r="C20" s="97" t="n"/>
-      <c r="D20" s="97" t="n"/>
-      <c r="E20" s="121">
+      <c r="C20" s="100" t="n"/>
+      <c r="D20" s="100" t="n"/>
+      <c r="E20" s="132">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="121">
+      <c r="F20" s="132">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="121">
+      <c r="G20" s="132">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="121">
+      <c r="H20" s="132">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="121">
+      <c r="I20" s="132">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
-      <c r="J20" s="97" t="n"/>
-      <c r="K20" s="97" t="n"/>
-      <c r="L20" s="97" t="inlineStr">
+      <c r="J20" s="100" t="n"/>
+      <c r="K20" s="100" t="n"/>
+      <c r="L20" s="100" t="inlineStr">
         <is>
           <t>Implied Gordon exit multiple</t>
         </is>
       </c>
-      <c r="M20" s="109">
+      <c r="M20" s="120">
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="122">
-        <f>AVERAGE(N18:N19)</f>
-        <v/>
-      </c>
-      <c r="O20" s="97" t="n"/>
+      <c r="N20" s="133" t="inlineStr">
+        <is>
+          <t>← ~bear check</t>
+        </is>
+      </c>
+      <c r="O20" s="100" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="97" t="n"/>
-      <c r="B21" s="97" t="inlineStr">
+      <c r="A21" s="100" t="n"/>
+      <c r="B21" s="100" t="inlineStr">
         <is>
           <t>EBIT (linked to 3-stmt)</t>
         </is>
       </c>
-      <c r="C21" s="97" t="n"/>
-      <c r="D21" s="97" t="n"/>
-      <c r="E21" s="109">
+      <c r="C21" s="100" t="n"/>
+      <c r="D21" s="100" t="n"/>
+      <c r="E21" s="120">
         <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F21" s="109">
+      <c r="F21" s="120">
         <f>'3 Statement Model'!K26-'3 Statement Model'!K28-'3 Statement Model'!K29-'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G21" s="109">
+      <c r="G21" s="120">
         <f>'3 Statement Model'!L26-'3 Statement Model'!L28-'3 Statement Model'!L29-'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H21" s="109">
+      <c r="H21" s="120">
         <f>'3 Statement Model'!M26-'3 Statement Model'!M28-'3 Statement Model'!M29-'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I21" s="109">
+      <c r="I21" s="120">
         <f>'3 Statement Model'!N26-'3 Statement Model'!N28-'3 Statement Model'!N29-'3 Statement Model'!N30</f>
         <v/>
       </c>
-      <c r="J21" s="97" t="n"/>
-      <c r="K21" s="97" t="n"/>
-      <c r="L21" s="97" t="inlineStr">
-        <is>
-          <t>Bull case TV @ 25x (sensitivity only)</t>
-        </is>
-      </c>
-      <c r="M21" s="109">
+      <c r="J21" s="100" t="n"/>
+      <c r="K21" s="100" t="n"/>
+      <c r="L21" s="100" t="inlineStr">
+        <is>
+          <t>BASE TV @ 17.5x (primary)</t>
+        </is>
+      </c>
+      <c r="M21" s="120">
+        <f>($I$21+$I$23)*17.5</f>
+        <v/>
+      </c>
+      <c r="N21" s="100" t="inlineStr">
+        <is>
+          <t>← = D8 policy</t>
+        </is>
+      </c>
+      <c r="O21" s="100" t="n"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="100" t="n"/>
+      <c r="B22" s="100" t="inlineStr">
+        <is>
+          <t>Less: Unlevered Cash Taxes (EBIT×t)</t>
+        </is>
+      </c>
+      <c r="C22" s="100" t="n"/>
+      <c r="D22" s="100" t="n"/>
+      <c r="E22" s="134">
+        <f>E21*$D$5</f>
+        <v/>
+      </c>
+      <c r="F22" s="134">
+        <f>F21*$D$5</f>
+        <v/>
+      </c>
+      <c r="G22" s="134">
+        <f>G21*$D$5</f>
+        <v/>
+      </c>
+      <c r="H22" s="134">
+        <f>H21*$D$5</f>
+        <v/>
+      </c>
+      <c r="I22" s="134">
+        <f>I21*$D$5</f>
+        <v/>
+      </c>
+      <c r="J22" s="100" t="n"/>
+      <c r="K22" s="100" t="n"/>
+      <c r="L22" s="100" t="inlineStr">
+        <is>
+          <t>BULL TV @ 25.0x (spot/policy)</t>
+        </is>
+      </c>
+      <c r="M22" s="120">
         <f>($I$21+$I$23)*25.0</f>
         <v/>
       </c>
-      <c r="N21" s="97" t="inlineStr">
-        <is>
-          <t>← not in base case</t>
-        </is>
-      </c>
-      <c r="O21" s="97" t="n"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="97" t="n"/>
-      <c r="B22" s="97" t="inlineStr">
-        <is>
-          <t>Less: Unlevered Cash Taxes (EBIT×t)</t>
-        </is>
-      </c>
-      <c r="C22" s="97" t="n"/>
-      <c r="D22" s="97" t="n"/>
-      <c r="E22" s="123">
-        <f>E21*$D$5</f>
-        <v/>
-      </c>
-      <c r="F22" s="123">
-        <f>F21*$D$5</f>
-        <v/>
-      </c>
-      <c r="G22" s="123">
-        <f>G21*$D$5</f>
-        <v/>
-      </c>
-      <c r="H22" s="123">
-        <f>H21*$D$5</f>
-        <v/>
-      </c>
-      <c r="I22" s="123">
-        <f>I21*$D$5</f>
-        <v/>
-      </c>
-      <c r="J22" s="97" t="n"/>
-      <c r="K22" s="97" t="n"/>
-      <c r="L22" s="97" t="n"/>
-      <c r="M22" s="97" t="n"/>
-      <c r="N22" s="97" t="n"/>
-      <c r="O22" s="97" t="n"/>
+      <c r="N22" s="100" t="inlineStr">
+        <is>
+          <t>← sensitivity only</t>
+        </is>
+      </c>
+      <c r="O22" s="100" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="97" t="n"/>
-      <c r="B23" s="97" t="inlineStr">
+      <c r="A23" s="100" t="n"/>
+      <c r="B23" s="100" t="inlineStr">
         <is>
           <t>Plus: D&amp;A (linked to 3-stmt)</t>
         </is>
       </c>
-      <c r="C23" s="97" t="n"/>
-      <c r="D23" s="97" t="n"/>
-      <c r="E23" s="123">
+      <c r="C23" s="100" t="n"/>
+      <c r="D23" s="100" t="n"/>
+      <c r="E23" s="134">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="123">
+      <c r="F23" s="134">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="123">
+      <c r="G23" s="134">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="123">
+      <c r="H23" s="134">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="123">
+      <c r="I23" s="134">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
-      <c r="J23" s="97" t="n"/>
-      <c r="K23" s="97" t="n"/>
-      <c r="L23" s="97" t="n"/>
-      <c r="M23" s="97" t="n"/>
-      <c r="N23" s="97" t="n"/>
-      <c r="O23" s="97" t="n"/>
+      <c r="J23" s="100" t="n"/>
+      <c r="K23" s="100" t="n"/>
+      <c r="L23" s="100" t="inlineStr">
+        <is>
+          <t>BEAR TV @ 12.8x (Gordon-implied)</t>
+        </is>
+      </c>
+      <c r="M23" s="120">
+        <f>($I$21+$I$23)*12.8</f>
+        <v/>
+      </c>
+      <c r="N23" s="100" t="inlineStr">
+        <is>
+          <t>← sensitivity only</t>
+        </is>
+      </c>
+      <c r="O23" s="100" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="97" t="n"/>
-      <c r="B24" s="97" t="inlineStr">
+      <c r="A24" s="100" t="n"/>
+      <c r="B24" s="100" t="inlineStr">
         <is>
           <t>Less: Capex (linked to 3-stmt CF)</t>
         </is>
       </c>
-      <c r="C24" s="97" t="n"/>
-      <c r="D24" s="97" t="n"/>
-      <c r="E24" s="109">
+      <c r="C24" s="100" t="n"/>
+      <c r="D24" s="100" t="n"/>
+      <c r="E24" s="120">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="F24" s="109">
+      <c r="F24" s="120">
         <f>'3 Statement Model'!K68</f>
         <v/>
       </c>
-      <c r="G24" s="109">
+      <c r="G24" s="120">
         <f>'3 Statement Model'!L68</f>
         <v/>
       </c>
-      <c r="H24" s="109">
+      <c r="H24" s="120">
         <f>'3 Statement Model'!M68</f>
         <v/>
       </c>
-      <c r="I24" s="109">
+      <c r="I24" s="120">
         <f>'3 Statement Model'!N68</f>
         <v/>
       </c>
-      <c r="J24" s="97" t="n"/>
-      <c r="K24" s="97" t="n"/>
-      <c r="L24" s="97" t="n"/>
-      <c r="M24" s="97" t="n"/>
-      <c r="N24" s="97" t="n"/>
-      <c r="O24" s="97" t="n"/>
+      <c r="J24" s="100" t="n"/>
+      <c r="K24" s="100" t="n"/>
+      <c r="L24" s="110" t="inlineStr">
+        <is>
+          <t>Reconciliation: Bull 25x → Base 17.5x (peer median ~18.1x) → Bear 12.8x</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="97" t="n"/>
-      <c r="B25" s="97" t="inlineStr">
+      <c r="A25" s="100" t="n"/>
+      <c r="B25" s="100" t="inlineStr">
         <is>
           <t>Less: ΔNWC (linked to 3-stmt CF)</t>
         </is>
       </c>
-      <c r="C25" s="97" t="n"/>
-      <c r="D25" s="97" t="n"/>
-      <c r="E25" s="109">
+      <c r="C25" s="100" t="n"/>
+      <c r="D25" s="100" t="n"/>
+      <c r="E25" s="120">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="F25" s="109">
+      <c r="F25" s="120">
         <f>'3 Statement Model'!K64</f>
         <v/>
       </c>
-      <c r="G25" s="109">
+      <c r="G25" s="120">
         <f>'3 Statement Model'!L64</f>
         <v/>
       </c>
-      <c r="H25" s="109">
+      <c r="H25" s="120">
         <f>'3 Statement Model'!M64</f>
         <v/>
       </c>
-      <c r="I25" s="109">
+      <c r="I25" s="120">
         <f>'3 Statement Model'!N64</f>
         <v/>
       </c>
-      <c r="J25" s="97" t="n"/>
-      <c r="K25" s="97" t="n"/>
-      <c r="L25" s="97" t="n"/>
-      <c r="M25" s="97" t="n"/>
-      <c r="N25" s="97" t="n"/>
-      <c r="O25" s="97" t="n"/>
+      <c r="J25" s="100" t="n"/>
+      <c r="K25" s="100" t="n"/>
+      <c r="L25" s="100" t="n"/>
+      <c r="M25" s="100" t="n"/>
+      <c r="N25" s="100" t="n"/>
+      <c r="O25" s="100" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="97" t="n"/>
-      <c r="B26" s="97" t="inlineStr">
+      <c r="A26" s="100" t="n"/>
+      <c r="B26" s="100" t="inlineStr">
         <is>
           <t>Unlevered FCF</t>
         </is>
       </c>
-      <c r="C26" s="97" t="n"/>
-      <c r="D26" s="97" t="n"/>
-      <c r="E26" s="122">
+      <c r="C26" s="100" t="n"/>
+      <c r="D26" s="100" t="n"/>
+      <c r="E26" s="133">
         <f>E21-E22+E23-E24-E25</f>
         <v/>
       </c>
-      <c r="F26" s="122">
+      <c r="F26" s="133">
         <f>F21-F22+F23-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="122">
+      <c r="G26" s="133">
         <f>G21-G22+G23-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="122">
+      <c r="H26" s="133">
         <f>H21-H22+H23-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="122">
+      <c r="I26" s="133">
         <f>I21-I22+I23-I24-I25</f>
         <v/>
       </c>
-      <c r="J26" s="97" t="n"/>
-      <c r="K26" s="97" t="n"/>
-      <c r="L26" s="97" t="n"/>
-      <c r="M26" s="97" t="n"/>
-      <c r="N26" s="97" t="n"/>
-      <c r="O26" s="97" t="n"/>
+      <c r="J26" s="100" t="n"/>
+      <c r="K26" s="100" t="n"/>
+      <c r="L26" s="100" t="n"/>
+      <c r="M26" s="100" t="n"/>
+      <c r="N26" s="100" t="n"/>
+      <c r="O26" s="100" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="97" t="n"/>
-      <c r="B27" s="97" t="inlineStr">
-        <is>
-          <t>(Entry)/Exit TV — Exit EV/EBITDA (primary 16x)</t>
-        </is>
-      </c>
-      <c r="C27" s="97" t="n"/>
-      <c r="D27" s="97">
+      <c r="A27" s="100" t="n"/>
+      <c r="B27" s="100" t="inlineStr">
+        <is>
+          <t>(Entry)/Exit TV — Exit EV/EBITDA (BASE 17.5x)</t>
+        </is>
+      </c>
+      <c r="C27" s="100" t="n"/>
+      <c r="D27" s="100">
         <f>-I35</f>
         <v/>
       </c>
-      <c r="E27" s="97" t="n"/>
-      <c r="F27" s="97" t="n"/>
-      <c r="G27" s="97" t="n"/>
-      <c r="H27" s="97" t="n"/>
-      <c r="I27" s="97" t="n"/>
-      <c r="J27" s="109">
+      <c r="E27" s="100" t="n"/>
+      <c r="F27" s="100" t="n"/>
+      <c r="G27" s="100" t="n"/>
+      <c r="H27" s="100" t="n"/>
+      <c r="I27" s="100" t="n"/>
+      <c r="J27" s="120">
         <f>($I$21+$I$23)*$D$8</f>
         <v/>
       </c>
-      <c r="K27" s="97" t="n"/>
-      <c r="L27" s="97" t="n"/>
-      <c r="M27" s="97" t="n"/>
-      <c r="N27" s="97" t="n"/>
-      <c r="O27" s="97" t="n"/>
+      <c r="K27" s="100" t="n"/>
+      <c r="L27" s="100" t="n"/>
+      <c r="M27" s="100" t="n"/>
+      <c r="N27" s="100" t="n"/>
+      <c r="O27" s="100" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="97" t="n"/>
-      <c r="B28" s="97" t="inlineStr">
+      <c r="A28" s="100" t="n"/>
+      <c r="B28" s="100" t="inlineStr">
         <is>
           <t>Transaction CF</t>
         </is>
       </c>
-      <c r="C28" s="97" t="n"/>
-      <c r="D28" s="122" t="n">
+      <c r="C28" s="100" t="n"/>
+      <c r="D28" s="133" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="124">
+      <c r="E28" s="135">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="124">
+      <c r="F28" s="135">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="124">
+      <c r="G28" s="135">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="124">
+      <c r="H28" s="135">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="124">
+      <c r="I28" s="135">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="124">
+      <c r="J28" s="135">
         <f>J27+J26</f>
         <v/>
       </c>
-      <c r="K28" s="97" t="n"/>
-      <c r="L28" s="97" t="n"/>
-      <c r="M28" s="97" t="n"/>
-      <c r="N28" s="97" t="n"/>
-      <c r="O28" s="97" t="n"/>
+      <c r="K28" s="100" t="n"/>
+      <c r="L28" s="100" t="n"/>
+      <c r="M28" s="100" t="n"/>
+      <c r="N28" s="100" t="n"/>
+      <c r="O28" s="100" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="97" t="n"/>
-      <c r="B29" s="97" t="inlineStr">
+      <c r="A29" s="100" t="n"/>
+      <c r="B29" s="100" t="inlineStr">
         <is>
           <t>Transaction CF</t>
         </is>
       </c>
-      <c r="C29" s="97" t="n"/>
-      <c r="D29" s="97">
+      <c r="C29" s="100" t="n"/>
+      <c r="D29" s="100">
         <f>D27+D26</f>
         <v/>
       </c>
-      <c r="E29" s="109">
+      <c r="E29" s="120">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F29" s="109">
+      <c r="F29" s="120">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G29" s="109">
+      <c r="G29" s="120">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H29" s="109">
+      <c r="H29" s="120">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I29" s="109">
+      <c r="I29" s="120">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J29" s="109">
+      <c r="J29" s="120">
         <f>J27</f>
         <v/>
       </c>
-      <c r="K29" s="97" t="n"/>
-      <c r="L29" s="97" t="n"/>
-      <c r="M29" s="97" t="n"/>
-      <c r="N29" s="97" t="n"/>
-      <c r="O29" s="97" t="n"/>
+      <c r="K29" s="100" t="n"/>
+      <c r="L29" s="100" t="n"/>
+      <c r="M29" s="100" t="n"/>
+      <c r="N29" s="100" t="n"/>
+      <c r="O29" s="100" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="97" t="n"/>
-      <c r="B30" s="97" t="n"/>
-      <c r="C30" s="97" t="n"/>
-      <c r="D30" s="99" t="n"/>
-      <c r="E30" s="97" t="n"/>
-      <c r="G30" s="97" t="n"/>
-      <c r="H30" s="97" t="n"/>
-      <c r="I30" s="97" t="n"/>
-      <c r="J30" s="97" t="n"/>
-      <c r="L30" s="97" t="n"/>
-      <c r="M30" s="97" t="n"/>
-      <c r="N30" s="97" t="n"/>
-      <c r="O30" s="97" t="n"/>
+      <c r="A30" s="100" t="n"/>
+      <c r="B30" s="100" t="n"/>
+      <c r="C30" s="100" t="n"/>
+      <c r="D30" s="102" t="n"/>
+      <c r="E30" s="100" t="n"/>
+      <c r="G30" s="100" t="n"/>
+      <c r="H30" s="100" t="n"/>
+      <c r="I30" s="100" t="n"/>
+      <c r="J30" s="100" t="n"/>
+      <c r="L30" s="100" t="n"/>
+      <c r="M30" s="100" t="n"/>
+      <c r="N30" s="100" t="n"/>
+      <c r="O30" s="100" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="97" t="n"/>
-      <c r="B31" s="110" t="inlineStr">
+      <c r="A31" s="100" t="n"/>
+      <c r="B31" s="121" t="inlineStr">
         <is>
           <t>Intrinsic Value</t>
         </is>
       </c>
-      <c r="C31" s="111" t="n"/>
-      <c r="D31" s="111" t="n"/>
-      <c r="E31" s="97" t="n"/>
-      <c r="G31" s="110" t="inlineStr">
+      <c r="C31" s="122" t="n"/>
+      <c r="D31" s="122" t="n"/>
+      <c r="E31" s="100" t="n"/>
+      <c r="G31" s="121" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="H31" s="111" t="n"/>
-      <c r="I31" s="111" t="n"/>
-      <c r="J31" s="97" t="n"/>
-      <c r="L31" s="110" t="inlineStr">
+      <c r="H31" s="122" t="n"/>
+      <c r="I31" s="122" t="n"/>
+      <c r="J31" s="100" t="n"/>
+      <c r="L31" s="121" t="inlineStr">
         <is>
           <t>Rate of Return</t>
         </is>
       </c>
-      <c r="M31" s="111" t="n"/>
-      <c r="N31" s="111" t="n"/>
-      <c r="O31" s="97" t="n"/>
+      <c r="M31" s="122" t="n"/>
+      <c r="N31" s="122" t="n"/>
+      <c r="O31" s="100" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="97" t="n"/>
-      <c r="B32" s="97" t="inlineStr">
+      <c r="A32" s="100" t="n"/>
+      <c r="B32" s="100" t="inlineStr">
         <is>
           <t>Enterprise Value (XNPV, mid-year EDATE dates)</t>
         </is>
       </c>
-      <c r="C32" s="97" t="n"/>
-      <c r="D32" s="109">
+      <c r="C32" s="100" t="n"/>
+      <c r="D32" s="120">
         <f>XNPV(D6,D28:J28,D18:J18)</f>
         <v/>
       </c>
-      <c r="E32" s="97" t="n"/>
-      <c r="G32" s="97" t="inlineStr">
+      <c r="E32" s="100" t="n"/>
+      <c r="G32" s="100" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="H32" s="97" t="n"/>
-      <c r="I32" s="97">
+      <c r="H32" s="100" t="n"/>
+      <c r="I32" s="100">
         <f>D12*D11</f>
         <v/>
       </c>
-      <c r="J32" s="97" t="n"/>
-      <c r="L32" s="97" t="inlineStr">
+      <c r="J32" s="100" t="n"/>
+      <c r="L32" s="100" t="inlineStr">
         <is>
           <t>Target Price Upside</t>
         </is>
       </c>
-      <c r="M32" s="97" t="n"/>
-      <c r="N32" s="125">
+      <c r="M32" s="100" t="n"/>
+      <c r="N32" s="136">
         <f>D37/I37-1</f>
         <v/>
       </c>
-      <c r="O32" s="97" t="n"/>
+      <c r="O32" s="100" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="97" t="n"/>
-      <c r="B33" s="97" t="inlineStr">
+      <c r="A33" s="100" t="n"/>
+      <c r="B33" s="100" t="inlineStr">
         <is>
           <t>Plus: Cash</t>
         </is>
       </c>
-      <c r="C33" s="97" t="n"/>
-      <c r="D33" s="97">
+      <c r="C33" s="100" t="n"/>
+      <c r="D33" s="100">
         <f>+D14</f>
         <v/>
       </c>
-      <c r="E33" s="97" t="n"/>
-      <c r="G33" s="97" t="inlineStr">
+      <c r="E33" s="100" t="n"/>
+      <c r="G33" s="100" t="inlineStr">
         <is>
           <t>Plus: Debt</t>
         </is>
       </c>
-      <c r="H33" s="97" t="n"/>
-      <c r="I33" s="97">
+      <c r="H33" s="100" t="n"/>
+      <c r="I33" s="100">
         <f>D13</f>
         <v/>
       </c>
-      <c r="J33" s="97" t="n"/>
-      <c r="L33" s="97" t="inlineStr">
+      <c r="J33" s="100" t="n"/>
+      <c r="L33" s="100" t="inlineStr">
         <is>
           <t>Internal Rate of Return (IRR)</t>
         </is>
       </c>
-      <c r="M33" s="97" t="n"/>
-      <c r="N33" s="125">
+      <c r="M33" s="100" t="n"/>
+      <c r="N33" s="136">
         <f>XIRR(D29:J29,D18:J18)</f>
         <v/>
       </c>
-      <c r="O33" s="97" t="n"/>
+      <c r="O33" s="100" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="97" t="n"/>
-      <c r="B34" s="97" t="inlineStr">
+      <c r="A34" s="100" t="n"/>
+      <c r="B34" s="100" t="inlineStr">
         <is>
           <t>Less: Debt</t>
         </is>
       </c>
-      <c r="C34" s="97" t="n"/>
-      <c r="D34" s="97">
+      <c r="C34" s="100" t="n"/>
+      <c r="D34" s="100">
         <f>+D13</f>
         <v/>
       </c>
-      <c r="E34" s="97" t="n"/>
-      <c r="G34" s="97" t="inlineStr">
+      <c r="E34" s="100" t="n"/>
+      <c r="G34" s="100" t="inlineStr">
         <is>
           <t>Less: Cash</t>
         </is>
       </c>
-      <c r="H34" s="97" t="n"/>
-      <c r="I34" s="97">
+      <c r="H34" s="100" t="n"/>
+      <c r="I34" s="100">
         <f>+D14</f>
         <v/>
       </c>
-      <c r="J34" s="97" t="n"/>
-      <c r="L34" s="97" t="n"/>
-      <c r="M34" s="97" t="n"/>
-      <c r="N34" s="97" t="n"/>
-      <c r="O34" s="97" t="n"/>
+      <c r="J34" s="100" t="n"/>
+      <c r="L34" s="100" t="n"/>
+      <c r="M34" s="100" t="n"/>
+      <c r="N34" s="100" t="n"/>
+      <c r="O34" s="100" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="97" t="n"/>
-      <c r="B35" s="97" t="inlineStr">
+      <c r="A35" s="100" t="n"/>
+      <c r="B35" s="100" t="inlineStr">
         <is>
           <t>Equity Value</t>
         </is>
       </c>
-      <c r="C35" s="97" t="n"/>
-      <c r="D35" s="122">
+      <c r="C35" s="100" t="n"/>
+      <c r="D35" s="133">
         <f>D32+D33-D34</f>
         <v/>
       </c>
-      <c r="E35" s="97" t="n"/>
-      <c r="G35" s="97" t="inlineStr">
+      <c r="E35" s="100" t="n"/>
+      <c r="G35" s="100" t="inlineStr">
         <is>
           <t>Enterprise Value</t>
         </is>
       </c>
-      <c r="H35" s="97" t="n"/>
-      <c r="I35" s="122">
+      <c r="H35" s="100" t="n"/>
+      <c r="I35" s="133">
         <f>I32+I33-I34</f>
         <v/>
       </c>
-      <c r="J35" s="97" t="n"/>
-      <c r="L35" s="110" t="inlineStr">
+      <c r="J35" s="100" t="n"/>
+      <c r="L35" s="121" t="inlineStr">
         <is>
           <t>Market Value vs Intrinsic Value</t>
         </is>
       </c>
-      <c r="M35" s="111" t="n"/>
-      <c r="N35" s="111" t="n"/>
-      <c r="O35" s="97" t="n"/>
+      <c r="M35" s="122" t="n"/>
+      <c r="N35" s="122" t="n"/>
+      <c r="O35" s="100" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="97" t="n"/>
-      <c r="B36" s="97" t="n"/>
-      <c r="C36" s="97" t="n"/>
-      <c r="D36" s="97" t="n"/>
-      <c r="E36" s="97" t="n"/>
-      <c r="G36" s="97" t="n"/>
-      <c r="H36" s="97" t="n"/>
-      <c r="I36" s="126" t="n"/>
-      <c r="J36" s="97" t="n"/>
-      <c r="L36" s="97" t="inlineStr">
+      <c r="A36" s="100" t="n"/>
+      <c r="B36" s="100" t="n"/>
+      <c r="C36" s="100" t="n"/>
+      <c r="D36" s="100" t="n"/>
+      <c r="E36" s="100" t="n"/>
+      <c r="G36" s="100" t="n"/>
+      <c r="H36" s="100" t="n"/>
+      <c r="I36" s="137" t="n"/>
+      <c r="J36" s="100" t="n"/>
+      <c r="L36" s="100" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="M36" s="97" t="n"/>
-      <c r="N36" s="126">
+      <c r="M36" s="100" t="n"/>
+      <c r="N36" s="137">
         <f>I37</f>
         <v/>
       </c>
-      <c r="O36" s="97" t="n"/>
+      <c r="O36" s="100" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="97" t="n"/>
-      <c r="B37" s="97" t="inlineStr">
+      <c r="A37" s="100" t="n"/>
+      <c r="B37" s="100" t="inlineStr">
         <is>
           <t>Equity Value/Share</t>
         </is>
       </c>
-      <c r="C37" s="97" t="n"/>
-      <c r="D37" s="126">
+      <c r="C37" s="100" t="n"/>
+      <c r="D37" s="137">
         <f>D35/D12</f>
         <v/>
       </c>
-      <c r="E37" s="97" t="n"/>
-      <c r="G37" s="97" t="inlineStr">
+      <c r="E37" s="100" t="n"/>
+      <c r="G37" s="100" t="inlineStr">
         <is>
           <t>Equity Value/Share</t>
         </is>
       </c>
-      <c r="H37" s="97" t="n"/>
-      <c r="I37" s="126">
+      <c r="H37" s="100" t="n"/>
+      <c r="I37" s="137">
         <f>D11</f>
         <v/>
       </c>
-      <c r="J37" s="97" t="n"/>
-      <c r="L37" s="97" t="inlineStr">
+      <c r="J37" s="100" t="n"/>
+      <c r="L37" s="100" t="inlineStr">
         <is>
           <t>Upside</t>
         </is>
       </c>
-      <c r="M37" s="97" t="n"/>
-      <c r="N37" s="126">
+      <c r="M37" s="100" t="n"/>
+      <c r="N37" s="137">
         <f>D37-I37</f>
         <v/>
       </c>
-      <c r="O37" s="97" t="n"/>
+      <c r="O37" s="100" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="97" t="n"/>
-      <c r="B38" s="97" t="n"/>
-      <c r="C38" s="97" t="n"/>
-      <c r="D38" s="97" t="n"/>
-      <c r="E38" s="97" t="n"/>
-      <c r="G38" s="97" t="n"/>
-      <c r="H38" s="97" t="n"/>
-      <c r="I38" s="97" t="n"/>
-      <c r="J38" s="97" t="n"/>
-      <c r="L38" s="97" t="inlineStr">
+      <c r="A38" s="100" t="n"/>
+      <c r="B38" s="100" t="n"/>
+      <c r="C38" s="100" t="n"/>
+      <c r="D38" s="100" t="n"/>
+      <c r="E38" s="100" t="n"/>
+      <c r="G38" s="100" t="n"/>
+      <c r="H38" s="100" t="n"/>
+      <c r="I38" s="100" t="n"/>
+      <c r="J38" s="100" t="n"/>
+      <c r="L38" s="100" t="inlineStr">
         <is>
           <t>Intrinsic Value</t>
         </is>
       </c>
-      <c r="M38" s="97" t="n"/>
-      <c r="N38" s="126">
+      <c r="M38" s="100" t="n"/>
+      <c r="N38" s="137">
         <f>SUM(N36:N37)</f>
         <v/>
       </c>
-      <c r="O38" s="97" t="n"/>
+      <c r="O38" s="100" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="97" t="n"/>
-      <c r="C39" s="97" t="n"/>
-      <c r="D39" s="99" t="n"/>
-      <c r="E39" s="97" t="n"/>
-      <c r="G39" s="97" t="n"/>
-      <c r="H39" s="97" t="n"/>
-      <c r="I39" s="98" t="n"/>
-      <c r="J39" s="97" t="n"/>
-      <c r="L39" s="97" t="n"/>
-      <c r="M39" s="97" t="n"/>
-      <c r="N39" s="97" t="n"/>
-      <c r="O39" s="97" t="n"/>
+      <c r="A39" s="100" t="n"/>
+      <c r="C39" s="100" t="n"/>
+      <c r="D39" s="102" t="n"/>
+      <c r="E39" s="100" t="n"/>
+      <c r="G39" s="100" t="n"/>
+      <c r="H39" s="100" t="n"/>
+      <c r="I39" s="101" t="n"/>
+      <c r="J39" s="100" t="n"/>
+      <c r="L39" s="100" t="n"/>
+      <c r="M39" s="100" t="n"/>
+      <c r="N39" s="100" t="n"/>
+      <c r="O39" s="100" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="97" t="n"/>
-      <c r="C40" s="97" t="n"/>
-      <c r="D40" s="99" t="n"/>
-      <c r="E40" s="97" t="n"/>
-      <c r="F40" s="97" t="n"/>
-      <c r="G40" s="97" t="n"/>
-      <c r="H40" s="98" t="n"/>
-      <c r="I40" s="97" t="n"/>
-      <c r="K40" s="97" t="n"/>
-      <c r="L40" s="97" t="n"/>
-      <c r="M40" s="97" t="n"/>
-      <c r="N40" s="97" t="n"/>
-      <c r="O40" s="97" t="n"/>
+      <c r="A40" s="100" t="n"/>
+      <c r="C40" s="100" t="n"/>
+      <c r="D40" s="102" t="n"/>
+      <c r="E40" s="100" t="n"/>
+      <c r="F40" s="100" t="n"/>
+      <c r="G40" s="100" t="n"/>
+      <c r="H40" s="101" t="n"/>
+      <c r="I40" s="100" t="n"/>
+      <c r="K40" s="100" t="n"/>
+      <c r="L40" s="100" t="n"/>
+      <c r="M40" s="100" t="n"/>
+      <c r="N40" s="100" t="n"/>
+      <c r="O40" s="100" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="97" t="n"/>
-      <c r="B41" s="110" t="inlineStr">
+      <c r="A41" s="100" t="n"/>
+      <c r="B41" s="121" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="C41" s="111" t="n"/>
-      <c r="D41" s="127" t="n"/>
-      <c r="E41" s="111" t="n"/>
-      <c r="F41" s="111" t="n"/>
-      <c r="G41" s="111" t="n"/>
-      <c r="H41" s="111" t="n"/>
-      <c r="I41" s="111" t="n"/>
-      <c r="J41" s="111" t="n"/>
-      <c r="K41" s="111" t="n"/>
-      <c r="L41" s="111" t="n"/>
-      <c r="M41" s="111" t="n"/>
-      <c r="N41" s="111" t="n"/>
-      <c r="O41" s="97" t="n"/>
+      <c r="C41" s="122" t="n"/>
+      <c r="D41" s="138" t="n"/>
+      <c r="E41" s="122" t="n"/>
+      <c r="F41" s="122" t="n"/>
+      <c r="G41" s="122" t="n"/>
+      <c r="H41" s="122" t="n"/>
+      <c r="I41" s="122" t="n"/>
+      <c r="J41" s="122" t="n"/>
+      <c r="K41" s="122" t="n"/>
+      <c r="L41" s="122" t="n"/>
+      <c r="M41" s="122" t="n"/>
+      <c r="N41" s="122" t="n"/>
+      <c r="O41" s="100" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="97" t="n"/>
-      <c r="B42" s="97" t="inlineStr">
+      <c r="A42" s="100" t="n"/>
+      <c r="B42" s="100" t="inlineStr">
         <is>
           <t>Step 1: Get EBIT and D&amp;A from the income statement</t>
         </is>
       </c>
-      <c r="C42" s="97" t="n"/>
-      <c r="D42" s="99" t="n"/>
-      <c r="E42" s="97" t="n"/>
-      <c r="F42" s="97" t="n"/>
-      <c r="G42" s="97" t="n"/>
-      <c r="H42" s="97" t="n"/>
-      <c r="N42" s="128" t="inlineStr">
+      <c r="C42" s="100" t="n"/>
+      <c r="D42" s="102" t="n"/>
+      <c r="E42" s="100" t="n"/>
+      <c r="F42" s="100" t="n"/>
+      <c r="G42" s="100" t="n"/>
+      <c r="H42" s="100" t="n"/>
+      <c r="N42" s="139" t="inlineStr">
         <is>
           <t>This file is for educational purposes only. E&amp;OE</t>
         </is>
       </c>
-      <c r="O42" s="97" t="n"/>
+      <c r="O42" s="100" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="97" t="n"/>
-      <c r="B43" s="97" t="inlineStr">
+      <c r="A43" s="100" t="n"/>
+      <c r="B43" s="100" t="inlineStr">
         <is>
           <t>Step 2: Calculate the net working capital</t>
         </is>
       </c>
-      <c r="C43" s="97" t="n"/>
-      <c r="D43" s="99" t="n"/>
-      <c r="E43" s="97" t="n"/>
-      <c r="F43" s="97" t="n"/>
-      <c r="G43" s="97" t="n"/>
-      <c r="H43" s="97" t="n"/>
+      <c r="C43" s="100" t="n"/>
+      <c r="D43" s="102" t="n"/>
+      <c r="E43" s="100" t="n"/>
+      <c r="F43" s="100" t="n"/>
+      <c r="G43" s="100" t="n"/>
+      <c r="H43" s="100" t="n"/>
       <c r="N43" s="69" t="n"/>
-      <c r="O43" s="97" t="n"/>
+      <c r="O43" s="100" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="97" t="n"/>
-      <c r="B44" s="129" t="inlineStr">
+      <c r="A44" s="100" t="n"/>
+      <c r="B44" s="140" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
       </c>
-      <c r="C44" s="97" t="n"/>
-      <c r="D44" s="99" t="n"/>
-      <c r="E44" s="97" t="n"/>
-      <c r="F44" s="97" t="n"/>
-      <c r="G44" s="97" t="n"/>
-      <c r="H44" s="97" t="n"/>
+      <c r="C44" s="100" t="n"/>
+      <c r="D44" s="102" t="n"/>
+      <c r="E44" s="100" t="n"/>
+      <c r="F44" s="100" t="n"/>
+      <c r="G44" s="100" t="n"/>
+      <c r="H44" s="100" t="n"/>
       <c r="N44" s="69" t="n"/>
-      <c r="O44" s="97" t="n"/>
+      <c r="O44" s="100" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="97" t="n"/>
-      <c r="B45" s="129" t="inlineStr">
+      <c r="A45" s="100" t="n"/>
+      <c r="B45" s="140" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
       </c>
-      <c r="C45" s="97" t="n"/>
-      <c r="D45" s="99" t="n"/>
-      <c r="E45" s="97" t="n"/>
-      <c r="F45" s="97" t="n"/>
-      <c r="G45" s="97" t="n"/>
-      <c r="H45" s="97" t="n"/>
+      <c r="C45" s="100" t="n"/>
+      <c r="D45" s="102" t="n"/>
+      <c r="E45" s="100" t="n"/>
+      <c r="F45" s="100" t="n"/>
+      <c r="G45" s="100" t="n"/>
+      <c r="H45" s="100" t="n"/>
       <c r="N45" s="69" t="n"/>
-      <c r="O45" s="97" t="n"/>
+      <c r="O45" s="100" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="97" t="n"/>
-      <c r="B46" s="129" t="inlineStr">
+      <c r="A46" s="100" t="n"/>
+      <c r="B46" s="140" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
       </c>
-      <c r="C46" s="97" t="n"/>
-      <c r="D46" s="99" t="n"/>
-      <c r="E46" s="97" t="n"/>
-      <c r="F46" s="97" t="n"/>
-      <c r="G46" s="97" t="n"/>
-      <c r="H46" s="97" t="n"/>
+      <c r="C46" s="100" t="n"/>
+      <c r="D46" s="102" t="n"/>
+      <c r="E46" s="100" t="n"/>
+      <c r="F46" s="100" t="n"/>
+      <c r="G46" s="100" t="n"/>
+      <c r="H46" s="100" t="n"/>
       <c r="N46" s="69" t="n"/>
-      <c r="O46" s="97" t="n"/>
+      <c r="O46" s="100" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="97" t="n"/>
-      <c r="B47" s="97" t="n"/>
-      <c r="C47" s="97" t="n"/>
-      <c r="D47" s="99" t="n"/>
-      <c r="E47" s="97" t="n"/>
-      <c r="F47" s="97" t="n"/>
-      <c r="G47" s="97" t="n"/>
-      <c r="H47" s="97" t="n"/>
+      <c r="A47" s="100" t="n"/>
+      <c r="B47" s="100" t="n"/>
+      <c r="C47" s="100" t="n"/>
+      <c r="D47" s="102" t="n"/>
+      <c r="E47" s="100" t="n"/>
+      <c r="F47" s="100" t="n"/>
+      <c r="G47" s="100" t="n"/>
+      <c r="H47" s="100" t="n"/>
       <c r="N47" s="69" t="n"/>
-      <c r="O47" s="97" t="n"/>
+      <c r="O47" s="100" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="97" t="n"/>
-      <c r="B48" s="97" t="n"/>
-      <c r="C48" s="97" t="n"/>
-      <c r="D48" s="99" t="n"/>
-      <c r="E48" s="97" t="n"/>
-      <c r="F48" s="97" t="n"/>
-      <c r="G48" s="97" t="n"/>
-      <c r="H48" s="97" t="n"/>
-      <c r="N48" s="130" t="inlineStr">
+      <c r="A48" s="100" t="n"/>
+      <c r="B48" s="100" t="n"/>
+      <c r="C48" s="100" t="n"/>
+      <c r="D48" s="102" t="n"/>
+      <c r="E48" s="100" t="n"/>
+      <c r="F48" s="100" t="n"/>
+      <c r="G48" s="100" t="n"/>
+      <c r="H48" s="100" t="n"/>
+      <c r="N48" s="141" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
       </c>
-      <c r="O48" s="97" t="n"/>
+      <c r="O48" s="100" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="97" t="n"/>
-      <c r="B49" s="97" t="n"/>
-      <c r="C49" s="97" t="n"/>
-      <c r="D49" s="99" t="n"/>
-      <c r="E49" s="97" t="n"/>
-      <c r="F49" s="97" t="n"/>
-      <c r="G49" s="97" t="n"/>
-      <c r="H49" s="97" t="n"/>
-      <c r="N49" s="131" t="inlineStr">
+      <c r="A49" s="100" t="n"/>
+      <c r="B49" s="100" t="n"/>
+      <c r="C49" s="100" t="n"/>
+      <c r="D49" s="102" t="n"/>
+      <c r="E49" s="100" t="n"/>
+      <c r="F49" s="100" t="n"/>
+      <c r="G49" s="100" t="n"/>
+      <c r="H49" s="100" t="n"/>
+      <c r="N49" s="142" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
       </c>
-      <c r="O49" s="97" t="n"/>
+      <c r="O49" s="100" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="97" t="n"/>
-      <c r="B50" s="97" t="n"/>
-      <c r="C50" s="97" t="n"/>
-      <c r="D50" s="99" t="n"/>
-      <c r="E50" s="97" t="n"/>
-      <c r="F50" s="97" t="n"/>
-      <c r="G50" s="97" t="n"/>
-      <c r="H50" s="97" t="n"/>
-      <c r="O50" s="97" t="n"/>
+      <c r="A50" s="100" t="n"/>
+      <c r="B50" s="100" t="n"/>
+      <c r="C50" s="100" t="n"/>
+      <c r="D50" s="102" t="n"/>
+      <c r="E50" s="100" t="n"/>
+      <c r="F50" s="100" t="n"/>
+      <c r="G50" s="100" t="n"/>
+      <c r="H50" s="100" t="n"/>
+      <c r="O50" s="100" t="n"/>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="97" t="n"/>
-      <c r="B51" s="97" t="n"/>
-      <c r="C51" s="97" t="n"/>
-      <c r="D51" s="99" t="n"/>
-      <c r="E51" s="97" t="n"/>
-      <c r="F51" s="97" t="n"/>
-      <c r="G51" s="97" t="n"/>
-      <c r="H51" s="97" t="n"/>
-      <c r="M51" s="97" t="n"/>
-      <c r="O51" s="97" t="n"/>
+      <c r="A51" s="100" t="n"/>
+      <c r="B51" s="100" t="n"/>
+      <c r="C51" s="100" t="n"/>
+      <c r="D51" s="102" t="n"/>
+      <c r="E51" s="100" t="n"/>
+      <c r="F51" s="100" t="n"/>
+      <c r="G51" s="100" t="n"/>
+      <c r="H51" s="100" t="n"/>
+      <c r="M51" s="100" t="n"/>
+      <c r="O51" s="100" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="97" t="n"/>
-      <c r="B52" s="97" t="n"/>
-      <c r="C52" s="97" t="n"/>
-      <c r="D52" s="99" t="n"/>
-      <c r="E52" s="97" t="n"/>
-      <c r="F52" s="97" t="n"/>
-      <c r="G52" s="97" t="n"/>
-      <c r="H52" s="97" t="n"/>
-      <c r="I52" s="97" t="n"/>
-      <c r="J52" s="97" t="n"/>
-      <c r="K52" s="97" t="n"/>
-      <c r="L52" s="97" t="n"/>
-      <c r="M52" s="97" t="n"/>
-      <c r="N52" s="97" t="n"/>
-      <c r="O52" s="97" t="n"/>
+      <c r="A52" s="100" t="n"/>
+      <c r="B52" s="100" t="n"/>
+      <c r="C52" s="100" t="n"/>
+      <c r="D52" s="102" t="n"/>
+      <c r="E52" s="100" t="n"/>
+      <c r="F52" s="100" t="n"/>
+      <c r="G52" s="100" t="n"/>
+      <c r="H52" s="100" t="n"/>
+      <c r="I52" s="100" t="n"/>
+      <c r="J52" s="100" t="n"/>
+      <c r="K52" s="100" t="n"/>
+      <c r="L52" s="100" t="n"/>
+      <c r="M52" s="100" t="n"/>
+      <c r="N52" s="100" t="n"/>
+      <c r="O52" s="100" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="97" t="n"/>
-      <c r="B53" s="97" t="n"/>
-      <c r="C53" s="97" t="n"/>
-      <c r="D53" s="99" t="n"/>
-      <c r="E53" s="97" t="n"/>
-      <c r="F53" s="97" t="n"/>
-      <c r="G53" s="97" t="n"/>
-      <c r="H53" s="97" t="n"/>
-      <c r="I53" s="97" t="n"/>
-      <c r="J53" s="97" t="n"/>
-      <c r="K53" s="97" t="n"/>
-      <c r="L53" s="97" t="n"/>
-      <c r="M53" s="97" t="n"/>
-      <c r="N53" s="97" t="n"/>
-      <c r="O53" s="97" t="n"/>
+      <c r="A53" s="100" t="n"/>
+      <c r="B53" s="100" t="n"/>
+      <c r="C53" s="100" t="n"/>
+      <c r="D53" s="102" t="n"/>
+      <c r="E53" s="100" t="n"/>
+      <c r="F53" s="100" t="n"/>
+      <c r="G53" s="100" t="n"/>
+      <c r="H53" s="100" t="n"/>
+      <c r="I53" s="100" t="n"/>
+      <c r="J53" s="100" t="n"/>
+      <c r="K53" s="100" t="n"/>
+      <c r="L53" s="100" t="n"/>
+      <c r="M53" s="100" t="n"/>
+      <c r="N53" s="100" t="n"/>
+      <c r="O53" s="100" t="n"/>
     </row>
     <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="97" t="n"/>
-      <c r="B54" s="97" t="n"/>
-      <c r="C54" s="97" t="n"/>
-      <c r="D54" s="99" t="n"/>
-      <c r="E54" s="97" t="n"/>
-      <c r="F54" s="97" t="n"/>
-      <c r="G54" s="97" t="n"/>
-      <c r="H54" s="97" t="n"/>
-      <c r="I54" s="97" t="n"/>
-      <c r="J54" s="97" t="n"/>
-      <c r="K54" s="97" t="n"/>
-      <c r="L54" s="97" t="n"/>
-      <c r="M54" s="97" t="n"/>
-      <c r="N54" s="97" t="n"/>
-      <c r="O54" s="97" t="n"/>
+      <c r="A54" s="100" t="n"/>
+      <c r="B54" s="100" t="n"/>
+      <c r="C54" s="100" t="n"/>
+      <c r="D54" s="102" t="n"/>
+      <c r="E54" s="100" t="n"/>
+      <c r="F54" s="100" t="n"/>
+      <c r="G54" s="100" t="n"/>
+      <c r="H54" s="100" t="n"/>
+      <c r="I54" s="100" t="n"/>
+      <c r="J54" s="100" t="n"/>
+      <c r="K54" s="100" t="n"/>
+      <c r="L54" s="100" t="n"/>
+      <c r="M54" s="100" t="n"/>
+      <c r="N54" s="100" t="n"/>
+      <c r="O54" s="100" t="n"/>
     </row>
     <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="97" t="n"/>
-      <c r="B55" s="97" t="n"/>
-      <c r="C55" s="97" t="n"/>
-      <c r="D55" s="99" t="n"/>
-      <c r="E55" s="97" t="n"/>
-      <c r="F55" s="97" t="n"/>
-      <c r="G55" s="97" t="n"/>
-      <c r="H55" s="97" t="n"/>
-      <c r="I55" s="97" t="n"/>
-      <c r="J55" s="97" t="n"/>
-      <c r="K55" s="97" t="n"/>
-      <c r="L55" s="97" t="n"/>
-      <c r="M55" s="97" t="n"/>
-      <c r="N55" s="97" t="n"/>
-      <c r="O55" s="97" t="n"/>
+      <c r="A55" s="100" t="n"/>
+      <c r="B55" s="100" t="n"/>
+      <c r="C55" s="100" t="n"/>
+      <c r="D55" s="102" t="n"/>
+      <c r="E55" s="100" t="n"/>
+      <c r="F55" s="100" t="n"/>
+      <c r="G55" s="100" t="n"/>
+      <c r="H55" s="100" t="n"/>
+      <c r="I55" s="100" t="n"/>
+      <c r="J55" s="100" t="n"/>
+      <c r="K55" s="100" t="n"/>
+      <c r="L55" s="143" t="inlineStr">
+        <is>
+          <t>SENSITIVITY — Enterprise Value ($000s)</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="97" t="n"/>
-      <c r="B56" s="97" t="n"/>
-      <c r="C56" s="97" t="n"/>
-      <c r="D56" s="99" t="n"/>
-      <c r="E56" s="97" t="n"/>
-      <c r="F56" s="97" t="n"/>
-      <c r="G56" s="97" t="n"/>
-      <c r="H56" s="97" t="n"/>
-      <c r="I56" s="97" t="n"/>
-      <c r="J56" s="97" t="n"/>
-      <c r="K56" s="97" t="n"/>
-      <c r="L56" s="97" t="n"/>
-      <c r="M56" s="97" t="n"/>
-      <c r="N56" s="97" t="n"/>
-      <c r="O56" s="97" t="n"/>
+      <c r="A56" s="100" t="n"/>
+      <c r="B56" s="100" t="n"/>
+      <c r="C56" s="100" t="n"/>
+      <c r="D56" s="102" t="n"/>
+      <c r="E56" s="100" t="n"/>
+      <c r="F56" s="100" t="n"/>
+      <c r="G56" s="100" t="n"/>
+      <c r="H56" s="100" t="n"/>
+      <c r="I56" s="100" t="n"/>
+      <c r="J56" s="100" t="n"/>
+      <c r="K56" s="100" t="n"/>
+      <c r="L56" s="113" t="inlineStr">
+        <is>
+          <t>WACC \ Exit EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="M56" s="144" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="N56" s="144" t="n">
+        <v>15</v>
+      </c>
+      <c r="O56" s="144" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="P56" s="144" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q56" s="144" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="R56" s="144" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="97" t="n"/>
-      <c r="B57" s="97" t="n"/>
-      <c r="C57" s="97" t="n"/>
-      <c r="D57" s="99" t="n"/>
-      <c r="E57" s="97" t="n"/>
-      <c r="F57" s="97" t="n"/>
-      <c r="G57" s="97" t="n"/>
-      <c r="H57" s="97" t="n"/>
-      <c r="I57" s="97" t="n"/>
-      <c r="J57" s="97" t="n"/>
-      <c r="K57" s="97" t="n"/>
-      <c r="L57" s="97" t="n"/>
-      <c r="M57" s="97" t="n"/>
-      <c r="N57" s="97" t="n"/>
-      <c r="O57" s="97" t="n"/>
+      <c r="A57" s="100" t="n"/>
+      <c r="B57" s="100" t="n"/>
+      <c r="C57" s="100" t="n"/>
+      <c r="D57" s="102" t="n"/>
+      <c r="E57" s="100" t="n"/>
+      <c r="F57" s="100" t="n"/>
+      <c r="G57" s="100" t="n"/>
+      <c r="H57" s="100" t="n"/>
+      <c r="I57" s="100" t="n"/>
+      <c r="J57" s="100" t="n"/>
+      <c r="K57" s="100" t="n"/>
+      <c r="L57" s="145" t="n">
+        <v>0.0824</v>
+      </c>
+      <c r="M57" s="146">
+        <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="N57" s="146">
+        <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="O57" s="146">
+        <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="P57" s="146">
+        <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="Q57" s="146">
+        <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="R57" s="146">
+        <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
     </row>
     <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="97" t="n"/>
-      <c r="B58" s="97" t="n"/>
-      <c r="C58" s="97" t="n"/>
-      <c r="D58" s="99" t="n"/>
-      <c r="E58" s="97" t="n"/>
-      <c r="F58" s="97" t="n"/>
-      <c r="G58" s="97" t="n"/>
-      <c r="H58" s="97" t="n"/>
-      <c r="I58" s="97" t="n"/>
-      <c r="J58" s="97" t="n"/>
-      <c r="K58" s="97" t="n"/>
-      <c r="L58" s="97" t="n"/>
-      <c r="M58" s="97" t="n"/>
-      <c r="N58" s="97" t="n"/>
-      <c r="O58" s="97" t="n"/>
+      <c r="A58" s="100" t="n"/>
+      <c r="B58" s="100" t="n"/>
+      <c r="C58" s="100" t="n"/>
+      <c r="D58" s="102" t="n"/>
+      <c r="E58" s="100" t="n"/>
+      <c r="F58" s="100" t="n"/>
+      <c r="G58" s="100" t="n"/>
+      <c r="H58" s="100" t="n"/>
+      <c r="I58" s="100" t="n"/>
+      <c r="J58" s="100" t="n"/>
+      <c r="K58" s="100" t="n"/>
+      <c r="L58" s="145" t="n">
+        <v>0.08740000000000001</v>
+      </c>
+      <c r="M58" s="146">
+        <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="N58" s="146">
+        <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="O58" s="146">
+        <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="P58" s="146">
+        <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="Q58" s="146">
+        <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="R58" s="146">
+        <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
     </row>
     <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="97" t="n"/>
-      <c r="B59" s="97" t="n"/>
-      <c r="C59" s="97" t="n"/>
-      <c r="D59" s="99" t="n"/>
-      <c r="E59" s="97" t="n"/>
-      <c r="F59" s="97" t="n"/>
-      <c r="G59" s="97" t="n"/>
-      <c r="H59" s="97" t="n"/>
-      <c r="I59" s="97" t="n"/>
-      <c r="J59" s="97" t="n"/>
-      <c r="K59" s="97" t="n"/>
-      <c r="L59" s="97" t="n"/>
-      <c r="M59" s="97" t="n"/>
-      <c r="N59" s="97" t="n"/>
-      <c r="O59" s="97" t="n"/>
+      <c r="A59" s="100" t="n"/>
+      <c r="B59" s="100" t="n"/>
+      <c r="C59" s="100" t="n"/>
+      <c r="D59" s="102" t="n"/>
+      <c r="E59" s="100" t="n"/>
+      <c r="F59" s="100" t="n"/>
+      <c r="G59" s="100" t="n"/>
+      <c r="H59" s="100" t="n"/>
+      <c r="I59" s="100" t="n"/>
+      <c r="J59" s="100" t="n"/>
+      <c r="K59" s="100" t="n"/>
+      <c r="L59" s="145" t="n">
+        <v>0.0924</v>
+      </c>
+      <c r="M59" s="146">
+        <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="N59" s="146">
+        <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="O59" s="147">
+        <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="P59" s="146">
+        <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="Q59" s="146">
+        <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="R59" s="146">
+        <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="97" t="n"/>
-      <c r="B60" s="97" t="n"/>
-      <c r="C60" s="97" t="n"/>
-      <c r="D60" s="99" t="n"/>
-      <c r="E60" s="97" t="n"/>
-      <c r="F60" s="97" t="n"/>
-      <c r="G60" s="97" t="n"/>
-      <c r="H60" s="97" t="n"/>
-      <c r="I60" s="97" t="n"/>
-      <c r="J60" s="97" t="n"/>
-      <c r="K60" s="97" t="n"/>
-      <c r="L60" s="97" t="n"/>
-      <c r="M60" s="97" t="n"/>
-      <c r="N60" s="97" t="n"/>
-      <c r="O60" s="97" t="n"/>
+      <c r="A60" s="100" t="n"/>
+      <c r="B60" s="100" t="n"/>
+      <c r="C60" s="100" t="n"/>
+      <c r="D60" s="102" t="n"/>
+      <c r="E60" s="100" t="n"/>
+      <c r="F60" s="100" t="n"/>
+      <c r="G60" s="100" t="n"/>
+      <c r="H60" s="100" t="n"/>
+      <c r="I60" s="100" t="n"/>
+      <c r="J60" s="100" t="n"/>
+      <c r="K60" s="100" t="n"/>
+      <c r="L60" s="145" t="n">
+        <v>0.0974</v>
+      </c>
+      <c r="M60" s="146">
+        <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="N60" s="146">
+        <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="O60" s="146">
+        <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="P60" s="146">
+        <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="Q60" s="146">
+        <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="R60" s="146">
+        <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
     </row>
     <row r="61" ht="16" customHeight="1">
-      <c r="B61" s="97" t="n"/>
-      <c r="C61" s="97" t="n"/>
-      <c r="D61" s="99" t="n"/>
-      <c r="E61" s="97" t="n"/>
-      <c r="F61" s="97" t="n"/>
-      <c r="G61" s="97" t="n"/>
-      <c r="H61" s="97" t="n"/>
-      <c r="I61" s="97" t="n"/>
-      <c r="J61" s="97" t="n"/>
-      <c r="K61" s="97" t="n"/>
-      <c r="L61" s="97" t="n"/>
+      <c r="B61" s="100" t="n"/>
+      <c r="C61" s="100" t="n"/>
+      <c r="D61" s="102" t="n"/>
+      <c r="E61" s="100" t="n"/>
+      <c r="F61" s="100" t="n"/>
+      <c r="G61" s="100" t="n"/>
+      <c r="H61" s="100" t="n"/>
+      <c r="I61" s="100" t="n"/>
+      <c r="J61" s="100" t="n"/>
+      <c r="K61" s="100" t="n"/>
+      <c r="L61" s="145" t="n">
+        <v>0.1024</v>
+      </c>
+      <c r="M61" s="146">
+        <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="N61" s="146">
+        <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="O61" s="146">
+        <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="P61" s="146">
+        <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="Q61" s="146">
+        <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="R61" s="146">
+        <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="L64" s="148" t="inlineStr">
+        <is>
+          <t>SENSITIVITY — Equity Value / Share ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="L65" s="149" t="inlineStr">
+        <is>
+          <t>WACC \ Exit EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="M65" s="150" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="N65" s="150" t="n">
+        <v>15</v>
+      </c>
+      <c r="O65" s="150" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="P65" s="150" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q65" s="150" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="R65" s="150" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="L66" s="145" t="n">
+        <v>0.0824</v>
+      </c>
+      <c r="M66" s="151">
+        <f>(M57+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="N66" s="151">
+        <f>(N57+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="O66" s="151">
+        <f>(O57+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="P66" s="151">
+        <f>(P57+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="Q66" s="151">
+        <f>(Q57+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="R66" s="151">
+        <f>(R57+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="L67" s="145" t="n">
+        <v>0.08740000000000001</v>
+      </c>
+      <c r="M67" s="151">
+        <f>(M58+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="N67" s="151">
+        <f>(N58+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="O67" s="151">
+        <f>(O58+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="P67" s="151">
+        <f>(P58+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="Q67" s="151">
+        <f>(Q58+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="R67" s="151">
+        <f>(R58+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="L68" s="145" t="n">
+        <v>0.0924</v>
+      </c>
+      <c r="M68" s="151">
+        <f>(M59+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="N68" s="151">
+        <f>(N59+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="O68" s="152">
+        <f>(O59+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="P68" s="151">
+        <f>(P59+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="Q68" s="151">
+        <f>(Q59+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="R68" s="151">
+        <f>(R59+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="L69" s="145" t="n">
+        <v>0.0974</v>
+      </c>
+      <c r="M69" s="151">
+        <f>(M60+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="N69" s="151">
+        <f>(N60+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="O69" s="151">
+        <f>(O60+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="P69" s="151">
+        <f>(P60+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="Q69" s="151">
+        <f>(Q60+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="R69" s="151">
+        <f>(R60+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="L70" s="145" t="n">
+        <v>0.1024</v>
+      </c>
+      <c r="M70" s="151">
+        <f>(M61+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="N70" s="151">
+        <f>(N61+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="O70" s="151">
+        <f>(O61+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="P70" s="151">
+        <f>(P61+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="Q70" s="151">
+        <f>(Q61+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+      <c r="R70" s="151">
+        <f>(R61+$D$33-$D$34)/$D$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="L72" s="153" t="inlineStr">
+        <is>
+          <t>Yellow = base (WACC≈9.24%, Exit 17.5x). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 17.5x; bull 25x; bear 12.8x.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="L55:R55"/>
+    <mergeCell ref="L64:R64"/>
+    <mergeCell ref="L72:R72"/>
+    <mergeCell ref="L24:O24"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="L1:O1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MODEL8: link DCF assumptions to 3-statement sources
Wire D5 tax to 3S!J13, EBIT to EBT+Interest, ΔNWC to WC row 90, and add
an on-sheet DCF←3S linkage audit. Stop CSV overwrite of live tax/WACC cells.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -100,7 +100,7 @@
     <numFmt numFmtId="178" formatCode="#,##0.0"/>
     <numFmt numFmtId="179" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="47">
+  <fonts count="48">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -357,13 +357,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="000000FF"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="8"/>
+      <color rgb="000000FF"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -395,6 +395,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="12">
@@ -534,7 +539,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -708,11 +713,14 @@
     <xf numFmtId="164" fontId="33" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="32" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="9" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="175" fontId="39" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="40" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -744,12 +752,21 @@
     <xf numFmtId="173" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="38" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="39" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="44" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="47" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="47" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="39" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -762,19 +779,17 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="177" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="178" fontId="38" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="177" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="179" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="179" fontId="38" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1580,6 +1595,14 @@
     <author>vengeanceaiUSCMODEL8</author>
   </authors>
   <commentList>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Tax rate for unlevered FCFF and WACC after-tax Rd.
+HOW: D5 = '3 Statement Model'!J13 (I35/I33 on hist, held in forecast).
+WHY: DCF must use the same t as the 3-statement so NOPAT/FCFF articulate.
+SOURCE: SEC 10-K FY2025 tax / EBT (via 3S hist).</t>
+      </text>
+    </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
         <t>Exit EV/EBITDA multiple (BASE)
@@ -6304,12 +6327,17 @@
       <c r="A5" s="100" t="n"/>
       <c r="B5" s="108" t="inlineStr">
         <is>
-          <t>Tax Rate (unlevered / on EBIT)</t>
-        </is>
-      </c>
-      <c r="C5" s="103" t="n"/>
-      <c r="D5" s="109" t="n">
-        <v>0.25</v>
+          <t>Tax Rate (from 3-Statement J13 = FY25 tax/EBT)</t>
+        </is>
+      </c>
+      <c r="C5" s="109" t="inlineStr">
+        <is>
+          <t>Linked to 3S — do not hardcode</t>
+        </is>
+      </c>
+      <c r="D5" s="110">
+        <f>'3 Statement Model'!J13</f>
+        <v/>
       </c>
       <c r="E5" s="103" t="n"/>
       <c r="F5" s="100" t="n"/>
@@ -6345,7 +6373,7 @@
         </is>
       </c>
       <c r="C6" s="100" t="n"/>
-      <c r="D6" s="109" t="n">
+      <c r="D6" s="111" t="n">
         <v>0.12</v>
       </c>
       <c r="E6" s="100" t="n"/>
@@ -6382,7 +6410,7 @@
         </is>
       </c>
       <c r="C7" s="100" t="n"/>
-      <c r="D7" s="109" t="n">
+      <c r="D7" s="111" t="n">
         <v>0.03</v>
       </c>
       <c r="E7" s="100" t="n"/>
@@ -6418,21 +6446,21 @@
           <t>Exit EV/EBITDA (BASE 17.5x — peer comps)</t>
         </is>
       </c>
-      <c r="C8" s="110" t="inlineStr">
+      <c r="C8" s="109" t="inlineStr">
         <is>
           <t>BASE 17.5x ≈ peer median 18.1x (VCP Scanner). Bull 25x / Bear 12.8x.</t>
         </is>
       </c>
-      <c r="D8" s="111" t="n">
+      <c r="D8" s="112" t="n">
         <v>17.5</v>
       </c>
       <c r="E8" s="100" t="n"/>
-      <c r="F8" s="112" t="inlineStr">
+      <c r="F8" s="113" t="inlineStr">
         <is>
           <t>Peer EV/EBITDA comps (click)</t>
         </is>
       </c>
-      <c r="G8" s="112" t="inlineStr">
+      <c r="G8" s="113" t="inlineStr">
         <is>
           <t>FICO spot EV/EBITDA (click)</t>
         </is>
@@ -6441,20 +6469,20 @@
       <c r="I8" s="100" t="n"/>
       <c r="J8" s="100" t="n"/>
       <c r="K8" s="100" t="n"/>
-      <c r="L8" s="113" t="inlineStr">
+      <c r="L8" s="114" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="M8" s="113" t="inlineStr">
+      <c r="M8" s="114" t="inlineStr">
         <is>
           <t>Peer set</t>
         </is>
       </c>
-      <c r="N8" s="114" t="n">
+      <c r="N8" s="115" t="n">
         <v>18.11</v>
       </c>
-      <c r="O8" s="113" t="inlineStr">
+      <c r="O8" s="114" t="inlineStr">
         <is>
           <t>Sorted median (SPGI)</t>
         </is>
@@ -6464,11 +6492,15 @@
       <c r="A9" s="100" t="n"/>
       <c r="B9" s="100" t="inlineStr">
         <is>
-          <t>Transaction Date</t>
-        </is>
-      </c>
-      <c r="C9" s="100" t="n"/>
-      <c r="D9" s="115" t="n">
+          <t>Transaction Date (= last hist FYE on 3S)</t>
+        </is>
+      </c>
+      <c r="C9" s="109" t="inlineStr">
+        <is>
+          <t>Matches 3S hist FYE (Sep 30)</t>
+        </is>
+      </c>
+      <c r="D9" s="116" t="n">
         <v>43100</v>
       </c>
       <c r="E9" s="100" t="n"/>
@@ -6478,16 +6510,16 @@
       <c r="I9" s="100" t="n"/>
       <c r="J9" s="100" t="n"/>
       <c r="K9" s="100" t="n"/>
-      <c r="L9" s="116" t="inlineStr">
+      <c r="L9" s="117" t="inlineStr">
         <is>
           <t>Base exit (D8)</t>
         </is>
       </c>
-      <c r="M9" s="116" t="n"/>
-      <c r="N9" s="117" t="n">
+      <c r="M9" s="117" t="n"/>
+      <c r="N9" s="118" t="n">
         <v>17.5</v>
       </c>
-      <c r="O9" s="116" t="inlineStr">
+      <c r="O9" s="117" t="inlineStr">
         <is>
           <t>Near peer median; audit 17.5x</t>
         </is>
@@ -6497,11 +6529,11 @@
       <c r="A10" s="100" t="n"/>
       <c r="B10" s="100" t="inlineStr">
         <is>
-          <t>Fiscal Year End</t>
+          <t>Fiscal Year End (first forecast FYE)</t>
         </is>
       </c>
       <c r="C10" s="100" t="n"/>
-      <c r="D10" s="115" t="n">
+      <c r="D10" s="116" t="n">
         <v>43281</v>
       </c>
       <c r="E10" s="100" t="n"/>
@@ -6511,12 +6543,12 @@
       <c r="I10" s="100" t="n"/>
       <c r="J10" s="100" t="n"/>
       <c r="K10" s="100" t="n"/>
-      <c r="L10" s="112" t="inlineStr">
+      <c r="L10" s="113" t="inlineStr">
         <is>
           <t>Peer comps (click)</t>
         </is>
       </c>
-      <c r="M10" s="112" t="inlineStr">
+      <c r="M10" s="113" t="inlineStr">
         <is>
           <t>FICO spot EV/EBITDA (click)</t>
         </is>
@@ -6532,7 +6564,7 @@
         </is>
       </c>
       <c r="C11" s="100" t="n"/>
-      <c r="D11" s="118" t="n">
+      <c r="D11" s="119" t="n">
         <v>25</v>
       </c>
       <c r="E11" s="100" t="n"/>
@@ -6555,7 +6587,7 @@
         </is>
       </c>
       <c r="C12" s="100" t="n"/>
-      <c r="D12" s="119" t="n">
+      <c r="D12" s="120" t="n">
         <v>20000</v>
       </c>
       <c r="E12" s="100" t="n"/>
@@ -6574,11 +6606,15 @@
       <c r="A13" s="100" t="n"/>
       <c r="B13" s="100" t="inlineStr">
         <is>
-          <t>Debt</t>
-        </is>
-      </c>
-      <c r="C13" s="100" t="n"/>
-      <c r="D13" s="119" t="n">
+          <t>Debt (10-Q bridge — not 3S FY25 I49)</t>
+        </is>
+      </c>
+      <c r="C13" s="109" t="inlineStr">
+        <is>
+          <t>See L39 for 3S FY25 debt ref</t>
+        </is>
+      </c>
+      <c r="D13" s="120" t="n">
         <v>30000</v>
       </c>
       <c r="E13" s="100" t="n"/>
@@ -6597,11 +6633,15 @@
       <c r="A14" s="100" t="n"/>
       <c r="B14" s="100" t="inlineStr">
         <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="C14" s="100" t="n"/>
-      <c r="D14" s="119" t="n">
+          <t>Cash+mkt secs (10-Q bridge — not 3S FY25 I41)</t>
+        </is>
+      </c>
+      <c r="C14" s="109" t="inlineStr">
+        <is>
+          <t>See L38 for 3S FY25 cash ref</t>
+        </is>
+      </c>
+      <c r="D14" s="120" t="n">
         <v>239549.5203651849</v>
       </c>
       <c r="E14" s="100" t="n"/>
@@ -6620,11 +6660,11 @@
       <c r="A15" s="100" t="n"/>
       <c r="B15" s="100" t="inlineStr">
         <is>
-          <t>Capex (FY1 forecast, linked)</t>
+          <t>Capex FY1 (linked to 3S J68)</t>
         </is>
       </c>
       <c r="C15" s="100" t="n"/>
-      <c r="D15" s="120">
+      <c r="D15" s="121">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
@@ -6644,7 +6684,7 @@
       <c r="A16" s="100" t="n"/>
       <c r="B16" s="100" t="n"/>
       <c r="C16" s="100" t="n"/>
-      <c r="D16" s="115" t="n"/>
+      <c r="D16" s="116" t="n"/>
       <c r="J16" s="100" t="n"/>
       <c r="K16" s="100" t="n"/>
       <c r="L16" s="100" t="n"/>
@@ -6654,44 +6694,44 @@
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="100" t="n"/>
-      <c r="B17" s="121" t="inlineStr">
+      <c r="B17" s="122" t="inlineStr">
         <is>
           <t>Discounted Cash Flow</t>
         </is>
       </c>
-      <c r="C17" s="122" t="n"/>
-      <c r="D17" s="123" t="inlineStr">
+      <c r="C17" s="123" t="n"/>
+      <c r="D17" s="124" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="E17" s="124">
+      <c r="E17" s="125">
         <f>YEAR(E18)</f>
         <v/>
       </c>
-      <c r="F17" s="124">
+      <c r="F17" s="125">
         <f>YEAR(F18)</f>
         <v/>
       </c>
-      <c r="G17" s="124">
+      <c r="G17" s="125">
         <f>YEAR(G18)</f>
         <v/>
       </c>
-      <c r="H17" s="124">
+      <c r="H17" s="125">
         <f>YEAR(H18)</f>
         <v/>
       </c>
-      <c r="I17" s="124">
+      <c r="I17" s="125">
         <f>YEAR(I18)</f>
         <v/>
       </c>
-      <c r="J17" s="123" t="inlineStr">
+      <c r="J17" s="124" t="inlineStr">
         <is>
           <t>Exit</t>
         </is>
       </c>
       <c r="K17" s="100" t="n"/>
-      <c r="L17" s="125" t="inlineStr">
+      <c r="L17" s="126" t="inlineStr">
         <is>
           <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL8)</t>
         </is>
@@ -6706,31 +6746,31 @@
         </is>
       </c>
       <c r="C18" s="100" t="n"/>
-      <c r="D18" s="126">
+      <c r="D18" s="127">
         <f>$D$9</f>
         <v/>
       </c>
-      <c r="E18" s="126">
+      <c r="E18" s="127">
         <f>EDATE($D$9,(E19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="F18" s="126">
+      <c r="F18" s="127">
         <f>EDATE($D$9,(F19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="G18" s="126">
+      <c r="G18" s="127">
         <f>EDATE($D$9,(G19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="H18" s="126">
+      <c r="H18" s="127">
         <f>EDATE($D$9,(H19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="I18" s="126">
+      <c r="I18" s="127">
         <f>EDATE($D$9,(I19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="J18" s="126">
+      <c r="J18" s="127">
         <f>I18</f>
         <v/>
       </c>
@@ -6740,7 +6780,7 @@
           <t>Exit EV/EBITDA @ D8 (BASE 17.5x)</t>
         </is>
       </c>
-      <c r="M18" s="120">
+      <c r="M18" s="121">
         <f>J27</f>
         <v/>
       </c>
@@ -6753,44 +6793,44 @@
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="100" t="n"/>
-      <c r="B19" s="127" t="inlineStr">
+      <c r="B19" s="128" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="127" t="n"/>
-      <c r="D19" s="128" t="n"/>
-      <c r="E19" s="129" t="n">
+      <c r="C19" s="128" t="n"/>
+      <c r="D19" s="129" t="n"/>
+      <c r="E19" s="130" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="130">
+      <c r="F19" s="131">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="130">
+      <c r="G19" s="131">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="130">
+      <c r="H19" s="131">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="130">
+      <c r="I19" s="131">
         <f>H19+1</f>
         <v/>
       </c>
-      <c r="J19" s="128" t="n"/>
+      <c r="J19" s="129" t="n"/>
       <c r="K19" s="100" t="n"/>
       <c r="L19" s="100" t="inlineStr">
         <is>
           <t>Gordon cross-check (g=D7)</t>
         </is>
       </c>
-      <c r="M19" s="120">
+      <c r="M19" s="121">
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="131" t="inlineStr">
+      <c r="N19" s="132" t="inlineStr">
         <is>
           <t>← sanity check</t>
         </is>
@@ -6799,30 +6839,30 @@
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="100" t="n"/>
-      <c r="B20" s="127" t="inlineStr">
+      <c r="B20" s="128" t="inlineStr">
         <is>
           <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
       <c r="C20" s="100" t="n"/>
       <c r="D20" s="100" t="n"/>
-      <c r="E20" s="132">
+      <c r="E20" s="133">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="132">
+      <c r="F20" s="133">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="132">
+      <c r="G20" s="133">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="132">
+      <c r="H20" s="133">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="132">
+      <c r="I20" s="133">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
@@ -6833,11 +6873,11 @@
           <t>Implied Gordon exit multiple</t>
         </is>
       </c>
-      <c r="M20" s="120">
+      <c r="M20" s="121">
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="133" t="inlineStr">
+      <c r="N20" s="134" t="inlineStr">
         <is>
           <t>← ~bear check</t>
         </is>
@@ -6848,29 +6888,29 @@
       <c r="A21" s="100" t="n"/>
       <c r="B21" s="100" t="inlineStr">
         <is>
-          <t>EBIT (linked to 3-stmt)</t>
+          <t>EBIT (3S: EBT + Interest)</t>
         </is>
       </c>
       <c r="C21" s="100" t="n"/>
       <c r="D21" s="100" t="n"/>
-      <c r="E21" s="120">
-        <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
-        <v/>
-      </c>
-      <c r="F21" s="120">
-        <f>'3 Statement Model'!K26-'3 Statement Model'!K28-'3 Statement Model'!K29-'3 Statement Model'!K30</f>
-        <v/>
-      </c>
-      <c r="G21" s="120">
-        <f>'3 Statement Model'!L26-'3 Statement Model'!L28-'3 Statement Model'!L29-'3 Statement Model'!L30</f>
-        <v/>
-      </c>
-      <c r="H21" s="120">
-        <f>'3 Statement Model'!M26-'3 Statement Model'!M28-'3 Statement Model'!M29-'3 Statement Model'!M30</f>
-        <v/>
-      </c>
-      <c r="I21" s="120">
-        <f>'3 Statement Model'!N26-'3 Statement Model'!N28-'3 Statement Model'!N29-'3 Statement Model'!N30</f>
+      <c r="E21" s="121">
+        <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
+        <v/>
+      </c>
+      <c r="F21" s="121">
+        <f>'3 Statement Model'!K33+'3 Statement Model'!K31</f>
+        <v/>
+      </c>
+      <c r="G21" s="121">
+        <f>'3 Statement Model'!L33+'3 Statement Model'!L31</f>
+        <v/>
+      </c>
+      <c r="H21" s="121">
+        <f>'3 Statement Model'!M33+'3 Statement Model'!M31</f>
+        <v/>
+      </c>
+      <c r="I21" s="121">
+        <f>'3 Statement Model'!N33+'3 Statement Model'!N31</f>
         <v/>
       </c>
       <c r="J21" s="100" t="n"/>
@@ -6880,7 +6920,7 @@
           <t>BASE TV @ 17.5x (primary)</t>
         </is>
       </c>
-      <c r="M21" s="120">
+      <c r="M21" s="121">
         <f>($I$21+$I$23)*17.5</f>
         <v/>
       </c>
@@ -6895,28 +6935,28 @@
       <c r="A22" s="100" t="n"/>
       <c r="B22" s="100" t="inlineStr">
         <is>
-          <t>Less: Unlevered Cash Taxes (EBIT×t)</t>
+          <t>Less: Unlevered Cash Taxes (EBIT × 3S tax rate)</t>
         </is>
       </c>
       <c r="C22" s="100" t="n"/>
       <c r="D22" s="100" t="n"/>
-      <c r="E22" s="134">
+      <c r="E22" s="135">
         <f>E21*$D$5</f>
         <v/>
       </c>
-      <c r="F22" s="134">
+      <c r="F22" s="135">
         <f>F21*$D$5</f>
         <v/>
       </c>
-      <c r="G22" s="134">
+      <c r="G22" s="135">
         <f>G21*$D$5</f>
         <v/>
       </c>
-      <c r="H22" s="134">
+      <c r="H22" s="135">
         <f>H21*$D$5</f>
         <v/>
       </c>
-      <c r="I22" s="134">
+      <c r="I22" s="135">
         <f>I21*$D$5</f>
         <v/>
       </c>
@@ -6927,7 +6967,7 @@
           <t>BULL TV @ 25.0x (spot/policy)</t>
         </is>
       </c>
-      <c r="M22" s="120">
+      <c r="M22" s="121">
         <f>($I$21+$I$23)*25.0</f>
         <v/>
       </c>
@@ -6942,28 +6982,28 @@
       <c r="A23" s="100" t="n"/>
       <c r="B23" s="100" t="inlineStr">
         <is>
-          <t>Plus: D&amp;A (linked to 3-stmt)</t>
+          <t>Plus: D&amp;A (3S IS row 30)</t>
         </is>
       </c>
       <c r="C23" s="100" t="n"/>
       <c r="D23" s="100" t="n"/>
-      <c r="E23" s="134">
+      <c r="E23" s="135">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="134">
+      <c r="F23" s="135">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="134">
+      <c r="G23" s="135">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="134">
+      <c r="H23" s="135">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="134">
+      <c r="I23" s="135">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
@@ -6974,7 +7014,7 @@
           <t>BEAR TV @ 12.8x (Gordon-implied)</t>
         </is>
       </c>
-      <c r="M23" s="120">
+      <c r="M23" s="121">
         <f>($I$21+$I$23)*12.8</f>
         <v/>
       </c>
@@ -6989,34 +7029,34 @@
       <c r="A24" s="100" t="n"/>
       <c r="B24" s="100" t="inlineStr">
         <is>
-          <t>Less: Capex (linked to 3-stmt CF)</t>
+          <t>Less: Capex (3S CF row 68)</t>
         </is>
       </c>
       <c r="C24" s="100" t="n"/>
       <c r="D24" s="100" t="n"/>
-      <c r="E24" s="120">
+      <c r="E24" s="121">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="F24" s="120">
+      <c r="F24" s="121">
         <f>'3 Statement Model'!K68</f>
         <v/>
       </c>
-      <c r="G24" s="120">
+      <c r="G24" s="121">
         <f>'3 Statement Model'!L68</f>
         <v/>
       </c>
-      <c r="H24" s="120">
+      <c r="H24" s="121">
         <f>'3 Statement Model'!M68</f>
         <v/>
       </c>
-      <c r="I24" s="120">
+      <c r="I24" s="121">
         <f>'3 Statement Model'!N68</f>
         <v/>
       </c>
       <c r="J24" s="100" t="n"/>
       <c r="K24" s="100" t="n"/>
-      <c r="L24" s="110" t="inlineStr">
+      <c r="L24" s="109" t="inlineStr">
         <is>
           <t>Reconciliation: Bull 25x → Base 17.5x (peer median ~18.1x) → Bear 12.8x</t>
         </is>
@@ -7026,29 +7066,29 @@
       <c r="A25" s="100" t="n"/>
       <c r="B25" s="100" t="inlineStr">
         <is>
-          <t>Less: ΔNWC (linked to 3-stmt CF)</t>
+          <t>Less: ΔNWC (3S WC row 90)</t>
         </is>
       </c>
       <c r="C25" s="100" t="n"/>
       <c r="D25" s="100" t="n"/>
-      <c r="E25" s="120">
-        <f>'3 Statement Model'!J64</f>
-        <v/>
-      </c>
-      <c r="F25" s="120">
-        <f>'3 Statement Model'!K64</f>
-        <v/>
-      </c>
-      <c r="G25" s="120">
-        <f>'3 Statement Model'!L64</f>
-        <v/>
-      </c>
-      <c r="H25" s="120">
-        <f>'3 Statement Model'!M64</f>
-        <v/>
-      </c>
-      <c r="I25" s="120">
-        <f>'3 Statement Model'!N64</f>
+      <c r="E25" s="121">
+        <f>'3 Statement Model'!J90</f>
+        <v/>
+      </c>
+      <c r="F25" s="121">
+        <f>'3 Statement Model'!K90</f>
+        <v/>
+      </c>
+      <c r="G25" s="121">
+        <f>'3 Statement Model'!L90</f>
+        <v/>
+      </c>
+      <c r="H25" s="121">
+        <f>'3 Statement Model'!M90</f>
+        <v/>
+      </c>
+      <c r="I25" s="121">
+        <f>'3 Statement Model'!N90</f>
         <v/>
       </c>
       <c r="J25" s="100" t="n"/>
@@ -7067,32 +7107,33 @@
       </c>
       <c r="C26" s="100" t="n"/>
       <c r="D26" s="100" t="n"/>
-      <c r="E26" s="133">
+      <c r="E26" s="134">
         <f>E21-E22+E23-E24-E25</f>
         <v/>
       </c>
-      <c r="F26" s="133">
+      <c r="F26" s="134">
         <f>F21-F22+F23-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="133">
+      <c r="G26" s="134">
         <f>G21-G22+G23-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="133">
+      <c r="H26" s="134">
         <f>H21-H22+H23-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="133">
+      <c r="I26" s="134">
         <f>I21-I22+I23-I24-I25</f>
         <v/>
       </c>
       <c r="J26" s="100" t="n"/>
       <c r="K26" s="100" t="n"/>
-      <c r="L26" s="100" t="n"/>
-      <c r="M26" s="100" t="n"/>
-      <c r="N26" s="100" t="n"/>
-      <c r="O26" s="100" t="n"/>
+      <c r="L26" s="136" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSCMODEL8 — DCF ← 3-Statement linkage audit</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="100" t="n"/>
@@ -7111,15 +7152,31 @@
       <c r="G27" s="100" t="n"/>
       <c r="H27" s="100" t="n"/>
       <c r="I27" s="100" t="n"/>
-      <c r="J27" s="120">
+      <c r="J27" s="121">
         <f>($I$21+$I$23)*$D$8</f>
         <v/>
       </c>
       <c r="K27" s="100" t="n"/>
-      <c r="L27" s="100" t="n"/>
-      <c r="M27" s="100" t="n"/>
-      <c r="N27" s="100" t="n"/>
-      <c r="O27" s="100" t="n"/>
+      <c r="L27" s="137" t="inlineStr">
+        <is>
+          <t>DCF item</t>
+        </is>
+      </c>
+      <c r="M27" s="137" t="inlineStr">
+        <is>
+          <t>Value / link</t>
+        </is>
+      </c>
+      <c r="N27" s="137" t="inlineStr">
+        <is>
+          <t>3-Statement source</t>
+        </is>
+      </c>
+      <c r="O27" s="137" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="100" t="n"/>
@@ -7129,38 +7186,52 @@
         </is>
       </c>
       <c r="C28" s="100" t="n"/>
-      <c r="D28" s="133" t="n">
+      <c r="D28" s="134" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="135">
+      <c r="E28" s="138">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="135">
+      <c r="F28" s="138">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="135">
+      <c r="G28" s="138">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="135">
+      <c r="H28" s="138">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="135">
+      <c r="I28" s="138">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="135">
+      <c r="J28" s="138">
         <f>J27+J26</f>
         <v/>
       </c>
       <c r="K28" s="100" t="n"/>
-      <c r="L28" s="100" t="n"/>
-      <c r="M28" s="100" t="n"/>
-      <c r="N28" s="100" t="n"/>
-      <c r="O28" s="100" t="n"/>
+      <c r="L28" s="104" t="inlineStr">
+        <is>
+          <t>Tax rate (D5)</t>
+        </is>
+      </c>
+      <c r="M28" s="139">
+        <f>$D$5</f>
+        <v/>
+      </c>
+      <c r="N28" s="140">
+        <f>'3 Statement Model'!J13</f>
+        <v/>
+      </c>
+      <c r="O28" s="141" t="inlineStr">
+        <is>
+          <t>Same FY25 effective rate as 3S forecast (I35/I33)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="100" t="n"/>
@@ -7174,35 +7245,49 @@
         <f>D27+D26</f>
         <v/>
       </c>
-      <c r="E29" s="120">
+      <c r="E29" s="121">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F29" s="120">
+      <c r="F29" s="121">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G29" s="120">
+      <c r="G29" s="121">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H29" s="120">
+      <c r="H29" s="121">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I29" s="120">
+      <c r="I29" s="121">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J29" s="120">
+      <c r="J29" s="121">
         <f>J27</f>
         <v/>
       </c>
       <c r="K29" s="100" t="n"/>
-      <c r="L29" s="100" t="n"/>
-      <c r="M29" s="100" t="n"/>
-      <c r="N29" s="100" t="n"/>
-      <c r="O29" s="100" t="n"/>
+      <c r="L29" s="104" t="inlineStr">
+        <is>
+          <t>NWC % of sales</t>
+        </is>
+      </c>
+      <c r="M29" s="139">
+        <f>'3 Statement Model'!J15</f>
+        <v/>
+      </c>
+      <c r="N29" s="140">
+        <f>'3 Statement Model'!J15</f>
+        <v/>
+      </c>
+      <c r="O29" s="141" t="inlineStr">
+        <is>
+          <t>Flat policy NWC%; drives ΔNWC in FCFF</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="100" t="n"/>
@@ -7214,37 +7299,61 @@
       <c r="H30" s="100" t="n"/>
       <c r="I30" s="100" t="n"/>
       <c r="J30" s="100" t="n"/>
-      <c r="L30" s="100" t="n"/>
-      <c r="M30" s="100" t="n"/>
-      <c r="N30" s="100" t="n"/>
-      <c r="O30" s="100" t="n"/>
+      <c r="L30" s="104" t="inlineStr">
+        <is>
+          <t>CapEx % (FY1)</t>
+        </is>
+      </c>
+      <c r="M30" s="139">
+        <f>'3 Statement Model'!J18</f>
+        <v/>
+      </c>
+      <c r="N30" s="140">
+        <f>'3 Statement Model'!J18</f>
+        <v/>
+      </c>
+      <c r="O30" s="141" t="inlineStr">
+        <is>
+          <t>3S CapEx fade path → CF CapEx $</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="100" t="n"/>
-      <c r="B31" s="121" t="inlineStr">
+      <c r="B31" s="122" t="inlineStr">
         <is>
           <t>Intrinsic Value</t>
         </is>
       </c>
-      <c r="C31" s="122" t="n"/>
-      <c r="D31" s="122" t="n"/>
+      <c r="C31" s="123" t="n"/>
+      <c r="D31" s="123" t="n"/>
       <c r="E31" s="100" t="n"/>
-      <c r="G31" s="121" t="inlineStr">
+      <c r="G31" s="122" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="H31" s="122" t="n"/>
-      <c r="I31" s="122" t="n"/>
+      <c r="H31" s="123" t="n"/>
+      <c r="I31" s="123" t="n"/>
       <c r="J31" s="100" t="n"/>
-      <c r="L31" s="121" t="inlineStr">
-        <is>
-          <t>Rate of Return</t>
-        </is>
-      </c>
-      <c r="M31" s="122" t="n"/>
-      <c r="N31" s="122" t="n"/>
-      <c r="O31" s="100" t="n"/>
+      <c r="L31" s="142" t="inlineStr">
+        <is>
+          <t>Revenue growth FY1</t>
+        </is>
+      </c>
+      <c r="M31" s="139">
+        <f>'3 Statement Model'!J7</f>
+        <v/>
+      </c>
+      <c r="N31" s="140">
+        <f>'3 Statement Model'!J7</f>
+        <v/>
+      </c>
+      <c r="O31" s="141" t="inlineStr">
+        <is>
+          <t>Policy path on 3S assumption row 7</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="100" t="n"/>
@@ -7254,7 +7363,7 @@
         </is>
       </c>
       <c r="C32" s="100" t="n"/>
-      <c r="D32" s="120">
+      <c r="D32" s="121">
         <f>XNPV(D6,D28:J28,D18:J18)</f>
         <v/>
       </c>
@@ -7270,17 +7379,24 @@
         <v/>
       </c>
       <c r="J32" s="100" t="n"/>
-      <c r="L32" s="100" t="inlineStr">
-        <is>
-          <t>Target Price Upside</t>
-        </is>
-      </c>
-      <c r="M32" s="100" t="n"/>
-      <c r="N32" s="136">
-        <f>D37/I37-1</f>
-        <v/>
-      </c>
-      <c r="O32" s="100" t="n"/>
+      <c r="L32" s="104" t="inlineStr">
+        <is>
+          <t>EBIT FY1 (DCF E21)</t>
+        </is>
+      </c>
+      <c r="M32" s="143">
+        <f>$E$21</f>
+        <v/>
+      </c>
+      <c r="N32" s="143">
+        <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
+        <v/>
+      </c>
+      <c r="O32" s="141" t="inlineStr">
+        <is>
+          <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="100" t="n"/>
@@ -7306,17 +7422,25 @@
         <v/>
       </c>
       <c r="J33" s="100" t="n"/>
-      <c r="L33" s="100" t="inlineStr">
-        <is>
-          <t>Internal Rate of Return (IRR)</t>
-        </is>
-      </c>
-      <c r="M33" s="100" t="n"/>
-      <c r="N33" s="136">
-        <f>XIRR(D29:J29,D18:J18)</f>
-        <v/>
-      </c>
-      <c r="O33" s="100" t="n"/>
+      <c r="L33" s="104" t="inlineStr">
+        <is>
+          <t>EBIT cross-check</t>
+        </is>
+      </c>
+      <c r="M33" s="143">
+        <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
+        <v/>
+      </c>
+      <c r="N33" s="144" t="inlineStr">
+        <is>
+          <t>GP−SGA−R&amp;D−DA</t>
+        </is>
+      </c>
+      <c r="O33" s="141" t="inlineStr">
+        <is>
+          <t>Must equal E21 (live check)</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="100" t="n"/>
@@ -7342,10 +7466,24 @@
         <v/>
       </c>
       <c r="J34" s="100" t="n"/>
-      <c r="L34" s="100" t="n"/>
-      <c r="M34" s="100" t="n"/>
-      <c r="N34" s="100" t="n"/>
-      <c r="O34" s="100" t="n"/>
+      <c r="L34" s="104" t="inlineStr">
+        <is>
+          <t>D&amp;A FY1</t>
+        </is>
+      </c>
+      <c r="M34" s="143">
+        <f>$E$23</f>
+        <v/>
+      </c>
+      <c r="N34" s="143">
+        <f>'3 Statement Model'!J30</f>
+        <v/>
+      </c>
+      <c r="O34" s="141" t="inlineStr">
+        <is>
+          <t>Avg-PP&amp;E D&amp;A from 3S IS</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="100" t="n"/>
@@ -7355,7 +7493,7 @@
         </is>
       </c>
       <c r="C35" s="100" t="n"/>
-      <c r="D35" s="133">
+      <c r="D35" s="134">
         <f>D32+D33-D34</f>
         <v/>
       </c>
@@ -7366,19 +7504,29 @@
         </is>
       </c>
       <c r="H35" s="100" t="n"/>
-      <c r="I35" s="133">
+      <c r="I35" s="134">
         <f>I32+I33-I34</f>
         <v/>
       </c>
       <c r="J35" s="100" t="n"/>
-      <c r="L35" s="121" t="inlineStr">
-        <is>
-          <t>Market Value vs Intrinsic Value</t>
-        </is>
-      </c>
-      <c r="M35" s="122" t="n"/>
-      <c r="N35" s="122" t="n"/>
-      <c r="O35" s="100" t="n"/>
+      <c r="L35" s="142" t="inlineStr">
+        <is>
+          <t>CapEx FY1</t>
+        </is>
+      </c>
+      <c r="M35" s="143">
+        <f>$E$24</f>
+        <v/>
+      </c>
+      <c r="N35" s="143">
+        <f>'3 Statement Model'!J68</f>
+        <v/>
+      </c>
+      <c r="O35" s="141" t="inlineStr">
+        <is>
+          <t>3S CF CapEx (also D15)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="100" t="n"/>
@@ -7388,19 +7536,26 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="137" t="n"/>
+      <c r="I36" s="145" t="n"/>
       <c r="J36" s="100" t="n"/>
-      <c r="L36" s="100" t="inlineStr">
-        <is>
-          <t>Market Value</t>
-        </is>
-      </c>
-      <c r="M36" s="100" t="n"/>
-      <c r="N36" s="137">
-        <f>I37</f>
-        <v/>
-      </c>
-      <c r="O36" s="100" t="n"/>
+      <c r="L36" s="104" t="inlineStr">
+        <is>
+          <t>ΔNWC FY1</t>
+        </is>
+      </c>
+      <c r="M36" s="143">
+        <f>$E$25</f>
+        <v/>
+      </c>
+      <c r="N36" s="143">
+        <f>'3 Statement Model'!J90</f>
+        <v/>
+      </c>
+      <c r="O36" s="141" t="inlineStr">
+        <is>
+          <t>WC schedule change (CF row 64 = J90)</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="100" t="n"/>
@@ -7410,7 +7565,7 @@
         </is>
       </c>
       <c r="C37" s="100" t="n"/>
-      <c r="D37" s="137">
+      <c r="D37" s="145">
         <f>D35/D12</f>
         <v/>
       </c>
@@ -7421,22 +7576,29 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="137">
+      <c r="I37" s="145">
         <f>D11</f>
         <v/>
       </c>
       <c r="J37" s="100" t="n"/>
-      <c r="L37" s="100" t="inlineStr">
-        <is>
-          <t>Upside</t>
-        </is>
-      </c>
-      <c r="M37" s="100" t="n"/>
-      <c r="N37" s="137">
-        <f>D37-I37</f>
-        <v/>
-      </c>
-      <c r="O37" s="100" t="n"/>
+      <c r="L37" s="104" t="inlineStr">
+        <is>
+          <t>EBITDA FY5 (TV base)</t>
+        </is>
+      </c>
+      <c r="M37" s="143">
+        <f>$I$21+$I$23</f>
+        <v/>
+      </c>
+      <c r="N37" s="143">
+        <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
+        <v/>
+      </c>
+      <c r="O37" s="141" t="inlineStr">
+        <is>
+          <t>EBIT+D&amp;A; Exit TV = this × D8</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="100" t="n"/>
@@ -7448,17 +7610,24 @@
       <c r="H38" s="100" t="n"/>
       <c r="I38" s="100" t="n"/>
       <c r="J38" s="100" t="n"/>
-      <c r="L38" s="100" t="inlineStr">
-        <is>
-          <t>Intrinsic Value</t>
-        </is>
-      </c>
-      <c r="M38" s="100" t="n"/>
-      <c r="N38" s="137">
-        <f>SUM(N36:N37)</f>
-        <v/>
-      </c>
-      <c r="O38" s="100" t="n"/>
+      <c r="L38" s="104" t="inlineStr">
+        <is>
+          <t>3S FY25 Cash (ref)</t>
+        </is>
+      </c>
+      <c r="M38" s="143">
+        <f>'3 Statement Model'!I41</f>
+        <v/>
+      </c>
+      <c r="N38" s="143">
+        <f>'3 Statement Model'!I41</f>
+        <v/>
+      </c>
+      <c r="O38" s="141" t="inlineStr">
+        <is>
+          <t>FYE reference only — bridge uses 10-Q D14</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="100" t="n"/>
@@ -7469,10 +7638,24 @@
       <c r="H39" s="100" t="n"/>
       <c r="I39" s="101" t="n"/>
       <c r="J39" s="100" t="n"/>
-      <c r="L39" s="100" t="n"/>
-      <c r="M39" s="100" t="n"/>
-      <c r="N39" s="100" t="n"/>
-      <c r="O39" s="100" t="n"/>
+      <c r="L39" s="104" t="inlineStr">
+        <is>
+          <t>3S FY25 Debt (ref)</t>
+        </is>
+      </c>
+      <c r="M39" s="143">
+        <f>'3 Statement Model'!I49</f>
+        <v/>
+      </c>
+      <c r="N39" s="143">
+        <f>'3 Statement Model'!I49</f>
+        <v/>
+      </c>
+      <c r="O39" s="141" t="inlineStr">
+        <is>
+          <t>FYE reference only — bridge uses 10-Q D13</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="100" t="n"/>
@@ -7484,31 +7667,43 @@
       <c r="H40" s="101" t="n"/>
       <c r="I40" s="100" t="n"/>
       <c r="K40" s="100" t="n"/>
-      <c r="L40" s="100" t="n"/>
-      <c r="M40" s="100" t="n"/>
-      <c r="N40" s="100" t="n"/>
-      <c r="O40" s="100" t="n"/>
+      <c r="L40" s="104" t="inlineStr">
+        <is>
+          <t>EBIT link OK?</t>
+        </is>
+      </c>
+      <c r="M40" s="140">
+        <f>IF(ABS(M32-M33)&lt;1,"OK","MISMATCH")</f>
+        <v/>
+      </c>
+      <c r="N40" s="146" t="inlineStr"/>
+      <c r="O40" s="141" t="inlineStr">
+        <is>
+          <t>Flags if EBIT link ≠ GP−opex build</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="100" t="n"/>
-      <c r="B41" s="121" t="inlineStr">
+      <c r="B41" s="122" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="C41" s="122" t="n"/>
-      <c r="D41" s="138" t="n"/>
-      <c r="E41" s="122" t="n"/>
-      <c r="F41" s="122" t="n"/>
-      <c r="G41" s="122" t="n"/>
-      <c r="H41" s="122" t="n"/>
-      <c r="I41" s="122" t="n"/>
-      <c r="J41" s="122" t="n"/>
-      <c r="K41" s="122" t="n"/>
-      <c r="L41" s="122" t="n"/>
-      <c r="M41" s="122" t="n"/>
-      <c r="N41" s="122" t="n"/>
-      <c r="O41" s="100" t="n"/>
+      <c r="C41" s="123" t="n"/>
+      <c r="D41" s="147" t="n"/>
+      <c r="E41" s="123" t="n"/>
+      <c r="F41" s="123" t="n"/>
+      <c r="G41" s="123" t="n"/>
+      <c r="H41" s="123" t="n"/>
+      <c r="I41" s="123" t="n"/>
+      <c r="J41" s="123" t="n"/>
+      <c r="K41" s="123" t="n"/>
+      <c r="L41" s="148" t="inlineStr">
+        <is>
+          <t>Green cells are live links. FCFF uses 3S EBIT/D&amp;A/CapEx/ΔNWC. D5 tax = 3S J13. D13/D14 stay 10-Q for a current equity bridge (3S I41/I49 shown above as FY25 reference).</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="100" t="n"/>
@@ -7523,7 +7718,7 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="N42" s="139" t="inlineStr">
+      <c r="N42" s="149" t="inlineStr">
         <is>
           <t>This file is for educational purposes only. E&amp;OE</t>
         </is>
@@ -7548,7 +7743,7 @@
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="140" t="inlineStr">
+      <c r="B44" s="150" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7564,7 +7759,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="140" t="inlineStr">
+      <c r="B45" s="150" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7580,7 +7775,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="140" t="inlineStr">
+      <c r="B46" s="150" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -7615,7 +7810,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="141" t="inlineStr">
+      <c r="N48" s="151" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -7631,7 +7826,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="142" t="inlineStr">
+      <c r="N49" s="152" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -7724,7 +7919,7 @@
       <c r="I55" s="100" t="n"/>
       <c r="J55" s="100" t="n"/>
       <c r="K55" s="100" t="n"/>
-      <c r="L55" s="143" t="inlineStr">
+      <c r="L55" s="136" t="inlineStr">
         <is>
           <t>SENSITIVITY — Enterprise Value ($000s)</t>
         </is>
@@ -7742,27 +7937,27 @@
       <c r="I56" s="100" t="n"/>
       <c r="J56" s="100" t="n"/>
       <c r="K56" s="100" t="n"/>
-      <c r="L56" s="113" t="inlineStr">
+      <c r="L56" s="114" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="144" t="n">
+      <c r="M56" s="153" t="n">
         <v>12.5</v>
       </c>
-      <c r="N56" s="144" t="n">
+      <c r="N56" s="153" t="n">
         <v>15</v>
       </c>
-      <c r="O56" s="144" t="n">
+      <c r="O56" s="153" t="n">
         <v>17.5</v>
       </c>
-      <c r="P56" s="144" t="n">
+      <c r="P56" s="153" t="n">
         <v>20</v>
       </c>
-      <c r="Q56" s="144" t="n">
+      <c r="Q56" s="153" t="n">
         <v>22.5</v>
       </c>
-      <c r="R56" s="144" t="n">
+      <c r="R56" s="153" t="n">
         <v>25</v>
       </c>
     </row>
@@ -7778,30 +7973,30 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="145" t="n">
+      <c r="L57" s="154" t="n">
         <v>0.0824</v>
       </c>
-      <c r="M57" s="146">
+      <c r="M57" s="143">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N57" s="146">
+      <c r="N57" s="143">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O57" s="146">
+      <c r="O57" s="143">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P57" s="146">
+      <c r="P57" s="143">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q57" s="146">
+      <c r="Q57" s="143">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R57" s="146">
+      <c r="R57" s="143">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -7818,30 +8013,30 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="145" t="n">
+      <c r="L58" s="154" t="n">
         <v>0.08740000000000001</v>
       </c>
-      <c r="M58" s="146">
+      <c r="M58" s="143">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N58" s="146">
+      <c r="N58" s="143">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O58" s="146">
+      <c r="O58" s="143">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P58" s="146">
+      <c r="P58" s="143">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q58" s="146">
+      <c r="Q58" s="143">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R58" s="146">
+      <c r="R58" s="143">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -7858,30 +8053,30 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="145" t="n">
+      <c r="L59" s="154" t="n">
         <v>0.0924</v>
       </c>
-      <c r="M59" s="146">
+      <c r="M59" s="143">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N59" s="146">
+      <c r="N59" s="143">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O59" s="147">
+      <c r="O59" s="155">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P59" s="146">
+      <c r="P59" s="143">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q59" s="146">
+      <c r="Q59" s="143">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R59" s="146">
+      <c r="R59" s="143">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -7898,30 +8093,30 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="145" t="n">
+      <c r="L60" s="154" t="n">
         <v>0.0974</v>
       </c>
-      <c r="M60" s="146">
+      <c r="M60" s="143">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N60" s="146">
+      <c r="N60" s="143">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="146">
+      <c r="O60" s="143">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P60" s="146">
+      <c r="P60" s="143">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q60" s="146">
+      <c r="Q60" s="143">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R60" s="146">
+      <c r="R60" s="143">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -7937,226 +8132,228 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="145" t="n">
+      <c r="L61" s="154" t="n">
         <v>0.1024</v>
       </c>
-      <c r="M61" s="146">
+      <c r="M61" s="143">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N61" s="146">
+      <c r="N61" s="143">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O61" s="146">
+      <c r="O61" s="143">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P61" s="146">
+      <c r="P61" s="143">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q61" s="146">
+      <c r="Q61" s="143">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R61" s="146">
+      <c r="R61" s="143">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="148" t="inlineStr">
+      <c r="L64" s="156" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="149" t="inlineStr">
+      <c r="L65" s="157" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="150" t="n">
+      <c r="M65" s="158" t="n">
         <v>12.5</v>
       </c>
-      <c r="N65" s="150" t="n">
+      <c r="N65" s="158" t="n">
         <v>15</v>
       </c>
-      <c r="O65" s="150" t="n">
+      <c r="O65" s="158" t="n">
         <v>17.5</v>
       </c>
-      <c r="P65" s="150" t="n">
+      <c r="P65" s="158" t="n">
         <v>20</v>
       </c>
-      <c r="Q65" s="150" t="n">
+      <c r="Q65" s="158" t="n">
         <v>22.5</v>
       </c>
-      <c r="R65" s="150" t="n">
+      <c r="R65" s="158" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="145" t="n">
+      <c r="L66" s="154" t="n">
         <v>0.0824</v>
       </c>
-      <c r="M66" s="151">
+      <c r="M66" s="159">
         <f>(M57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N66" s="151">
+      <c r="N66" s="159">
         <f>(N57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O66" s="151">
+      <c r="O66" s="159">
         <f>(O57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P66" s="151">
+      <c r="P66" s="159">
         <f>(P57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q66" s="151">
+      <c r="Q66" s="159">
         <f>(Q57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R66" s="151">
+      <c r="R66" s="159">
         <f>(R57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="145" t="n">
+      <c r="L67" s="154" t="n">
         <v>0.08740000000000001</v>
       </c>
-      <c r="M67" s="151">
+      <c r="M67" s="159">
         <f>(M58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N67" s="151">
+      <c r="N67" s="159">
         <f>(N58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O67" s="151">
+      <c r="O67" s="159">
         <f>(O58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P67" s="151">
+      <c r="P67" s="159">
         <f>(P58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q67" s="151">
+      <c r="Q67" s="159">
         <f>(Q58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R67" s="151">
+      <c r="R67" s="159">
         <f>(R58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="145" t="n">
+      <c r="L68" s="154" t="n">
         <v>0.0924</v>
       </c>
-      <c r="M68" s="151">
+      <c r="M68" s="159">
         <f>(M59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N68" s="151">
+      <c r="N68" s="159">
         <f>(N59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O68" s="152">
+      <c r="O68" s="160">
         <f>(O59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P68" s="151">
+      <c r="P68" s="159">
         <f>(P59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q68" s="151">
+      <c r="Q68" s="159">
         <f>(Q59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R68" s="151">
+      <c r="R68" s="159">
         <f>(R59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="145" t="n">
+      <c r="L69" s="154" t="n">
         <v>0.0974</v>
       </c>
-      <c r="M69" s="151">
+      <c r="M69" s="159">
         <f>(M60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N69" s="151">
+      <c r="N69" s="159">
         <f>(N60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O69" s="151">
+      <c r="O69" s="159">
         <f>(O60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P69" s="151">
+      <c r="P69" s="159">
         <f>(P60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q69" s="151">
+      <c r="Q69" s="159">
         <f>(Q60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R69" s="151">
+      <c r="R69" s="159">
         <f>(R60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="145" t="n">
+      <c r="L70" s="154" t="n">
         <v>0.1024</v>
       </c>
-      <c r="M70" s="151">
+      <c r="M70" s="159">
         <f>(M61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N70" s="151">
+      <c r="N70" s="159">
         <f>(N61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O70" s="151">
+      <c r="O70" s="159">
         <f>(O61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P70" s="151">
+      <c r="P70" s="159">
         <f>(P61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q70" s="151">
+      <c r="Q70" s="159">
         <f>(Q61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R70" s="151">
+      <c r="R70" s="159">
         <f>(R61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="153" t="inlineStr">
+      <c r="L72" s="161" t="inlineStr">
         <is>
           <t>Yellow = base (WACC≈9.24%, Exit 17.5x). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 17.5x; bull 25x; bear 12.8x.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="L26:O26"/>
     <mergeCell ref="L55:R55"/>
     <mergeCell ref="L64:R64"/>
     <mergeCell ref="L72:R72"/>
     <mergeCell ref="L24:O24"/>
     <mergeCell ref="L17:N17"/>
     <mergeCell ref="L1:O1"/>
+    <mergeCell ref="L41:O41"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId1"/>

</xml_diff>

<commit_message>
MODEL8: add downloadable Assumptions List PDF linked on every row
Generate a chart-free PDF/MD list of all 3S + DCF assumptions and add
clickable download links on Cover, DCF, and every 3S assumption row (col W).

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -1617,6 +1617,54 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>714374</colOff>
+      <row>3</row>
+      <rowOff>19050</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>661827</colOff>
+      <row>9</row>
+      <rowOff>114300</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Picture 1">
+          <a:hlinkClick r:id="rId1"/>
+        </cNvPr>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1447799" y="762000"/>
+          <a:ext cx="3359943" cy="1581150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
@@ -1670,6 +1718,49 @@
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38101</colOff>
+      <row>131</row>
+      <rowOff>129314</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>783591</colOff>
+      <row>135</row>
+      <rowOff>144144</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Picture 3">
+          <a:hlinkClick r:id="rId1"/>
+        </cNvPr>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="647701" y="5158514"/>
+          <a:ext cx="742950" cy="813659"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
     <clientData/>
   </twoCellAnchor>
 </wsDr>
@@ -2459,6 +2550,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" scale="64"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
MODEL10: rebuild Excel, CSVs, and Assumptions PDF
Regenerate completed workbook with SBC CFO/FCFF add-back, DA% of sales,
flat CapEx, cash tax rate, financing run-rates, and MODEL10_* artifacts.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -37,7 +37,7 @@
     <definedName name="BS_Debt_Start">'3 Statement Model'!$E$49</definedName>
     <definedName name="BS_EquityCapital_Start">'3 Statement Model'!$E$52</definedName>
     <definedName name="BS_RE_Start">'3 Statement Model'!$E$53</definedName>
-    <definedName name="CF_DeltaNWC_Start">'3 Statement Model'!$E$64</definedName>
+    <definedName name="CF_DeltaNWC_Start">'3 Statement Model'!$E$65</definedName>
     <definedName name="CF_Capex_Start">'3 Statement Model'!$E$68</definedName>
     <definedName name="CF_DebtIssuance_Start">'3 Statement Model'!$E$72</definedName>
     <definedName name="CF_EquityIssuance_Start">'3 Statement Model'!$E$73</definedName>
@@ -353,7 +353,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00000000"/>
+      <color rgb="000000FF"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -363,7 +363,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="000000FF"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -441,12 +441,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -539,7 +539,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -720,22 +720,22 @@
     <xf numFmtId="9" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="175" fontId="40" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="176" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="30" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="30" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -743,7 +743,7 @@
     </xf>
     <xf numFmtId="0" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="46" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -751,25 +751,27 @@
     <xf numFmtId="168" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="40" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="38" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="47" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="39" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="47" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="47" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="39" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="5"/>
     </xf>
@@ -783,13 +785,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="38" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="177" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="38" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="38" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1592,15 +1593,16 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>vengeanceaiUSCMODEL9</author>
+    <author>vengeanceaiUSCMODEL10</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
       <text>
-        <t>Tax rate for unlevered FCFF and WACC after-tax Rd.
-HOW: D5 = '3 Statement Model'!J13 (I35/I33 on hist, held in forecast).
-WHY: DCF must use the same t as the 3-statement so NOPAT/FCFF articulate.
-SOURCE: SEC 10-K FY2025 tax / EBT (via 3S hist).</t>
+        <t>Cash tax rate for unlevered FCFF.
+HOW: Yellow POLICY D5 = 22.87% (3yr FY23–25 avg of IncomeTaxesPaidNet ÷ EBT from 10-K).
+WHY: Book tax (~19%) understates cash taxes paid; FCFF should use cash taxes.
+3S row 13 remains book tax for Net Income. WACC after-tax Rd still uses D5.
+SOURCE: SEC companyfacts IncomeTaxesPaidNet / EBT.</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
@@ -6308,7 +6310,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL9 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL10 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6419,17 +6421,16 @@
       <c r="A5" s="100" t="n"/>
       <c r="B5" s="108" t="inlineStr">
         <is>
-          <t>Tax Rate (from 3-Statement J13 = FY25 tax/EBT)</t>
+          <t>Cash Tax Rate (3yr avg IncomeTaxesPaid/EBT = 22.87%)</t>
         </is>
       </c>
       <c r="C5" s="109" t="inlineStr">
         <is>
-          <t>Linked to 3S — do not hardcode</t>
-        </is>
-      </c>
-      <c r="D5" s="110">
-        <f>'3 Statement Model'!J13</f>
-        <v/>
+          <t>MODEL10 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
+        </is>
+      </c>
+      <c r="D5" s="110" t="n">
+        <v>0.22873</v>
       </c>
       <c r="E5" s="103" t="n"/>
       <c r="F5" s="100" t="n"/>
@@ -6825,7 +6826,7 @@
       <c r="K17" s="100" t="n"/>
       <c r="L17" s="126" t="inlineStr">
         <is>
-          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL9)</t>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL10)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -7027,7 +7028,7 @@
       <c r="A22" s="100" t="n"/>
       <c r="B22" s="100" t="inlineStr">
         <is>
-          <t>Less: Unlevered Cash Taxes (EBIT × 3S tax rate)</t>
+          <t>Less: Unlevered Cash Taxes (EBIT × cash tax rate D5)</t>
         </is>
       </c>
       <c r="C22" s="100" t="n"/>
@@ -7194,36 +7195,40 @@
       <c r="A26" s="100" t="n"/>
       <c r="B26" s="100" t="inlineStr">
         <is>
-          <t>Unlevered FCF</t>
-        </is>
-      </c>
-      <c r="C26" s="100" t="n"/>
+          <t>Unlevered FCF (includes SBC add-back from 3S row 64)</t>
+        </is>
+      </c>
+      <c r="C26" s="100" t="inlineStr">
+        <is>
+          <t>FCFF=EBIT−cashTax+DA+SBC−CapEx−ΔNWC</t>
+        </is>
+      </c>
       <c r="D26" s="100" t="n"/>
-      <c r="E26" s="134">
-        <f>E21-E22+E23-E24-E25</f>
-        <v/>
-      </c>
-      <c r="F26" s="134">
-        <f>F21-F22+F23-F24-F25</f>
-        <v/>
-      </c>
-      <c r="G26" s="134">
-        <f>G21-G22+G23-G24-G25</f>
-        <v/>
-      </c>
-      <c r="H26" s="134">
-        <f>H21-H22+H23-H24-H25</f>
-        <v/>
-      </c>
-      <c r="I26" s="134">
-        <f>I21-I22+I23-I24-I25</f>
+      <c r="E26" s="136">
+        <f>E21-E22+E23+'3 Statement Model'!J64-E24-E25</f>
+        <v/>
+      </c>
+      <c r="F26" s="136">
+        <f>F21-F22+F23+'3 Statement Model'!K64-F24-F25</f>
+        <v/>
+      </c>
+      <c r="G26" s="136">
+        <f>G21-G22+G23+'3 Statement Model'!L64-G24-G25</f>
+        <v/>
+      </c>
+      <c r="H26" s="136">
+        <f>H21-H22+H23+'3 Statement Model'!M64-H24-H25</f>
+        <v/>
+      </c>
+      <c r="I26" s="136">
+        <f>I21-I22+I23+'3 Statement Model'!N64-I24-I25</f>
         <v/>
       </c>
       <c r="J26" s="100" t="n"/>
       <c r="K26" s="100" t="n"/>
-      <c r="L26" s="136" t="inlineStr">
-        <is>
-          <t>vengeanceaiUSCMODEL9 — DCF ← 3-Statement linkage audit</t>
+      <c r="L26" s="137" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSCMODEL10 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7249,22 +7254,22 @@
         <v/>
       </c>
       <c r="K27" s="100" t="n"/>
-      <c r="L27" s="137" t="inlineStr">
+      <c r="L27" s="138" t="inlineStr">
         <is>
           <t>DCF item</t>
         </is>
       </c>
-      <c r="M27" s="137" t="inlineStr">
+      <c r="M27" s="138" t="inlineStr">
         <is>
           <t>Value / link</t>
         </is>
       </c>
-      <c r="N27" s="137" t="inlineStr">
+      <c r="N27" s="138" t="inlineStr">
         <is>
           <t>3-Statement source</t>
         </is>
       </c>
-      <c r="O27" s="137" t="inlineStr">
+      <c r="O27" s="138" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -7281,47 +7286,48 @@
       <c r="D28" s="134" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="138">
+      <c r="E28" s="136">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="138">
+      <c r="F28" s="136">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="138">
+      <c r="G28" s="136">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="138">
+      <c r="H28" s="136">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="138">
+      <c r="I28" s="136">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="138">
+      <c r="J28" s="136">
         <f>J27+J26</f>
         <v/>
       </c>
       <c r="K28" s="100" t="n"/>
       <c r="L28" s="104" t="inlineStr">
         <is>
-          <t>Tax rate (D5)</t>
+          <t>Cash tax rate (D5)</t>
         </is>
       </c>
       <c r="M28" s="139">
         <f>$D$5</f>
         <v/>
       </c>
-      <c r="N28" s="140">
-        <f>'3 Statement Model'!J13</f>
-        <v/>
+      <c r="N28" s="140" t="inlineStr">
+        <is>
+          <t>22.87%</t>
+        </is>
       </c>
       <c r="O28" s="141" t="inlineStr">
         <is>
-          <t>Same FY25 effective rate as 3S forecast (I35/I33)</t>
+          <t>3yr avg IncomeTaxesPaidNet/EBT (not book J13)</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7377,7 @@
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="N29" s="140">
+      <c r="N29" s="142">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
@@ -7393,20 +7399,20 @@
       <c r="J30" s="100" t="n"/>
       <c r="L30" s="104" t="inlineStr">
         <is>
-          <t>CapEx % (FY1)</t>
+          <t>SBC % of sales</t>
         </is>
       </c>
       <c r="M30" s="139">
-        <f>'3 Statement Model'!J18</f>
-        <v/>
-      </c>
-      <c r="N30" s="140">
-        <f>'3 Statement Model'!J18</f>
+        <f>'3 Statement Model'!J21</f>
+        <v/>
+      </c>
+      <c r="N30" s="142">
+        <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
       <c r="O30" s="141" t="inlineStr">
         <is>
-          <t>3S CapEx fade path → CF CapEx $</t>
+          <t>SBC add-back in CFO row 64 and FCFF</t>
         </is>
       </c>
     </row>
@@ -7428,22 +7434,22 @@
       <c r="H31" s="123" t="n"/>
       <c r="I31" s="123" t="n"/>
       <c r="J31" s="100" t="n"/>
-      <c r="L31" s="142" t="inlineStr">
-        <is>
-          <t>Revenue growth FY1</t>
+      <c r="L31" s="143" t="inlineStr">
+        <is>
+          <t>CapEx % (FY1)</t>
         </is>
       </c>
       <c r="M31" s="139">
-        <f>'3 Statement Model'!J7</f>
-        <v/>
-      </c>
-      <c r="N31" s="140">
-        <f>'3 Statement Model'!J7</f>
+        <f>'3 Statement Model'!J18</f>
+        <v/>
+      </c>
+      <c r="N31" s="142">
+        <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
       <c r="O31" s="141" t="inlineStr">
         <is>
-          <t>Policy path on 3S assumption row 7</t>
+          <t>Flat 3yr hist avg CapEx% → CF CapEx $</t>
         </is>
       </c>
     </row>
@@ -7473,20 +7479,20 @@
       <c r="J32" s="100" t="n"/>
       <c r="L32" s="104" t="inlineStr">
         <is>
-          <t>EBIT FY1 (DCF E21)</t>
-        </is>
-      </c>
-      <c r="M32" s="143">
-        <f>$E$21</f>
-        <v/>
-      </c>
-      <c r="N32" s="143">
-        <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
+          <t>Revenue growth FY1</t>
+        </is>
+      </c>
+      <c r="M32" s="142">
+        <f>'3 Statement Model'!J7</f>
+        <v/>
+      </c>
+      <c r="N32" s="144">
+        <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
       <c r="O32" s="141" t="inlineStr">
         <is>
-          <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
+          <t>Policy path on 3S assumption row 7</t>
         </is>
       </c>
     </row>
@@ -7516,21 +7522,20 @@
       <c r="J33" s="100" t="n"/>
       <c r="L33" s="104" t="inlineStr">
         <is>
-          <t>EBIT cross-check</t>
-        </is>
-      </c>
-      <c r="M33" s="143">
-        <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
-        <v/>
-      </c>
-      <c r="N33" s="144" t="inlineStr">
-        <is>
-          <t>GP−SGA−R&amp;D−DA</t>
-        </is>
+          <t>EBIT FY1 (DCF E21)</t>
+        </is>
+      </c>
+      <c r="M33" s="145">
+        <f>$E$21</f>
+        <v/>
+      </c>
+      <c r="N33" s="145">
+        <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
+        <v/>
       </c>
       <c r="O33" s="141" t="inlineStr">
         <is>
-          <t>Must equal E21 (live check)</t>
+          <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
         </is>
       </c>
     </row>
@@ -7560,20 +7565,21 @@
       <c r="J34" s="100" t="n"/>
       <c r="L34" s="104" t="inlineStr">
         <is>
-          <t>D&amp;A FY1</t>
-        </is>
-      </c>
-      <c r="M34" s="143">
-        <f>$E$23</f>
-        <v/>
-      </c>
-      <c r="N34" s="143">
-        <f>'3 Statement Model'!J30</f>
-        <v/>
+          <t>EBIT cross-check</t>
+        </is>
+      </c>
+      <c r="M34" s="145">
+        <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
+        <v/>
+      </c>
+      <c r="N34" s="140" t="inlineStr">
+        <is>
+          <t>GP−SGA−R&amp;D−DA</t>
+        </is>
       </c>
       <c r="O34" s="141" t="inlineStr">
         <is>
-          <t>(Open+CapEx/2)×DA% from 3S IS</t>
+          <t>Must equal E21 (live check)</t>
         </is>
       </c>
     </row>
@@ -7601,22 +7607,22 @@
         <v/>
       </c>
       <c r="J35" s="100" t="n"/>
-      <c r="L35" s="142" t="inlineStr">
-        <is>
-          <t>CapEx FY1</t>
-        </is>
-      </c>
-      <c r="M35" s="143">
-        <f>$E$24</f>
-        <v/>
-      </c>
-      <c r="N35" s="143">
-        <f>'3 Statement Model'!J68</f>
+      <c r="L35" s="143" t="inlineStr">
+        <is>
+          <t>D&amp;A FY1</t>
+        </is>
+      </c>
+      <c r="M35" s="145">
+        <f>$E$23</f>
+        <v/>
+      </c>
+      <c r="N35" s="145">
+        <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
       <c r="O35" s="141" t="inlineStr">
         <is>
-          <t>3S CF CapEx (also D15)</t>
+          <t>Rev × DA% (total D&amp;A / sales) from 3S IS</t>
         </is>
       </c>
     </row>
@@ -7628,24 +7634,24 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="145" t="n"/>
+      <c r="I36" s="146" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
-          <t>ΔNWC FY1</t>
-        </is>
-      </c>
-      <c r="M36" s="143">
-        <f>$E$25</f>
-        <v/>
-      </c>
-      <c r="N36" s="143">
-        <f>'3 Statement Model'!J90</f>
+          <t>SBC FY1</t>
+        </is>
+      </c>
+      <c r="M36" s="145">
+        <f>'3 Statement Model'!J64</f>
+        <v/>
+      </c>
+      <c r="N36" s="145">
+        <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
       <c r="O36" s="141" t="inlineStr">
         <is>
-          <t>WC schedule change (CF row 64 = J90)</t>
+          <t>Rev × SBC%; added in FCFF</t>
         </is>
       </c>
     </row>
@@ -7657,7 +7663,7 @@
         </is>
       </c>
       <c r="C37" s="100" t="n"/>
-      <c r="D37" s="145">
+      <c r="D37" s="146">
         <f>D35/D12</f>
         <v/>
       </c>
@@ -7668,27 +7674,27 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="145">
+      <c r="I37" s="146">
         <f>D11</f>
         <v/>
       </c>
       <c r="J37" s="100" t="n"/>
       <c r="L37" s="104" t="inlineStr">
         <is>
-          <t>EBITDA FY5 (TV base)</t>
-        </is>
-      </c>
-      <c r="M37" s="143">
-        <f>$I$21+$I$23</f>
-        <v/>
-      </c>
-      <c r="N37" s="143">
-        <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
+          <t>CapEx FY1</t>
+        </is>
+      </c>
+      <c r="M37" s="145">
+        <f>$E$24</f>
+        <v/>
+      </c>
+      <c r="N37" s="145">
+        <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
       <c r="O37" s="141" t="inlineStr">
         <is>
-          <t>EBIT+D&amp;A; Exit TV = this × D8</t>
+          <t>3S CF CapEx (also D15)</t>
         </is>
       </c>
     </row>
@@ -7704,20 +7710,20 @@
       <c r="J38" s="100" t="n"/>
       <c r="L38" s="104" t="inlineStr">
         <is>
-          <t>3S FY25 Cash (ref)</t>
-        </is>
-      </c>
-      <c r="M38" s="143">
-        <f>'3 Statement Model'!I41</f>
-        <v/>
-      </c>
-      <c r="N38" s="143">
-        <f>'3 Statement Model'!I41</f>
+          <t>ΔNWC FY1</t>
+        </is>
+      </c>
+      <c r="M38" s="145">
+        <f>$E$25</f>
+        <v/>
+      </c>
+      <c r="N38" s="145">
+        <f>'3 Statement Model'!J90</f>
         <v/>
       </c>
       <c r="O38" s="141" t="inlineStr">
         <is>
-          <t>FYE reference only — bridge uses 10-Q D14</t>
+          <t>WC schedule change (CF row 65 = J90)</t>
         </is>
       </c>
     </row>
@@ -7732,20 +7738,20 @@
       <c r="J39" s="100" t="n"/>
       <c r="L39" s="104" t="inlineStr">
         <is>
-          <t>3S FY25 Debt (ref)</t>
-        </is>
-      </c>
-      <c r="M39" s="143">
-        <f>'3 Statement Model'!I49</f>
-        <v/>
-      </c>
-      <c r="N39" s="143">
-        <f>'3 Statement Model'!I49</f>
+          <t>EBITDA FY5 (TV base)</t>
+        </is>
+      </c>
+      <c r="M39" s="145">
+        <f>$I$21+$I$23</f>
+        <v/>
+      </c>
+      <c r="N39" s="145">
+        <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
         <v/>
       </c>
       <c r="O39" s="141" t="inlineStr">
         <is>
-          <t>FYE reference only — bridge uses 10-Q D13</t>
+          <t>EBIT+D&amp;A; Exit TV = this × D8</t>
         </is>
       </c>
     </row>
@@ -7761,17 +7767,20 @@
       <c r="K40" s="100" t="n"/>
       <c r="L40" s="104" t="inlineStr">
         <is>
-          <t>EBIT link OK?</t>
-        </is>
-      </c>
-      <c r="M40" s="140">
-        <f>IF(ABS(M32-M33)&lt;1,"OK","MISMATCH")</f>
-        <v/>
-      </c>
-      <c r="N40" s="146" t="inlineStr"/>
+          <t>3S FY25 Cash (ref)</t>
+        </is>
+      </c>
+      <c r="M40" s="145">
+        <f>'3 Statement Model'!I41</f>
+        <v/>
+      </c>
+      <c r="N40" s="145">
+        <f>'3 Statement Model'!I41</f>
+        <v/>
+      </c>
       <c r="O40" s="141" t="inlineStr">
         <is>
-          <t>Flags if EBIT link ≠ GP−opex build</t>
+          <t>FYE reference only — bridge uses 10-Q D14</t>
         </is>
       </c>
     </row>
@@ -7791,9 +7800,22 @@
       <c r="I41" s="123" t="n"/>
       <c r="J41" s="123" t="n"/>
       <c r="K41" s="123" t="n"/>
-      <c r="L41" s="148" t="inlineStr">
-        <is>
-          <t>Green cells are live links. FCFF uses 3S EBIT/D&amp;A/CapEx/ΔNWC. D5 tax = 3S J13. D13/D14 stay 10-Q for a current equity bridge (3S I41/I49 shown above as FY25 reference).</t>
+      <c r="L41" s="143" t="inlineStr">
+        <is>
+          <t>3S FY25 Debt (ref)</t>
+        </is>
+      </c>
+      <c r="M41" s="145">
+        <f>'3 Statement Model'!I49</f>
+        <v/>
+      </c>
+      <c r="N41" s="145">
+        <f>'3 Statement Model'!I49</f>
+        <v/>
+      </c>
+      <c r="O41" s="141" t="inlineStr">
+        <is>
+          <t>FYE reference only — bridge uses 10-Q D13</t>
         </is>
       </c>
     </row>
@@ -7810,12 +7832,21 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="N42" s="149" t="inlineStr">
-        <is>
-          <t>This file is for educational purposes only. E&amp;OE</t>
-        </is>
-      </c>
-      <c r="O42" s="100" t="n"/>
+      <c r="L42" s="148" t="inlineStr">
+        <is>
+          <t>EBIT link OK?</t>
+        </is>
+      </c>
+      <c r="M42" s="149">
+        <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
+        <v/>
+      </c>
+      <c r="N42" s="150" t="inlineStr"/>
+      <c r="O42" s="141" t="inlineStr">
+        <is>
+          <t>Flags if EBIT link ≠ GP−opex build</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="100" t="n"/>
@@ -7830,12 +7861,15 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="N43" s="69" t="n"/>
-      <c r="O43" s="100" t="n"/>
+      <c r="L43" s="151" t="inlineStr">
+        <is>
+          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔNWC. D5 = historical cash tax rate (not book J13). D13/D14 stay 10-Q for the equity bridge.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="150" t="inlineStr">
+      <c r="B44" s="152" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7851,7 +7885,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="150" t="inlineStr">
+      <c r="B45" s="152" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7867,7 +7901,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="150" t="inlineStr">
+      <c r="B46" s="152" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -7902,7 +7936,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="151" t="inlineStr">
+      <c r="N48" s="153" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -7918,7 +7952,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="152" t="inlineStr">
+      <c r="N49" s="154" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8011,7 +8045,7 @@
       <c r="I55" s="100" t="n"/>
       <c r="J55" s="100" t="n"/>
       <c r="K55" s="100" t="n"/>
-      <c r="L55" s="136" t="inlineStr">
+      <c r="L55" s="137" t="inlineStr">
         <is>
           <t>SENSITIVITY — Enterprise Value ($000s)</t>
         </is>
@@ -8034,22 +8068,22 @@
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="153" t="n">
+      <c r="M56" s="155" t="n">
         <v>12.5</v>
       </c>
-      <c r="N56" s="153" t="n">
+      <c r="N56" s="155" t="n">
         <v>15</v>
       </c>
-      <c r="O56" s="153" t="n">
+      <c r="O56" s="155" t="n">
         <v>17.5</v>
       </c>
-      <c r="P56" s="153" t="n">
+      <c r="P56" s="155" t="n">
         <v>20</v>
       </c>
-      <c r="Q56" s="153" t="n">
+      <c r="Q56" s="155" t="n">
         <v>22.5</v>
       </c>
-      <c r="R56" s="153" t="n">
+      <c r="R56" s="155" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8065,30 +8099,30 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="154" t="n">
+      <c r="L57" s="156" t="n">
         <v>0.0824</v>
       </c>
-      <c r="M57" s="143">
+      <c r="M57" s="145">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N57" s="143">
+      <c r="N57" s="145">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O57" s="143">
+      <c r="O57" s="145">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P57" s="143">
+      <c r="P57" s="145">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q57" s="143">
+      <c r="Q57" s="145">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R57" s="143">
+      <c r="R57" s="145">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8105,30 +8139,30 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="154" t="n">
+      <c r="L58" s="156" t="n">
         <v>0.08740000000000001</v>
       </c>
-      <c r="M58" s="143">
+      <c r="M58" s="145">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N58" s="143">
+      <c r="N58" s="145">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O58" s="143">
+      <c r="O58" s="145">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P58" s="143">
+      <c r="P58" s="145">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q58" s="143">
+      <c r="Q58" s="145">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R58" s="143">
+      <c r="R58" s="145">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8145,30 +8179,30 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="154" t="n">
+      <c r="L59" s="156" t="n">
         <v>0.0924</v>
       </c>
-      <c r="M59" s="143">
+      <c r="M59" s="145">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N59" s="143">
+      <c r="N59" s="145">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O59" s="155">
+      <c r="O59" s="157">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P59" s="143">
+      <c r="P59" s="145">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q59" s="143">
+      <c r="Q59" s="145">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R59" s="143">
+      <c r="R59" s="145">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8185,30 +8219,30 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="154" t="n">
+      <c r="L60" s="156" t="n">
         <v>0.0974</v>
       </c>
-      <c r="M60" s="143">
+      <c r="M60" s="145">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N60" s="143">
+      <c r="N60" s="145">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="143">
+      <c r="O60" s="145">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P60" s="143">
+      <c r="P60" s="145">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q60" s="143">
+      <c r="Q60" s="145">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R60" s="143">
+      <c r="R60" s="145">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8224,213 +8258,213 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="154" t="n">
+      <c r="L61" s="156" t="n">
         <v>0.1024</v>
       </c>
-      <c r="M61" s="143">
+      <c r="M61" s="145">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N61" s="143">
+      <c r="N61" s="145">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O61" s="143">
+      <c r="O61" s="145">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P61" s="143">
+      <c r="P61" s="145">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q61" s="143">
+      <c r="Q61" s="145">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R61" s="143">
+      <c r="R61" s="145">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="156" t="inlineStr">
+      <c r="L64" s="158" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="157" t="inlineStr">
+      <c r="L65" s="159" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="158" t="n">
+      <c r="M65" s="160" t="n">
         <v>12.5</v>
       </c>
-      <c r="N65" s="158" t="n">
+      <c r="N65" s="160" t="n">
         <v>15</v>
       </c>
-      <c r="O65" s="158" t="n">
+      <c r="O65" s="160" t="n">
         <v>17.5</v>
       </c>
-      <c r="P65" s="158" t="n">
+      <c r="P65" s="160" t="n">
         <v>20</v>
       </c>
-      <c r="Q65" s="158" t="n">
+      <c r="Q65" s="160" t="n">
         <v>22.5</v>
       </c>
-      <c r="R65" s="158" t="n">
+      <c r="R65" s="160" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="154" t="n">
+      <c r="L66" s="156" t="n">
         <v>0.0824</v>
       </c>
-      <c r="M66" s="159">
+      <c r="M66" s="161">
         <f>(M57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N66" s="159">
+      <c r="N66" s="161">
         <f>(N57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O66" s="159">
+      <c r="O66" s="161">
         <f>(O57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P66" s="159">
+      <c r="P66" s="161">
         <f>(P57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q66" s="159">
+      <c r="Q66" s="161">
         <f>(Q57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R66" s="159">
+      <c r="R66" s="161">
         <f>(R57+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="154" t="n">
+      <c r="L67" s="156" t="n">
         <v>0.08740000000000001</v>
       </c>
-      <c r="M67" s="159">
+      <c r="M67" s="161">
         <f>(M58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N67" s="159">
+      <c r="N67" s="161">
         <f>(N58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O67" s="159">
+      <c r="O67" s="161">
         <f>(O58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P67" s="159">
+      <c r="P67" s="161">
         <f>(P58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q67" s="159">
+      <c r="Q67" s="161">
         <f>(Q58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R67" s="159">
+      <c r="R67" s="161">
         <f>(R58+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="154" t="n">
+      <c r="L68" s="156" t="n">
         <v>0.0924</v>
       </c>
-      <c r="M68" s="159">
+      <c r="M68" s="161">
         <f>(M59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N68" s="159">
+      <c r="N68" s="161">
         <f>(N59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O68" s="160">
+      <c r="O68" s="162">
         <f>(O59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P68" s="159">
+      <c r="P68" s="161">
         <f>(P59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q68" s="159">
+      <c r="Q68" s="161">
         <f>(Q59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R68" s="159">
+      <c r="R68" s="161">
         <f>(R59+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="154" t="n">
+      <c r="L69" s="156" t="n">
         <v>0.0974</v>
       </c>
-      <c r="M69" s="159">
+      <c r="M69" s="161">
         <f>(M60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N69" s="159">
+      <c r="N69" s="161">
         <f>(N60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O69" s="159">
+      <c r="O69" s="161">
         <f>(O60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P69" s="159">
+      <c r="P69" s="161">
         <f>(P60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q69" s="159">
+      <c r="Q69" s="161">
         <f>(Q60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R69" s="159">
+      <c r="R69" s="161">
         <f>(R60+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="154" t="n">
+      <c r="L70" s="156" t="n">
         <v>0.1024</v>
       </c>
-      <c r="M70" s="159">
+      <c r="M70" s="161">
         <f>(M61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="N70" s="159">
+      <c r="N70" s="161">
         <f>(N61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="O70" s="159">
+      <c r="O70" s="161">
         <f>(O61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="P70" s="159">
+      <c r="P70" s="161">
         <f>(P61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="Q70" s="159">
+      <c r="Q70" s="161">
         <f>(Q61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
-      <c r="R70" s="159">
+      <c r="R70" s="161">
         <f>(R61+$D$33-$D$34)/$D$12</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="161" t="inlineStr">
+      <c r="L72" s="151" t="inlineStr">
         <is>
           <t>Yellow = base (WACC≈9.24%, Exit 17.5x). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 17.5x; bull 25x; bear 12.8x.</t>
         </is>
@@ -8440,12 +8474,12 @@
   <mergeCells count="8">
     <mergeCell ref="L26:O26"/>
     <mergeCell ref="L55:R55"/>
+    <mergeCell ref="L43:O43"/>
     <mergeCell ref="L64:R64"/>
     <mergeCell ref="L72:R72"/>
     <mergeCell ref="L24:O24"/>
     <mergeCell ref="L17:N17"/>
     <mergeCell ref="L1:O1"/>
-    <mergeCell ref="L41:O41"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId1"/>

</xml_diff>

<commit_message>
MODEL11: segment cash conversion, Deferred NWC, SBC share dilution
Disaggregate FY25 10-K revenue mix (SaaS, B2C myFICO, B2B Scores,
Professional Services, on-prem) into blended DSO/COGS drivers that
offset within Total Revenue. Deferred Revenue is a BS liability in
Total Liab and NWC, driven only by SaaS+on-prem mix. DCF shares roll
forward with SBC$/price so Equity Value/Share uses Year-5 diluted
shares. Assumptions PDF/Cover cite the FY2025 10-K and IR filings hub.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -82,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="16">
+  <numFmts count="17">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\(#,##0\)_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.0000_ ;\-0.0000\ "/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -95,10 +95,11 @@
     <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0.00_-;\(#,##0.00\)_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="175" formatCode="0.0"/>
-    <numFmt numFmtId="176" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="177" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="178" formatCode="#,##0.0"/>
-    <numFmt numFmtId="179" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="#,##0.000"/>
+    <numFmt numFmtId="177" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="178" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="179" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="180" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="48">
     <font>
@@ -539,7 +540,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -709,7 +710,7 @@
     </xf>
     <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="33" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="32" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -725,10 +726,10 @@
     </xf>
     <xf numFmtId="164" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -736,6 +737,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -761,8 +763,9 @@
     <xf numFmtId="164" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -781,16 +784,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="177" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="179" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1614,6 +1617,15 @@
 SOURCE (FICO spot): https://www.alphaspread.com/security/nyse/fico/relative-valuation/ratio/enterprise-value-to-ebitda</t>
       </text>
     </comment>
+    <comment ref="D16" authorId="0" shapeId="0">
+      <text>
+        <t>SBC-linked share dilution schedule.
+HOW: D16 = starting shares (D12). Each forecast year adds SBC$000s (3S row 64 = Rev × 8.25%) ÷ Current Price (D11).
+WHY: SBC is added back in FCFF; ignoring dilution overstates $/share.
+Equity Value/Share (D37) and sensitivity use I16 (Year-5 diluted shares).
+SOURCE: 3S SBC row 64; SEC 10-K ShareBasedCompensation.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -6676,10 +6688,14 @@
       <c r="A12" s="100" t="n"/>
       <c r="B12" s="100" t="inlineStr">
         <is>
-          <t>Shares Outstanding</t>
-        </is>
-      </c>
-      <c r="C12" s="100" t="n"/>
+          <t>Shares Outstanding — starting (000s)</t>
+        </is>
+      </c>
+      <c r="C12" s="109" t="inlineStr">
+        <is>
+          <t>Diluted forward via row 16 (SBC$ ÷ Price each year)</t>
+        </is>
+      </c>
       <c r="D12" s="120" t="n">
         <v>20000</v>
       </c>
@@ -6775,9 +6791,40 @@
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="100" t="n"/>
-      <c r="B16" s="100" t="n"/>
-      <c r="C16" s="100" t="n"/>
-      <c r="D16" s="116" t="n"/>
+      <c r="B16" s="100" t="inlineStr">
+        <is>
+          <t>Shares Outstanding — SBC-diluted (000s)</t>
+        </is>
+      </c>
+      <c r="C16" s="109" t="inlineStr">
+        <is>
+          <t>Shares_t = Shares_t−1 + SBC_t($000s) / Price; SBC from 3S row 64</t>
+        </is>
+      </c>
+      <c r="D16" s="122">
+        <f>$D$12</f>
+        <v/>
+      </c>
+      <c r="E16" s="122">
+        <f>D16+'3 Statement Model'!J64/$D$11</f>
+        <v/>
+      </c>
+      <c r="F16" s="122">
+        <f>E16+'3 Statement Model'!K64/$D$11</f>
+        <v/>
+      </c>
+      <c r="G16" s="122">
+        <f>F16+'3 Statement Model'!L64/$D$11</f>
+        <v/>
+      </c>
+      <c r="H16" s="122">
+        <f>G16+'3 Statement Model'!M64/$D$11</f>
+        <v/>
+      </c>
+      <c r="I16" s="122">
+        <f>H16+'3 Statement Model'!N64/$D$11</f>
+        <v/>
+      </c>
       <c r="J16" s="100" t="n"/>
       <c r="K16" s="100" t="n"/>
       <c r="L16" s="100" t="n"/>
@@ -6787,44 +6834,44 @@
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="100" t="n"/>
-      <c r="B17" s="122" t="inlineStr">
+      <c r="B17" s="123" t="inlineStr">
         <is>
           <t>Discounted Cash Flow</t>
         </is>
       </c>
-      <c r="C17" s="123" t="n"/>
-      <c r="D17" s="124" t="inlineStr">
+      <c r="C17" s="124" t="n"/>
+      <c r="D17" s="125" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="E17" s="125">
+      <c r="E17" s="126">
         <f>YEAR(E18)</f>
         <v/>
       </c>
-      <c r="F17" s="125">
+      <c r="F17" s="126">
         <f>YEAR(F18)</f>
         <v/>
       </c>
-      <c r="G17" s="125">
+      <c r="G17" s="126">
         <f>YEAR(G18)</f>
         <v/>
       </c>
-      <c r="H17" s="125">
+      <c r="H17" s="126">
         <f>YEAR(H18)</f>
         <v/>
       </c>
-      <c r="I17" s="125">
+      <c r="I17" s="126">
         <f>YEAR(I18)</f>
         <v/>
       </c>
-      <c r="J17" s="124" t="inlineStr">
+      <c r="J17" s="125" t="inlineStr">
         <is>
           <t>Exit</t>
         </is>
       </c>
       <c r="K17" s="100" t="n"/>
-      <c r="L17" s="126" t="inlineStr">
+      <c r="L17" s="127" t="inlineStr">
         <is>
           <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL11)</t>
         </is>
@@ -6839,31 +6886,31 @@
         </is>
       </c>
       <c r="C18" s="100" t="n"/>
-      <c r="D18" s="127">
+      <c r="D18" s="128">
         <f>$D$9</f>
         <v/>
       </c>
-      <c r="E18" s="127">
+      <c r="E18" s="128">
         <f>EDATE($D$9,(E19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="F18" s="127">
+      <c r="F18" s="128">
         <f>EDATE($D$9,(F19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="G18" s="127">
+      <c r="G18" s="128">
         <f>EDATE($D$9,(G19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="H18" s="127">
+      <c r="H18" s="128">
         <f>EDATE($D$9,(H19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="I18" s="127">
+      <c r="I18" s="128">
         <f>EDATE($D$9,(I19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="J18" s="127">
+      <c r="J18" s="128">
         <f>I18</f>
         <v/>
       </c>
@@ -6886,33 +6933,33 @@
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="100" t="n"/>
-      <c r="B19" s="128" t="inlineStr">
+      <c r="B19" s="129" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="128" t="n"/>
-      <c r="D19" s="129" t="n"/>
-      <c r="E19" s="130" t="n">
+      <c r="C19" s="129" t="n"/>
+      <c r="D19" s="130" t="n"/>
+      <c r="E19" s="131" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="131">
+      <c r="F19" s="132">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="131">
+      <c r="G19" s="132">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="131">
+      <c r="H19" s="132">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="131">
+      <c r="I19" s="132">
         <f>H19+1</f>
         <v/>
       </c>
-      <c r="J19" s="129" t="n"/>
+      <c r="J19" s="130" t="n"/>
       <c r="K19" s="100" t="n"/>
       <c r="L19" s="100" t="inlineStr">
         <is>
@@ -6923,7 +6970,7 @@
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="132" t="inlineStr">
+      <c r="N19" s="133" t="inlineStr">
         <is>
           <t>← sanity check</t>
         </is>
@@ -6932,30 +6979,30 @@
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="100" t="n"/>
-      <c r="B20" s="128" t="inlineStr">
+      <c r="B20" s="129" t="inlineStr">
         <is>
           <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
       <c r="C20" s="100" t="n"/>
       <c r="D20" s="100" t="n"/>
-      <c r="E20" s="133">
+      <c r="E20" s="134">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="133">
+      <c r="F20" s="134">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="133">
+      <c r="G20" s="134">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="133">
+      <c r="H20" s="134">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="133">
+      <c r="I20" s="134">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
@@ -6970,7 +7017,7 @@
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="134" t="inlineStr">
+      <c r="N20" s="135" t="inlineStr">
         <is>
           <t>← ~bear check</t>
         </is>
@@ -7033,23 +7080,23 @@
       </c>
       <c r="C22" s="100" t="n"/>
       <c r="D22" s="100" t="n"/>
-      <c r="E22" s="135">
+      <c r="E22" s="136">
         <f>E21*$D$5</f>
         <v/>
       </c>
-      <c r="F22" s="135">
+      <c r="F22" s="136">
         <f>F21*$D$5</f>
         <v/>
       </c>
-      <c r="G22" s="135">
+      <c r="G22" s="136">
         <f>G21*$D$5</f>
         <v/>
       </c>
-      <c r="H22" s="135">
+      <c r="H22" s="136">
         <f>H21*$D$5</f>
         <v/>
       </c>
-      <c r="I22" s="135">
+      <c r="I22" s="136">
         <f>I21*$D$5</f>
         <v/>
       </c>
@@ -7080,23 +7127,23 @@
       </c>
       <c r="C23" s="100" t="n"/>
       <c r="D23" s="100" t="n"/>
-      <c r="E23" s="135">
+      <c r="E23" s="136">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="135">
+      <c r="F23" s="136">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="135">
+      <c r="G23" s="136">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="135">
+      <c r="H23" s="136">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="135">
+      <c r="I23" s="136">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
@@ -7159,7 +7206,7 @@
       <c r="A25" s="100" t="n"/>
       <c r="B25" s="100" t="inlineStr">
         <is>
-          <t>Less: ΔNWC (3S WC row 90)</t>
+          <t>Less: ΔNWC (3S WC row 90 = AR+Inv−AP−Deferred)</t>
         </is>
       </c>
       <c r="C25" s="100" t="n"/>
@@ -7204,29 +7251,29 @@
         </is>
       </c>
       <c r="D26" s="100" t="n"/>
-      <c r="E26" s="136">
+      <c r="E26" s="137">
         <f>E21-E22+E23+'3 Statement Model'!J64-E24-E25</f>
         <v/>
       </c>
-      <c r="F26" s="136">
+      <c r="F26" s="137">
         <f>F21-F22+F23+'3 Statement Model'!K64-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="136">
+      <c r="G26" s="137">
         <f>G21-G22+G23+'3 Statement Model'!L64-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="136">
+      <c r="H26" s="137">
         <f>H21-H22+H23+'3 Statement Model'!M64-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="136">
+      <c r="I26" s="137">
         <f>I21-I22+I23+'3 Statement Model'!N64-I24-I25</f>
         <v/>
       </c>
       <c r="J26" s="100" t="n"/>
       <c r="K26" s="100" t="n"/>
-      <c r="L26" s="137" t="inlineStr">
+      <c r="L26" s="138" t="inlineStr">
         <is>
           <t>vengeanceaiUSCMODEL11 — DCF ← 3-Statement linkage audit</t>
         </is>
@@ -7254,22 +7301,22 @@
         <v/>
       </c>
       <c r="K27" s="100" t="n"/>
-      <c r="L27" s="138" t="inlineStr">
+      <c r="L27" s="139" t="inlineStr">
         <is>
           <t>DCF item</t>
         </is>
       </c>
-      <c r="M27" s="138" t="inlineStr">
+      <c r="M27" s="139" t="inlineStr">
         <is>
           <t>Value / link</t>
         </is>
       </c>
-      <c r="N27" s="138" t="inlineStr">
+      <c r="N27" s="139" t="inlineStr">
         <is>
           <t>3-Statement source</t>
         </is>
       </c>
-      <c r="O27" s="138" t="inlineStr">
+      <c r="O27" s="139" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -7283,30 +7330,30 @@
         </is>
       </c>
       <c r="C28" s="100" t="n"/>
-      <c r="D28" s="134" t="n">
+      <c r="D28" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="136">
+      <c r="E28" s="137">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="136">
+      <c r="F28" s="137">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="136">
+      <c r="G28" s="137">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="136">
+      <c r="H28" s="137">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="136">
+      <c r="I28" s="137">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="136">
+      <c r="J28" s="137">
         <f>J27+J26</f>
         <v/>
       </c>
@@ -7316,16 +7363,16 @@
           <t>Cash tax rate (D5)</t>
         </is>
       </c>
-      <c r="M28" s="139">
+      <c r="M28" s="140">
         <f>$D$5</f>
         <v/>
       </c>
-      <c r="N28" s="140" t="inlineStr">
+      <c r="N28" s="141" t="inlineStr">
         <is>
           <t>22.87%</t>
         </is>
       </c>
-      <c r="O28" s="141" t="inlineStr">
+      <c r="O28" s="142" t="inlineStr">
         <is>
           <t>3yr avg IncomeTaxesPaidNet/EBT (not book J13)</t>
         </is>
@@ -7373,15 +7420,15 @@
           <t>DSO (AR days)</t>
         </is>
       </c>
-      <c r="M29" s="139">
+      <c r="M29" s="140">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="N29" s="142">
+      <c r="N29" s="143">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="O29" s="141" t="inlineStr">
+      <c r="O29" s="142" t="inlineStr">
         <is>
           <t>AR days driver; NWC = AR+Inv−AP−Def (organic ΔNWC → FCFF)</t>
         </is>
@@ -7402,15 +7449,15 @@
           <t>SBC % of sales</t>
         </is>
       </c>
-      <c r="M30" s="139">
+      <c r="M30" s="140">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="N30" s="142">
+      <c r="N30" s="143">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="O30" s="141" t="inlineStr">
+      <c r="O30" s="142" t="inlineStr">
         <is>
           <t>SBC add-back in CFO row 64 and FCFF</t>
         </is>
@@ -7418,36 +7465,36 @@
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="100" t="n"/>
-      <c r="B31" s="122" t="inlineStr">
+      <c r="B31" s="123" t="inlineStr">
         <is>
           <t>Intrinsic Value</t>
         </is>
       </c>
-      <c r="C31" s="123" t="n"/>
-      <c r="D31" s="123" t="n"/>
+      <c r="C31" s="124" t="n"/>
+      <c r="D31" s="124" t="n"/>
       <c r="E31" s="100" t="n"/>
-      <c r="G31" s="122" t="inlineStr">
+      <c r="G31" s="123" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="H31" s="123" t="n"/>
-      <c r="I31" s="123" t="n"/>
+      <c r="H31" s="124" t="n"/>
+      <c r="I31" s="124" t="n"/>
       <c r="J31" s="100" t="n"/>
-      <c r="L31" s="143" t="inlineStr">
+      <c r="L31" s="144" t="inlineStr">
         <is>
           <t>CapEx % (FY1)</t>
         </is>
       </c>
-      <c r="M31" s="139">
+      <c r="M31" s="140">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="N31" s="142">
+      <c r="N31" s="143">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="O31" s="141" t="inlineStr">
+      <c r="O31" s="142" t="inlineStr">
         <is>
           <t>Flat 3yr hist avg CapEx% → CF CapEx $</t>
         </is>
@@ -7482,15 +7529,15 @@
           <t>Revenue growth FY1</t>
         </is>
       </c>
-      <c r="M32" s="142">
+      <c r="M32" s="143">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="N32" s="144">
+      <c r="N32" s="145">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="O32" s="141" t="inlineStr">
+      <c r="O32" s="142" t="inlineStr">
         <is>
           <t>Policy path on 3S assumption row 7</t>
         </is>
@@ -7525,15 +7572,15 @@
           <t>EBIT FY1 (DCF E21)</t>
         </is>
       </c>
-      <c r="M33" s="145">
+      <c r="M33" s="146">
         <f>$E$21</f>
         <v/>
       </c>
-      <c r="N33" s="145">
+      <c r="N33" s="146">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="O33" s="141" t="inlineStr">
+      <c r="O33" s="142" t="inlineStr">
         <is>
           <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
         </is>
@@ -7568,16 +7615,16 @@
           <t>EBIT cross-check</t>
         </is>
       </c>
-      <c r="M34" s="145">
+      <c r="M34" s="146">
         <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="N34" s="140" t="inlineStr">
+      <c r="N34" s="141" t="inlineStr">
         <is>
           <t>GP−SGA−R&amp;D−DA</t>
         </is>
       </c>
-      <c r="O34" s="141" t="inlineStr">
+      <c r="O34" s="142" t="inlineStr">
         <is>
           <t>Must equal E21 (live check)</t>
         </is>
@@ -7591,7 +7638,7 @@
         </is>
       </c>
       <c r="C35" s="100" t="n"/>
-      <c r="D35" s="134">
+      <c r="D35" s="135">
         <f>D32+D33-D34</f>
         <v/>
       </c>
@@ -7602,25 +7649,25 @@
         </is>
       </c>
       <c r="H35" s="100" t="n"/>
-      <c r="I35" s="134">
+      <c r="I35" s="135">
         <f>I32+I33-I34</f>
         <v/>
       </c>
       <c r="J35" s="100" t="n"/>
-      <c r="L35" s="143" t="inlineStr">
+      <c r="L35" s="144" t="inlineStr">
         <is>
           <t>D&amp;A FY1</t>
         </is>
       </c>
-      <c r="M35" s="145">
+      <c r="M35" s="146">
         <f>$E$23</f>
         <v/>
       </c>
-      <c r="N35" s="145">
+      <c r="N35" s="146">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="O35" s="141" t="inlineStr">
+      <c r="O35" s="142" t="inlineStr">
         <is>
           <t>Rev × DA% (total D&amp;A / sales) from 3S IS</t>
         </is>
@@ -7634,22 +7681,22 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="146" t="n"/>
+      <c r="I36" s="147" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
           <t>SBC FY1</t>
         </is>
       </c>
-      <c r="M36" s="145">
+      <c r="M36" s="146">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="N36" s="145">
+      <c r="N36" s="146">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="O36" s="141" t="inlineStr">
+      <c r="O36" s="142" t="inlineStr">
         <is>
           <t>Rev × SBC%; added in FCFF</t>
         </is>
@@ -7659,12 +7706,16 @@
       <c r="A37" s="100" t="n"/>
       <c r="B37" s="100" t="inlineStr">
         <is>
-          <t>Equity Value/Share</t>
-        </is>
-      </c>
-      <c r="C37" s="100" t="n"/>
-      <c r="D37" s="146">
-        <f>D35/D12</f>
+          <t>Equity Value/Share (÷ Y5 SBC-diluted shares I16)</t>
+        </is>
+      </c>
+      <c r="C37" s="109" t="inlineStr">
+        <is>
+          <t>MODEL11: starting D12 grows with SBC add-back / price</t>
+        </is>
+      </c>
+      <c r="D37" s="148">
+        <f>$D$35/$I$16</f>
         <v/>
       </c>
       <c r="E37" s="100" t="n"/>
@@ -7674,7 +7725,7 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="146">
+      <c r="I37" s="147">
         <f>D11</f>
         <v/>
       </c>
@@ -7684,15 +7735,15 @@
           <t>CapEx FY1</t>
         </is>
       </c>
-      <c r="M37" s="145">
+      <c r="M37" s="146">
         <f>$E$24</f>
         <v/>
       </c>
-      <c r="N37" s="145">
+      <c r="N37" s="146">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="O37" s="141" t="inlineStr">
+      <c r="O37" s="142" t="inlineStr">
         <is>
           <t>3S CF CapEx (also D15)</t>
         </is>
@@ -7713,15 +7764,15 @@
           <t>ΔNWC FY1</t>
         </is>
       </c>
-      <c r="M38" s="145">
+      <c r="M38" s="146">
         <f>$E$25</f>
         <v/>
       </c>
-      <c r="N38" s="145">
+      <c r="N38" s="146">
         <f>'3 Statement Model'!J90</f>
         <v/>
       </c>
-      <c r="O38" s="141" t="inlineStr">
+      <c r="O38" s="142" t="inlineStr">
         <is>
           <t>WC schedule change (CF row 65 = J90)</t>
         </is>
@@ -7741,15 +7792,15 @@
           <t>EBITDA FY5 (TV base)</t>
         </is>
       </c>
-      <c r="M39" s="145">
+      <c r="M39" s="146">
         <f>$I$21+$I$23</f>
         <v/>
       </c>
-      <c r="N39" s="145">
+      <c r="N39" s="146">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
         <v/>
       </c>
-      <c r="O39" s="141" t="inlineStr">
+      <c r="O39" s="142" t="inlineStr">
         <is>
           <t>EBIT+D&amp;A; Exit TV = this × D8</t>
         </is>
@@ -7770,15 +7821,15 @@
           <t>3S FY25 Cash (ref)</t>
         </is>
       </c>
-      <c r="M40" s="145">
+      <c r="M40" s="146">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="N40" s="145">
+      <c r="N40" s="146">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="O40" s="141" t="inlineStr">
+      <c r="O40" s="142" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D14</t>
         </is>
@@ -7786,34 +7837,34 @@
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="100" t="n"/>
-      <c r="B41" s="122" t="inlineStr">
+      <c r="B41" s="123" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="C41" s="123" t="n"/>
-      <c r="D41" s="147" t="n"/>
-      <c r="E41" s="123" t="n"/>
-      <c r="F41" s="123" t="n"/>
-      <c r="G41" s="123" t="n"/>
-      <c r="H41" s="123" t="n"/>
-      <c r="I41" s="123" t="n"/>
-      <c r="J41" s="123" t="n"/>
-      <c r="K41" s="123" t="n"/>
-      <c r="L41" s="143" t="inlineStr">
+      <c r="C41" s="124" t="n"/>
+      <c r="D41" s="149" t="n"/>
+      <c r="E41" s="124" t="n"/>
+      <c r="F41" s="124" t="n"/>
+      <c r="G41" s="124" t="n"/>
+      <c r="H41" s="124" t="n"/>
+      <c r="I41" s="124" t="n"/>
+      <c r="J41" s="124" t="n"/>
+      <c r="K41" s="124" t="n"/>
+      <c r="L41" s="144" t="inlineStr">
         <is>
           <t>3S FY25 Debt (ref)</t>
         </is>
       </c>
-      <c r="M41" s="145">
+      <c r="M41" s="146">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="N41" s="145">
+      <c r="N41" s="146">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="O41" s="141" t="inlineStr">
+      <c r="O41" s="142" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D13</t>
         </is>
@@ -7832,17 +7883,17 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="L42" s="148" t="inlineStr">
+      <c r="L42" s="150" t="inlineStr">
         <is>
           <t>EBIT link OK?</t>
         </is>
       </c>
-      <c r="M42" s="149">
+      <c r="M42" s="151">
         <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
         <v/>
       </c>
-      <c r="N42" s="150" t="inlineStr"/>
-      <c r="O42" s="141" t="inlineStr">
+      <c r="N42" s="152" t="inlineStr"/>
+      <c r="O42" s="142" t="inlineStr">
         <is>
           <t>Flags if EBIT link ≠ GP−opex build</t>
         </is>
@@ -7861,15 +7912,15 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="L43" s="151" t="inlineStr">
-        <is>
-          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔNWC. D5 = historical cash tax rate (not book J13). D13/D14 stay 10-Q for the equity bridge.</t>
+      <c r="L43" s="153" t="inlineStr">
+        <is>
+          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔNWC. D5 = cash tax (not book J13). $/share uses I16 (Y5 SBC-diluted shares), not static D12. D13/D14 stay 10-Q for the equity bridge.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="152" t="inlineStr">
+      <c r="B44" s="154" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7885,7 +7936,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="152" t="inlineStr">
+      <c r="B45" s="154" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7901,7 +7952,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="152" t="inlineStr">
+      <c r="B46" s="154" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -7936,7 +7987,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="153" t="inlineStr">
+      <c r="N48" s="155" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -7952,7 +8003,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="154" t="inlineStr">
+      <c r="N49" s="156" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8045,7 +8096,7 @@
       <c r="I55" s="100" t="n"/>
       <c r="J55" s="100" t="n"/>
       <c r="K55" s="100" t="n"/>
-      <c r="L55" s="137" t="inlineStr">
+      <c r="L55" s="138" t="inlineStr">
         <is>
           <t>SENSITIVITY — Enterprise Value ($000s)</t>
         </is>
@@ -8068,22 +8119,22 @@
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="155" t="n">
+      <c r="M56" s="157" t="n">
         <v>12.5</v>
       </c>
-      <c r="N56" s="155" t="n">
+      <c r="N56" s="157" t="n">
         <v>15</v>
       </c>
-      <c r="O56" s="155" t="n">
+      <c r="O56" s="157" t="n">
         <v>17.5</v>
       </c>
-      <c r="P56" s="155" t="n">
+      <c r="P56" s="157" t="n">
         <v>20</v>
       </c>
-      <c r="Q56" s="155" t="n">
+      <c r="Q56" s="157" t="n">
         <v>22.5</v>
       </c>
-      <c r="R56" s="155" t="n">
+      <c r="R56" s="157" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8099,30 +8150,30 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="156" t="n">
+      <c r="L57" s="158" t="n">
         <v>0.0824</v>
       </c>
-      <c r="M57" s="145">
+      <c r="M57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N57" s="145">
+      <c r="N57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O57" s="145">
+      <c r="O57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P57" s="145">
+      <c r="P57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q57" s="145">
+      <c r="Q57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R57" s="145">
+      <c r="R57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8139,30 +8190,30 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="156" t="n">
+      <c r="L58" s="158" t="n">
         <v>0.08740000000000001</v>
       </c>
-      <c r="M58" s="145">
+      <c r="M58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N58" s="145">
+      <c r="N58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O58" s="145">
+      <c r="O58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P58" s="145">
+      <c r="P58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q58" s="145">
+      <c r="Q58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R58" s="145">
+      <c r="R58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8179,30 +8230,30 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="156" t="n">
+      <c r="L59" s="158" t="n">
         <v>0.0924</v>
       </c>
-      <c r="M59" s="145">
+      <c r="M59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N59" s="145">
+      <c r="N59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O59" s="157">
+      <c r="O59" s="159">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P59" s="145">
+      <c r="P59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q59" s="145">
+      <c r="Q59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R59" s="145">
+      <c r="R59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8219,30 +8270,30 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="156" t="n">
+      <c r="L60" s="158" t="n">
         <v>0.0974</v>
       </c>
-      <c r="M60" s="145">
+      <c r="M60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N60" s="145">
+      <c r="N60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="145">
+      <c r="O60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P60" s="145">
+      <c r="P60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q60" s="145">
+      <c r="Q60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R60" s="145">
+      <c r="R60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8258,213 +8309,213 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="156" t="n">
+      <c r="L61" s="158" t="n">
         <v>0.1024</v>
       </c>
-      <c r="M61" s="145">
+      <c r="M61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N61" s="145">
+      <c r="N61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O61" s="145">
+      <c r="O61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P61" s="145">
+      <c r="P61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q61" s="145">
+      <c r="Q61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R61" s="145">
+      <c r="R61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="158" t="inlineStr">
+      <c r="L64" s="160" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="159" t="inlineStr">
+      <c r="L65" s="161" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="160" t="n">
+      <c r="M65" s="162" t="n">
         <v>12.5</v>
       </c>
-      <c r="N65" s="160" t="n">
+      <c r="N65" s="162" t="n">
         <v>15</v>
       </c>
-      <c r="O65" s="160" t="n">
+      <c r="O65" s="162" t="n">
         <v>17.5</v>
       </c>
-      <c r="P65" s="160" t="n">
+      <c r="P65" s="162" t="n">
         <v>20</v>
       </c>
-      <c r="Q65" s="160" t="n">
+      <c r="Q65" s="162" t="n">
         <v>22.5</v>
       </c>
-      <c r="R65" s="160" t="n">
+      <c r="R65" s="162" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="156" t="n">
+      <c r="L66" s="158" t="n">
         <v>0.0824</v>
       </c>
-      <c r="M66" s="161">
-        <f>(M57+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="N66" s="161">
-        <f>(N57+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="O66" s="161">
-        <f>(O57+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="P66" s="161">
-        <f>(P57+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="Q66" s="161">
-        <f>(Q57+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="R66" s="161">
-        <f>(R57+$D$33-$D$34)/$D$12</f>
+      <c r="M66" s="163">
+        <f>(M57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N66" s="163">
+        <f>(N57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O66" s="163">
+        <f>(O57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P66" s="163">
+        <f>(P57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q66" s="163">
+        <f>(Q57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R66" s="163">
+        <f>(R57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="156" t="n">
+      <c r="L67" s="158" t="n">
         <v>0.08740000000000001</v>
       </c>
-      <c r="M67" s="161">
-        <f>(M58+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="N67" s="161">
-        <f>(N58+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="O67" s="161">
-        <f>(O58+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="P67" s="161">
-        <f>(P58+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="Q67" s="161">
-        <f>(Q58+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="R67" s="161">
-        <f>(R58+$D$33-$D$34)/$D$12</f>
+      <c r="M67" s="163">
+        <f>(M58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N67" s="163">
+        <f>(N58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O67" s="163">
+        <f>(O58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P67" s="163">
+        <f>(P58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q67" s="163">
+        <f>(Q58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R67" s="163">
+        <f>(R58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="156" t="n">
+      <c r="L68" s="158" t="n">
         <v>0.0924</v>
       </c>
-      <c r="M68" s="161">
-        <f>(M59+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="N68" s="161">
-        <f>(N59+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="O68" s="162">
-        <f>(O59+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="P68" s="161">
-        <f>(P59+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="Q68" s="161">
-        <f>(Q59+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="R68" s="161">
-        <f>(R59+$D$33-$D$34)/$D$12</f>
+      <c r="M68" s="163">
+        <f>(M59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N68" s="163">
+        <f>(N59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O68" s="164">
+        <f>(O59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P68" s="163">
+        <f>(P59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q68" s="163">
+        <f>(Q59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R68" s="163">
+        <f>(R59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="156" t="n">
+      <c r="L69" s="158" t="n">
         <v>0.0974</v>
       </c>
-      <c r="M69" s="161">
-        <f>(M60+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="N69" s="161">
-        <f>(N60+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="O69" s="161">
-        <f>(O60+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="P69" s="161">
-        <f>(P60+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="Q69" s="161">
-        <f>(Q60+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="R69" s="161">
-        <f>(R60+$D$33-$D$34)/$D$12</f>
+      <c r="M69" s="163">
+        <f>(M60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N69" s="163">
+        <f>(N60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O69" s="163">
+        <f>(O60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P69" s="163">
+        <f>(P60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q69" s="163">
+        <f>(Q60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R69" s="163">
+        <f>(R60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="156" t="n">
+      <c r="L70" s="158" t="n">
         <v>0.1024</v>
       </c>
-      <c r="M70" s="161">
-        <f>(M61+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="N70" s="161">
-        <f>(N61+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="O70" s="161">
-        <f>(O61+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="P70" s="161">
-        <f>(P61+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="Q70" s="161">
-        <f>(Q61+$D$33-$D$34)/$D$12</f>
-        <v/>
-      </c>
-      <c r="R70" s="161">
-        <f>(R61+$D$33-$D$34)/$D$12</f>
+      <c r="M70" s="163">
+        <f>(M61+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N70" s="163">
+        <f>(N61+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O70" s="163">
+        <f>(O61+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P70" s="163">
+        <f>(P61+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q70" s="163">
+        <f>(Q61+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R70" s="163">
+        <f>(R61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="151" t="inlineStr">
+      <c r="L72" s="153" t="inlineStr">
         <is>
           <t>Yellow = base (WACC≈9.24%, Exit 17.5x). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 17.5x; bull 25x; bear 12.8x.</t>
         </is>

</xml_diff>

<commit_message>
MODEL13 rebuild: phased DSO fix, OpNWC hist, Excel outputs
Fix DSO path (86.6→45d), align hist Op NWC, refresh bake_equations
FCFF labels, and publish MODEL13 CSVs/PDF/xlsx with BS-balanced forecast.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -1596,7 +1596,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>VengeanceUSCModel12.0</author>
+    <author>vengeanceaiUSCMODEL13.0</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
@@ -1608,11 +1608,19 @@
 SOURCE: SEC companyfacts IncomeTaxesPaidNet / EBT.</t>
       </text>
     </comment>
+    <comment ref="D6" authorId="0" shapeId="0">
+      <text>
+        <t>Yacktman AAA-equity discount rate.
+HOW: Yellow POLICY D6 = 7.80% (band 7.5–8.2%). CAPM stack remains at R15 (≈9.24%) as a reference only.
+WHY: Don Yacktman — treat high-quality equities like bonds. FICO's Scores toll-bridge has ultra-low default risk and inflation-protected pricing; CAPM with β≈1.32 misprices the 20–30yr hold.
+SOURCE: Yacktman framework + FICO 10-K Scores pricing commentary.</t>
+      </text>
+    </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
         <t>Exit EV/EBITDA multiple (BASE)
-HOW: Yellow POLICY input D8 = 17.5x; TV = Year-5 EBITDA × D8.
-WHY: Sourced from public peer EV/EBITDA (EFX/VRSK/SPGI/MCO/MSCI). Peer median ≈ 18.1x → base 17.5x (also ≈ 50/50 of bull 25x and bear/Gordon 12.8x). NOT FICO spot (~25–27x).
+HOW: Yellow POLICY input D8 = 21.0x; TV = Year-5 EBITDA × D8.
+WHY: Bond-like perpetual pricing power commands a premium to the public peer median (~18.1x). Raised from MODEL12 17.5x into the 20–22x Yacktman band. Bull 26x / Bear 15.5x. NOT FICO spot (~25–27x).
 SOURCE (peer comps): https://vcpscanner.com/valuation/fico/relative
 SOURCE (FICO spot): https://www.alphaspread.com/security/nyse/fico/relative-valuation/ratio/enterprise-value-to-ebitda</t>
       </text>
@@ -6321,7 +6329,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>VengeanceUSCModel12.0 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL13.0 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6437,7 +6445,7 @@
       </c>
       <c r="C5" s="109" t="inlineStr">
         <is>
-          <t>MODEL12 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
+          <t>MODEL13 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
         </is>
       </c>
       <c r="D5" s="110" t="n">
@@ -6473,12 +6481,16 @@
       <c r="A6" s="100" t="n"/>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>Discount Rate</t>
-        </is>
-      </c>
-      <c r="C6" s="100" t="n"/>
-      <c r="D6" s="111" t="n">
-        <v>0.12</v>
+          <t>Discount Rate (Yacktman AAA-equity WACC = 7.80%; CAPM ref R15≈9.24%)</t>
+        </is>
+      </c>
+      <c r="C6" s="109" t="inlineStr">
+        <is>
+          <t>MODEL13 Yacktman: bond-like Scores monopoly → 7.80% (band 7.5–8.2%); CAPM β≈1.32 overstates LT risk</t>
+        </is>
+      </c>
+      <c r="D6" s="110" t="n">
+        <v>0.078</v>
       </c>
       <c r="E6" s="100" t="n"/>
       <c r="F6" s="100" t="n"/>
@@ -6547,16 +6559,16 @@
       <c r="A8" s="100" t="n"/>
       <c r="B8" s="100" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA (BASE 17.5x — peer comps)</t>
+          <t>Exit EV/EBITDA (BASE 21.0x — Yacktman premium)</t>
         </is>
       </c>
       <c r="C8" s="109" t="inlineStr">
         <is>
-          <t>BASE 17.5x ≈ peer median 18.1x (VCP Scanner). Bull 25x / Bear 12.8x.</t>
+          <t>BASE 21.0x = Yacktman premium vs peer median 18.1x. Bull 26x / Bear 15.5x.</t>
         </is>
       </c>
       <c r="D8" s="112" t="n">
-        <v>17.5</v>
+        <v>21</v>
       </c>
       <c r="E8" s="100" t="n"/>
       <c r="F8" s="113" t="inlineStr">
@@ -6621,11 +6633,11 @@
       </c>
       <c r="M9" s="117" t="n"/>
       <c r="N9" s="118" t="n">
-        <v>17.5</v>
+        <v>21</v>
       </c>
       <c r="O9" s="117" t="inlineStr">
         <is>
-          <t>Near peer median; audit 17.5x</t>
+          <t>Yacktman premium vs peer median; audit 21.0x</t>
         </is>
       </c>
     </row>
@@ -6872,7 +6884,7 @@
       <c r="K17" s="100" t="n"/>
       <c r="L17" s="127" t="inlineStr">
         <is>
-          <t>Terminal value &amp; scenarios (VengeanceUSCModel12.0)</t>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL13.0)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -6916,7 +6928,7 @@
       <c r="K18" s="100" t="n"/>
       <c r="L18" s="100" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA @ D8 (BASE 17.5x)</t>
+          <t>Exit EV/EBITDA @ D8 (BASE 21.0x)</t>
         </is>
       </c>
       <c r="M18" s="121">
@@ -7056,11 +7068,11 @@
       <c r="K21" s="100" t="n"/>
       <c r="L21" s="100" t="inlineStr">
         <is>
-          <t>BASE TV @ 17.5x (primary)</t>
+          <t>BASE TV @ 21.0x (primary)</t>
         </is>
       </c>
       <c r="M21" s="121">
-        <f>($I$21+$I$23)*17.5</f>
+        <f>($I$21+$I$23)*21.0</f>
         <v/>
       </c>
       <c r="N21" s="100" t="inlineStr">
@@ -7103,11 +7115,11 @@
       <c r="K22" s="100" t="n"/>
       <c r="L22" s="100" t="inlineStr">
         <is>
-          <t>BULL TV @ 25.0x (spot/policy)</t>
+          <t>BULL TV @ 26.0x (spot/policy)</t>
         </is>
       </c>
       <c r="M22" s="121">
-        <f>($I$21+$I$23)*25.0</f>
+        <f>($I$21+$I$23)*26.0</f>
         <v/>
       </c>
       <c r="N22" s="100" t="inlineStr">
@@ -7150,11 +7162,11 @@
       <c r="K23" s="100" t="n"/>
       <c r="L23" s="100" t="inlineStr">
         <is>
-          <t>BEAR TV @ 12.8x (Gordon-implied)</t>
+          <t>BEAR TV @ 15.5x (Gordon-implied)</t>
         </is>
       </c>
       <c r="M23" s="121">
-        <f>($I$21+$I$23)*12.8</f>
+        <f>($I$21+$I$23)*15.5</f>
         <v/>
       </c>
       <c r="N23" s="100" t="inlineStr">
@@ -7197,7 +7209,7 @@
       <c r="K24" s="100" t="n"/>
       <c r="L24" s="109" t="inlineStr">
         <is>
-          <t>Reconciliation: Bull 25x → Base 17.5x (peer median ~18.1x) → Bear 12.8x</t>
+          <t>Reconciliation: Bull 26x → Base 21.0x (Yacktman premium vs peer median ~18.1x) → Bear 15.5x</t>
         </is>
       </c>
     </row>
@@ -7205,29 +7217,29 @@
       <c r="A25" s="100" t="n"/>
       <c r="B25" s="100" t="inlineStr">
         <is>
-          <t>Less: ΔNWC (3S WC row 90 = AR+Inv−AP−Deferred)</t>
+          <t>Less: ΔOpNWC − ΔDeferred (3S 90 − 81; AR≠Deferred)</t>
         </is>
       </c>
       <c r="C25" s="100" t="n"/>
       <c r="D25" s="100" t="n"/>
       <c r="E25" s="121">
-        <f>'3 Statement Model'!J90</f>
+        <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
       <c r="F25" s="121">
-        <f>'3 Statement Model'!K90</f>
+        <f>'3 Statement Model'!K90-('3 Statement Model'!K88-'3 Statement Model'!J88)</f>
         <v/>
       </c>
       <c r="G25" s="121">
-        <f>'3 Statement Model'!L90</f>
+        <f>'3 Statement Model'!L90-('3 Statement Model'!L88-'3 Statement Model'!K88)</f>
         <v/>
       </c>
       <c r="H25" s="121">
-        <f>'3 Statement Model'!M90</f>
+        <f>'3 Statement Model'!M90-('3 Statement Model'!M88-'3 Statement Model'!L88)</f>
         <v/>
       </c>
       <c r="I25" s="121">
-        <f>'3 Statement Model'!N90</f>
+        <f>'3 Statement Model'!N90-('3 Statement Model'!N88-'3 Statement Model'!M88)</f>
         <v/>
       </c>
       <c r="J25" s="100" t="n"/>
@@ -7241,12 +7253,12 @@
       <c r="A26" s="100" t="n"/>
       <c r="B26" s="100" t="inlineStr">
         <is>
-          <t>Unlevered FCF (includes SBC add-back from 3S row 64)</t>
+          <t>Unlevered FCF (SBC add-back + Deferred cash source)</t>
         </is>
       </c>
       <c r="C26" s="100" t="inlineStr">
         <is>
-          <t>FCFF=EBIT−cashTax+DA+SBC−CapEx−ΔNWC</t>
+          <t>FCFF=EBIT−cashTax+DA+SBC−CapEx−ΔOpNWC+ΔDeferred</t>
         </is>
       </c>
       <c r="D26" s="100" t="n"/>
@@ -7274,7 +7286,7 @@
       <c r="K26" s="100" t="n"/>
       <c r="L26" s="138" t="inlineStr">
         <is>
-          <t>VengeanceUSCModel12.0 — DCF ← 3-Statement linkage audit</t>
+          <t>vengeanceaiUSCMODEL13.0 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7282,7 +7294,7 @@
       <c r="A27" s="100" t="n"/>
       <c r="B27" s="100" t="inlineStr">
         <is>
-          <t>(Entry)/Exit TV — Exit EV/EBITDA (BASE 17.5x)</t>
+          <t>(Entry)/Exit TV — Exit EV/EBITDA (BASE 21.0x)</t>
         </is>
       </c>
       <c r="C27" s="100" t="n"/>
@@ -7429,7 +7441,7 @@
       </c>
       <c r="O29" s="142" t="inlineStr">
         <is>
-          <t>AR days driver; NWC = AR+Inv−AP−Def (organic ΔNWC → FCFF)</t>
+          <t>Phased DSO hist→45d; Op NWC excludes Deferred</t>
         </is>
       </c>
     </row>
@@ -7495,7 +7507,7 @@
       </c>
       <c r="O31" s="142" t="inlineStr">
         <is>
-          <t>Flat 3yr hist avg CapEx% → CF CapEx $</t>
+          <t>CapEx% fade path → CF CapEx $</t>
         </is>
       </c>
     </row>
@@ -7710,7 +7722,7 @@
       </c>
       <c r="C37" s="109" t="inlineStr">
         <is>
-          <t>MODEL12: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
+          <t>MODEL13: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
         </is>
       </c>
       <c r="D37" s="148">
@@ -7760,7 +7772,7 @@
       <c r="J38" s="100" t="n"/>
       <c r="L38" s="104" t="inlineStr">
         <is>
-          <t>ΔNWC FY1</t>
+          <t>Net WC use FY1</t>
         </is>
       </c>
       <c r="M38" s="146">
@@ -7768,12 +7780,12 @@
         <v/>
       </c>
       <c r="N38" s="146">
-        <f>'3 Statement Model'!J90</f>
+        <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
       <c r="O38" s="142" t="inlineStr">
         <is>
-          <t>WC schedule change (CF row 65 = J90)</t>
+          <t>ΔOpNWC − ΔDeferred (AR≠Deferred)</t>
         </is>
       </c>
     </row>
@@ -7913,7 +7925,7 @@
       <c r="H43" s="100" t="n"/>
       <c r="L43" s="153" t="inlineStr">
         <is>
-          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A(incl. amort) + SBC − CapEx − ΔNWC. D5 = cash tax. $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute shares. D13/D14 stay 10-Q for the equity bridge.</t>
+          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman WACC 7.8%. $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute shares.</t>
         </is>
       </c>
     </row>
@@ -8119,22 +8131,22 @@
         </is>
       </c>
       <c r="M56" s="157" t="n">
-        <v>12.5</v>
+        <v>15.5</v>
       </c>
       <c r="N56" s="157" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O56" s="157" t="n">
-        <v>17.5</v>
+        <v>21</v>
       </c>
       <c r="P56" s="157" t="n">
-        <v>20</v>
+        <v>23.5</v>
       </c>
       <c r="Q56" s="157" t="n">
-        <v>22.5</v>
+        <v>26</v>
       </c>
       <c r="R56" s="157" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
@@ -8150,7 +8162,7 @@
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
       <c r="L57" s="158" t="n">
-        <v>0.0824</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
@@ -8190,7 +8202,7 @@
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
       <c r="L58" s="158" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.074</v>
       </c>
       <c r="M58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
@@ -8230,7 +8242,7 @@
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
       <c r="L59" s="158" t="n">
-        <v>0.0924</v>
+        <v>0.078</v>
       </c>
       <c r="M59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
@@ -8270,7 +8282,7 @@
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
       <c r="L60" s="158" t="n">
-        <v>0.0974</v>
+        <v>0.082</v>
       </c>
       <c r="M60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
@@ -8309,7 +8321,7 @@
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
       <c r="L61" s="158" t="n">
-        <v>0.1024</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="M61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
@@ -8350,27 +8362,27 @@
         </is>
       </c>
       <c r="M65" s="162" t="n">
-        <v>12.5</v>
+        <v>15.5</v>
       </c>
       <c r="N65" s="162" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O65" s="162" t="n">
-        <v>17.5</v>
+        <v>21</v>
       </c>
       <c r="P65" s="162" t="n">
-        <v>20</v>
+        <v>23.5</v>
       </c>
       <c r="Q65" s="162" t="n">
-        <v>22.5</v>
+        <v>26</v>
       </c>
       <c r="R65" s="162" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="66">
       <c r="L66" s="158" t="n">
-        <v>0.0824</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M66" s="163">
         <f>(M57+$D$33-$D$34)/$I$16</f>
@@ -8399,7 +8411,7 @@
     </row>
     <row r="67">
       <c r="L67" s="158" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.074</v>
       </c>
       <c r="M67" s="163">
         <f>(M58+$D$33-$D$34)/$I$16</f>
@@ -8428,7 +8440,7 @@
     </row>
     <row r="68">
       <c r="L68" s="158" t="n">
-        <v>0.0924</v>
+        <v>0.078</v>
       </c>
       <c r="M68" s="163">
         <f>(M59+$D$33-$D$34)/$I$16</f>
@@ -8457,7 +8469,7 @@
     </row>
     <row r="69">
       <c r="L69" s="158" t="n">
-        <v>0.0974</v>
+        <v>0.082</v>
       </c>
       <c r="M69" s="163">
         <f>(M60+$D$33-$D$34)/$I$16</f>
@@ -8486,7 +8498,7 @@
     </row>
     <row r="70">
       <c r="L70" s="158" t="n">
-        <v>0.1024</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="M70" s="163">
         <f>(M61+$D$33-$D$34)/$I$16</f>
@@ -8516,7 +8528,7 @@
     <row r="72">
       <c r="L72" s="153" t="inlineStr">
         <is>
-          <t>Yellow = base (WACC≈9.24%, Exit 17.5x). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 17.5x; bull 25x; bear 12.8x.</t>
+          <t>Yellow = base (Yacktman WACC=7.80%, Exit 21.0x; CAPM ref ≈9.24%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 21.0x; bull 26x; bear 15.5x.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MODEL14 rebuild: publish CSVs/PDF/xlsx with AAA toll-road assumptions
Syntax fix in assumptions export; rebuilt workbook with WACC 7.1%, g 3.5%,
exit 22x, mortgage royalty path, R&D fade, post-Q3 shares; BS balanced.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -95,8 +95,8 @@
     <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0.00_-;\(#,##0.00\)_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="175" formatCode="0.0"/>
-    <numFmt numFmtId="176" formatCode="#,##0.000"/>
-    <numFmt numFmtId="177" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="177" formatCode="#,##0.000"/>
     <numFmt numFmtId="178" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="179" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="180" formatCode="#,##0.0"/>
@@ -540,7 +540,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -718,7 +718,7 @@
     <xf numFmtId="10" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="175" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -730,14 +730,17 @@
     <xf numFmtId="14" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="179" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="177" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -765,7 +768,7 @@
     <xf numFmtId="9" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="180" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -792,8 +795,8 @@
     <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="179" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1596,7 +1599,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>vengeanceaiUSCMODEL13.0</author>
+    <author>vengeanceaiUSCMODEL14.0</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
@@ -1611,16 +1614,16 @@
     <comment ref="D6" authorId="0" shapeId="0">
       <text>
         <t>Yacktman AAA-equity discount rate.
-HOW: Yellow POLICY D6 = 7.80% (band 7.5–8.2%). CAPM stack remains at R15 (≈9.24%) as a reference only.
-WHY: Don Yacktman — treat high-quality equities like bonds. FICO's Scores toll-bridge has ultra-low default risk and inflation-protected pricing; CAPM with β≈1.32 misprices the 20–30yr hold.
-SOURCE: Yacktman framework + FICO 10-K Scores pricing commentary.</t>
+HOW: Yellow POLICY D6 = 7.10% (band 7.0%–7.2%). CAPM stack remains at R15 (≈9.24%) as a reference only.
+WHY: Don Yacktman — treat high-quality equities like bonds. FICO's GSE-mandated Scores toll-bridge is AAA-equivalent cash; MODEL13's 7.8% was still too punitive for a 20–30yr hold.
+SOURCE: Yacktman framework + Q3 FY2026 EX-99.1 / mortgage royalty disclosures.</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
         <t>Exit EV/EBITDA multiple (BASE)
-HOW: Yellow POLICY input D8 = 21.0x; TV = Year-5 EBITDA × D8.
-WHY: Bond-like perpetual pricing power commands a premium to the public peer median (~18.1x). Raised from MODEL12 17.5x into the 20–22x Yacktman band. Bull 26x / Bear 15.5x. NOT FICO spot (~25–27x).
+HOW: Yellow POLICY input D8 = 22.0x; TV = Year-5 EBITDA × D8.
+WHY: AAA toll-road pricing power premium vs peer median (~18.1x). Branch Process: MODEL13 21.0x → MODEL14 22.0x. Bull 27x / Bear 16.0x. NOT FICO spot (~25–27x).
 SOURCE (peer comps): https://vcpscanner.com/valuation/fico/relative
 SOURCE (FICO spot): https://www.alphaspread.com/security/nyse/fico/relative-valuation/ratio/enterprise-value-to-ebitda</t>
       </text>
@@ -1628,9 +1631,9 @@
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>Buyback-adjusted share schedule (Yacktman — no SBC double penalty).
-HOW: D16 = starting shares (D12 = FYE25 23,764k). Each year: Shares += 3S EquityIssuance (row 20) / Price. Row 20 is residual FCF buybacks (negative) so the share count falls.
-WHY: SBC is already added back in FCFF — diluting by SBC$/Price would double-penalize. Massive repurchases ($1.4B in FY25) are the real share-count driver.
-SOURCE: 10-K FY2025 — Repurchases of common stock; shares outstanding.</t>
+HOW: D16 = starting shares (D12 = 21,597.6k post–Q3 FY2026). Price D11 = $1,149 (Q3 avg repurchase). Each year: Shares += 3S EquityIssuance (row 20) / Price. Row 20 is residual FCF buybacks (negative) so the share count falls.
+WHY: SBC is already added back in FCFF — diluting by SBC$/Price would double-penalize. Q3 FY2026 alone: $1.96B / 1.705M shares @ $1,149; FCF $370.3M (EX-99.1).
+SOURCE: SEC EX-99.1 Q3 FY2026; IR earnings release.</t>
       </text>
     </comment>
   </commentList>
@@ -6329,7 +6332,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL13.0 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL14.0 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6445,7 +6448,7 @@
       </c>
       <c r="C5" s="109" t="inlineStr">
         <is>
-          <t>MODEL13 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
+          <t>MODEL14 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
         </is>
       </c>
       <c r="D5" s="110" t="n">
@@ -6481,16 +6484,16 @@
       <c r="A6" s="100" t="n"/>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>Discount Rate (Yacktman AAA-equity WACC = 7.80%; CAPM ref R15≈9.24%)</t>
+          <t>Discount Rate (Yacktman AAA-equity WACC = 7.10%; CAPM ref R15≈9.24%)</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
         <is>
-          <t>MODEL13 Yacktman: bond-like Scores monopoly → 7.80% (band 7.5–8.2%); CAPM β≈1.32 overstates LT risk</t>
+          <t>MODEL14 Yacktman AAA: 7.10% (band 7.0%–7.2%; MODEL13 was 7.8%); CAPM β≈1.32 overstates LT risk</t>
         </is>
       </c>
       <c r="D6" s="110" t="n">
-        <v>0.078</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="E6" s="100" t="n"/>
       <c r="F6" s="100" t="n"/>
@@ -6522,12 +6525,16 @@
       <c r="A7" s="100" t="n"/>
       <c r="B7" s="100" t="inlineStr">
         <is>
-          <t>Perpetural Growth Rate</t>
-        </is>
-      </c>
-      <c r="C7" s="100" t="n"/>
+          <t>Perpetual Growth g = 3.5% (MODEL13 was 3.0% — pricing power &gt; inflation)</t>
+        </is>
+      </c>
+      <c r="C7" s="109" t="inlineStr">
+        <is>
+          <t>Gordon cross-check only; primary TV uses exit multiple D8</t>
+        </is>
+      </c>
       <c r="D7" s="111" t="n">
-        <v>0.03</v>
+        <v>0.035</v>
       </c>
       <c r="E7" s="100" t="n"/>
       <c r="F7" s="100" t="n"/>
@@ -6559,16 +6566,16 @@
       <c r="A8" s="100" t="n"/>
       <c r="B8" s="100" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA (BASE 21.0x — Yacktman premium)</t>
+          <t>Exit EV/EBITDA (BASE 22.0x — Yacktman premium)</t>
         </is>
       </c>
       <c r="C8" s="109" t="inlineStr">
         <is>
-          <t>BASE 21.0x = Yacktman premium vs peer median 18.1x. Bull 26x / Bear 15.5x.</t>
+          <t>BASE 22.0x = Yacktman premium vs peer median 18.1x. Bull 27x / Bear 16.0x.</t>
         </is>
       </c>
       <c r="D8" s="112" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" s="100" t="n"/>
       <c r="F8" s="113" t="inlineStr">
@@ -6633,11 +6640,11 @@
       </c>
       <c r="M9" s="117" t="n"/>
       <c r="N9" s="118" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O9" s="117" t="inlineStr">
         <is>
-          <t>Yacktman premium vs peer median; audit 21.0x</t>
+          <t>Yacktman premium vs peer median; audit 22.0x</t>
         </is>
       </c>
     </row>
@@ -6676,12 +6683,12 @@
       <c r="A11" s="100" t="n"/>
       <c r="B11" s="100" t="inlineStr">
         <is>
-          <t>Current Price</t>
+          <t>Share Price (Q3 FY2026 avg repurchase $1,149)</t>
         </is>
       </c>
       <c r="C11" s="100" t="n"/>
       <c r="D11" s="119" t="n">
-        <v>25</v>
+        <v>1149</v>
       </c>
       <c r="E11" s="100" t="n"/>
       <c r="F11" s="100" t="n"/>
@@ -6699,16 +6706,16 @@
       <c r="A12" s="100" t="n"/>
       <c r="B12" s="100" t="inlineStr">
         <is>
-          <t>Shares Outstanding — starting (000s, FYE25 10-K)</t>
+          <t>Shares Outstanding — starting (000s, post–Q3 FY2026 buybacks)</t>
         </is>
       </c>
       <c r="C12" s="109" t="inlineStr">
         <is>
-          <t>Row 16: buybacks reduce shares; SBC add-back does NOT dilute</t>
+          <t>MODEL14: 21,597.6k after Q3 $1.96B / 1.705M-sh buyback (MODEL13 used 23,764k FYE25)</t>
         </is>
       </c>
       <c r="D12" s="120" t="n">
-        <v>20000</v>
+        <v>21597.635</v>
       </c>
       <c r="E12" s="100" t="n"/>
       <c r="F12" s="100" t="n"/>
@@ -6734,7 +6741,7 @@
           <t>See L39 for 3S FY25 debt ref</t>
         </is>
       </c>
-      <c r="D13" s="120" t="n">
+      <c r="D13" s="121" t="n">
         <v>30000</v>
       </c>
       <c r="E13" s="100" t="n"/>
@@ -6761,7 +6768,7 @@
           <t>See L38 for 3S FY25 cash ref</t>
         </is>
       </c>
-      <c r="D14" s="120" t="n">
+      <c r="D14" s="121" t="n">
         <v>239549.5203651849</v>
       </c>
       <c r="E14" s="100" t="n"/>
@@ -6784,7 +6791,7 @@
         </is>
       </c>
       <c r="C15" s="100" t="n"/>
-      <c r="D15" s="121">
+      <c r="D15" s="122">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
@@ -6812,27 +6819,27 @@
           <t>Shares_t = Shares_t−1 + EquityCF_t/Price; EquityCF = 3S buybacks (row 20, &lt;0)</t>
         </is>
       </c>
-      <c r="D16" s="122">
+      <c r="D16" s="123">
         <f>$D$12</f>
         <v/>
       </c>
-      <c r="E16" s="122">
+      <c r="E16" s="123">
         <f>MAX(1000,D16+'3 Statement Model'!J20/$D$11)</f>
         <v/>
       </c>
-      <c r="F16" s="122">
+      <c r="F16" s="123">
         <f>MAX(1000,E16+'3 Statement Model'!K20/$D$11)</f>
         <v/>
       </c>
-      <c r="G16" s="122">
+      <c r="G16" s="123">
         <f>MAX(1000,F16+'3 Statement Model'!L20/$D$11)</f>
         <v/>
       </c>
-      <c r="H16" s="122">
+      <c r="H16" s="123">
         <f>MAX(1000,G16+'3 Statement Model'!M20/$D$11)</f>
         <v/>
       </c>
-      <c r="I16" s="122">
+      <c r="I16" s="123">
         <f>MAX(1000,H16+'3 Statement Model'!N20/$D$11)</f>
         <v/>
       </c>
@@ -6845,46 +6852,46 @@
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="100" t="n"/>
-      <c r="B17" s="123" t="inlineStr">
+      <c r="B17" s="124" t="inlineStr">
         <is>
           <t>Discounted Cash Flow</t>
         </is>
       </c>
-      <c r="C17" s="124" t="n"/>
-      <c r="D17" s="125" t="inlineStr">
+      <c r="C17" s="125" t="n"/>
+      <c r="D17" s="126" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="E17" s="126">
+      <c r="E17" s="127">
         <f>YEAR(E18)</f>
         <v/>
       </c>
-      <c r="F17" s="126">
+      <c r="F17" s="127">
         <f>YEAR(F18)</f>
         <v/>
       </c>
-      <c r="G17" s="126">
+      <c r="G17" s="127">
         <f>YEAR(G18)</f>
         <v/>
       </c>
-      <c r="H17" s="126">
+      <c r="H17" s="127">
         <f>YEAR(H18)</f>
         <v/>
       </c>
-      <c r="I17" s="126">
+      <c r="I17" s="127">
         <f>YEAR(I18)</f>
         <v/>
       </c>
-      <c r="J17" s="125" t="inlineStr">
+      <c r="J17" s="126" t="inlineStr">
         <is>
           <t>Exit</t>
         </is>
       </c>
       <c r="K17" s="100" t="n"/>
-      <c r="L17" s="127" t="inlineStr">
-        <is>
-          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL13.0)</t>
+      <c r="L17" s="128" t="inlineStr">
+        <is>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL14.0)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -6897,41 +6904,41 @@
         </is>
       </c>
       <c r="C18" s="100" t="n"/>
-      <c r="D18" s="128">
+      <c r="D18" s="129">
         <f>$D$9</f>
         <v/>
       </c>
-      <c r="E18" s="128">
+      <c r="E18" s="129">
         <f>EDATE($D$9,(E19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="F18" s="128">
+      <c r="F18" s="129">
         <f>EDATE($D$9,(F19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="G18" s="128">
+      <c r="G18" s="129">
         <f>EDATE($D$9,(G19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="H18" s="128">
+      <c r="H18" s="129">
         <f>EDATE($D$9,(H19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="I18" s="128">
+      <c r="I18" s="129">
         <f>EDATE($D$9,(I19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="J18" s="128">
+      <c r="J18" s="129">
         <f>I18</f>
         <v/>
       </c>
       <c r="K18" s="100" t="n"/>
       <c r="L18" s="100" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA @ D8 (BASE 21.0x)</t>
-        </is>
-      </c>
-      <c r="M18" s="121">
+          <t>Exit EV/EBITDA @ D8 (BASE 22.0x)</t>
+        </is>
+      </c>
+      <c r="M18" s="122">
         <f>J27</f>
         <v/>
       </c>
@@ -6944,44 +6951,44 @@
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="100" t="n"/>
-      <c r="B19" s="129" t="inlineStr">
+      <c r="B19" s="130" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="129" t="n"/>
-      <c r="D19" s="130" t="n"/>
-      <c r="E19" s="131" t="n">
+      <c r="C19" s="130" t="n"/>
+      <c r="D19" s="131" t="n"/>
+      <c r="E19" s="132" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="132">
+      <c r="F19" s="133">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="132">
+      <c r="G19" s="133">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="132">
+      <c r="H19" s="133">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="132">
+      <c r="I19" s="133">
         <f>H19+1</f>
         <v/>
       </c>
-      <c r="J19" s="130" t="n"/>
+      <c r="J19" s="131" t="n"/>
       <c r="K19" s="100" t="n"/>
       <c r="L19" s="100" t="inlineStr">
         <is>
           <t>Gordon cross-check (g=D7)</t>
         </is>
       </c>
-      <c r="M19" s="121">
+      <c r="M19" s="122">
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="133" t="inlineStr">
+      <c r="N19" s="134" t="inlineStr">
         <is>
           <t>← sanity check</t>
         </is>
@@ -6990,30 +6997,30 @@
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="100" t="n"/>
-      <c r="B20" s="129" t="inlineStr">
+      <c r="B20" s="130" t="inlineStr">
         <is>
           <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
       <c r="C20" s="100" t="n"/>
       <c r="D20" s="100" t="n"/>
-      <c r="E20" s="134">
+      <c r="E20" s="135">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="134">
+      <c r="F20" s="135">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="134">
+      <c r="G20" s="135">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="134">
+      <c r="H20" s="135">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="134">
+      <c r="I20" s="135">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
@@ -7024,11 +7031,11 @@
           <t>Implied Gordon exit multiple</t>
         </is>
       </c>
-      <c r="M20" s="121">
+      <c r="M20" s="122">
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="135" t="inlineStr">
+      <c r="N20" s="136" t="inlineStr">
         <is>
           <t>← ~bear check</t>
         </is>
@@ -7044,23 +7051,23 @@
       </c>
       <c r="C21" s="100" t="n"/>
       <c r="D21" s="100" t="n"/>
-      <c r="E21" s="121">
+      <c r="E21" s="122">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="F21" s="121">
+      <c r="F21" s="122">
         <f>'3 Statement Model'!K33+'3 Statement Model'!K31</f>
         <v/>
       </c>
-      <c r="G21" s="121">
+      <c r="G21" s="122">
         <f>'3 Statement Model'!L33+'3 Statement Model'!L31</f>
         <v/>
       </c>
-      <c r="H21" s="121">
+      <c r="H21" s="122">
         <f>'3 Statement Model'!M33+'3 Statement Model'!M31</f>
         <v/>
       </c>
-      <c r="I21" s="121">
+      <c r="I21" s="122">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31</f>
         <v/>
       </c>
@@ -7068,11 +7075,11 @@
       <c r="K21" s="100" t="n"/>
       <c r="L21" s="100" t="inlineStr">
         <is>
-          <t>BASE TV @ 21.0x (primary)</t>
-        </is>
-      </c>
-      <c r="M21" s="121">
-        <f>($I$21+$I$23)*21.0</f>
+          <t>BASE TV @ 22.0x (primary)</t>
+        </is>
+      </c>
+      <c r="M21" s="122">
+        <f>($I$21+$I$23)*22.0</f>
         <v/>
       </c>
       <c r="N21" s="100" t="inlineStr">
@@ -7091,23 +7098,23 @@
       </c>
       <c r="C22" s="100" t="n"/>
       <c r="D22" s="100" t="n"/>
-      <c r="E22" s="136">
+      <c r="E22" s="137">
         <f>E21*$D$5</f>
         <v/>
       </c>
-      <c r="F22" s="136">
+      <c r="F22" s="137">
         <f>F21*$D$5</f>
         <v/>
       </c>
-      <c r="G22" s="136">
+      <c r="G22" s="137">
         <f>G21*$D$5</f>
         <v/>
       </c>
-      <c r="H22" s="136">
+      <c r="H22" s="137">
         <f>H21*$D$5</f>
         <v/>
       </c>
-      <c r="I22" s="136">
+      <c r="I22" s="137">
         <f>I21*$D$5</f>
         <v/>
       </c>
@@ -7115,11 +7122,11 @@
       <c r="K22" s="100" t="n"/>
       <c r="L22" s="100" t="inlineStr">
         <is>
-          <t>BULL TV @ 26.0x (spot/policy)</t>
-        </is>
-      </c>
-      <c r="M22" s="121">
-        <f>($I$21+$I$23)*26.0</f>
+          <t>BULL TV @ 27.0x (spot/policy)</t>
+        </is>
+      </c>
+      <c r="M22" s="122">
+        <f>($I$21+$I$23)*27.0</f>
         <v/>
       </c>
       <c r="N22" s="100" t="inlineStr">
@@ -7138,23 +7145,23 @@
       </c>
       <c r="C23" s="100" t="n"/>
       <c r="D23" s="100" t="n"/>
-      <c r="E23" s="136">
+      <c r="E23" s="137">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="136">
+      <c r="F23" s="137">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="136">
+      <c r="G23" s="137">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="136">
+      <c r="H23" s="137">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="136">
+      <c r="I23" s="137">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
@@ -7162,11 +7169,11 @@
       <c r="K23" s="100" t="n"/>
       <c r="L23" s="100" t="inlineStr">
         <is>
-          <t>BEAR TV @ 15.5x (Gordon-implied)</t>
-        </is>
-      </c>
-      <c r="M23" s="121">
-        <f>($I$21+$I$23)*15.5</f>
+          <t>BEAR TV @ 16.0x (Gordon-implied)</t>
+        </is>
+      </c>
+      <c r="M23" s="122">
+        <f>($I$21+$I$23)*16.0</f>
         <v/>
       </c>
       <c r="N23" s="100" t="inlineStr">
@@ -7185,23 +7192,23 @@
       </c>
       <c r="C24" s="100" t="n"/>
       <c r="D24" s="100" t="n"/>
-      <c r="E24" s="121">
+      <c r="E24" s="122">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="F24" s="121">
+      <c r="F24" s="122">
         <f>'3 Statement Model'!K68</f>
         <v/>
       </c>
-      <c r="G24" s="121">
+      <c r="G24" s="122">
         <f>'3 Statement Model'!L68</f>
         <v/>
       </c>
-      <c r="H24" s="121">
+      <c r="H24" s="122">
         <f>'3 Statement Model'!M68</f>
         <v/>
       </c>
-      <c r="I24" s="121">
+      <c r="I24" s="122">
         <f>'3 Statement Model'!N68</f>
         <v/>
       </c>
@@ -7209,7 +7216,7 @@
       <c r="K24" s="100" t="n"/>
       <c r="L24" s="109" t="inlineStr">
         <is>
-          <t>Reconciliation: Bull 26x → Base 21.0x (Yacktman premium vs peer median ~18.1x) → Bear 15.5x</t>
+          <t>Reconciliation: Bull 27x → Base 22.0x (Yacktman premium vs peer median ~18.1x) → Bear 16.0x</t>
         </is>
       </c>
     </row>
@@ -7222,23 +7229,23 @@
       </c>
       <c r="C25" s="100" t="n"/>
       <c r="D25" s="100" t="n"/>
-      <c r="E25" s="121">
+      <c r="E25" s="122">
         <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
-      <c r="F25" s="121">
+      <c r="F25" s="122">
         <f>'3 Statement Model'!K90-('3 Statement Model'!K88-'3 Statement Model'!J88)</f>
         <v/>
       </c>
-      <c r="G25" s="121">
+      <c r="G25" s="122">
         <f>'3 Statement Model'!L90-('3 Statement Model'!L88-'3 Statement Model'!K88)</f>
         <v/>
       </c>
-      <c r="H25" s="121">
+      <c r="H25" s="122">
         <f>'3 Statement Model'!M90-('3 Statement Model'!M88-'3 Statement Model'!L88)</f>
         <v/>
       </c>
-      <c r="I25" s="121">
+      <c r="I25" s="122">
         <f>'3 Statement Model'!N90-('3 Statement Model'!N88-'3 Statement Model'!M88)</f>
         <v/>
       </c>
@@ -7262,31 +7269,31 @@
         </is>
       </c>
       <c r="D26" s="100" t="n"/>
-      <c r="E26" s="137">
+      <c r="E26" s="138">
         <f>E21-E22+E23+'3 Statement Model'!J64-E24-E25</f>
         <v/>
       </c>
-      <c r="F26" s="137">
+      <c r="F26" s="138">
         <f>F21-F22+F23+'3 Statement Model'!K64-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="137">
+      <c r="G26" s="138">
         <f>G21-G22+G23+'3 Statement Model'!L64-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="137">
+      <c r="H26" s="138">
         <f>H21-H22+H23+'3 Statement Model'!M64-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="137">
+      <c r="I26" s="138">
         <f>I21-I22+I23+'3 Statement Model'!N64-I24-I25</f>
         <v/>
       </c>
       <c r="J26" s="100" t="n"/>
       <c r="K26" s="100" t="n"/>
-      <c r="L26" s="138" t="inlineStr">
-        <is>
-          <t>vengeanceaiUSCMODEL13.0 — DCF ← 3-Statement linkage audit</t>
+      <c r="L26" s="139" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSCMODEL14.0 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7294,7 +7301,7 @@
       <c r="A27" s="100" t="n"/>
       <c r="B27" s="100" t="inlineStr">
         <is>
-          <t>(Entry)/Exit TV — Exit EV/EBITDA (BASE 21.0x)</t>
+          <t>(Entry)/Exit TV — Exit EV/EBITDA (BASE 22.0x)</t>
         </is>
       </c>
       <c r="C27" s="100" t="n"/>
@@ -7307,27 +7314,27 @@
       <c r="G27" s="100" t="n"/>
       <c r="H27" s="100" t="n"/>
       <c r="I27" s="100" t="n"/>
-      <c r="J27" s="121">
+      <c r="J27" s="122">
         <f>($I$21+$I$23)*$D$8</f>
         <v/>
       </c>
       <c r="K27" s="100" t="n"/>
-      <c r="L27" s="139" t="inlineStr">
+      <c r="L27" s="140" t="inlineStr">
         <is>
           <t>DCF item</t>
         </is>
       </c>
-      <c r="M27" s="139" t="inlineStr">
+      <c r="M27" s="140" t="inlineStr">
         <is>
           <t>Value / link</t>
         </is>
       </c>
-      <c r="N27" s="139" t="inlineStr">
+      <c r="N27" s="140" t="inlineStr">
         <is>
           <t>3-Statement source</t>
         </is>
       </c>
-      <c r="O27" s="139" t="inlineStr">
+      <c r="O27" s="140" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -7341,30 +7348,30 @@
         </is>
       </c>
       <c r="C28" s="100" t="n"/>
-      <c r="D28" s="135" t="n">
+      <c r="D28" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="137">
+      <c r="E28" s="138">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="137">
+      <c r="F28" s="138">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="137">
+      <c r="G28" s="138">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="137">
+      <c r="H28" s="138">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="137">
+      <c r="I28" s="138">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="137">
+      <c r="J28" s="138">
         <f>J27+J26</f>
         <v/>
       </c>
@@ -7374,16 +7381,16 @@
           <t>Cash tax rate (D5)</t>
         </is>
       </c>
-      <c r="M28" s="140">
+      <c r="M28" s="141">
         <f>$D$5</f>
         <v/>
       </c>
-      <c r="N28" s="141" t="inlineStr">
+      <c r="N28" s="142" t="inlineStr">
         <is>
           <t>22.87%</t>
         </is>
       </c>
-      <c r="O28" s="142" t="inlineStr">
+      <c r="O28" s="143" t="inlineStr">
         <is>
           <t>3yr avg IncomeTaxesPaidNet/EBT (not book J13)</t>
         </is>
@@ -7401,27 +7408,27 @@
         <f>D27+D26</f>
         <v/>
       </c>
-      <c r="E29" s="121">
+      <c r="E29" s="122">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F29" s="121">
+      <c r="F29" s="122">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G29" s="121">
+      <c r="G29" s="122">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H29" s="121">
+      <c r="H29" s="122">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I29" s="121">
+      <c r="I29" s="122">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J29" s="121">
+      <c r="J29" s="122">
         <f>J27</f>
         <v/>
       </c>
@@ -7431,15 +7438,15 @@
           <t>DSO (AR days)</t>
         </is>
       </c>
-      <c r="M29" s="140">
+      <c r="M29" s="141">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="N29" s="143">
+      <c r="N29" s="144">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="O29" s="142" t="inlineStr">
+      <c r="O29" s="143" t="inlineStr">
         <is>
           <t>Phased DSO hist→45d; Op NWC excludes Deferred</t>
         </is>
@@ -7460,15 +7467,15 @@
           <t>SBC % of sales</t>
         </is>
       </c>
-      <c r="M30" s="140">
+      <c r="M30" s="141">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="N30" s="143">
+      <c r="N30" s="144">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="O30" s="142" t="inlineStr">
+      <c r="O30" s="143" t="inlineStr">
         <is>
           <t>SBC add-back in CFO row 64 and FCFF</t>
         </is>
@@ -7476,36 +7483,36 @@
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="100" t="n"/>
-      <c r="B31" s="123" t="inlineStr">
+      <c r="B31" s="124" t="inlineStr">
         <is>
           <t>Intrinsic Value</t>
         </is>
       </c>
-      <c r="C31" s="124" t="n"/>
-      <c r="D31" s="124" t="n"/>
+      <c r="C31" s="125" t="n"/>
+      <c r="D31" s="125" t="n"/>
       <c r="E31" s="100" t="n"/>
-      <c r="G31" s="123" t="inlineStr">
+      <c r="G31" s="124" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="H31" s="124" t="n"/>
-      <c r="I31" s="124" t="n"/>
+      <c r="H31" s="125" t="n"/>
+      <c r="I31" s="125" t="n"/>
       <c r="J31" s="100" t="n"/>
-      <c r="L31" s="144" t="inlineStr">
+      <c r="L31" s="145" t="inlineStr">
         <is>
           <t>CapEx % (FY1)</t>
         </is>
       </c>
-      <c r="M31" s="140">
+      <c r="M31" s="141">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="N31" s="143">
+      <c r="N31" s="144">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="O31" s="142" t="inlineStr">
+      <c r="O31" s="143" t="inlineStr">
         <is>
           <t>CapEx% fade path → CF CapEx $</t>
         </is>
@@ -7519,7 +7526,7 @@
         </is>
       </c>
       <c r="C32" s="100" t="n"/>
-      <c r="D32" s="121">
+      <c r="D32" s="122">
         <f>XNPV(D6,D28:J28,D18:J18)</f>
         <v/>
       </c>
@@ -7540,15 +7547,15 @@
           <t>Revenue growth FY1</t>
         </is>
       </c>
-      <c r="M32" s="143">
+      <c r="M32" s="144">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="N32" s="145">
+      <c r="N32" s="146">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="O32" s="142" t="inlineStr">
+      <c r="O32" s="143" t="inlineStr">
         <is>
           <t>Policy path on 3S assumption row 7</t>
         </is>
@@ -7583,15 +7590,15 @@
           <t>EBIT FY1 (DCF E21)</t>
         </is>
       </c>
-      <c r="M33" s="146">
+      <c r="M33" s="147">
         <f>$E$21</f>
         <v/>
       </c>
-      <c r="N33" s="146">
+      <c r="N33" s="147">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="O33" s="142" t="inlineStr">
+      <c r="O33" s="143" t="inlineStr">
         <is>
           <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
         </is>
@@ -7626,16 +7633,16 @@
           <t>EBIT cross-check</t>
         </is>
       </c>
-      <c r="M34" s="146">
+      <c r="M34" s="147">
         <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="N34" s="141" t="inlineStr">
+      <c r="N34" s="142" t="inlineStr">
         <is>
           <t>GP−SGA−R&amp;D−DA</t>
         </is>
       </c>
-      <c r="O34" s="142" t="inlineStr">
+      <c r="O34" s="143" t="inlineStr">
         <is>
           <t>Must equal E21 (live check)</t>
         </is>
@@ -7649,7 +7656,7 @@
         </is>
       </c>
       <c r="C35" s="100" t="n"/>
-      <c r="D35" s="135">
+      <c r="D35" s="136">
         <f>D32+D33-D34</f>
         <v/>
       </c>
@@ -7660,25 +7667,25 @@
         </is>
       </c>
       <c r="H35" s="100" t="n"/>
-      <c r="I35" s="135">
+      <c r="I35" s="136">
         <f>I32+I33-I34</f>
         <v/>
       </c>
       <c r="J35" s="100" t="n"/>
-      <c r="L35" s="144" t="inlineStr">
+      <c r="L35" s="145" t="inlineStr">
         <is>
           <t>D&amp;A FY1</t>
         </is>
       </c>
-      <c r="M35" s="146">
+      <c r="M35" s="147">
         <f>$E$23</f>
         <v/>
       </c>
-      <c r="N35" s="146">
+      <c r="N35" s="147">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="O35" s="142" t="inlineStr">
+      <c r="O35" s="143" t="inlineStr">
         <is>
           <t>Rev × DA% (total D&amp;A / sales) from 3S IS</t>
         </is>
@@ -7692,22 +7699,22 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="147" t="n"/>
+      <c r="I36" s="148" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
           <t>SBC FY1</t>
         </is>
       </c>
-      <c r="M36" s="146">
+      <c r="M36" s="147">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="N36" s="146">
+      <c r="N36" s="147">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="O36" s="142" t="inlineStr">
+      <c r="O36" s="143" t="inlineStr">
         <is>
           <t>Rev × SBC%; added in FCFF</t>
         </is>
@@ -7722,10 +7729,10 @@
       </c>
       <c r="C37" s="109" t="inlineStr">
         <is>
-          <t>MODEL13: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
-        </is>
-      </c>
-      <c r="D37" s="148">
+          <t>MODEL14: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
+        </is>
+      </c>
+      <c r="D37" s="149">
         <f>$D$35/$I$16</f>
         <v/>
       </c>
@@ -7736,7 +7743,7 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="147">
+      <c r="I37" s="148">
         <f>D11</f>
         <v/>
       </c>
@@ -7746,15 +7753,15 @@
           <t>CapEx FY1</t>
         </is>
       </c>
-      <c r="M37" s="146">
+      <c r="M37" s="147">
         <f>$E$24</f>
         <v/>
       </c>
-      <c r="N37" s="146">
+      <c r="N37" s="147">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="O37" s="142" t="inlineStr">
+      <c r="O37" s="143" t="inlineStr">
         <is>
           <t>3S CF CapEx (also D15)</t>
         </is>
@@ -7775,15 +7782,15 @@
           <t>Net WC use FY1</t>
         </is>
       </c>
-      <c r="M38" s="146">
+      <c r="M38" s="147">
         <f>$E$25</f>
         <v/>
       </c>
-      <c r="N38" s="146">
+      <c r="N38" s="147">
         <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
-      <c r="O38" s="142" t="inlineStr">
+      <c r="O38" s="143" t="inlineStr">
         <is>
           <t>ΔOpNWC − ΔDeferred (AR≠Deferred)</t>
         </is>
@@ -7803,15 +7810,15 @@
           <t>EBITDA FY5 (TV base)</t>
         </is>
       </c>
-      <c r="M39" s="146">
+      <c r="M39" s="147">
         <f>$I$21+$I$23</f>
         <v/>
       </c>
-      <c r="N39" s="146">
+      <c r="N39" s="147">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
         <v/>
       </c>
-      <c r="O39" s="142" t="inlineStr">
+      <c r="O39" s="143" t="inlineStr">
         <is>
           <t>EBIT+D&amp;A; Exit TV = this × D8</t>
         </is>
@@ -7832,15 +7839,15 @@
           <t>3S FY25 Cash (ref)</t>
         </is>
       </c>
-      <c r="M40" s="146">
+      <c r="M40" s="147">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="N40" s="146">
+      <c r="N40" s="147">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="O40" s="142" t="inlineStr">
+      <c r="O40" s="143" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D14</t>
         </is>
@@ -7848,34 +7855,34 @@
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="100" t="n"/>
-      <c r="B41" s="123" t="inlineStr">
+      <c r="B41" s="124" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="C41" s="124" t="n"/>
-      <c r="D41" s="149" t="n"/>
-      <c r="E41" s="124" t="n"/>
-      <c r="F41" s="124" t="n"/>
-      <c r="G41" s="124" t="n"/>
-      <c r="H41" s="124" t="n"/>
-      <c r="I41" s="124" t="n"/>
-      <c r="J41" s="124" t="n"/>
-      <c r="K41" s="124" t="n"/>
-      <c r="L41" s="144" t="inlineStr">
+      <c r="C41" s="125" t="n"/>
+      <c r="D41" s="150" t="n"/>
+      <c r="E41" s="125" t="n"/>
+      <c r="F41" s="125" t="n"/>
+      <c r="G41" s="125" t="n"/>
+      <c r="H41" s="125" t="n"/>
+      <c r="I41" s="125" t="n"/>
+      <c r="J41" s="125" t="n"/>
+      <c r="K41" s="125" t="n"/>
+      <c r="L41" s="145" t="inlineStr">
         <is>
           <t>3S FY25 Debt (ref)</t>
         </is>
       </c>
-      <c r="M41" s="146">
+      <c r="M41" s="147">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="N41" s="146">
+      <c r="N41" s="147">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="O41" s="142" t="inlineStr">
+      <c r="O41" s="143" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D13</t>
         </is>
@@ -7894,17 +7901,17 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="L42" s="150" t="inlineStr">
+      <c r="L42" s="151" t="inlineStr">
         <is>
           <t>EBIT link OK?</t>
         </is>
       </c>
-      <c r="M42" s="151">
+      <c r="M42" s="152">
         <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
         <v/>
       </c>
-      <c r="N42" s="152" t="inlineStr"/>
-      <c r="O42" s="142" t="inlineStr">
+      <c r="N42" s="153" t="inlineStr"/>
+      <c r="O42" s="143" t="inlineStr">
         <is>
           <t>Flags if EBIT link ≠ GP−opex build</t>
         </is>
@@ -7923,15 +7930,15 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="L43" s="153" t="inlineStr">
-        <is>
-          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman WACC 7.8%. $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute shares.</t>
+      <c r="L43" s="154" t="inlineStr">
+        <is>
+          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman WACC 7.10%; g=3.5%. $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute shares.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="154" t="inlineStr">
+      <c r="B44" s="155" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7947,7 +7954,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="154" t="inlineStr">
+      <c r="B45" s="155" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7963,7 +7970,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="154" t="inlineStr">
+      <c r="B46" s="155" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -7998,7 +8005,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="155" t="inlineStr">
+      <c r="N48" s="156" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -8014,7 +8021,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="156" t="inlineStr">
+      <c r="N49" s="157" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8107,7 +8114,7 @@
       <c r="I55" s="100" t="n"/>
       <c r="J55" s="100" t="n"/>
       <c r="K55" s="100" t="n"/>
-      <c r="L55" s="138" t="inlineStr">
+      <c r="L55" s="139" t="inlineStr">
         <is>
           <t>SENSITIVITY — Enterprise Value ($000s)</t>
         </is>
@@ -8130,23 +8137,23 @@
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="157" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="N56" s="157" t="n">
-        <v>18</v>
-      </c>
-      <c r="O56" s="157" t="n">
-        <v>21</v>
-      </c>
-      <c r="P56" s="157" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="Q56" s="157" t="n">
-        <v>26</v>
-      </c>
-      <c r="R56" s="157" t="n">
-        <v>28</v>
+      <c r="M56" s="158" t="n">
+        <v>16</v>
+      </c>
+      <c r="N56" s="158" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="O56" s="158" t="n">
+        <v>22</v>
+      </c>
+      <c r="P56" s="158" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="Q56" s="158" t="n">
+        <v>27</v>
+      </c>
+      <c r="R56" s="158" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
@@ -8161,30 +8168,30 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="158" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="M57" s="146">
+      <c r="L57" s="159" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="M57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N57" s="146">
+      <c r="N57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O57" s="146">
+      <c r="O57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P57" s="146">
+      <c r="P57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q57" s="146">
+      <c r="Q57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R57" s="146">
+      <c r="R57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8201,30 +8208,30 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="158" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="M58" s="146">
+      <c r="L58" s="159" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="M58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N58" s="146">
+      <c r="N58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O58" s="146">
+      <c r="O58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P58" s="146">
+      <c r="P58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q58" s="146">
+      <c r="Q58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R58" s="146">
+      <c r="R58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8241,30 +8248,30 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="158" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="M59" s="146">
+      <c r="L59" s="159" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="M59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N59" s="146">
+      <c r="N59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O59" s="159">
+      <c r="O59" s="160">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P59" s="146">
+      <c r="P59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q59" s="146">
+      <c r="Q59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R59" s="146">
+      <c r="R59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8281,30 +8288,30 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="158" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="M60" s="146">
+      <c r="L60" s="159" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="M60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N60" s="146">
+      <c r="N60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="146">
+      <c r="O60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P60" s="146">
+      <c r="P60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q60" s="146">
+      <c r="Q60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R60" s="146">
+      <c r="R60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8320,215 +8327,215 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="158" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="M61" s="146">
+      <c r="L61" s="159" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="M61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N61" s="146">
+      <c r="N61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O61" s="146">
+      <c r="O61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P61" s="146">
+      <c r="P61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q61" s="146">
+      <c r="Q61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R61" s="146">
+      <c r="R61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="160" t="inlineStr">
+      <c r="L64" s="161" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="161" t="inlineStr">
+      <c r="L65" s="162" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="162" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="N65" s="162" t="n">
-        <v>18</v>
-      </c>
-      <c r="O65" s="162" t="n">
-        <v>21</v>
-      </c>
-      <c r="P65" s="162" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="Q65" s="162" t="n">
-        <v>26</v>
-      </c>
-      <c r="R65" s="162" t="n">
-        <v>28</v>
+      <c r="M65" s="163" t="n">
+        <v>16</v>
+      </c>
+      <c r="N65" s="163" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="O65" s="163" t="n">
+        <v>22</v>
+      </c>
+      <c r="P65" s="163" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="Q65" s="163" t="n">
+        <v>27</v>
+      </c>
+      <c r="R65" s="163" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="158" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="M66" s="163">
+      <c r="L66" s="159" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="M66" s="164">
         <f>(M57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N66" s="163">
+      <c r="N66" s="164">
         <f>(N57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O66" s="163">
+      <c r="O66" s="164">
         <f>(O57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P66" s="163">
+      <c r="P66" s="164">
         <f>(P57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q66" s="163">
+      <c r="Q66" s="164">
         <f>(Q57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R66" s="163">
+      <c r="R66" s="164">
         <f>(R57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="158" t="n">
+      <c r="L67" s="159" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="M67" s="164">
+        <f>(M58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N67" s="164">
+        <f>(N58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O67" s="164">
+        <f>(O58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P67" s="164">
+        <f>(P58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q67" s="164">
+        <f>(Q58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R67" s="164">
+        <f>(R58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="L68" s="159" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="M68" s="164">
+        <f>(M59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N68" s="164">
+        <f>(N59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O68" s="165">
+        <f>(O59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P68" s="164">
+        <f>(P59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q68" s="164">
+        <f>(Q59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R68" s="164">
+        <f>(R59+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="L69" s="159" t="n">
         <v>0.074</v>
       </c>
-      <c r="M67" s="163">
-        <f>(M58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="N67" s="163">
-        <f>(N58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="O67" s="163">
-        <f>(O58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="P67" s="163">
-        <f>(P58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="Q67" s="163">
-        <f>(Q58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="R67" s="163">
-        <f>(R58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="L68" s="158" t="n">
+      <c r="M69" s="164">
+        <f>(M60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N69" s="164">
+        <f>(N60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O69" s="164">
+        <f>(O60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P69" s="164">
+        <f>(P60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q69" s="164">
+        <f>(Q60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R69" s="164">
+        <f>(R60+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="L70" s="159" t="n">
         <v>0.078</v>
       </c>
-      <c r="M68" s="163">
-        <f>(M59+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="N68" s="163">
-        <f>(N59+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="O68" s="164">
-        <f>(O59+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="P68" s="163">
-        <f>(P59+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="Q68" s="163">
-        <f>(Q59+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="R68" s="163">
-        <f>(R59+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="L69" s="158" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="M69" s="163">
-        <f>(M60+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="N69" s="163">
-        <f>(N60+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="O69" s="163">
-        <f>(O60+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="P69" s="163">
-        <f>(P60+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="Q69" s="163">
-        <f>(Q60+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="R69" s="163">
-        <f>(R60+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="L70" s="158" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="M70" s="163">
+      <c r="M70" s="164">
         <f>(M61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N70" s="163">
+      <c r="N70" s="164">
         <f>(N61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O70" s="163">
+      <c r="O70" s="164">
         <f>(O61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P70" s="163">
+      <c r="P70" s="164">
         <f>(P61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q70" s="163">
+      <c r="Q70" s="164">
         <f>(Q61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R70" s="163">
+      <c r="R70" s="164">
         <f>(R61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="153" t="inlineStr">
-        <is>
-          <t>Yellow = base (Yacktman WACC=7.80%, Exit 21.0x; CAPM ref ≈9.24%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 21.0x; bull 26x; bear 15.5x.</t>
+      <c r="L72" s="154" t="inlineStr">
+        <is>
+          <t>Yellow = base (Yacktman WACC=7.10%, Exit 22.0x; CAPM ref ≈9.24%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 22.0x; bull 27x; bear 16.0x.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MODEL15 rebuild: publish xlsx, CSVs, and assumptions PDF
Excel-path verification: BS OK / cash check 0 all years; WACC 6.65%,
g 3.75%, exit 23.5x; levered buybacks 1.4×FCF; intrinsic ≈ $6,275/sh.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -540,7 +540,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -716,9 +716,6 @@
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="175" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1599,7 +1596,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>vengeanceaiUSCMODEL14.0</author>
+    <author>vengeanceaiUSCMODEL15.0</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
@@ -1614,16 +1611,16 @@
     <comment ref="D6" authorId="0" shapeId="0">
       <text>
         <t>Yacktman AAA-equity discount rate.
-HOW: Yellow POLICY D6 = 7.10% (band 7.0%–7.2%). CAPM stack remains at R15 (≈9.24%) as a reference only.
-WHY: Don Yacktman — treat high-quality equities like bonds. FICO's GSE-mandated Scores toll-bridge is AAA-equivalent cash; MODEL13's 7.8% was still too punitive for a 20–30yr hold.
-SOURCE: Yacktman framework + Q3 FY2026 EX-99.1 / mortgage royalty disclosures.</t>
+HOW: Yellow POLICY D6 = 6.65% (band 6.5%–6.8%). CAPM stack remains at R15 (≈9.24%) as a reference only.
+WHY: In Model 14, WACC was 7.10%; in Model 15 it is 6.65% (AAA + thin ERP) for GSE-mandated Scores coupons under a 20–30yr Yacktman hold.
+SOURCE: Yacktman framework + Q3 FY2026 EX-99.1 / IR Scores OM ~91%.</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
         <t>Exit EV/EBITDA multiple (BASE)
-HOW: Yellow POLICY input D8 = 22.0x; TV = Year-5 EBITDA × D8.
-WHY: AAA toll-road pricing power premium vs peer median (~18.1x). Branch Process: MODEL13 21.0x → MODEL14 22.0x. Bull 27x / Bear 16.0x. NOT FICO spot (~25–27x).
+HOW: Yellow POLICY input D8 = 23.5x; TV = Year-5 EBITDA × D8.
+WHY: AAA toll-road pricing power premium vs peer median (~18.1x). Branch Process: MODEL14 22.0x → MODEL15 23.5x. Bull 28x / Bear 17.0x. NOT FICO spot (~25–27x).
 SOURCE (peer comps): https://vcpscanner.com/valuation/fico/relative
 SOURCE (FICO spot): https://www.alphaspread.com/security/nyse/fico/relative-valuation/ratio/enterprise-value-to-ebitda</t>
       </text>
@@ -1631,8 +1628,8 @@
     <comment ref="D16" authorId="0" shapeId="0">
       <text>
         <t>Buyback-adjusted share schedule (Yacktman — no SBC double penalty).
-HOW: D16 = starting shares (D12 = 21,597.6k post–Q3 FY2026). Price D11 = $1,149 (Q3 avg repurchase). Each year: Shares += 3S EquityIssuance (row 20) / Price. Row 20 is residual FCF buybacks (negative) so the share count falls.
-WHY: SBC is already added back in FCFF — diluting by SBC$/Price would double-penalize. Q3 FY2026 alone: $1.96B / 1.705M shares @ $1,149; FCF $370.3M (EX-99.1).
+HOW: D16 = starting shares (D12 = 21,597.6k post–Q3 FY2026). Price D11 = $1,149 (Q3 avg repurchase). Each year: Shares += 3S EquityIssuance (row 20) / Price. Row 20 = −1.40×(CFO−CapEx); debt funds the excess so ΔCash≈0.
+WHY: SBC is already added back in FCFF — diluting by SBC$/Price would double-penalize. Q3 FY2026 alone: $1.96B / 1.705M shares @ $1,149; FCF $370.3M (EX-99.1) — buybacks ≫ FCF via leverage.
 SOURCE: SEC EX-99.1 Q3 FY2026; IR earnings release.</t>
       </text>
     </comment>
@@ -6332,7 +6329,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL14.0 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL15.0 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6448,7 +6445,7 @@
       </c>
       <c r="C5" s="109" t="inlineStr">
         <is>
-          <t>MODEL14 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
+          <t>MODEL15 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
         </is>
       </c>
       <c r="D5" s="110" t="n">
@@ -6484,16 +6481,16 @@
       <c r="A6" s="100" t="n"/>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>Discount Rate (Yacktman AAA-equity WACC = 7.10%; CAPM ref R15≈9.24%)</t>
+          <t>Discount Rate (Yacktman AAA-equity WACC = 6.65%; CAPM ref R15≈9.24%)</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
         <is>
-          <t>MODEL14 Yacktman AAA: 7.10% (band 7.0%–7.2%; MODEL13 was 7.8%); CAPM β≈1.32 overstates LT risk</t>
+          <t>MODEL15 Yacktman AAA: 6.65% (band 6.5%–6.8%; MODEL14 was 7.10%); CAPM β≈1.32 overstates LT risk</t>
         </is>
       </c>
       <c r="D6" s="110" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.0665</v>
       </c>
       <c r="E6" s="100" t="n"/>
       <c r="F6" s="100" t="n"/>
@@ -6525,7 +6522,7 @@
       <c r="A7" s="100" t="n"/>
       <c r="B7" s="100" t="inlineStr">
         <is>
-          <t>Perpetual Growth g = 3.5% (MODEL13 was 3.0% — pricing power &gt; inflation)</t>
+          <t>Perpetual Growth g = 3.75% (MODEL14 was 3.5% — pricing power &gt; inflation)</t>
         </is>
       </c>
       <c r="C7" s="109" t="inlineStr">
@@ -6533,8 +6530,8 @@
           <t>Gordon cross-check only; primary TV uses exit multiple D8</t>
         </is>
       </c>
-      <c r="D7" s="111" t="n">
-        <v>0.035</v>
+      <c r="D7" s="110" t="n">
+        <v>0.0375</v>
       </c>
       <c r="E7" s="100" t="n"/>
       <c r="F7" s="100" t="n"/>
@@ -6566,24 +6563,24 @@
       <c r="A8" s="100" t="n"/>
       <c r="B8" s="100" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA (BASE 22.0x — Yacktman premium)</t>
+          <t>Exit EV/EBITDA (BASE 23.5x — Yacktman premium)</t>
         </is>
       </c>
       <c r="C8" s="109" t="inlineStr">
         <is>
-          <t>BASE 22.0x = Yacktman premium vs peer median 18.1x. Bull 27x / Bear 16.0x.</t>
-        </is>
-      </c>
-      <c r="D8" s="112" t="n">
-        <v>22</v>
+          <t>BASE 23.5x = Yacktman premium vs peer median 18.1x. Bull 28x / Bear 17.0x.</t>
+        </is>
+      </c>
+      <c r="D8" s="111" t="n">
+        <v>23.5</v>
       </c>
       <c r="E8" s="100" t="n"/>
-      <c r="F8" s="113" t="inlineStr">
+      <c r="F8" s="112" t="inlineStr">
         <is>
           <t>Peer EV/EBITDA comps (click)</t>
         </is>
       </c>
-      <c r="G8" s="113" t="inlineStr">
+      <c r="G8" s="112" t="inlineStr">
         <is>
           <t>FICO spot EV/EBITDA (click)</t>
         </is>
@@ -6592,20 +6589,20 @@
       <c r="I8" s="100" t="n"/>
       <c r="J8" s="100" t="n"/>
       <c r="K8" s="100" t="n"/>
-      <c r="L8" s="114" t="inlineStr">
+      <c r="L8" s="113" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="M8" s="114" t="inlineStr">
+      <c r="M8" s="113" t="inlineStr">
         <is>
           <t>Peer set</t>
         </is>
       </c>
-      <c r="N8" s="115" t="n">
+      <c r="N8" s="114" t="n">
         <v>18.11</v>
       </c>
-      <c r="O8" s="114" t="inlineStr">
+      <c r="O8" s="113" t="inlineStr">
         <is>
           <t>Sorted median (SPGI)</t>
         </is>
@@ -6623,7 +6620,7 @@
           <t>Matches 3S hist FYE (Sep 30)</t>
         </is>
       </c>
-      <c r="D9" s="116" t="n">
+      <c r="D9" s="115" t="n">
         <v>43100</v>
       </c>
       <c r="E9" s="100" t="n"/>
@@ -6633,18 +6630,18 @@
       <c r="I9" s="100" t="n"/>
       <c r="J9" s="100" t="n"/>
       <c r="K9" s="100" t="n"/>
-      <c r="L9" s="117" t="inlineStr">
+      <c r="L9" s="116" t="inlineStr">
         <is>
           <t>Base exit (D8)</t>
         </is>
       </c>
-      <c r="M9" s="117" t="n"/>
-      <c r="N9" s="118" t="n">
-        <v>22</v>
-      </c>
-      <c r="O9" s="117" t="inlineStr">
-        <is>
-          <t>Yacktman premium vs peer median; audit 22.0x</t>
+      <c r="M9" s="116" t="n"/>
+      <c r="N9" s="117" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="O9" s="116" t="inlineStr">
+        <is>
+          <t>Yacktman premium vs peer median; audit 23.5x</t>
         </is>
       </c>
     </row>
@@ -6656,7 +6653,7 @@
         </is>
       </c>
       <c r="C10" s="100" t="n"/>
-      <c r="D10" s="116" t="n">
+      <c r="D10" s="115" t="n">
         <v>43281</v>
       </c>
       <c r="E10" s="100" t="n"/>
@@ -6666,12 +6663,12 @@
       <c r="I10" s="100" t="n"/>
       <c r="J10" s="100" t="n"/>
       <c r="K10" s="100" t="n"/>
-      <c r="L10" s="113" t="inlineStr">
+      <c r="L10" s="112" t="inlineStr">
         <is>
           <t>Peer comps (click)</t>
         </is>
       </c>
-      <c r="M10" s="113" t="inlineStr">
+      <c r="M10" s="112" t="inlineStr">
         <is>
           <t>FICO spot EV/EBITDA (click)</t>
         </is>
@@ -6687,7 +6684,7 @@
         </is>
       </c>
       <c r="C11" s="100" t="n"/>
-      <c r="D11" s="119" t="n">
+      <c r="D11" s="118" t="n">
         <v>1149</v>
       </c>
       <c r="E11" s="100" t="n"/>
@@ -6711,10 +6708,10 @@
       </c>
       <c r="C12" s="109" t="inlineStr">
         <is>
-          <t>MODEL14: 21,597.6k after Q3 $1.96B / 1.705M-sh buyback (MODEL13 used 23,764k FYE25)</t>
-        </is>
-      </c>
-      <c r="D12" s="120" t="n">
+          <t>MODEL15: 21,597.6k after Q3 $1.96B / 1.705M-sh buyback; levered buybacks 1.4×FCF (MODEL14 was residual ≈1.0×)</t>
+        </is>
+      </c>
+      <c r="D12" s="119" t="n">
         <v>21597.635</v>
       </c>
       <c r="E12" s="100" t="n"/>
@@ -6741,7 +6738,7 @@
           <t>See L39 for 3S FY25 debt ref</t>
         </is>
       </c>
-      <c r="D13" s="121" t="n">
+      <c r="D13" s="120" t="n">
         <v>30000</v>
       </c>
       <c r="E13" s="100" t="n"/>
@@ -6768,7 +6765,7 @@
           <t>See L38 for 3S FY25 cash ref</t>
         </is>
       </c>
-      <c r="D14" s="121" t="n">
+      <c r="D14" s="120" t="n">
         <v>239549.5203651849</v>
       </c>
       <c r="E14" s="100" t="n"/>
@@ -6791,7 +6788,7 @@
         </is>
       </c>
       <c r="C15" s="100" t="n"/>
-      <c r="D15" s="122">
+      <c r="D15" s="121">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
@@ -6819,27 +6816,27 @@
           <t>Shares_t = Shares_t−1 + EquityCF_t/Price; EquityCF = 3S buybacks (row 20, &lt;0)</t>
         </is>
       </c>
-      <c r="D16" s="123">
+      <c r="D16" s="122">
         <f>$D$12</f>
         <v/>
       </c>
-      <c r="E16" s="123">
+      <c r="E16" s="122">
         <f>MAX(1000,D16+'3 Statement Model'!J20/$D$11)</f>
         <v/>
       </c>
-      <c r="F16" s="123">
+      <c r="F16" s="122">
         <f>MAX(1000,E16+'3 Statement Model'!K20/$D$11)</f>
         <v/>
       </c>
-      <c r="G16" s="123">
+      <c r="G16" s="122">
         <f>MAX(1000,F16+'3 Statement Model'!L20/$D$11)</f>
         <v/>
       </c>
-      <c r="H16" s="123">
+      <c r="H16" s="122">
         <f>MAX(1000,G16+'3 Statement Model'!M20/$D$11)</f>
         <v/>
       </c>
-      <c r="I16" s="123">
+      <c r="I16" s="122">
         <f>MAX(1000,H16+'3 Statement Model'!N20/$D$11)</f>
         <v/>
       </c>
@@ -6852,46 +6849,46 @@
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="100" t="n"/>
-      <c r="B17" s="124" t="inlineStr">
+      <c r="B17" s="123" t="inlineStr">
         <is>
           <t>Discounted Cash Flow</t>
         </is>
       </c>
-      <c r="C17" s="125" t="n"/>
-      <c r="D17" s="126" t="inlineStr">
+      <c r="C17" s="124" t="n"/>
+      <c r="D17" s="125" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="E17" s="127">
+      <c r="E17" s="126">
         <f>YEAR(E18)</f>
         <v/>
       </c>
-      <c r="F17" s="127">
+      <c r="F17" s="126">
         <f>YEAR(F18)</f>
         <v/>
       </c>
-      <c r="G17" s="127">
+      <c r="G17" s="126">
         <f>YEAR(G18)</f>
         <v/>
       </c>
-      <c r="H17" s="127">
+      <c r="H17" s="126">
         <f>YEAR(H18)</f>
         <v/>
       </c>
-      <c r="I17" s="127">
+      <c r="I17" s="126">
         <f>YEAR(I18)</f>
         <v/>
       </c>
-      <c r="J17" s="126" t="inlineStr">
+      <c r="J17" s="125" t="inlineStr">
         <is>
           <t>Exit</t>
         </is>
       </c>
       <c r="K17" s="100" t="n"/>
-      <c r="L17" s="128" t="inlineStr">
-        <is>
-          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL14.0)</t>
+      <c r="L17" s="127" t="inlineStr">
+        <is>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL15.0)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -6904,41 +6901,41 @@
         </is>
       </c>
       <c r="C18" s="100" t="n"/>
-      <c r="D18" s="129">
+      <c r="D18" s="128">
         <f>$D$9</f>
         <v/>
       </c>
-      <c r="E18" s="129">
+      <c r="E18" s="128">
         <f>EDATE($D$9,(E19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="F18" s="129">
+      <c r="F18" s="128">
         <f>EDATE($D$9,(F19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="G18" s="129">
+      <c r="G18" s="128">
         <f>EDATE($D$9,(G19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="H18" s="129">
+      <c r="H18" s="128">
         <f>EDATE($D$9,(H19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="I18" s="129">
+      <c r="I18" s="128">
         <f>EDATE($D$9,(I19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="J18" s="129">
+      <c r="J18" s="128">
         <f>I18</f>
         <v/>
       </c>
       <c r="K18" s="100" t="n"/>
       <c r="L18" s="100" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA @ D8 (BASE 22.0x)</t>
-        </is>
-      </c>
-      <c r="M18" s="122">
+          <t>Exit EV/EBITDA @ D8 (BASE 23.5x)</t>
+        </is>
+      </c>
+      <c r="M18" s="121">
         <f>J27</f>
         <v/>
       </c>
@@ -6951,44 +6948,44 @@
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="100" t="n"/>
-      <c r="B19" s="130" t="inlineStr">
+      <c r="B19" s="129" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="130" t="n"/>
-      <c r="D19" s="131" t="n"/>
-      <c r="E19" s="132" t="n">
+      <c r="C19" s="129" t="n"/>
+      <c r="D19" s="130" t="n"/>
+      <c r="E19" s="131" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="133">
+      <c r="F19" s="132">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="133">
+      <c r="G19" s="132">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="133">
+      <c r="H19" s="132">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="133">
+      <c r="I19" s="132">
         <f>H19+1</f>
         <v/>
       </c>
-      <c r="J19" s="131" t="n"/>
+      <c r="J19" s="130" t="n"/>
       <c r="K19" s="100" t="n"/>
       <c r="L19" s="100" t="inlineStr">
         <is>
           <t>Gordon cross-check (g=D7)</t>
         </is>
       </c>
-      <c r="M19" s="122">
+      <c r="M19" s="121">
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="134" t="inlineStr">
+      <c r="N19" s="133" t="inlineStr">
         <is>
           <t>← sanity check</t>
         </is>
@@ -6997,30 +6994,30 @@
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="100" t="n"/>
-      <c r="B20" s="130" t="inlineStr">
+      <c r="B20" s="129" t="inlineStr">
         <is>
           <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
       <c r="C20" s="100" t="n"/>
       <c r="D20" s="100" t="n"/>
-      <c r="E20" s="135">
+      <c r="E20" s="134">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="135">
+      <c r="F20" s="134">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="135">
+      <c r="G20" s="134">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="135">
+      <c r="H20" s="134">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="135">
+      <c r="I20" s="134">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
@@ -7031,11 +7028,11 @@
           <t>Implied Gordon exit multiple</t>
         </is>
       </c>
-      <c r="M20" s="122">
+      <c r="M20" s="121">
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="136" t="inlineStr">
+      <c r="N20" s="135" t="inlineStr">
         <is>
           <t>← ~bear check</t>
         </is>
@@ -7051,23 +7048,23 @@
       </c>
       <c r="C21" s="100" t="n"/>
       <c r="D21" s="100" t="n"/>
-      <c r="E21" s="122">
+      <c r="E21" s="121">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="F21" s="122">
+      <c r="F21" s="121">
         <f>'3 Statement Model'!K33+'3 Statement Model'!K31</f>
         <v/>
       </c>
-      <c r="G21" s="122">
+      <c r="G21" s="121">
         <f>'3 Statement Model'!L33+'3 Statement Model'!L31</f>
         <v/>
       </c>
-      <c r="H21" s="122">
+      <c r="H21" s="121">
         <f>'3 Statement Model'!M33+'3 Statement Model'!M31</f>
         <v/>
       </c>
-      <c r="I21" s="122">
+      <c r="I21" s="121">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31</f>
         <v/>
       </c>
@@ -7075,11 +7072,11 @@
       <c r="K21" s="100" t="n"/>
       <c r="L21" s="100" t="inlineStr">
         <is>
-          <t>BASE TV @ 22.0x (primary)</t>
-        </is>
-      </c>
-      <c r="M21" s="122">
-        <f>($I$21+$I$23)*22.0</f>
+          <t>BASE TV @ 23.5x (primary)</t>
+        </is>
+      </c>
+      <c r="M21" s="121">
+        <f>($I$21+$I$23)*23.5</f>
         <v/>
       </c>
       <c r="N21" s="100" t="inlineStr">
@@ -7098,23 +7095,23 @@
       </c>
       <c r="C22" s="100" t="n"/>
       <c r="D22" s="100" t="n"/>
-      <c r="E22" s="137">
+      <c r="E22" s="136">
         <f>E21*$D$5</f>
         <v/>
       </c>
-      <c r="F22" s="137">
+      <c r="F22" s="136">
         <f>F21*$D$5</f>
         <v/>
       </c>
-      <c r="G22" s="137">
+      <c r="G22" s="136">
         <f>G21*$D$5</f>
         <v/>
       </c>
-      <c r="H22" s="137">
+      <c r="H22" s="136">
         <f>H21*$D$5</f>
         <v/>
       </c>
-      <c r="I22" s="137">
+      <c r="I22" s="136">
         <f>I21*$D$5</f>
         <v/>
       </c>
@@ -7122,11 +7119,11 @@
       <c r="K22" s="100" t="n"/>
       <c r="L22" s="100" t="inlineStr">
         <is>
-          <t>BULL TV @ 27.0x (spot/policy)</t>
-        </is>
-      </c>
-      <c r="M22" s="122">
-        <f>($I$21+$I$23)*27.0</f>
+          <t>BULL TV @ 28.0x (spot/policy)</t>
+        </is>
+      </c>
+      <c r="M22" s="121">
+        <f>($I$21+$I$23)*28.0</f>
         <v/>
       </c>
       <c r="N22" s="100" t="inlineStr">
@@ -7145,23 +7142,23 @@
       </c>
       <c r="C23" s="100" t="n"/>
       <c r="D23" s="100" t="n"/>
-      <c r="E23" s="137">
+      <c r="E23" s="136">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="137">
+      <c r="F23" s="136">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="137">
+      <c r="G23" s="136">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="137">
+      <c r="H23" s="136">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="137">
+      <c r="I23" s="136">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
@@ -7169,11 +7166,11 @@
       <c r="K23" s="100" t="n"/>
       <c r="L23" s="100" t="inlineStr">
         <is>
-          <t>BEAR TV @ 16.0x (Gordon-implied)</t>
-        </is>
-      </c>
-      <c r="M23" s="122">
-        <f>($I$21+$I$23)*16.0</f>
+          <t>BEAR TV @ 17.0x (Gordon-implied)</t>
+        </is>
+      </c>
+      <c r="M23" s="121">
+        <f>($I$21+$I$23)*17.0</f>
         <v/>
       </c>
       <c r="N23" s="100" t="inlineStr">
@@ -7192,23 +7189,23 @@
       </c>
       <c r="C24" s="100" t="n"/>
       <c r="D24" s="100" t="n"/>
-      <c r="E24" s="122">
+      <c r="E24" s="121">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="F24" s="122">
+      <c r="F24" s="121">
         <f>'3 Statement Model'!K68</f>
         <v/>
       </c>
-      <c r="G24" s="122">
+      <c r="G24" s="121">
         <f>'3 Statement Model'!L68</f>
         <v/>
       </c>
-      <c r="H24" s="122">
+      <c r="H24" s="121">
         <f>'3 Statement Model'!M68</f>
         <v/>
       </c>
-      <c r="I24" s="122">
+      <c r="I24" s="121">
         <f>'3 Statement Model'!N68</f>
         <v/>
       </c>
@@ -7216,7 +7213,7 @@
       <c r="K24" s="100" t="n"/>
       <c r="L24" s="109" t="inlineStr">
         <is>
-          <t>Reconciliation: Bull 27x → Base 22.0x (Yacktman premium vs peer median ~18.1x) → Bear 16.0x</t>
+          <t>Reconciliation: Bull 28x → Base 23.5x (Yacktman premium vs peer median ~18.1x) → Bear 17.0x</t>
         </is>
       </c>
     </row>
@@ -7229,23 +7226,23 @@
       </c>
       <c r="C25" s="100" t="n"/>
       <c r="D25" s="100" t="n"/>
-      <c r="E25" s="122">
+      <c r="E25" s="121">
         <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
-      <c r="F25" s="122">
+      <c r="F25" s="121">
         <f>'3 Statement Model'!K90-('3 Statement Model'!K88-'3 Statement Model'!J88)</f>
         <v/>
       </c>
-      <c r="G25" s="122">
+      <c r="G25" s="121">
         <f>'3 Statement Model'!L90-('3 Statement Model'!L88-'3 Statement Model'!K88)</f>
         <v/>
       </c>
-      <c r="H25" s="122">
+      <c r="H25" s="121">
         <f>'3 Statement Model'!M90-('3 Statement Model'!M88-'3 Statement Model'!L88)</f>
         <v/>
       </c>
-      <c r="I25" s="122">
+      <c r="I25" s="121">
         <f>'3 Statement Model'!N90-('3 Statement Model'!N88-'3 Statement Model'!M88)</f>
         <v/>
       </c>
@@ -7269,31 +7266,31 @@
         </is>
       </c>
       <c r="D26" s="100" t="n"/>
-      <c r="E26" s="138">
+      <c r="E26" s="137">
         <f>E21-E22+E23+'3 Statement Model'!J64-E24-E25</f>
         <v/>
       </c>
-      <c r="F26" s="138">
+      <c r="F26" s="137">
         <f>F21-F22+F23+'3 Statement Model'!K64-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="138">
+      <c r="G26" s="137">
         <f>G21-G22+G23+'3 Statement Model'!L64-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="138">
+      <c r="H26" s="137">
         <f>H21-H22+H23+'3 Statement Model'!M64-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="138">
+      <c r="I26" s="137">
         <f>I21-I22+I23+'3 Statement Model'!N64-I24-I25</f>
         <v/>
       </c>
       <c r="J26" s="100" t="n"/>
       <c r="K26" s="100" t="n"/>
-      <c r="L26" s="139" t="inlineStr">
-        <is>
-          <t>vengeanceaiUSCMODEL14.0 — DCF ← 3-Statement linkage audit</t>
+      <c r="L26" s="138" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSCMODEL15.0 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7301,7 +7298,7 @@
       <c r="A27" s="100" t="n"/>
       <c r="B27" s="100" t="inlineStr">
         <is>
-          <t>(Entry)/Exit TV — Exit EV/EBITDA (BASE 22.0x)</t>
+          <t>(Entry)/Exit TV — Exit EV/EBITDA (BASE 23.5x)</t>
         </is>
       </c>
       <c r="C27" s="100" t="n"/>
@@ -7314,27 +7311,27 @@
       <c r="G27" s="100" t="n"/>
       <c r="H27" s="100" t="n"/>
       <c r="I27" s="100" t="n"/>
-      <c r="J27" s="122">
+      <c r="J27" s="121">
         <f>($I$21+$I$23)*$D$8</f>
         <v/>
       </c>
       <c r="K27" s="100" t="n"/>
-      <c r="L27" s="140" t="inlineStr">
+      <c r="L27" s="139" t="inlineStr">
         <is>
           <t>DCF item</t>
         </is>
       </c>
-      <c r="M27" s="140" t="inlineStr">
+      <c r="M27" s="139" t="inlineStr">
         <is>
           <t>Value / link</t>
         </is>
       </c>
-      <c r="N27" s="140" t="inlineStr">
+      <c r="N27" s="139" t="inlineStr">
         <is>
           <t>3-Statement source</t>
         </is>
       </c>
-      <c r="O27" s="140" t="inlineStr">
+      <c r="O27" s="139" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -7348,30 +7345,30 @@
         </is>
       </c>
       <c r="C28" s="100" t="n"/>
-      <c r="D28" s="136" t="n">
+      <c r="D28" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="138">
+      <c r="E28" s="137">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="138">
+      <c r="F28" s="137">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="138">
+      <c r="G28" s="137">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="138">
+      <c r="H28" s="137">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="138">
+      <c r="I28" s="137">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="138">
+      <c r="J28" s="137">
         <f>J27+J26</f>
         <v/>
       </c>
@@ -7381,16 +7378,16 @@
           <t>Cash tax rate (D5)</t>
         </is>
       </c>
-      <c r="M28" s="141">
+      <c r="M28" s="140">
         <f>$D$5</f>
         <v/>
       </c>
-      <c r="N28" s="142" t="inlineStr">
+      <c r="N28" s="141" t="inlineStr">
         <is>
           <t>22.87%</t>
         </is>
       </c>
-      <c r="O28" s="143" t="inlineStr">
+      <c r="O28" s="142" t="inlineStr">
         <is>
           <t>3yr avg IncomeTaxesPaidNet/EBT (not book J13)</t>
         </is>
@@ -7408,27 +7405,27 @@
         <f>D27+D26</f>
         <v/>
       </c>
-      <c r="E29" s="122">
+      <c r="E29" s="121">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F29" s="122">
+      <c r="F29" s="121">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G29" s="122">
+      <c r="G29" s="121">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H29" s="122">
+      <c r="H29" s="121">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I29" s="122">
+      <c r="I29" s="121">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J29" s="122">
+      <c r="J29" s="121">
         <f>J27</f>
         <v/>
       </c>
@@ -7438,15 +7435,15 @@
           <t>DSO (AR days)</t>
         </is>
       </c>
-      <c r="M29" s="141">
+      <c r="M29" s="140">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="N29" s="144">
+      <c r="N29" s="143">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="O29" s="143" t="inlineStr">
+      <c r="O29" s="142" t="inlineStr">
         <is>
           <t>Phased DSO hist→45d; Op NWC excludes Deferred</t>
         </is>
@@ -7467,15 +7464,15 @@
           <t>SBC % of sales</t>
         </is>
       </c>
-      <c r="M30" s="141">
+      <c r="M30" s="140">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="N30" s="144">
+      <c r="N30" s="143">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="O30" s="143" t="inlineStr">
+      <c r="O30" s="142" t="inlineStr">
         <is>
           <t>SBC add-back in CFO row 64 and FCFF</t>
         </is>
@@ -7483,36 +7480,36 @@
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="100" t="n"/>
-      <c r="B31" s="124" t="inlineStr">
+      <c r="B31" s="123" t="inlineStr">
         <is>
           <t>Intrinsic Value</t>
         </is>
       </c>
-      <c r="C31" s="125" t="n"/>
-      <c r="D31" s="125" t="n"/>
+      <c r="C31" s="124" t="n"/>
+      <c r="D31" s="124" t="n"/>
       <c r="E31" s="100" t="n"/>
-      <c r="G31" s="124" t="inlineStr">
+      <c r="G31" s="123" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="H31" s="125" t="n"/>
-      <c r="I31" s="125" t="n"/>
+      <c r="H31" s="124" t="n"/>
+      <c r="I31" s="124" t="n"/>
       <c r="J31" s="100" t="n"/>
-      <c r="L31" s="145" t="inlineStr">
+      <c r="L31" s="144" t="inlineStr">
         <is>
           <t>CapEx % (FY1)</t>
         </is>
       </c>
-      <c r="M31" s="141">
+      <c r="M31" s="140">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="N31" s="144">
+      <c r="N31" s="143">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="O31" s="143" t="inlineStr">
+      <c r="O31" s="142" t="inlineStr">
         <is>
           <t>CapEx% fade path → CF CapEx $</t>
         </is>
@@ -7526,7 +7523,7 @@
         </is>
       </c>
       <c r="C32" s="100" t="n"/>
-      <c r="D32" s="122">
+      <c r="D32" s="121">
         <f>XNPV(D6,D28:J28,D18:J18)</f>
         <v/>
       </c>
@@ -7547,15 +7544,15 @@
           <t>Revenue growth FY1</t>
         </is>
       </c>
-      <c r="M32" s="144">
+      <c r="M32" s="143">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="N32" s="146">
+      <c r="N32" s="145">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="O32" s="143" t="inlineStr">
+      <c r="O32" s="142" t="inlineStr">
         <is>
           <t>Policy path on 3S assumption row 7</t>
         </is>
@@ -7590,15 +7587,15 @@
           <t>EBIT FY1 (DCF E21)</t>
         </is>
       </c>
-      <c r="M33" s="147">
+      <c r="M33" s="146">
         <f>$E$21</f>
         <v/>
       </c>
-      <c r="N33" s="147">
+      <c r="N33" s="146">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="O33" s="143" t="inlineStr">
+      <c r="O33" s="142" t="inlineStr">
         <is>
           <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
         </is>
@@ -7633,16 +7630,16 @@
           <t>EBIT cross-check</t>
         </is>
       </c>
-      <c r="M34" s="147">
+      <c r="M34" s="146">
         <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="N34" s="142" t="inlineStr">
+      <c r="N34" s="141" t="inlineStr">
         <is>
           <t>GP−SGA−R&amp;D−DA</t>
         </is>
       </c>
-      <c r="O34" s="143" t="inlineStr">
+      <c r="O34" s="142" t="inlineStr">
         <is>
           <t>Must equal E21 (live check)</t>
         </is>
@@ -7656,7 +7653,7 @@
         </is>
       </c>
       <c r="C35" s="100" t="n"/>
-      <c r="D35" s="136">
+      <c r="D35" s="135">
         <f>D32+D33-D34</f>
         <v/>
       </c>
@@ -7667,25 +7664,25 @@
         </is>
       </c>
       <c r="H35" s="100" t="n"/>
-      <c r="I35" s="136">
+      <c r="I35" s="135">
         <f>I32+I33-I34</f>
         <v/>
       </c>
       <c r="J35" s="100" t="n"/>
-      <c r="L35" s="145" t="inlineStr">
+      <c r="L35" s="144" t="inlineStr">
         <is>
           <t>D&amp;A FY1</t>
         </is>
       </c>
-      <c r="M35" s="147">
+      <c r="M35" s="146">
         <f>$E$23</f>
         <v/>
       </c>
-      <c r="N35" s="147">
+      <c r="N35" s="146">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="O35" s="143" t="inlineStr">
+      <c r="O35" s="142" t="inlineStr">
         <is>
           <t>Rev × DA% (total D&amp;A / sales) from 3S IS</t>
         </is>
@@ -7699,22 +7696,22 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="148" t="n"/>
+      <c r="I36" s="147" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
           <t>SBC FY1</t>
         </is>
       </c>
-      <c r="M36" s="147">
+      <c r="M36" s="146">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="N36" s="147">
+      <c r="N36" s="146">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="O36" s="143" t="inlineStr">
+      <c r="O36" s="142" t="inlineStr">
         <is>
           <t>Rev × SBC%; added in FCFF</t>
         </is>
@@ -7729,10 +7726,10 @@
       </c>
       <c r="C37" s="109" t="inlineStr">
         <is>
-          <t>MODEL14: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
-        </is>
-      </c>
-      <c r="D37" s="149">
+          <t>MODEL15: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
+        </is>
+      </c>
+      <c r="D37" s="148">
         <f>$D$35/$I$16</f>
         <v/>
       </c>
@@ -7743,7 +7740,7 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="148">
+      <c r="I37" s="147">
         <f>D11</f>
         <v/>
       </c>
@@ -7753,15 +7750,15 @@
           <t>CapEx FY1</t>
         </is>
       </c>
-      <c r="M37" s="147">
+      <c r="M37" s="146">
         <f>$E$24</f>
         <v/>
       </c>
-      <c r="N37" s="147">
+      <c r="N37" s="146">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="O37" s="143" t="inlineStr">
+      <c r="O37" s="142" t="inlineStr">
         <is>
           <t>3S CF CapEx (also D15)</t>
         </is>
@@ -7782,15 +7779,15 @@
           <t>Net WC use FY1</t>
         </is>
       </c>
-      <c r="M38" s="147">
+      <c r="M38" s="146">
         <f>$E$25</f>
         <v/>
       </c>
-      <c r="N38" s="147">
+      <c r="N38" s="146">
         <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
-      <c r="O38" s="143" t="inlineStr">
+      <c r="O38" s="142" t="inlineStr">
         <is>
           <t>ΔOpNWC − ΔDeferred (AR≠Deferred)</t>
         </is>
@@ -7810,15 +7807,15 @@
           <t>EBITDA FY5 (TV base)</t>
         </is>
       </c>
-      <c r="M39" s="147">
+      <c r="M39" s="146">
         <f>$I$21+$I$23</f>
         <v/>
       </c>
-      <c r="N39" s="147">
+      <c r="N39" s="146">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
         <v/>
       </c>
-      <c r="O39" s="143" t="inlineStr">
+      <c r="O39" s="142" t="inlineStr">
         <is>
           <t>EBIT+D&amp;A; Exit TV = this × D8</t>
         </is>
@@ -7839,15 +7836,15 @@
           <t>3S FY25 Cash (ref)</t>
         </is>
       </c>
-      <c r="M40" s="147">
+      <c r="M40" s="146">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="N40" s="147">
+      <c r="N40" s="146">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="O40" s="143" t="inlineStr">
+      <c r="O40" s="142" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D14</t>
         </is>
@@ -7855,34 +7852,34 @@
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="100" t="n"/>
-      <c r="B41" s="124" t="inlineStr">
+      <c r="B41" s="123" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="C41" s="125" t="n"/>
-      <c r="D41" s="150" t="n"/>
-      <c r="E41" s="125" t="n"/>
-      <c r="F41" s="125" t="n"/>
-      <c r="G41" s="125" t="n"/>
-      <c r="H41" s="125" t="n"/>
-      <c r="I41" s="125" t="n"/>
-      <c r="J41" s="125" t="n"/>
-      <c r="K41" s="125" t="n"/>
-      <c r="L41" s="145" t="inlineStr">
+      <c r="C41" s="124" t="n"/>
+      <c r="D41" s="149" t="n"/>
+      <c r="E41" s="124" t="n"/>
+      <c r="F41" s="124" t="n"/>
+      <c r="G41" s="124" t="n"/>
+      <c r="H41" s="124" t="n"/>
+      <c r="I41" s="124" t="n"/>
+      <c r="J41" s="124" t="n"/>
+      <c r="K41" s="124" t="n"/>
+      <c r="L41" s="144" t="inlineStr">
         <is>
           <t>3S FY25 Debt (ref)</t>
         </is>
       </c>
-      <c r="M41" s="147">
+      <c r="M41" s="146">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="N41" s="147">
+      <c r="N41" s="146">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="O41" s="143" t="inlineStr">
+      <c r="O41" s="142" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D13</t>
         </is>
@@ -7901,17 +7898,17 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="L42" s="151" t="inlineStr">
+      <c r="L42" s="150" t="inlineStr">
         <is>
           <t>EBIT link OK?</t>
         </is>
       </c>
-      <c r="M42" s="152">
+      <c r="M42" s="151">
         <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
         <v/>
       </c>
-      <c r="N42" s="153" t="inlineStr"/>
-      <c r="O42" s="143" t="inlineStr">
+      <c r="N42" s="152" t="inlineStr"/>
+      <c r="O42" s="142" t="inlineStr">
         <is>
           <t>Flags if EBIT link ≠ GP−opex build</t>
         </is>
@@ -7930,15 +7927,15 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="L43" s="154" t="inlineStr">
-        <is>
-          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman WACC 7.10%; g=3.5%. $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute shares.</t>
+      <c r="L43" s="153" t="inlineStr">
+        <is>
+          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman WACC 6.65%; g=3.8%. $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute shares.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="155" t="inlineStr">
+      <c r="B44" s="154" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7954,7 +7951,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="155" t="inlineStr">
+      <c r="B45" s="154" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7970,7 +7967,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="155" t="inlineStr">
+      <c r="B46" s="154" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -8005,7 +8002,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="156" t="inlineStr">
+      <c r="N48" s="155" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -8021,7 +8018,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="157" t="inlineStr">
+      <c r="N49" s="156" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8114,7 +8111,7 @@
       <c r="I55" s="100" t="n"/>
       <c r="J55" s="100" t="n"/>
       <c r="K55" s="100" t="n"/>
-      <c r="L55" s="139" t="inlineStr">
+      <c r="L55" s="138" t="inlineStr">
         <is>
           <t>SENSITIVITY — Enterprise Value ($000s)</t>
         </is>
@@ -8132,28 +8129,28 @@
       <c r="I56" s="100" t="n"/>
       <c r="J56" s="100" t="n"/>
       <c r="K56" s="100" t="n"/>
-      <c r="L56" s="114" t="inlineStr">
+      <c r="L56" s="113" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="158" t="n">
-        <v>16</v>
-      </c>
-      <c r="N56" s="158" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="O56" s="158" t="n">
-        <v>22</v>
-      </c>
-      <c r="P56" s="158" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="Q56" s="158" t="n">
-        <v>27</v>
-      </c>
-      <c r="R56" s="158" t="n">
-        <v>29</v>
+      <c r="M56" s="157" t="n">
+        <v>17</v>
+      </c>
+      <c r="N56" s="157" t="n">
+        <v>20</v>
+      </c>
+      <c r="O56" s="157" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="P56" s="157" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q56" s="157" t="n">
+        <v>28</v>
+      </c>
+      <c r="R56" s="157" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
@@ -8168,30 +8165,30 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="159" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="M57" s="147">
+      <c r="L57" s="158" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N57" s="147">
+      <c r="N57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O57" s="147">
+      <c r="O57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P57" s="147">
+      <c r="P57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q57" s="147">
+      <c r="Q57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R57" s="147">
+      <c r="R57" s="146">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8208,30 +8205,30 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="159" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="M58" s="147">
+      <c r="L58" s="158" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N58" s="147">
+      <c r="N58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O58" s="147">
+      <c r="O58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P58" s="147">
+      <c r="P58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q58" s="147">
+      <c r="Q58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R58" s="147">
+      <c r="R58" s="146">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8248,30 +8245,30 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="159" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="M59" s="147">
+      <c r="L59" s="158" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="M59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N59" s="147">
+      <c r="N59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O59" s="160">
+      <c r="O59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P59" s="147">
+      <c r="P59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q59" s="147">
+      <c r="Q59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R59" s="147">
+      <c r="R59" s="146">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8288,30 +8285,30 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="159" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="M60" s="147">
+      <c r="L60" s="158" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="M60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N60" s="147">
+      <c r="N60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="147">
+      <c r="O60" s="159">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P60" s="147">
+      <c r="P60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q60" s="147">
+      <c r="Q60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R60" s="147">
+      <c r="R60" s="146">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8327,162 +8324,191 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="159" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="M61" s="147">
+      <c r="L61" s="158" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="M61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N61" s="147">
+      <c r="N61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O61" s="147">
+      <c r="O61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P61" s="147">
+      <c r="P61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q61" s="147">
+      <c r="Q61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R61" s="147">
+      <c r="R61" s="146">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="L62" s="158" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="M62" s="146">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="N62" s="146">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="O62" s="146">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="P62" s="146">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="Q62" s="146">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="R62" s="146">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+    </row>
     <row r="64">
-      <c r="L64" s="161" t="inlineStr">
+      <c r="L64" s="160" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="162" t="inlineStr">
+      <c r="L65" s="161" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="163" t="n">
-        <v>16</v>
-      </c>
-      <c r="N65" s="163" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="O65" s="163" t="n">
-        <v>22</v>
-      </c>
-      <c r="P65" s="163" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="Q65" s="163" t="n">
-        <v>27</v>
-      </c>
-      <c r="R65" s="163" t="n">
-        <v>29</v>
+      <c r="M65" s="162" t="n">
+        <v>17</v>
+      </c>
+      <c r="N65" s="162" t="n">
+        <v>20</v>
+      </c>
+      <c r="O65" s="162" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="P65" s="162" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q65" s="162" t="n">
+        <v>28</v>
+      </c>
+      <c r="R65" s="162" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="159" t="n">
+      <c r="L66" s="158" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M66" s="163">
+        <f>(M57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N66" s="163">
+        <f>(N57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O66" s="163">
+        <f>(O57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P66" s="163">
+        <f>(P57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q66" s="163">
+        <f>(Q57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R66" s="163">
+        <f>(R57+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="L67" s="158" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M67" s="163">
+        <f>(M58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N67" s="163">
+        <f>(N58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O67" s="163">
+        <f>(O58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P67" s="163">
+        <f>(P58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q67" s="163">
+        <f>(Q58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R67" s="163">
+        <f>(R58+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="L68" s="158" t="n">
         <v>0.065</v>
       </c>
-      <c r="M66" s="164">
-        <f>(M57+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="N66" s="164">
-        <f>(N57+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="O66" s="164">
-        <f>(O57+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="P66" s="164">
-        <f>(P57+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="Q66" s="164">
-        <f>(Q57+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="R66" s="164">
-        <f>(R57+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="L67" s="159" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="M67" s="164">
-        <f>(M58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="N67" s="164">
-        <f>(N58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="O67" s="164">
-        <f>(O58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="P67" s="164">
-        <f>(P58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="Q67" s="164">
-        <f>(Q58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-      <c r="R67" s="164">
-        <f>(R58+$D$33-$D$34)/$I$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="L68" s="159" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="M68" s="164">
+      <c r="M68" s="163">
         <f>(M59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N68" s="164">
+      <c r="N68" s="163">
         <f>(N59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O68" s="165">
+      <c r="O68" s="163">
         <f>(O59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P68" s="164">
+      <c r="P68" s="163">
         <f>(P59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q68" s="164">
+      <c r="Q68" s="163">
         <f>(Q59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R68" s="164">
+      <c r="R68" s="163">
         <f>(R59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="159" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="M69" s="164">
+      <c r="L69" s="158" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="M69" s="163">
         <f>(M60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N69" s="164">
+      <c r="N69" s="163">
         <f>(N60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
@@ -8490,52 +8516,81 @@
         <f>(O60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P69" s="164">
+      <c r="P69" s="163">
         <f>(P60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q69" s="164">
+      <c r="Q69" s="163">
         <f>(Q60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R69" s="164">
+      <c r="R69" s="163">
         <f>(R60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="159" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="M70" s="164">
+      <c r="L70" s="158" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="M70" s="163">
         <f>(M61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N70" s="164">
+      <c r="N70" s="163">
         <f>(N61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O70" s="164">
+      <c r="O70" s="163">
         <f>(O61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P70" s="164">
+      <c r="P70" s="163">
         <f>(P61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q70" s="164">
+      <c r="Q70" s="163">
         <f>(Q61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R70" s="164">
+      <c r="R70" s="163">
         <f>(R61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
+    <row r="71">
+      <c r="L71" s="158" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="M71" s="163">
+        <f>(M62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N71" s="163">
+        <f>(N62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O71" s="163">
+        <f>(O62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P71" s="163">
+        <f>(P62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q71" s="163">
+        <f>(Q62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R71" s="163">
+        <f>(R62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+    </row>
     <row r="72">
-      <c r="L72" s="154" t="inlineStr">
-        <is>
-          <t>Yellow = base (Yacktman WACC=7.10%, Exit 22.0x; CAPM ref ≈9.24%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 22.0x; bull 27x; bear 16.0x.</t>
+      <c r="L72" s="153" t="inlineStr">
+        <is>
+          <t>Yellow = base (Yacktman WACC=6.65%, Exit 23.5x; CAPM ref ≈9.24%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 23.5x; bull 28x; bear 17.0x.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MODEL16 rebuild: publish xlsx, CSVs, and assumptions PDF
Verified: BS OK / cash check 0; D6=R15 CAPM≈9.22%; DSO 97→28d;
Excel intrinsic ≈ $1,916/sh. Cover/Source Index MODEL16 only (no Model15).

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -540,7 +540,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -716,6 +716,9 @@
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="40" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="9" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1596,7 +1599,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>vengeanceaiUSCMODEL13.0</author>
+    <author>vengeanceaiUSCMODEL16.0</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
@@ -1610,17 +1613,17 @@
     </comment>
     <comment ref="D6" authorId="0" shapeId="0">
       <text>
-        <t>Yacktman AAA-equity discount rate.
-HOW: Yellow POLICY D6 = 7.80% (band 7.5–8.2%). CAPM stack remains at R15 (≈9.24%) as a reference only.
-WHY: Don Yacktman — treat high-quality equities like bonds. FICO's Scores toll-bridge has ultra-low default risk and inflation-protected pricing; CAPM with β≈1.32 misprices the 20–30yr hold.
-SOURCE: Yacktman framework + FICO 10-K Scores pricing commentary.</t>
+        <t>CAPM WACC (MODEL16 primary discount rate).
+HOW: D6 = R15 = We×Ke + Wd×Rd(1−t). Rf=4.67% (FRED DGS10/^TNX), β=1.32 (Yahoo 5Y), ERP=4.28% (Damodaran), Rd=6.250% (8-K 6.250% notes).
+WHY: Updated from Model13 (Previous: Yacktman 7.80%) to Model16 (New: live CAPM 9.27%) for Yacktman yield-based bond comparison — no hardcoded override.
+SOURCE: FRED DGS10; Yahoo FICO beta; Damodaran ERP; SEC 8-K notes.</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
         <t>Exit EV/EBITDA multiple (BASE)
 HOW: Yellow POLICY input D8 = 21.0x; TV = Year-5 EBITDA × D8.
-WHY: Bond-like perpetual pricing power commands a premium to the public peer median (~18.1x). Raised from MODEL12 17.5x into the 20–22x Yacktman band. Bull 26x / Bear 15.5x. NOT FICO spot (~25–27x).
+WHY: Perpetual pricing power premium vs peer median (~18.1x). Unchanged vs Model13 21.0x. Bull 26x / Bear 15.5x. NOT FICO spot (~25–27x).
 SOURCE (peer comps): https://vcpscanner.com/valuation/fico/relative
 SOURCE (FICO spot): https://www.alphaspread.com/security/nyse/fico/relative-valuation/ratio/enterprise-value-to-ebitda</t>
       </text>
@@ -6329,7 +6332,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL13.0 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL16.0 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6445,7 +6448,7 @@
       </c>
       <c r="C5" s="109" t="inlineStr">
         <is>
-          <t>MODEL13 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
+          <t>MODEL16 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
         </is>
       </c>
       <c r="D5" s="110" t="n">
@@ -6481,16 +6484,17 @@
       <c r="A6" s="100" t="n"/>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>Discount Rate (Yacktman AAA-equity WACC = 7.80%; CAPM ref R15≈9.24%)</t>
+          <t>Discount Rate (CAPM WACC = R15 ≈ 9.27%; Model13 was Yacktman 7.80%)</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
         <is>
-          <t>MODEL13 Yacktman: bond-like Scores monopoly → 7.80% (band 7.5–8.2%); CAPM β≈1.32 overstates LT risk</t>
-        </is>
-      </c>
-      <c r="D6" s="110" t="n">
-        <v>0.078</v>
+          <t>Updated WACC from Model13 (Previous: 7.80%) to Model16 (New: CAPM 9.27% = Rf 4.67% + β 1.32 × ERP 4.28%; Rd 6.250%)</t>
+        </is>
+      </c>
+      <c r="D6" s="111">
+        <f>R15</f>
+        <v/>
       </c>
       <c r="E6" s="100" t="n"/>
       <c r="F6" s="100" t="n"/>
@@ -6526,7 +6530,7 @@
         </is>
       </c>
       <c r="C7" s="100" t="n"/>
-      <c r="D7" s="111" t="n">
+      <c r="D7" s="112" t="n">
         <v>0.03</v>
       </c>
       <c r="E7" s="100" t="n"/>
@@ -6567,16 +6571,16 @@
           <t>BASE 21.0x = Yacktman premium vs peer median 18.1x. Bull 26x / Bear 15.5x.</t>
         </is>
       </c>
-      <c r="D8" s="112" t="n">
+      <c r="D8" s="113" t="n">
         <v>21</v>
       </c>
       <c r="E8" s="100" t="n"/>
-      <c r="F8" s="113" t="inlineStr">
+      <c r="F8" s="114" t="inlineStr">
         <is>
           <t>Peer EV/EBITDA comps (click)</t>
         </is>
       </c>
-      <c r="G8" s="113" t="inlineStr">
+      <c r="G8" s="114" t="inlineStr">
         <is>
           <t>FICO spot EV/EBITDA (click)</t>
         </is>
@@ -6585,20 +6589,20 @@
       <c r="I8" s="100" t="n"/>
       <c r="J8" s="100" t="n"/>
       <c r="K8" s="100" t="n"/>
-      <c r="L8" s="114" t="inlineStr">
+      <c r="L8" s="115" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="M8" s="114" t="inlineStr">
+      <c r="M8" s="115" t="inlineStr">
         <is>
           <t>Peer set</t>
         </is>
       </c>
-      <c r="N8" s="115" t="n">
+      <c r="N8" s="116" t="n">
         <v>18.11</v>
       </c>
-      <c r="O8" s="114" t="inlineStr">
+      <c r="O8" s="115" t="inlineStr">
         <is>
           <t>Sorted median (SPGI)</t>
         </is>
@@ -6616,7 +6620,7 @@
           <t>Matches 3S hist FYE (Sep 30)</t>
         </is>
       </c>
-      <c r="D9" s="116" t="n">
+      <c r="D9" s="117" t="n">
         <v>43100</v>
       </c>
       <c r="E9" s="100" t="n"/>
@@ -6626,16 +6630,16 @@
       <c r="I9" s="100" t="n"/>
       <c r="J9" s="100" t="n"/>
       <c r="K9" s="100" t="n"/>
-      <c r="L9" s="117" t="inlineStr">
+      <c r="L9" s="118" t="inlineStr">
         <is>
           <t>Base exit (D8)</t>
         </is>
       </c>
-      <c r="M9" s="117" t="n"/>
-      <c r="N9" s="118" t="n">
+      <c r="M9" s="118" t="n"/>
+      <c r="N9" s="119" t="n">
         <v>21</v>
       </c>
-      <c r="O9" s="117" t="inlineStr">
+      <c r="O9" s="118" t="inlineStr">
         <is>
           <t>Yacktman premium vs peer median; audit 21.0x</t>
         </is>
@@ -6649,7 +6653,7 @@
         </is>
       </c>
       <c r="C10" s="100" t="n"/>
-      <c r="D10" s="116" t="n">
+      <c r="D10" s="117" t="n">
         <v>43281</v>
       </c>
       <c r="E10" s="100" t="n"/>
@@ -6659,12 +6663,12 @@
       <c r="I10" s="100" t="n"/>
       <c r="J10" s="100" t="n"/>
       <c r="K10" s="100" t="n"/>
-      <c r="L10" s="113" t="inlineStr">
+      <c r="L10" s="114" t="inlineStr">
         <is>
           <t>Peer comps (click)</t>
         </is>
       </c>
-      <c r="M10" s="113" t="inlineStr">
+      <c r="M10" s="114" t="inlineStr">
         <is>
           <t>FICO spot EV/EBITDA (click)</t>
         </is>
@@ -6680,7 +6684,7 @@
         </is>
       </c>
       <c r="C11" s="100" t="n"/>
-      <c r="D11" s="119" t="n">
+      <c r="D11" s="120" t="n">
         <v>25</v>
       </c>
       <c r="E11" s="100" t="n"/>
@@ -6707,7 +6711,7 @@
           <t>Row 16: buybacks reduce shares; SBC add-back does NOT dilute</t>
         </is>
       </c>
-      <c r="D12" s="120" t="n">
+      <c r="D12" s="121" t="n">
         <v>20000</v>
       </c>
       <c r="E12" s="100" t="n"/>
@@ -6734,7 +6738,7 @@
           <t>See L39 for 3S FY25 debt ref</t>
         </is>
       </c>
-      <c r="D13" s="120" t="n">
+      <c r="D13" s="121" t="n">
         <v>30000</v>
       </c>
       <c r="E13" s="100" t="n"/>
@@ -6761,7 +6765,7 @@
           <t>See L38 for 3S FY25 cash ref</t>
         </is>
       </c>
-      <c r="D14" s="120" t="n">
+      <c r="D14" s="121" t="n">
         <v>239549.5203651849</v>
       </c>
       <c r="E14" s="100" t="n"/>
@@ -6784,7 +6788,7 @@
         </is>
       </c>
       <c r="C15" s="100" t="n"/>
-      <c r="D15" s="121">
+      <c r="D15" s="122">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
@@ -6812,27 +6816,27 @@
           <t>Shares_t = Shares_t−1 + EquityCF_t/Price; EquityCF = 3S buybacks (row 20, &lt;0)</t>
         </is>
       </c>
-      <c r="D16" s="122">
+      <c r="D16" s="123">
         <f>$D$12</f>
         <v/>
       </c>
-      <c r="E16" s="122">
+      <c r="E16" s="123">
         <f>MAX(1000,D16+'3 Statement Model'!J20/$D$11)</f>
         <v/>
       </c>
-      <c r="F16" s="122">
+      <c r="F16" s="123">
         <f>MAX(1000,E16+'3 Statement Model'!K20/$D$11)</f>
         <v/>
       </c>
-      <c r="G16" s="122">
+      <c r="G16" s="123">
         <f>MAX(1000,F16+'3 Statement Model'!L20/$D$11)</f>
         <v/>
       </c>
-      <c r="H16" s="122">
+      <c r="H16" s="123">
         <f>MAX(1000,G16+'3 Statement Model'!M20/$D$11)</f>
         <v/>
       </c>
-      <c r="I16" s="122">
+      <c r="I16" s="123">
         <f>MAX(1000,H16+'3 Statement Model'!N20/$D$11)</f>
         <v/>
       </c>
@@ -6845,46 +6849,46 @@
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="100" t="n"/>
-      <c r="B17" s="123" t="inlineStr">
+      <c r="B17" s="124" t="inlineStr">
         <is>
           <t>Discounted Cash Flow</t>
         </is>
       </c>
-      <c r="C17" s="124" t="n"/>
-      <c r="D17" s="125" t="inlineStr">
+      <c r="C17" s="125" t="n"/>
+      <c r="D17" s="126" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="E17" s="126">
+      <c r="E17" s="127">
         <f>YEAR(E18)</f>
         <v/>
       </c>
-      <c r="F17" s="126">
+      <c r="F17" s="127">
         <f>YEAR(F18)</f>
         <v/>
       </c>
-      <c r="G17" s="126">
+      <c r="G17" s="127">
         <f>YEAR(G18)</f>
         <v/>
       </c>
-      <c r="H17" s="126">
+      <c r="H17" s="127">
         <f>YEAR(H18)</f>
         <v/>
       </c>
-      <c r="I17" s="126">
+      <c r="I17" s="127">
         <f>YEAR(I18)</f>
         <v/>
       </c>
-      <c r="J17" s="125" t="inlineStr">
+      <c r="J17" s="126" t="inlineStr">
         <is>
           <t>Exit</t>
         </is>
       </c>
       <c r="K17" s="100" t="n"/>
-      <c r="L17" s="127" t="inlineStr">
-        <is>
-          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL13.0)</t>
+      <c r="L17" s="128" t="inlineStr">
+        <is>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL16.0)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -6897,31 +6901,31 @@
         </is>
       </c>
       <c r="C18" s="100" t="n"/>
-      <c r="D18" s="128">
+      <c r="D18" s="129">
         <f>$D$9</f>
         <v/>
       </c>
-      <c r="E18" s="128">
+      <c r="E18" s="129">
         <f>EDATE($D$9,(E19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="F18" s="128">
+      <c r="F18" s="129">
         <f>EDATE($D$9,(F19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="G18" s="128">
+      <c r="G18" s="129">
         <f>EDATE($D$9,(G19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="H18" s="128">
+      <c r="H18" s="129">
         <f>EDATE($D$9,(H19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="I18" s="128">
+      <c r="I18" s="129">
         <f>EDATE($D$9,(I19+0.5)*12)</f>
         <v/>
       </c>
-      <c r="J18" s="128">
+      <c r="J18" s="129">
         <f>I18</f>
         <v/>
       </c>
@@ -6931,7 +6935,7 @@
           <t>Exit EV/EBITDA @ D8 (BASE 21.0x)</t>
         </is>
       </c>
-      <c r="M18" s="121">
+      <c r="M18" s="122">
         <f>J27</f>
         <v/>
       </c>
@@ -6944,44 +6948,44 @@
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="100" t="n"/>
-      <c r="B19" s="129" t="inlineStr">
+      <c r="B19" s="130" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="129" t="n"/>
-      <c r="D19" s="130" t="n"/>
-      <c r="E19" s="131" t="n">
+      <c r="C19" s="130" t="n"/>
+      <c r="D19" s="131" t="n"/>
+      <c r="E19" s="132" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="132">
+      <c r="F19" s="133">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="132">
+      <c r="G19" s="133">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="132">
+      <c r="H19" s="133">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="132">
+      <c r="I19" s="133">
         <f>H19+1</f>
         <v/>
       </c>
-      <c r="J19" s="130" t="n"/>
+      <c r="J19" s="131" t="n"/>
       <c r="K19" s="100" t="n"/>
       <c r="L19" s="100" t="inlineStr">
         <is>
           <t>Gordon cross-check (g=D7)</t>
         </is>
       </c>
-      <c r="M19" s="121">
+      <c r="M19" s="122">
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="133" t="inlineStr">
+      <c r="N19" s="134" t="inlineStr">
         <is>
           <t>← sanity check</t>
         </is>
@@ -6990,30 +6994,30 @@
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="100" t="n"/>
-      <c r="B20" s="129" t="inlineStr">
+      <c r="B20" s="130" t="inlineStr">
         <is>
           <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
       <c r="C20" s="100" t="n"/>
       <c r="D20" s="100" t="n"/>
-      <c r="E20" s="134">
+      <c r="E20" s="135">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="134">
+      <c r="F20" s="135">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="134">
+      <c r="G20" s="135">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="134">
+      <c r="H20" s="135">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="134">
+      <c r="I20" s="135">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
@@ -7024,11 +7028,11 @@
           <t>Implied Gordon exit multiple</t>
         </is>
       </c>
-      <c r="M20" s="121">
+      <c r="M20" s="122">
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="135" t="inlineStr">
+      <c r="N20" s="136" t="inlineStr">
         <is>
           <t>← ~bear check</t>
         </is>
@@ -7044,23 +7048,23 @@
       </c>
       <c r="C21" s="100" t="n"/>
       <c r="D21" s="100" t="n"/>
-      <c r="E21" s="121">
+      <c r="E21" s="122">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="F21" s="121">
+      <c r="F21" s="122">
         <f>'3 Statement Model'!K33+'3 Statement Model'!K31</f>
         <v/>
       </c>
-      <c r="G21" s="121">
+      <c r="G21" s="122">
         <f>'3 Statement Model'!L33+'3 Statement Model'!L31</f>
         <v/>
       </c>
-      <c r="H21" s="121">
+      <c r="H21" s="122">
         <f>'3 Statement Model'!M33+'3 Statement Model'!M31</f>
         <v/>
       </c>
-      <c r="I21" s="121">
+      <c r="I21" s="122">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31</f>
         <v/>
       </c>
@@ -7071,7 +7075,7 @@
           <t>BASE TV @ 21.0x (primary)</t>
         </is>
       </c>
-      <c r="M21" s="121">
+      <c r="M21" s="122">
         <f>($I$21+$I$23)*21.0</f>
         <v/>
       </c>
@@ -7091,23 +7095,23 @@
       </c>
       <c r="C22" s="100" t="n"/>
       <c r="D22" s="100" t="n"/>
-      <c r="E22" s="136">
+      <c r="E22" s="137">
         <f>E21*$D$5</f>
         <v/>
       </c>
-      <c r="F22" s="136">
+      <c r="F22" s="137">
         <f>F21*$D$5</f>
         <v/>
       </c>
-      <c r="G22" s="136">
+      <c r="G22" s="137">
         <f>G21*$D$5</f>
         <v/>
       </c>
-      <c r="H22" s="136">
+      <c r="H22" s="137">
         <f>H21*$D$5</f>
         <v/>
       </c>
-      <c r="I22" s="136">
+      <c r="I22" s="137">
         <f>I21*$D$5</f>
         <v/>
       </c>
@@ -7118,7 +7122,7 @@
           <t>BULL TV @ 26.0x (spot/policy)</t>
         </is>
       </c>
-      <c r="M22" s="121">
+      <c r="M22" s="122">
         <f>($I$21+$I$23)*26.0</f>
         <v/>
       </c>
@@ -7138,23 +7142,23 @@
       </c>
       <c r="C23" s="100" t="n"/>
       <c r="D23" s="100" t="n"/>
-      <c r="E23" s="136">
+      <c r="E23" s="137">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="136">
+      <c r="F23" s="137">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="136">
+      <c r="G23" s="137">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="136">
+      <c r="H23" s="137">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="136">
+      <c r="I23" s="137">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
@@ -7165,7 +7169,7 @@
           <t>BEAR TV @ 15.5x (Gordon-implied)</t>
         </is>
       </c>
-      <c r="M23" s="121">
+      <c r="M23" s="122">
         <f>($I$21+$I$23)*15.5</f>
         <v/>
       </c>
@@ -7185,23 +7189,23 @@
       </c>
       <c r="C24" s="100" t="n"/>
       <c r="D24" s="100" t="n"/>
-      <c r="E24" s="121">
+      <c r="E24" s="122">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="F24" s="121">
+      <c r="F24" s="122">
         <f>'3 Statement Model'!K68</f>
         <v/>
       </c>
-      <c r="G24" s="121">
+      <c r="G24" s="122">
         <f>'3 Statement Model'!L68</f>
         <v/>
       </c>
-      <c r="H24" s="121">
+      <c r="H24" s="122">
         <f>'3 Statement Model'!M68</f>
         <v/>
       </c>
-      <c r="I24" s="121">
+      <c r="I24" s="122">
         <f>'3 Statement Model'!N68</f>
         <v/>
       </c>
@@ -7222,23 +7226,23 @@
       </c>
       <c r="C25" s="100" t="n"/>
       <c r="D25" s="100" t="n"/>
-      <c r="E25" s="121">
+      <c r="E25" s="122">
         <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
-      <c r="F25" s="121">
+      <c r="F25" s="122">
         <f>'3 Statement Model'!K90-('3 Statement Model'!K88-'3 Statement Model'!J88)</f>
         <v/>
       </c>
-      <c r="G25" s="121">
+      <c r="G25" s="122">
         <f>'3 Statement Model'!L90-('3 Statement Model'!L88-'3 Statement Model'!K88)</f>
         <v/>
       </c>
-      <c r="H25" s="121">
+      <c r="H25" s="122">
         <f>'3 Statement Model'!M90-('3 Statement Model'!M88-'3 Statement Model'!L88)</f>
         <v/>
       </c>
-      <c r="I25" s="121">
+      <c r="I25" s="122">
         <f>'3 Statement Model'!N90-('3 Statement Model'!N88-'3 Statement Model'!M88)</f>
         <v/>
       </c>
@@ -7262,31 +7266,31 @@
         </is>
       </c>
       <c r="D26" s="100" t="n"/>
-      <c r="E26" s="137">
+      <c r="E26" s="138">
         <f>E21-E22+E23+'3 Statement Model'!J64-E24-E25</f>
         <v/>
       </c>
-      <c r="F26" s="137">
+      <c r="F26" s="138">
         <f>F21-F22+F23+'3 Statement Model'!K64-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="137">
+      <c r="G26" s="138">
         <f>G21-G22+G23+'3 Statement Model'!L64-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="137">
+      <c r="H26" s="138">
         <f>H21-H22+H23+'3 Statement Model'!M64-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="137">
+      <c r="I26" s="138">
         <f>I21-I22+I23+'3 Statement Model'!N64-I24-I25</f>
         <v/>
       </c>
       <c r="J26" s="100" t="n"/>
       <c r="K26" s="100" t="n"/>
-      <c r="L26" s="138" t="inlineStr">
-        <is>
-          <t>vengeanceaiUSCMODEL13.0 — DCF ← 3-Statement linkage audit</t>
+      <c r="L26" s="139" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSCMODEL16.0 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7307,27 +7311,27 @@
       <c r="G27" s="100" t="n"/>
       <c r="H27" s="100" t="n"/>
       <c r="I27" s="100" t="n"/>
-      <c r="J27" s="121">
+      <c r="J27" s="122">
         <f>($I$21+$I$23)*$D$8</f>
         <v/>
       </c>
       <c r="K27" s="100" t="n"/>
-      <c r="L27" s="139" t="inlineStr">
+      <c r="L27" s="140" t="inlineStr">
         <is>
           <t>DCF item</t>
         </is>
       </c>
-      <c r="M27" s="139" t="inlineStr">
+      <c r="M27" s="140" t="inlineStr">
         <is>
           <t>Value / link</t>
         </is>
       </c>
-      <c r="N27" s="139" t="inlineStr">
+      <c r="N27" s="140" t="inlineStr">
         <is>
           <t>3-Statement source</t>
         </is>
       </c>
-      <c r="O27" s="139" t="inlineStr">
+      <c r="O27" s="140" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -7341,30 +7345,30 @@
         </is>
       </c>
       <c r="C28" s="100" t="n"/>
-      <c r="D28" s="135" t="n">
+      <c r="D28" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="137">
+      <c r="E28" s="138">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="137">
+      <c r="F28" s="138">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="137">
+      <c r="G28" s="138">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="137">
+      <c r="H28" s="138">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="137">
+      <c r="I28" s="138">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="137">
+      <c r="J28" s="138">
         <f>J27+J26</f>
         <v/>
       </c>
@@ -7374,16 +7378,16 @@
           <t>Cash tax rate (D5)</t>
         </is>
       </c>
-      <c r="M28" s="140">
+      <c r="M28" s="141">
         <f>$D$5</f>
         <v/>
       </c>
-      <c r="N28" s="141" t="inlineStr">
+      <c r="N28" s="142" t="inlineStr">
         <is>
           <t>22.87%</t>
         </is>
       </c>
-      <c r="O28" s="142" t="inlineStr">
+      <c r="O28" s="143" t="inlineStr">
         <is>
           <t>3yr avg IncomeTaxesPaidNet/EBT (not book J13)</t>
         </is>
@@ -7401,27 +7405,27 @@
         <f>D27+D26</f>
         <v/>
       </c>
-      <c r="E29" s="121">
+      <c r="E29" s="122">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F29" s="121">
+      <c r="F29" s="122">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G29" s="121">
+      <c r="G29" s="122">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H29" s="121">
+      <c r="H29" s="122">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I29" s="121">
+      <c r="I29" s="122">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J29" s="121">
+      <c r="J29" s="122">
         <f>J27</f>
         <v/>
       </c>
@@ -7431,15 +7435,15 @@
           <t>DSO (AR days)</t>
         </is>
       </c>
-      <c r="M29" s="140">
+      <c r="M29" s="141">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="N29" s="143">
+      <c r="N29" s="144">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="O29" s="142" t="inlineStr">
+      <c r="O29" s="143" t="inlineStr">
         <is>
           <t>Phased DSO hist→45d; Op NWC excludes Deferred</t>
         </is>
@@ -7460,15 +7464,15 @@
           <t>SBC % of sales</t>
         </is>
       </c>
-      <c r="M30" s="140">
+      <c r="M30" s="141">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="N30" s="143">
+      <c r="N30" s="144">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="O30" s="142" t="inlineStr">
+      <c r="O30" s="143" t="inlineStr">
         <is>
           <t>SBC add-back in CFO row 64 and FCFF</t>
         </is>
@@ -7476,36 +7480,36 @@
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="100" t="n"/>
-      <c r="B31" s="123" t="inlineStr">
+      <c r="B31" s="124" t="inlineStr">
         <is>
           <t>Intrinsic Value</t>
         </is>
       </c>
-      <c r="C31" s="124" t="n"/>
-      <c r="D31" s="124" t="n"/>
+      <c r="C31" s="125" t="n"/>
+      <c r="D31" s="125" t="n"/>
       <c r="E31" s="100" t="n"/>
-      <c r="G31" s="123" t="inlineStr">
+      <c r="G31" s="124" t="inlineStr">
         <is>
           <t>Market Value</t>
         </is>
       </c>
-      <c r="H31" s="124" t="n"/>
-      <c r="I31" s="124" t="n"/>
+      <c r="H31" s="125" t="n"/>
+      <c r="I31" s="125" t="n"/>
       <c r="J31" s="100" t="n"/>
-      <c r="L31" s="144" t="inlineStr">
+      <c r="L31" s="145" t="inlineStr">
         <is>
           <t>CapEx % (FY1)</t>
         </is>
       </c>
-      <c r="M31" s="140">
+      <c r="M31" s="141">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="N31" s="143">
+      <c r="N31" s="144">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="O31" s="142" t="inlineStr">
+      <c r="O31" s="143" t="inlineStr">
         <is>
           <t>CapEx% fade path → CF CapEx $</t>
         </is>
@@ -7519,7 +7523,7 @@
         </is>
       </c>
       <c r="C32" s="100" t="n"/>
-      <c r="D32" s="121">
+      <c r="D32" s="122">
         <f>XNPV(D6,D28:J28,D18:J18)</f>
         <v/>
       </c>
@@ -7540,15 +7544,15 @@
           <t>Revenue growth FY1</t>
         </is>
       </c>
-      <c r="M32" s="143">
+      <c r="M32" s="144">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="N32" s="145">
+      <c r="N32" s="146">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="O32" s="142" t="inlineStr">
+      <c r="O32" s="143" t="inlineStr">
         <is>
           <t>Policy path on 3S assumption row 7</t>
         </is>
@@ -7583,15 +7587,15 @@
           <t>EBIT FY1 (DCF E21)</t>
         </is>
       </c>
-      <c r="M33" s="146">
+      <c r="M33" s="147">
         <f>$E$21</f>
         <v/>
       </c>
-      <c r="N33" s="146">
+      <c r="N33" s="147">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="O33" s="142" t="inlineStr">
+      <c r="O33" s="143" t="inlineStr">
         <is>
           <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
         </is>
@@ -7626,16 +7630,16 @@
           <t>EBIT cross-check</t>
         </is>
       </c>
-      <c r="M34" s="146">
+      <c r="M34" s="147">
         <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="N34" s="141" t="inlineStr">
+      <c r="N34" s="142" t="inlineStr">
         <is>
           <t>GP−SGA−R&amp;D−DA</t>
         </is>
       </c>
-      <c r="O34" s="142" t="inlineStr">
+      <c r="O34" s="143" t="inlineStr">
         <is>
           <t>Must equal E21 (live check)</t>
         </is>
@@ -7649,7 +7653,7 @@
         </is>
       </c>
       <c r="C35" s="100" t="n"/>
-      <c r="D35" s="135">
+      <c r="D35" s="136">
         <f>D32+D33-D34</f>
         <v/>
       </c>
@@ -7660,25 +7664,25 @@
         </is>
       </c>
       <c r="H35" s="100" t="n"/>
-      <c r="I35" s="135">
+      <c r="I35" s="136">
         <f>I32+I33-I34</f>
         <v/>
       </c>
       <c r="J35" s="100" t="n"/>
-      <c r="L35" s="144" t="inlineStr">
+      <c r="L35" s="145" t="inlineStr">
         <is>
           <t>D&amp;A FY1</t>
         </is>
       </c>
-      <c r="M35" s="146">
+      <c r="M35" s="147">
         <f>$E$23</f>
         <v/>
       </c>
-      <c r="N35" s="146">
+      <c r="N35" s="147">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="O35" s="142" t="inlineStr">
+      <c r="O35" s="143" t="inlineStr">
         <is>
           <t>Rev × DA% (total D&amp;A / sales) from 3S IS</t>
         </is>
@@ -7692,22 +7696,22 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="147" t="n"/>
+      <c r="I36" s="148" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
           <t>SBC FY1</t>
         </is>
       </c>
-      <c r="M36" s="146">
+      <c r="M36" s="147">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="N36" s="146">
+      <c r="N36" s="147">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="O36" s="142" t="inlineStr">
+      <c r="O36" s="143" t="inlineStr">
         <is>
           <t>Rev × SBC%; added in FCFF</t>
         </is>
@@ -7722,10 +7726,10 @@
       </c>
       <c r="C37" s="109" t="inlineStr">
         <is>
-          <t>MODEL13: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
-        </is>
-      </c>
-      <c r="D37" s="148">
+          <t>MODEL16: SBC add-back in FCFF; buybacks cut shares (no SBC dilution)</t>
+        </is>
+      </c>
+      <c r="D37" s="149">
         <f>$D$35/$I$16</f>
         <v/>
       </c>
@@ -7736,7 +7740,7 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="147">
+      <c r="I37" s="148">
         <f>D11</f>
         <v/>
       </c>
@@ -7746,15 +7750,15 @@
           <t>CapEx FY1</t>
         </is>
       </c>
-      <c r="M37" s="146">
+      <c r="M37" s="147">
         <f>$E$24</f>
         <v/>
       </c>
-      <c r="N37" s="146">
+      <c r="N37" s="147">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="O37" s="142" t="inlineStr">
+      <c r="O37" s="143" t="inlineStr">
         <is>
           <t>3S CF CapEx (also D15)</t>
         </is>
@@ -7775,15 +7779,15 @@
           <t>Net WC use FY1</t>
         </is>
       </c>
-      <c r="M38" s="146">
+      <c r="M38" s="147">
         <f>$E$25</f>
         <v/>
       </c>
-      <c r="N38" s="146">
+      <c r="N38" s="147">
         <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
-      <c r="O38" s="142" t="inlineStr">
+      <c r="O38" s="143" t="inlineStr">
         <is>
           <t>ΔOpNWC − ΔDeferred (AR≠Deferred)</t>
         </is>
@@ -7803,15 +7807,15 @@
           <t>EBITDA FY5 (TV base)</t>
         </is>
       </c>
-      <c r="M39" s="146">
+      <c r="M39" s="147">
         <f>$I$21+$I$23</f>
         <v/>
       </c>
-      <c r="N39" s="146">
+      <c r="N39" s="147">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
         <v/>
       </c>
-      <c r="O39" s="142" t="inlineStr">
+      <c r="O39" s="143" t="inlineStr">
         <is>
           <t>EBIT+D&amp;A; Exit TV = this × D8</t>
         </is>
@@ -7832,15 +7836,15 @@
           <t>3S FY25 Cash (ref)</t>
         </is>
       </c>
-      <c r="M40" s="146">
+      <c r="M40" s="147">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="N40" s="146">
+      <c r="N40" s="147">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="O40" s="142" t="inlineStr">
+      <c r="O40" s="143" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D14</t>
         </is>
@@ -7848,34 +7852,34 @@
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="100" t="n"/>
-      <c r="B41" s="123" t="inlineStr">
+      <c r="B41" s="124" t="inlineStr">
         <is>
           <t>Instructions</t>
         </is>
       </c>
-      <c r="C41" s="124" t="n"/>
-      <c r="D41" s="149" t="n"/>
-      <c r="E41" s="124" t="n"/>
-      <c r="F41" s="124" t="n"/>
-      <c r="G41" s="124" t="n"/>
-      <c r="H41" s="124" t="n"/>
-      <c r="I41" s="124" t="n"/>
-      <c r="J41" s="124" t="n"/>
-      <c r="K41" s="124" t="n"/>
-      <c r="L41" s="144" t="inlineStr">
+      <c r="C41" s="125" t="n"/>
+      <c r="D41" s="150" t="n"/>
+      <c r="E41" s="125" t="n"/>
+      <c r="F41" s="125" t="n"/>
+      <c r="G41" s="125" t="n"/>
+      <c r="H41" s="125" t="n"/>
+      <c r="I41" s="125" t="n"/>
+      <c r="J41" s="125" t="n"/>
+      <c r="K41" s="125" t="n"/>
+      <c r="L41" s="145" t="inlineStr">
         <is>
           <t>3S FY25 Debt (ref)</t>
         </is>
       </c>
-      <c r="M41" s="146">
+      <c r="M41" s="147">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="N41" s="146">
+      <c r="N41" s="147">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="O41" s="142" t="inlineStr">
+      <c r="O41" s="143" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D13</t>
         </is>
@@ -7894,17 +7898,17 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="L42" s="150" t="inlineStr">
+      <c r="L42" s="151" t="inlineStr">
         <is>
           <t>EBIT link OK?</t>
         </is>
       </c>
-      <c r="M42" s="151">
+      <c r="M42" s="152">
         <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
         <v/>
       </c>
-      <c r="N42" s="152" t="inlineStr"/>
-      <c r="O42" s="142" t="inlineStr">
+      <c r="N42" s="153" t="inlineStr"/>
+      <c r="O42" s="143" t="inlineStr">
         <is>
           <t>Flags if EBIT link ≠ GP−opex build</t>
         </is>
@@ -7923,15 +7927,15 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="L43" s="153" t="inlineStr">
-        <is>
-          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman WACC 7.8%. $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute shares.</t>
+      <c r="L43" s="154" t="inlineStr">
+        <is>
+          <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = CAPM WACC 9.27% (D6←R15). $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="154" t="inlineStr">
+      <c r="B44" s="155" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7947,7 +7951,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="154" t="inlineStr">
+      <c r="B45" s="155" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7963,7 +7967,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="154" t="inlineStr">
+      <c r="B46" s="155" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -7998,7 +8002,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="155" t="inlineStr">
+      <c r="N48" s="156" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -8014,7 +8018,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="156" t="inlineStr">
+      <c r="N49" s="157" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8107,7 +8111,7 @@
       <c r="I55" s="100" t="n"/>
       <c r="J55" s="100" t="n"/>
       <c r="K55" s="100" t="n"/>
-      <c r="L55" s="138" t="inlineStr">
+      <c r="L55" s="139" t="inlineStr">
         <is>
           <t>SENSITIVITY — Enterprise Value ($000s)</t>
         </is>
@@ -8125,27 +8129,27 @@
       <c r="I56" s="100" t="n"/>
       <c r="J56" s="100" t="n"/>
       <c r="K56" s="100" t="n"/>
-      <c r="L56" s="114" t="inlineStr">
+      <c r="L56" s="115" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="157" t="n">
+      <c r="M56" s="158" t="n">
         <v>15.5</v>
       </c>
-      <c r="N56" s="157" t="n">
+      <c r="N56" s="158" t="n">
         <v>18</v>
       </c>
-      <c r="O56" s="157" t="n">
+      <c r="O56" s="158" t="n">
         <v>21</v>
       </c>
-      <c r="P56" s="157" t="n">
+      <c r="P56" s="158" t="n">
         <v>23.5</v>
       </c>
-      <c r="Q56" s="157" t="n">
+      <c r="Q56" s="158" t="n">
         <v>26</v>
       </c>
-      <c r="R56" s="157" t="n">
+      <c r="R56" s="158" t="n">
         <v>28</v>
       </c>
     </row>
@@ -8161,30 +8165,30 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="158" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="M57" s="146">
+      <c r="L57" s="159" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="M57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N57" s="146">
+      <c r="N57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O57" s="146">
+      <c r="O57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P57" s="146">
+      <c r="P57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q57" s="146">
+      <c r="Q57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R57" s="146">
+      <c r="R57" s="147">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8201,30 +8205,30 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="158" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="M58" s="146">
+      <c r="L58" s="159" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="M58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N58" s="146">
+      <c r="N58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O58" s="146">
+      <c r="O58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P58" s="146">
+      <c r="P58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q58" s="146">
+      <c r="Q58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R58" s="146">
+      <c r="R58" s="147">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8241,30 +8245,30 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="158" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="M59" s="146">
+      <c r="L59" s="159" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N59" s="146">
+      <c r="N59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O59" s="159">
+      <c r="O59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P59" s="146">
+      <c r="P59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q59" s="146">
+      <c r="Q59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R59" s="146">
+      <c r="R59" s="147">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8281,30 +8285,30 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="158" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="M60" s="146">
+      <c r="L60" s="159" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="M60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N60" s="146">
+      <c r="N60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="146">
+      <c r="O60" s="160">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P60" s="146">
+      <c r="P60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q60" s="146">
+      <c r="Q60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R60" s="146">
+      <c r="R60" s="147">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8320,133 +8324,162 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="158" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="M61" s="146">
+      <c r="L61" s="159" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N61" s="146">
+      <c r="N61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O61" s="146">
+      <c r="O61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P61" s="146">
+      <c r="P61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q61" s="146">
+      <c r="Q61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R61" s="146">
+      <c r="R61" s="147">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="L62" s="159" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="M62" s="147">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="N62" s="147">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="O62" s="147">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="P62" s="147">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="Q62" s="147">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+      <c r="R62" s="147">
+        <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
+        <v/>
+      </c>
+    </row>
     <row r="64">
-      <c r="L64" s="160" t="inlineStr">
+      <c r="L64" s="161" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="161" t="inlineStr">
+      <c r="L65" s="162" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="162" t="n">
+      <c r="M65" s="163" t="n">
         <v>15.5</v>
       </c>
-      <c r="N65" s="162" t="n">
+      <c r="N65" s="163" t="n">
         <v>18</v>
       </c>
-      <c r="O65" s="162" t="n">
+      <c r="O65" s="163" t="n">
         <v>21</v>
       </c>
-      <c r="P65" s="162" t="n">
+      <c r="P65" s="163" t="n">
         <v>23.5</v>
       </c>
-      <c r="Q65" s="162" t="n">
+      <c r="Q65" s="163" t="n">
         <v>26</v>
       </c>
-      <c r="R65" s="162" t="n">
+      <c r="R65" s="163" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="158" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="M66" s="163">
+      <c r="L66" s="159" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="M66" s="164">
         <f>(M57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N66" s="163">
+      <c r="N66" s="164">
         <f>(N57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O66" s="163">
+      <c r="O66" s="164">
         <f>(O57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P66" s="163">
+      <c r="P66" s="164">
         <f>(P57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q66" s="163">
+      <c r="Q66" s="164">
         <f>(Q57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R66" s="163">
+      <c r="R66" s="164">
         <f>(R57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="158" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="M67" s="163">
+      <c r="L67" s="159" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="M67" s="164">
         <f>(M58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N67" s="163">
+      <c r="N67" s="164">
         <f>(N58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O67" s="163">
+      <c r="O67" s="164">
         <f>(O58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P67" s="163">
+      <c r="P67" s="164">
         <f>(P58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q67" s="163">
+      <c r="Q67" s="164">
         <f>(Q58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R67" s="163">
+      <c r="R67" s="164">
         <f>(R58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="158" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="M68" s="163">
+      <c r="L68" s="159" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M68" s="164">
         <f>(M59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N68" s="163">
+      <c r="N68" s="164">
         <f>(N59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
@@ -8454,81 +8487,110 @@
         <f>(O59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P68" s="163">
+      <c r="P68" s="164">
         <f>(P59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q68" s="163">
+      <c r="Q68" s="164">
         <f>(Q59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R68" s="163">
+      <c r="R68" s="164">
         <f>(R59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="158" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="M69" s="163">
+      <c r="L69" s="159" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="M69" s="164">
         <f>(M60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N69" s="163">
+      <c r="N69" s="164">
         <f>(N60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O69" s="163">
+      <c r="O69" s="165">
         <f>(O60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P69" s="163">
+      <c r="P69" s="164">
         <f>(P60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q69" s="163">
+      <c r="Q69" s="164">
         <f>(Q60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R69" s="163">
+      <c r="R69" s="164">
         <f>(R60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="158" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="M70" s="163">
+      <c r="L70" s="159" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M70" s="164">
         <f>(M61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N70" s="163">
+      <c r="N70" s="164">
         <f>(N61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O70" s="163">
+      <c r="O70" s="164">
         <f>(O61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P70" s="163">
+      <c r="P70" s="164">
         <f>(P61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q70" s="163">
+      <c r="Q70" s="164">
         <f>(Q61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R70" s="163">
+      <c r="R70" s="164">
         <f>(R61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
+    <row r="71">
+      <c r="L71" s="159" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="M71" s="164">
+        <f>(M62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="N71" s="164">
+        <f>(N62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="O71" s="164">
+        <f>(O62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="P71" s="164">
+        <f>(P62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="Q71" s="164">
+        <f>(Q62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+      <c r="R71" s="164">
+        <f>(R62+$D$33-$D$34)/$I$16</f>
+        <v/>
+      </c>
+    </row>
     <row r="72">
-      <c r="L72" s="153" t="inlineStr">
-        <is>
-          <t>Yellow = base (Yacktman WACC=7.80%, Exit 21.0x; CAPM ref ≈9.24%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 21.0x; bull 26x; bear 15.5x.</t>
+      <c r="L72" s="154" t="inlineStr">
+        <is>
+          <t>Yellow = base (CAPM WACC=9.27%, Exit 21.0x; CAPM ref ≈9.27%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 21.0x; bull 26x; bear 15.5x.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MODEL18 rebuild: publish xlsx, CSVs, and assumptions PDF
Excel verifies BS≈0, cash check=0, D9=2026-08-06, Y1 FCFF×64.66%,
mid-stub 2026-12-02, WACC~7.62%, SBC 7→5%; intrinsic ≈ $4,692/sh.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -82,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="17">
+  <numFmts count="18">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\(#,##0\)_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.0000_ ;\-0.0000\ "/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -94,12 +94,13 @@
     <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0.00_-;\(#,##0.00\)_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="175" formatCode="0.0"/>
-    <numFmt numFmtId="176" formatCode="#,##0.000"/>
-    <numFmt numFmtId="177" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="178" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="179" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="180" formatCode="#,##0.0"/>
+    <numFmt numFmtId="175" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="176" formatCode="0.0"/>
+    <numFmt numFmtId="177" formatCode="#,##0.000"/>
+    <numFmt numFmtId="178" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="179" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="180" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="181" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="48">
     <font>
@@ -540,7 +541,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="167">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -710,7 +711,7 @@
     </xf>
     <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="33" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="32" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -724,15 +725,15 @@
     <xf numFmtId="166" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="175" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -740,7 +741,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="176" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -749,6 +750,7 @@
     <xf numFmtId="0" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="46" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="37" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -766,9 +768,9 @@
     <xf numFmtId="164" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="180" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -787,16 +789,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="179" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="180" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="180" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1599,7 +1601,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>vengeanceaiUSCMODEL17.0</author>
+    <author>vengeanceaiUSCMODEL18.0</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
@@ -1613,19 +1615,28 @@
     </comment>
     <comment ref="D6" authorId="0" shapeId="0">
       <text>
-        <t>Yacktman-adjusted CAPM WACC (MODEL17 primary discount rate).
+        <t>Yacktman-adjusted CAPM WACC (MODEL18 primary discount rate).
 HOW: D6 = R15 = We×Ke + Wd×Rd(1−t). β_Yacktman=0.854 (Blume+AAA blend; Yahoo raw 1.32). Rf=4.67%, ERP=4.28%, Rd=6.250%.
-WHY: Updated from Model16 (Previous: raw CAPM 9.27%) to Model17 (New: Yacktman-adj 7.68%) — Scores royalties ≈ AAA coupon; every term algebraic, no naked hardcoded WACC%.
-SOURCE: Blume 1971; IR Scores OM; FRED DGS10; Yahoo β; Damodaran ERP; 8-K notes.</t>
+WHY: Same algebraic CAPM as Model17 (7.68%); MODEL18 changes stub timing / SBC / SaaS mix — not a naked WACC override.
+SOURCE: Blume 1971; FRED DGS10; Yahoo β; Damodaran ERP; 8-K notes.</t>
       </text>
     </comment>
     <comment ref="D8" authorId="0" shapeId="0">
       <text>
         <t>Exit EV/EBITDA multiple (BASE)
 HOW: Yellow POLICY input D8 = 23.0x; TV = Year-5 EBITDA × D8.
-WHY: Updated from Model16 (Previous: 21.0x) to Model17 (New: 23.0x) — pricing-power premium vs peer median (~18.1x). Bull 27x / Bear 17.0x. NOT FICO spot (~25–27x).
+WHY: Exit unchanged vs Model17 (Previous: 23.0x) — pricing-power premium vs peer median (~18.1x). Bull 27x / Bear 17.0x. NOT FICO spot (~25–27x).
 SOURCE (peer comps): https://vcpscanner.com/valuation/fico/relative
 SOURCE (FICO spot): https://www.alphaspread.com/security/nyse/fico/relative-valuation/ratio/enterprise-value-to-ebitda</t>
+      </text>
+    </comment>
+    <comment ref="D9" authorId="0" shapeId="0">
+      <text>
+        <t>MODEL18 stub-period valuation date.
+HOW: D9 = 2026-08-06. FY stub starts 2026-03-30; 129 of 365 days elapsed (35.34%); 64.66% remains.
+Y1 FCFF scaled by 0.6466; E18 = D9+118d (mid-stub 2026-12-02).
+WHY: Do not discount cash that has already occurred.
+SOURCE: Model calendar stub 3/30/2026→3/29/2027; valuation 8/6/2026.</t>
       </text>
     </comment>
     <comment ref="D16" authorId="0" shapeId="0">
@@ -6332,7 +6343,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL17.0 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL18.0 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6448,7 +6459,7 @@
       </c>
       <c r="C5" s="109" t="inlineStr">
         <is>
-          <t>MODEL17 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
+          <t>MODEL18 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
         </is>
       </c>
       <c r="D5" s="110" t="n">
@@ -6484,12 +6495,12 @@
       <c r="A6" s="100" t="n"/>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>Discount Rate (Yacktman-adj CAPM WACC = R15 ≈ 7.68%; Model16 raw CAPM was 9.27%)</t>
+          <t>Discount Rate (Yacktman-adj CAPM WACC = R15 ≈ 7.68%; Model17 was 7.68%)</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
         <is>
-          <t>Updated WACC from Model16 (Previous: raw CAPM 9.27%, β=1.32) to Model17 (New: Yacktman-adj CAPM 7.68% = Rf 4.67% + β 0.854 × ERP 4.28%; Rd 6.250%)</t>
+          <t>WACC algebra unchanged vs Model17 (Previous: 7.68%) in Model18 (New: 7.68% = Rf 4.67% + β 0.854 × ERP 4.28%; Rd 6.250%). Stub fix is temporal, not WACC.</t>
         </is>
       </c>
       <c r="D6" s="111">
@@ -6531,7 +6542,7 @@
       </c>
       <c r="C7" s="109" t="inlineStr">
         <is>
-          <t>Updated g from Model16 (Previous: 3.0%) to Model17 (New: 3.5%)</t>
+          <t>g unchanged vs Model17 (Previous: 3.5%) in Model18</t>
         </is>
       </c>
       <c r="D7" s="112" t="n">
@@ -6616,16 +6627,16 @@
       <c r="A9" s="100" t="n"/>
       <c r="B9" s="100" t="inlineStr">
         <is>
-          <t>Transaction Date (= last hist FYE on 3S)</t>
+          <t>Valuation Date (stub clock; 2026-08-06)</t>
         </is>
       </c>
       <c r="C9" s="109" t="inlineStr">
         <is>
-          <t>Matches 3S hist FYE (Sep 30)</t>
+          <t>Updated from Model17 (Previous: hist FYE 2025-09-30) to Model18 (New: 2026-08-06; 129/365=35.34% elapsed)</t>
         </is>
       </c>
       <c r="D9" s="117" t="n">
-        <v>43100</v>
+        <v>46240</v>
       </c>
       <c r="E9" s="100" t="n"/>
       <c r="F9" s="100" t="n"/>
@@ -6653,12 +6664,16 @@
       <c r="A10" s="100" t="n"/>
       <c r="B10" s="100" t="inlineStr">
         <is>
-          <t>Fiscal Year End (first forecast FYE)</t>
-        </is>
-      </c>
-      <c r="C10" s="100" t="n"/>
+          <t>Stub FY End (first forward year end)</t>
+        </is>
+      </c>
+      <c r="C10" s="109" t="inlineStr">
+        <is>
+          <t>Stub year ends 2027-03-29</t>
+        </is>
+      </c>
       <c r="D10" s="117" t="n">
-        <v>43281</v>
+        <v>46475</v>
       </c>
       <c r="E10" s="100" t="n"/>
       <c r="F10" s="100" t="n"/>
@@ -6788,7 +6803,7 @@
       <c r="A15" s="100" t="n"/>
       <c r="B15" s="100" t="inlineStr">
         <is>
-          <t>Capex FY1 (linked to 3S J68)</t>
+          <t>Capex FY1 (linked to 3S J68; stub scales FCFF not CapEx cell)</t>
         </is>
       </c>
       <c r="C15" s="100" t="n"/>
@@ -6817,7 +6832,7 @@
       </c>
       <c r="C16" s="109" t="inlineStr">
         <is>
-          <t>Shares_t = Shares_t−1 + EquityCF_t/Price; EquityCF = 3S 1.4×FCF buybacks (row 20)</t>
+          <t>Shares_t = prior + EquityCF/Price; Y1 EquityCF × 64.66% stub</t>
         </is>
       </c>
       <c r="D16" s="123">
@@ -6825,7 +6840,7 @@
         <v/>
       </c>
       <c r="E16" s="123">
-        <f>MAX(1000,D16+'3 Statement Model'!J20/$D$11)</f>
+        <f>MAX(1000,D16+0.646575*'3 Statement Model'!J20/$D$11)</f>
         <v/>
       </c>
       <c r="F16" s="123">
@@ -6892,7 +6907,7 @@
       <c r="K17" s="100" t="n"/>
       <c r="L17" s="128" t="inlineStr">
         <is>
-          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL17.0)</t>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL18.0)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -6901,7 +6916,7 @@
       <c r="A18" s="100" t="n"/>
       <c r="B18" s="100" t="inlineStr">
         <is>
-          <t>Date (mid-year via EDATE; periods are 0-based)</t>
+          <t>Date (Y1 mid-stub +118d; Y2–Y5 EDATE mid-year)</t>
         </is>
       </c>
       <c r="C18" s="100" t="n"/>
@@ -6909,24 +6924,23 @@
         <f>$D$9</f>
         <v/>
       </c>
-      <c r="E18" s="129">
-        <f>EDATE($D$9,(E19+0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="F18" s="129">
-        <f>EDATE($D$9,(F19+0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="G18" s="129">
-        <f>EDATE($D$9,(G19+0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="H18" s="129">
-        <f>EDATE($D$9,(H19+0.5)*12)</f>
-        <v/>
-      </c>
-      <c r="I18" s="129">
-        <f>EDATE($D$9,(I19+0.5)*12)</f>
+      <c r="E18" s="130" t="n">
+        <v>46358</v>
+      </c>
+      <c r="F18" s="130">
+        <f>EDATE(DATE(2027,3,30),6)</f>
+        <v/>
+      </c>
+      <c r="G18" s="130">
+        <f>EDATE(DATE(2028,3,30),6)</f>
+        <v/>
+      </c>
+      <c r="H18" s="130">
+        <f>EDATE(DATE(2029,3,30),6)</f>
+        <v/>
+      </c>
+      <c r="I18" s="130">
+        <f>EDATE(DATE(2030,3,30),6)</f>
         <v/>
       </c>
       <c r="J18" s="129">
@@ -6952,33 +6966,33 @@
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="100" t="n"/>
-      <c r="B19" s="130" t="inlineStr">
+      <c r="B19" s="131" t="inlineStr">
         <is>
           <t>Time Periods</t>
         </is>
       </c>
-      <c r="C19" s="130" t="n"/>
-      <c r="D19" s="131" t="n"/>
-      <c r="E19" s="132" t="n">
+      <c r="C19" s="131" t="n"/>
+      <c r="D19" s="132" t="n"/>
+      <c r="E19" s="133" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="133">
+      <c r="F19" s="134">
         <f>E19+1</f>
         <v/>
       </c>
-      <c r="G19" s="133">
+      <c r="G19" s="134">
         <f>F19+1</f>
         <v/>
       </c>
-      <c r="H19" s="133">
+      <c r="H19" s="134">
         <f>G19+1</f>
         <v/>
       </c>
-      <c r="I19" s="133">
+      <c r="I19" s="134">
         <f>H19+1</f>
         <v/>
       </c>
-      <c r="J19" s="131" t="n"/>
+      <c r="J19" s="132" t="n"/>
       <c r="K19" s="100" t="n"/>
       <c r="L19" s="100" t="inlineStr">
         <is>
@@ -6989,7 +7003,7 @@
         <f>IF(($D$6-$D$7)&lt;=0,"WACC must exceed g",$I$26*(1+$D$7)/($D$6-$D$7))</f>
         <v/>
       </c>
-      <c r="N19" s="134" t="inlineStr">
+      <c r="N19" s="135" t="inlineStr">
         <is>
           <t>← sanity check</t>
         </is>
@@ -6998,30 +7012,30 @@
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="100" t="n"/>
-      <c r="B20" s="130" t="inlineStr">
+      <c r="B20" s="131" t="inlineStr">
         <is>
           <t>Year Fraction (display only; XNPV uses exact dates below)</t>
         </is>
       </c>
       <c r="C20" s="100" t="n"/>
       <c r="D20" s="100" t="n"/>
-      <c r="E20" s="135">
+      <c r="E20" s="136">
         <f>YEARFRAC(D18,E18)</f>
         <v/>
       </c>
-      <c r="F20" s="135">
+      <c r="F20" s="136">
         <f>YEARFRAC(E18,F18)</f>
         <v/>
       </c>
-      <c r="G20" s="135">
+      <c r="G20" s="136">
         <f>YEARFRAC(F18,G18)</f>
         <v/>
       </c>
-      <c r="H20" s="135">
+      <c r="H20" s="136">
         <f>YEARFRAC(G18,H18)</f>
         <v/>
       </c>
-      <c r="I20" s="135">
+      <c r="I20" s="136">
         <f>YEARFRAC(H18,I18)</f>
         <v/>
       </c>
@@ -7036,7 +7050,7 @@
         <f>IF(($I$21+$I$23)=0,0,M19/($I$21+$I$23))</f>
         <v/>
       </c>
-      <c r="N20" s="136" t="inlineStr">
+      <c r="N20" s="137" t="inlineStr">
         <is>
           <t>← ~bear check</t>
         </is>
@@ -7099,23 +7113,23 @@
       </c>
       <c r="C22" s="100" t="n"/>
       <c r="D22" s="100" t="n"/>
-      <c r="E22" s="137">
+      <c r="E22" s="138">
         <f>E21*$D$5</f>
         <v/>
       </c>
-      <c r="F22" s="137">
+      <c r="F22" s="138">
         <f>F21*$D$5</f>
         <v/>
       </c>
-      <c r="G22" s="137">
+      <c r="G22" s="138">
         <f>G21*$D$5</f>
         <v/>
       </c>
-      <c r="H22" s="137">
+      <c r="H22" s="138">
         <f>H21*$D$5</f>
         <v/>
       </c>
-      <c r="I22" s="137">
+      <c r="I22" s="138">
         <f>I21*$D$5</f>
         <v/>
       </c>
@@ -7146,23 +7160,23 @@
       </c>
       <c r="C23" s="100" t="n"/>
       <c r="D23" s="100" t="n"/>
-      <c r="E23" s="137">
+      <c r="E23" s="138">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="F23" s="137">
+      <c r="F23" s="138">
         <f>'3 Statement Model'!K30</f>
         <v/>
       </c>
-      <c r="G23" s="137">
+      <c r="G23" s="138">
         <f>'3 Statement Model'!L30</f>
         <v/>
       </c>
-      <c r="H23" s="137">
+      <c r="H23" s="138">
         <f>'3 Statement Model'!M30</f>
         <v/>
       </c>
-      <c r="I23" s="137">
+      <c r="I23" s="138">
         <f>'3 Statement Model'!N30</f>
         <v/>
       </c>
@@ -7261,40 +7275,40 @@
       <c r="A26" s="100" t="n"/>
       <c r="B26" s="100" t="inlineStr">
         <is>
-          <t>Unlevered FCF (SBC add-back + Deferred cash source)</t>
+          <t>Unlevered FCF (Y1 × 64.66% stub remaining; SBC + Deferred)</t>
         </is>
       </c>
       <c r="C26" s="100" t="inlineStr">
         <is>
-          <t>FCFF=EBIT−cashTax+DA+SBC−CapEx−ΔOpNWC+ΔDeferred</t>
+          <t>Y1 FCFF=stub(0.6466)×(EBIT−cashTax+DA+SBC−CapEx−ΔOpNWC+ΔDef); Y2–Y5 full year</t>
         </is>
       </c>
       <c r="D26" s="100" t="n"/>
-      <c r="E26" s="138">
-        <f>E21-E22+E23+'3 Statement Model'!J64-E24-E25</f>
-        <v/>
-      </c>
-      <c r="F26" s="138">
+      <c r="E26" s="139">
+        <f>0.646575*(E21-E22+E23+'3 Statement Model'!J64-E24-E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="139">
         <f>F21-F22+F23+'3 Statement Model'!K64-F24-F25</f>
         <v/>
       </c>
-      <c r="G26" s="138">
+      <c r="G26" s="139">
         <f>G21-G22+G23+'3 Statement Model'!L64-G24-G25</f>
         <v/>
       </c>
-      <c r="H26" s="138">
+      <c r="H26" s="139">
         <f>H21-H22+H23+'3 Statement Model'!M64-H24-H25</f>
         <v/>
       </c>
-      <c r="I26" s="138">
+      <c r="I26" s="139">
         <f>I21-I22+I23+'3 Statement Model'!N64-I24-I25</f>
         <v/>
       </c>
       <c r="J26" s="100" t="n"/>
       <c r="K26" s="100" t="n"/>
-      <c r="L26" s="139" t="inlineStr">
-        <is>
-          <t>vengeanceaiUSCMODEL17.0 — DCF ← 3-Statement linkage audit</t>
+      <c r="L26" s="140" t="inlineStr">
+        <is>
+          <t>vengeanceaiUSCMODEL18.0 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7320,22 +7334,22 @@
         <v/>
       </c>
       <c r="K27" s="100" t="n"/>
-      <c r="L27" s="140" t="inlineStr">
+      <c r="L27" s="141" t="inlineStr">
         <is>
           <t>DCF item</t>
         </is>
       </c>
-      <c r="M27" s="140" t="inlineStr">
+      <c r="M27" s="141" t="inlineStr">
         <is>
           <t>Value / link</t>
         </is>
       </c>
-      <c r="N27" s="140" t="inlineStr">
+      <c r="N27" s="141" t="inlineStr">
         <is>
           <t>3-Statement source</t>
         </is>
       </c>
-      <c r="O27" s="140" t="inlineStr">
+      <c r="O27" s="141" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -7349,30 +7363,30 @@
         </is>
       </c>
       <c r="C28" s="100" t="n"/>
-      <c r="D28" s="136" t="n">
+      <c r="D28" s="137" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="138">
+      <c r="E28" s="139">
         <f>E27+E26</f>
         <v/>
       </c>
-      <c r="F28" s="138">
+      <c r="F28" s="139">
         <f>F27+F26</f>
         <v/>
       </c>
-      <c r="G28" s="138">
+      <c r="G28" s="139">
         <f>G27+G26</f>
         <v/>
       </c>
-      <c r="H28" s="138">
+      <c r="H28" s="139">
         <f>H27+H26</f>
         <v/>
       </c>
-      <c r="I28" s="138">
+      <c r="I28" s="139">
         <f>I27+I26</f>
         <v/>
       </c>
-      <c r="J28" s="138">
+      <c r="J28" s="139">
         <f>J27+J26</f>
         <v/>
       </c>
@@ -7382,16 +7396,16 @@
           <t>Cash tax rate (D5)</t>
         </is>
       </c>
-      <c r="M28" s="141">
+      <c r="M28" s="142">
         <f>$D$5</f>
         <v/>
       </c>
-      <c r="N28" s="142" t="inlineStr">
+      <c r="N28" s="143" t="inlineStr">
         <is>
           <t>22.87%</t>
         </is>
       </c>
-      <c r="O28" s="143" t="inlineStr">
+      <c r="O28" s="144" t="inlineStr">
         <is>
           <t>3yr avg IncomeTaxesPaidNet/EBT (not book J13)</t>
         </is>
@@ -7439,15 +7453,15 @@
           <t>DSO (AR days)</t>
         </is>
       </c>
-      <c r="M29" s="141">
+      <c r="M29" s="142">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="N29" s="144">
+      <c r="N29" s="145">
         <f>'3 Statement Model'!J15</f>
         <v/>
       </c>
-      <c r="O29" s="143" t="inlineStr">
+      <c r="O29" s="144" t="inlineStr">
         <is>
           <t>Phased DSO hist→45d; Op NWC excludes Deferred</t>
         </is>
@@ -7468,15 +7482,15 @@
           <t>SBC % of sales</t>
         </is>
       </c>
-      <c r="M30" s="141">
+      <c r="M30" s="142">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="N30" s="144">
+      <c r="N30" s="145">
         <f>'3 Statement Model'!J21</f>
         <v/>
       </c>
-      <c r="O30" s="143" t="inlineStr">
+      <c r="O30" s="144" t="inlineStr">
         <is>
           <t>SBC add-back in CFO row 64 and FCFF</t>
         </is>
@@ -7500,20 +7514,20 @@
       <c r="H31" s="125" t="n"/>
       <c r="I31" s="125" t="n"/>
       <c r="J31" s="100" t="n"/>
-      <c r="L31" s="145" t="inlineStr">
+      <c r="L31" s="146" t="inlineStr">
         <is>
           <t>CapEx % (FY1)</t>
         </is>
       </c>
-      <c r="M31" s="141">
+      <c r="M31" s="142">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="N31" s="144">
+      <c r="N31" s="145">
         <f>'3 Statement Model'!J18</f>
         <v/>
       </c>
-      <c r="O31" s="143" t="inlineStr">
+      <c r="O31" s="144" t="inlineStr">
         <is>
           <t>CapEx% fade path → CF CapEx $</t>
         </is>
@@ -7523,7 +7537,7 @@
       <c r="A32" s="100" t="n"/>
       <c r="B32" s="100" t="inlineStr">
         <is>
-          <t>Enterprise Value (XNPV, mid-year EDATE dates)</t>
+          <t>Enterprise Value (XNPV; Y1 mid-stub dates)</t>
         </is>
       </c>
       <c r="C32" s="100" t="n"/>
@@ -7548,15 +7562,15 @@
           <t>Revenue growth FY1</t>
         </is>
       </c>
-      <c r="M32" s="144">
+      <c r="M32" s="145">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="N32" s="146">
+      <c r="N32" s="147">
         <f>'3 Statement Model'!J7</f>
         <v/>
       </c>
-      <c r="O32" s="143" t="inlineStr">
+      <c r="O32" s="144" t="inlineStr">
         <is>
           <t>Policy path on 3S assumption row 7</t>
         </is>
@@ -7591,15 +7605,15 @@
           <t>EBIT FY1 (DCF E21)</t>
         </is>
       </c>
-      <c r="M33" s="147">
+      <c r="M33" s="148">
         <f>$E$21</f>
         <v/>
       </c>
-      <c r="N33" s="147">
+      <c r="N33" s="148">
         <f>'3 Statement Model'!J33+'3 Statement Model'!J31</f>
         <v/>
       </c>
-      <c r="O33" s="143" t="inlineStr">
+      <c r="O33" s="144" t="inlineStr">
         <is>
           <t>EBT + Interest = GP − SG&amp;A − R&amp;D − D&amp;A</t>
         </is>
@@ -7634,16 +7648,16 @@
           <t>EBIT cross-check</t>
         </is>
       </c>
-      <c r="M34" s="147">
+      <c r="M34" s="148">
         <f>'3 Statement Model'!J26-'3 Statement Model'!J28-'3 Statement Model'!J29-'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="N34" s="142" t="inlineStr">
+      <c r="N34" s="143" t="inlineStr">
         <is>
           <t>GP−SGA−R&amp;D−DA</t>
         </is>
       </c>
-      <c r="O34" s="143" t="inlineStr">
+      <c r="O34" s="144" t="inlineStr">
         <is>
           <t>Must equal E21 (live check)</t>
         </is>
@@ -7657,7 +7671,7 @@
         </is>
       </c>
       <c r="C35" s="100" t="n"/>
-      <c r="D35" s="136">
+      <c r="D35" s="137">
         <f>D32+D33-D34</f>
         <v/>
       </c>
@@ -7668,25 +7682,25 @@
         </is>
       </c>
       <c r="H35" s="100" t="n"/>
-      <c r="I35" s="136">
+      <c r="I35" s="137">
         <f>I32+I33-I34</f>
         <v/>
       </c>
       <c r="J35" s="100" t="n"/>
-      <c r="L35" s="145" t="inlineStr">
+      <c r="L35" s="146" t="inlineStr">
         <is>
           <t>D&amp;A FY1</t>
         </is>
       </c>
-      <c r="M35" s="147">
+      <c r="M35" s="148">
         <f>$E$23</f>
         <v/>
       </c>
-      <c r="N35" s="147">
+      <c r="N35" s="148">
         <f>'3 Statement Model'!J30</f>
         <v/>
       </c>
-      <c r="O35" s="143" t="inlineStr">
+      <c r="O35" s="144" t="inlineStr">
         <is>
           <t>Rev × DA% (total D&amp;A / sales) from 3S IS</t>
         </is>
@@ -7700,22 +7714,22 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="148" t="n"/>
+      <c r="I36" s="149" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
           <t>SBC FY1</t>
         </is>
       </c>
-      <c r="M36" s="147">
+      <c r="M36" s="148">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="N36" s="147">
+      <c r="N36" s="148">
         <f>'3 Statement Model'!J64</f>
         <v/>
       </c>
-      <c r="O36" s="143" t="inlineStr">
+      <c r="O36" s="144" t="inlineStr">
         <is>
           <t>Rev × SBC%; added in FCFF</t>
         </is>
@@ -7730,10 +7744,10 @@
       </c>
       <c r="C37" s="109" t="inlineStr">
         <is>
-          <t>MODEL17: SBC add-back in FCFF; 1.4×FCF buybacks cut shares (no SBC dilution)</t>
-        </is>
-      </c>
-      <c r="D37" s="149">
+          <t>MODEL18: SBC add-back in FCFF; 1.4×FCF buybacks cut shares (no SBC dilution)</t>
+        </is>
+      </c>
+      <c r="D37" s="150">
         <f>$D$35/$I$16</f>
         <v/>
       </c>
@@ -7744,7 +7758,7 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="148">
+      <c r="I37" s="149">
         <f>D11</f>
         <v/>
       </c>
@@ -7754,15 +7768,15 @@
           <t>CapEx FY1</t>
         </is>
       </c>
-      <c r="M37" s="147">
+      <c r="M37" s="148">
         <f>$E$24</f>
         <v/>
       </c>
-      <c r="N37" s="147">
+      <c r="N37" s="148">
         <f>'3 Statement Model'!J68</f>
         <v/>
       </c>
-      <c r="O37" s="143" t="inlineStr">
+      <c r="O37" s="144" t="inlineStr">
         <is>
           <t>3S CF CapEx (also D15)</t>
         </is>
@@ -7783,15 +7797,15 @@
           <t>Net WC use FY1</t>
         </is>
       </c>
-      <c r="M38" s="147">
+      <c r="M38" s="148">
         <f>$E$25</f>
         <v/>
       </c>
-      <c r="N38" s="147">
+      <c r="N38" s="148">
         <f>'3 Statement Model'!J90-('3 Statement Model'!J88-'3 Statement Model'!I88)</f>
         <v/>
       </c>
-      <c r="O38" s="143" t="inlineStr">
+      <c r="O38" s="144" t="inlineStr">
         <is>
           <t>ΔOpNWC − ΔDeferred (AR≠Deferred)</t>
         </is>
@@ -7811,15 +7825,15 @@
           <t>EBITDA FY5 (TV base)</t>
         </is>
       </c>
-      <c r="M39" s="147">
+      <c r="M39" s="148">
         <f>$I$21+$I$23</f>
         <v/>
       </c>
-      <c r="N39" s="147">
+      <c r="N39" s="148">
         <f>'3 Statement Model'!N33+'3 Statement Model'!N31+'3 Statement Model'!N30</f>
         <v/>
       </c>
-      <c r="O39" s="143" t="inlineStr">
+      <c r="O39" s="144" t="inlineStr">
         <is>
           <t>EBIT+D&amp;A; Exit TV = this × D8</t>
         </is>
@@ -7840,15 +7854,15 @@
           <t>3S FY25 Cash (ref)</t>
         </is>
       </c>
-      <c r="M40" s="147">
+      <c r="M40" s="148">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="N40" s="147">
+      <c r="N40" s="148">
         <f>'3 Statement Model'!I41</f>
         <v/>
       </c>
-      <c r="O40" s="143" t="inlineStr">
+      <c r="O40" s="144" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D14</t>
         </is>
@@ -7862,7 +7876,7 @@
         </is>
       </c>
       <c r="C41" s="125" t="n"/>
-      <c r="D41" s="150" t="n"/>
+      <c r="D41" s="151" t="n"/>
       <c r="E41" s="125" t="n"/>
       <c r="F41" s="125" t="n"/>
       <c r="G41" s="125" t="n"/>
@@ -7870,20 +7884,20 @@
       <c r="I41" s="125" t="n"/>
       <c r="J41" s="125" t="n"/>
       <c r="K41" s="125" t="n"/>
-      <c r="L41" s="145" t="inlineStr">
+      <c r="L41" s="146" t="inlineStr">
         <is>
           <t>3S FY25 Debt (ref)</t>
         </is>
       </c>
-      <c r="M41" s="147">
+      <c r="M41" s="148">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="N41" s="147">
+      <c r="N41" s="148">
         <f>'3 Statement Model'!I49</f>
         <v/>
       </c>
-      <c r="O41" s="143" t="inlineStr">
+      <c r="O41" s="144" t="inlineStr">
         <is>
           <t>FYE reference only — bridge uses 10-Q D13</t>
         </is>
@@ -7902,17 +7916,17 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="L42" s="151" t="inlineStr">
+      <c r="L42" s="152" t="inlineStr">
         <is>
           <t>EBIT link OK?</t>
         </is>
       </c>
-      <c r="M42" s="152">
+      <c r="M42" s="153">
         <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
         <v/>
       </c>
-      <c r="N42" s="153" t="inlineStr"/>
-      <c r="O42" s="143" t="inlineStr">
+      <c r="N42" s="154" t="inlineStr"/>
+      <c r="O42" s="144" t="inlineStr">
         <is>
           <t>Flags if EBIT link ≠ GP−opex build</t>
         </is>
@@ -7931,7 +7945,7 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="L43" s="154" t="inlineStr">
+      <c r="L43" s="155" t="inlineStr">
         <is>
           <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman-adj CAPM 7.68% (D6←R15; raw CAPM ref 9.27%). $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute.</t>
         </is>
@@ -7939,7 +7953,7 @@
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="155" t="inlineStr">
+      <c r="B44" s="156" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7955,7 +7969,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="155" t="inlineStr">
+      <c r="B45" s="156" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7971,7 +7985,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="155" t="inlineStr">
+      <c r="B46" s="156" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -8006,7 +8020,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="156" t="inlineStr">
+      <c r="N48" s="157" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -8022,7 +8036,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="157" t="inlineStr">
+      <c r="N49" s="158" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8115,7 +8129,7 @@
       <c r="I55" s="100" t="n"/>
       <c r="J55" s="100" t="n"/>
       <c r="K55" s="100" t="n"/>
-      <c r="L55" s="139" t="inlineStr">
+      <c r="L55" s="140" t="inlineStr">
         <is>
           <t>SENSITIVITY — Enterprise Value ($000s)</t>
         </is>
@@ -8138,22 +8152,22 @@
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="158" t="n">
+      <c r="M56" s="159" t="n">
         <v>17</v>
       </c>
-      <c r="N56" s="158" t="n">
+      <c r="N56" s="159" t="n">
         <v>20</v>
       </c>
-      <c r="O56" s="158" t="n">
+      <c r="O56" s="159" t="n">
         <v>23</v>
       </c>
-      <c r="P56" s="158" t="n">
+      <c r="P56" s="159" t="n">
         <v>25</v>
       </c>
-      <c r="Q56" s="158" t="n">
+      <c r="Q56" s="159" t="n">
         <v>27</v>
       </c>
-      <c r="R56" s="158" t="n">
+      <c r="R56" s="159" t="n">
         <v>29</v>
       </c>
     </row>
@@ -8169,30 +8183,30 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="159" t="n">
+      <c r="L57" s="160" t="n">
         <v>0.065</v>
       </c>
-      <c r="M57" s="147">
+      <c r="M57" s="148">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N57" s="147">
+      <c r="N57" s="148">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O57" s="147">
+      <c r="O57" s="148">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P57" s="147">
+      <c r="P57" s="148">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q57" s="147">
+      <c r="Q57" s="148">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R57" s="147">
+      <c r="R57" s="148">
         <f>XNPV($L57,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L57)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8209,30 +8223,30 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="159" t="n">
+      <c r="L58" s="160" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="M58" s="147">
+      <c r="M58" s="148">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N58" s="147">
+      <c r="N58" s="148">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O58" s="147">
+      <c r="O58" s="148">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P58" s="147">
+      <c r="P58" s="148">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q58" s="147">
+      <c r="Q58" s="148">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R58" s="147">
+      <c r="R58" s="148">
         <f>XNPV($L58,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L58)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8249,30 +8263,30 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="159" t="n">
+      <c r="L59" s="160" t="n">
         <v>0.075</v>
       </c>
-      <c r="M59" s="147">
+      <c r="M59" s="148">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N59" s="147">
+      <c r="N59" s="148">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O59" s="147">
+      <c r="O59" s="148">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P59" s="147">
+      <c r="P59" s="148">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q59" s="147">
+      <c r="Q59" s="148">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R59" s="147">
+      <c r="R59" s="148">
         <f>XNPV($L59,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L59)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8289,30 +8303,30 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="159" t="n">
+      <c r="L60" s="160" t="n">
         <v>0.07679999999999999</v>
       </c>
-      <c r="M60" s="147">
+      <c r="M60" s="148">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N60" s="147">
+      <c r="N60" s="148">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="160">
+      <c r="O60" s="161">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P60" s="147">
+      <c r="P60" s="148">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q60" s="147">
+      <c r="Q60" s="148">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R60" s="147">
+      <c r="R60" s="148">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8328,271 +8342,271 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="159" t="n">
+      <c r="L61" s="160" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="M61" s="147">
+      <c r="M61" s="148">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N61" s="147">
+      <c r="N61" s="148">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O61" s="147">
+      <c r="O61" s="148">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P61" s="147">
+      <c r="P61" s="148">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q61" s="147">
+      <c r="Q61" s="148">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R61" s="147">
+      <c r="R61" s="148">
         <f>XNPV($L61,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L61)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="L62" s="159" t="n">
+      <c r="L62" s="160" t="n">
         <v>0.095</v>
       </c>
-      <c r="M62" s="147">
+      <c r="M62" s="148">
         <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*M$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="N62" s="147">
+      <c r="N62" s="148">
         <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O62" s="147">
+      <c r="O62" s="148">
         <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="P62" s="147">
+      <c r="P62" s="148">
         <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*P$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="Q62" s="147">
+      <c r="Q62" s="148">
         <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*Q$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="R62" s="147">
+      <c r="R62" s="148">
         <f>XNPV($L62,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*R$56)/((1+$L62)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="161" t="inlineStr">
+      <c r="L64" s="162" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="162" t="inlineStr">
+      <c r="L65" s="163" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="163" t="n">
+      <c r="M65" s="164" t="n">
         <v>17</v>
       </c>
-      <c r="N65" s="163" t="n">
+      <c r="N65" s="164" t="n">
         <v>20</v>
       </c>
-      <c r="O65" s="163" t="n">
+      <c r="O65" s="164" t="n">
         <v>23</v>
       </c>
-      <c r="P65" s="163" t="n">
+      <c r="P65" s="164" t="n">
         <v>25</v>
       </c>
-      <c r="Q65" s="163" t="n">
+      <c r="Q65" s="164" t="n">
         <v>27</v>
       </c>
-      <c r="R65" s="163" t="n">
+      <c r="R65" s="164" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="159" t="n">
+      <c r="L66" s="160" t="n">
         <v>0.065</v>
       </c>
-      <c r="M66" s="164">
+      <c r="M66" s="165">
         <f>(M57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N66" s="164">
+      <c r="N66" s="165">
         <f>(N57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O66" s="164">
+      <c r="O66" s="165">
         <f>(O57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P66" s="164">
+      <c r="P66" s="165">
         <f>(P57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q66" s="164">
+      <c r="Q66" s="165">
         <f>(Q57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R66" s="164">
+      <c r="R66" s="165">
         <f>(R57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="159" t="n">
+      <c r="L67" s="160" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="M67" s="164">
+      <c r="M67" s="165">
         <f>(M58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N67" s="164">
+      <c r="N67" s="165">
         <f>(N58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O67" s="164">
+      <c r="O67" s="165">
         <f>(O58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P67" s="164">
+      <c r="P67" s="165">
         <f>(P58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q67" s="164">
+      <c r="Q67" s="165">
         <f>(Q58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R67" s="164">
+      <c r="R67" s="165">
         <f>(R58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="159" t="n">
+      <c r="L68" s="160" t="n">
         <v>0.075</v>
       </c>
-      <c r="M68" s="164">
+      <c r="M68" s="165">
         <f>(M59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N68" s="164">
+      <c r="N68" s="165">
         <f>(N59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O68" s="164">
+      <c r="O68" s="165">
         <f>(O59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P68" s="164">
+      <c r="P68" s="165">
         <f>(P59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q68" s="164">
+      <c r="Q68" s="165">
         <f>(Q59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R68" s="164">
+      <c r="R68" s="165">
         <f>(R59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="159" t="n">
+      <c r="L69" s="160" t="n">
         <v>0.07679999999999999</v>
       </c>
-      <c r="M69" s="164">
+      <c r="M69" s="165">
         <f>(M60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N69" s="164">
+      <c r="N69" s="165">
         <f>(N60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O69" s="165">
+      <c r="O69" s="166">
         <f>(O60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P69" s="164">
+      <c r="P69" s="165">
         <f>(P60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q69" s="164">
+      <c r="Q69" s="165">
         <f>(Q60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R69" s="164">
+      <c r="R69" s="165">
         <f>(R60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="159" t="n">
+      <c r="L70" s="160" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="M70" s="164">
+      <c r="M70" s="165">
         <f>(M61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N70" s="164">
+      <c r="N70" s="165">
         <f>(N61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O70" s="164">
+      <c r="O70" s="165">
         <f>(O61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P70" s="164">
+      <c r="P70" s="165">
         <f>(P61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q70" s="164">
+      <c r="Q70" s="165">
         <f>(Q61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R70" s="164">
+      <c r="R70" s="165">
         <f>(R61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="L71" s="159" t="n">
+      <c r="L71" s="160" t="n">
         <v>0.095</v>
       </c>
-      <c r="M71" s="164">
+      <c r="M71" s="165">
         <f>(M62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N71" s="164">
+      <c r="N71" s="165">
         <f>(N62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O71" s="164">
+      <c r="O71" s="165">
         <f>(O62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P71" s="164">
+      <c r="P71" s="165">
         <f>(P62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q71" s="164">
+      <c r="Q71" s="165">
         <f>(Q62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R71" s="164">
+      <c r="R71" s="165">
         <f>(R62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="154" t="inlineStr">
+      <c r="L72" s="155" t="inlineStr">
         <is>
           <t>Yellow = base (Yacktman WACC=7.68%, Exit 23.0x; CAPM ref ≈9.27%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 23.0x; bull 27x; bear 17.0x.</t>
         </is>

</xml_diff>

<commit_message>
MODEL20: subtract forecast buyback-funded debt in equity bridge
MODEL18 shrank shares via 1.4×FCF levered buybacks but left D34 = today's
10-Q debt only. D34 now equals D13 + stub×Y1 debt CF + Y2–Y5 debt CF so
$/share pairs Y5 shares with the debt that funded the buybacks.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22296" windowHeight="8376" tabRatio="685" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover Page" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3 Statement Model" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DCF Model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover Page" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Statement Model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF Model" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="IS_BaseYear">'3 Statement Model'!$E$2</definedName>
@@ -95,12 +95,12 @@
     <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0.00_-;\(#,##0.00\)_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="175" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="176" formatCode="0.0"/>
-    <numFmt numFmtId="177" formatCode="#,##0.000"/>
-    <numFmt numFmtId="178" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="179" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="180" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="181" formatCode="#,##0.0"/>
+    <numFmt numFmtId="176" formatCode="#,##0.0"/>
+    <numFmt numFmtId="177" formatCode="0.0"/>
+    <numFmt numFmtId="178" formatCode="#,##0.000"/>
+    <numFmt numFmtId="179" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="180" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="181" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="48">
     <font>
@@ -541,7 +541,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -711,7 +711,7 @@
     </xf>
     <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="33" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="32" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -725,15 +725,15 @@
     <xf numFmtId="166" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="177" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="175" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="180" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -741,7 +741,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -768,9 +768,10 @@
     <xf numFmtId="164" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="181" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -789,16 +790,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="180" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="181" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="180" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -839,14 +840,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -869,16 +870,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -920,10 +921,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent1"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -974,10 +975,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent3"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1028,10 +1029,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent2"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1091,8 +1092,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -1104,9 +1105,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1145,16 +1146,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1183,16 +1184,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -1217,8 +1218,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1228,14 +1229,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -1263,16 +1264,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -1306,10 +1307,10 @@
             <v>Operating</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent2"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1352,10 +1353,10 @@
             <v>Investing</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent3"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1398,10 +1399,10 @@
             <v>FInancing</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1462,8 +1463,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -1475,9 +1476,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1516,16 +1517,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1554,16 +1555,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -1588,8 +1589,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1601,7 +1602,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>vengeanceaiUSCMODEL18.0</author>
+    <author>vengeanceaiUSCMODEL20.0</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
@@ -1615,9 +1616,9 @@
     </comment>
     <comment ref="D6" authorId="0" shapeId="0">
       <text>
-        <t>Yacktman-adjusted CAPM WACC (MODEL18 primary discount rate).
+        <t>Yacktman-adjusted CAPM WACC (MODEL20 primary discount rate).
 HOW: D6 = R15 = We×Ke + Wd×Rd(1−t). β_Yacktman=0.854 (Blume+AAA blend; Yahoo raw 1.32). Rf=4.67%, ERP=4.28%, Rd=6.250%.
-WHY: Same algebraic CAPM as Model17 (7.68%); MODEL18 changes stub timing / SBC / SaaS mix — not a naked WACC override.
+WHY: Same algebraic CAPM as Model17 (7.68%); MODEL20 changes stub timing / SBC / SaaS mix — not a naked WACC override.
 SOURCE: Blume 1971; FRED DGS10; Yahoo β; Damodaran ERP; 8-K notes.</t>
       </text>
     </comment>
@@ -1632,7 +1633,7 @@
     </comment>
     <comment ref="D9" authorId="0" shapeId="0">
       <text>
-        <t>MODEL18 stub-period valuation date.
+        <t>MODEL20 stub-period valuation date.
 HOW: D9 = 2026-08-06. FY stub starts 2026-03-30; 129 of 365 days elapsed (35.34%); 64.66% remains.
 Y1 FCFF scaled by 0.6466; E18 = D9+118d (mid-stub 2026-12-02).
 WHY: Do not discount cash that has already occurred.
@@ -1643,8 +1644,16 @@
       <text>
         <t>Buyback-adjusted share schedule (Yacktman — no SBC double penalty).
 HOW: D16 = starting shares (D12 ≈ 21,597.6k post–Q3 @ $1,149). Each year: Shares += 3S EquityIssuance (row 20) / Price. Row 20 = −1.4×(CFO−CapEx) levered buybacks so the share count falls faster.
-WHY: SBC is already added back in FCFF — diluting by SBC$/Price would double-penalize. Q3 FY2026 buybacks &gt;&gt; FCF prove levered repurchase capacity.
+WHY: SBC is already added back in FCFF — diluting by SBC$/Price would double-penalize. MODEL20 pairs I16 with D34 = today debt + forecast issuance (row 19) so leverage is not free.
 SOURCE: EX-99.1 Q3 FY2026; 10-K FY2025 repurchase footnote.</t>
+      </text>
+    </comment>
+    <comment ref="D34" authorId="0" shapeId="0">
+      <text>
+        <t>MODEL20 equity-bridge debt (pairs with Y5 buyback-adjusted shares).
+HOW: D34 = D13 + 0.6466×3S!J19 + K19+L19+M19+N19. Row 19 = (1.4−1)×FCF debt that funds levered buybacks; Y1 stub-scaled like Y1 share buybacks.
+WHY: Model18 cut shares ~21.6M→~11M but still subtracted only today's debt — overstated $/share. Cash D33 stays 10-Q (ΔCash≈0 by design).
+SOURCE: 3S financing rows 19–20; 10-Q debt D13.</t>
       </text>
     </comment>
   </commentList>
@@ -1652,7 +1661,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -1669,27 +1678,27 @@
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Picture 1">
-          <a:hlinkClick r:id="rId1"/>
+          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </cNvPr>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="1447799" y="762000"/>
           <a:ext cx="3359943" cy="1581150"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1700,7 +1709,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>1</col>
@@ -1720,9 +1729,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1747,9 +1756,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1771,27 +1780,27 @@
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Picture 3">
-          <a:hlinkClick r:id="rId1"/>
+          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </cNvPr>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="647701" y="5158514"/>
           <a:ext cx="742950" cy="813659"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -6343,7 +6352,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL18.0 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL20.0 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6459,7 +6468,7 @@
       </c>
       <c r="C5" s="109" t="inlineStr">
         <is>
-          <t>MODEL18 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
+          <t>MODEL20 — cash taxes ≠ book tax (3S J13 still book for NI)</t>
         </is>
       </c>
       <c r="D5" s="110" t="n">
@@ -6500,7 +6509,7 @@
       </c>
       <c r="C6" s="109" t="inlineStr">
         <is>
-          <t>WACC algebra unchanged vs Model17 (Previous: 7.68%) in Model18 (New: 7.68% = Rf 4.67% + β 0.854 × ERP 4.28%; Rd 6.250%). Stub fix is temporal, not WACC.</t>
+          <t>WACC algebra unchanged vs Model17 (Previous: 7.68%) in Model20 (New: 7.68% = Rf 4.67% + β 0.854 × ERP 4.28%; Rd 6.250%). Stub fix is temporal, not WACC.</t>
         </is>
       </c>
       <c r="D6" s="111">
@@ -6542,7 +6551,7 @@
       </c>
       <c r="C7" s="109" t="inlineStr">
         <is>
-          <t>g unchanged vs Model17 (Previous: 3.5%) in Model18</t>
+          <t>g unchanged vs Model17 (Previous: 3.5%) in Model20</t>
         </is>
       </c>
       <c r="D7" s="112" t="n">
@@ -6632,7 +6641,7 @@
       </c>
       <c r="C9" s="109" t="inlineStr">
         <is>
-          <t>Updated from Model17 (Previous: hist FYE 2025-09-30) to Model18 (New: 2026-08-06; 129/365=35.34% elapsed)</t>
+          <t>Updated from Model17 (Previous: hist FYE 2025-09-30) to Model20 (New: 2026-08-06; 129/365=35.34% elapsed)</t>
         </is>
       </c>
       <c r="D9" s="117" t="n">
@@ -6749,12 +6758,12 @@
       <c r="A13" s="100" t="n"/>
       <c r="B13" s="100" t="inlineStr">
         <is>
-          <t>Debt (10-Q bridge — not 3S FY25 I49)</t>
+          <t>Debt today (10-Q bridge — opening gross debt)</t>
         </is>
       </c>
       <c r="C13" s="109" t="inlineStr">
         <is>
-          <t>See L39 for 3S FY25 debt ref</t>
+          <t>D34 = D13 + stub×3S!J19 + K19:N19 (adds buyback-funded debt)</t>
         </is>
       </c>
       <c r="D13" s="121" t="n">
@@ -6776,12 +6785,12 @@
       <c r="A14" s="100" t="n"/>
       <c r="B14" s="100" t="inlineStr">
         <is>
-          <t>Cash+mkt secs (10-Q bridge — not 3S FY25 I41)</t>
+          <t>Cash+mkt secs (10-Q bridge — ΔCash≈0 under levered buybacks)</t>
         </is>
       </c>
       <c r="C14" s="109" t="inlineStr">
         <is>
-          <t>See L38 for 3S FY25 cash ref</t>
+          <t>See L38 for 3S FY25 cash ref; bridge cash stays current</t>
         </is>
       </c>
       <c r="D14" s="121" t="n">
@@ -6907,7 +6916,7 @@
       <c r="K17" s="100" t="n"/>
       <c r="L17" s="128" t="inlineStr">
         <is>
-          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL18.0)</t>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL20.0)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -7308,7 +7317,7 @@
       <c r="K26" s="100" t="n"/>
       <c r="L26" s="140" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL18.0 — DCF ← 3-Statement linkage audit</t>
+          <t>vengeanceaiUSCMODEL20.0 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7623,12 +7632,16 @@
       <c r="A34" s="100" t="n"/>
       <c r="B34" s="100" t="inlineStr">
         <is>
-          <t>Less: Debt</t>
-        </is>
-      </c>
-      <c r="C34" s="100" t="n"/>
-      <c r="D34" s="100">
-        <f>+D13</f>
+          <t>Less: Debt (today + forecast buyback-funded issuance)</t>
+        </is>
+      </c>
+      <c r="C34" s="109" t="inlineStr">
+        <is>
+          <t>Updated from Model18 (Previous: D34=D13 only) to Model20 (New: D34=D13+stub×Y1 debt CF + Y2–Y5 debt CF)</t>
+        </is>
+      </c>
+      <c r="D34" s="149">
+        <f>$D$13+0.646575*'3 Statement Model'!J19+'3 Statement Model'!K19+'3 Statement Model'!L19+'3 Statement Model'!M19+'3 Statement Model'!N19</f>
         <v/>
       </c>
       <c r="E34" s="100" t="n"/>
@@ -7714,7 +7727,7 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="149" t="n"/>
+      <c r="I36" s="150" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
@@ -7744,10 +7757,10 @@
       </c>
       <c r="C37" s="109" t="inlineStr">
         <is>
-          <t>MODEL18: SBC add-back in FCFF; 1.4×FCF buybacks cut shares (no SBC dilution)</t>
-        </is>
-      </c>
-      <c r="D37" s="150">
+          <t>MODEL20: $/share uses I16; D34 includes forecast debt that funded buybacks</t>
+        </is>
+      </c>
+      <c r="D37" s="151">
         <f>$D$35/$I$16</f>
         <v/>
       </c>
@@ -7758,7 +7771,7 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="149">
+      <c r="I37" s="150">
         <f>D11</f>
         <v/>
       </c>
@@ -7876,7 +7889,7 @@
         </is>
       </c>
       <c r="C41" s="125" t="n"/>
-      <c r="D41" s="151" t="n"/>
+      <c r="D41" s="152" t="n"/>
       <c r="E41" s="125" t="n"/>
       <c r="F41" s="125" t="n"/>
       <c r="G41" s="125" t="n"/>
@@ -7899,7 +7912,7 @@
       </c>
       <c r="O41" s="144" t="inlineStr">
         <is>
-          <t>FYE reference only — bridge uses 10-Q D13</t>
+          <t>FYE reference only — D13 is opening debt; D34 adds forecast issuance</t>
         </is>
       </c>
     </row>
@@ -7916,16 +7929,16 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="L42" s="152" t="inlineStr">
+      <c r="L42" s="153" t="inlineStr">
         <is>
           <t>EBIT link OK?</t>
         </is>
       </c>
-      <c r="M42" s="153">
+      <c r="M42" s="154">
         <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
         <v/>
       </c>
-      <c r="N42" s="154" t="inlineStr"/>
+      <c r="N42" s="155" t="inlineStr"/>
       <c r="O42" s="144" t="inlineStr">
         <is>
           <t>Flags if EBIT link ≠ GP−opex build</t>
@@ -7945,7 +7958,7 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="L43" s="155" t="inlineStr">
+      <c r="L43" s="156" t="inlineStr">
         <is>
           <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman-adj CAPM 7.68% (D6←R15; raw CAPM ref 9.27%). $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute.</t>
         </is>
@@ -7953,7 +7966,7 @@
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="156" t="inlineStr">
+      <c r="B44" s="157" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7969,7 +7982,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="156" t="inlineStr">
+      <c r="B45" s="157" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7985,7 +7998,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="156" t="inlineStr">
+      <c r="B46" s="157" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -8020,7 +8033,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="157" t="inlineStr">
+      <c r="N48" s="158" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -8036,7 +8049,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="158" t="inlineStr">
+      <c r="N49" s="159" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8152,22 +8165,22 @@
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="159" t="n">
+      <c r="M56" s="160" t="n">
         <v>17</v>
       </c>
-      <c r="N56" s="159" t="n">
+      <c r="N56" s="160" t="n">
         <v>20</v>
       </c>
-      <c r="O56" s="159" t="n">
+      <c r="O56" s="160" t="n">
         <v>23</v>
       </c>
-      <c r="P56" s="159" t="n">
+      <c r="P56" s="160" t="n">
         <v>25</v>
       </c>
-      <c r="Q56" s="159" t="n">
+      <c r="Q56" s="160" t="n">
         <v>27</v>
       </c>
-      <c r="R56" s="159" t="n">
+      <c r="R56" s="160" t="n">
         <v>29</v>
       </c>
     </row>
@@ -8183,7 +8196,7 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="160" t="n">
+      <c r="L57" s="161" t="n">
         <v>0.065</v>
       </c>
       <c r="M57" s="148">
@@ -8223,7 +8236,7 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="160" t="n">
+      <c r="L58" s="161" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="M58" s="148">
@@ -8263,7 +8276,7 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="160" t="n">
+      <c r="L59" s="161" t="n">
         <v>0.075</v>
       </c>
       <c r="M59" s="148">
@@ -8303,7 +8316,7 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="160" t="n">
+      <c r="L60" s="161" t="n">
         <v>0.07679999999999999</v>
       </c>
       <c r="M60" s="148">
@@ -8314,7 +8327,7 @@
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="161">
+      <c r="O60" s="162">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8342,7 +8355,7 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="160" t="n">
+      <c r="L61" s="161" t="n">
         <v>0.08500000000000001</v>
       </c>
       <c r="M61" s="148">
@@ -8371,7 +8384,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="L62" s="160" t="n">
+      <c r="L62" s="161" t="n">
         <v>0.095</v>
       </c>
       <c r="M62" s="148">
@@ -8400,213 +8413,213 @@
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="162" t="inlineStr">
+      <c r="L64" s="163" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="163" t="inlineStr">
+      <c r="L65" s="164" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="164" t="n">
+      <c r="M65" s="165" t="n">
         <v>17</v>
       </c>
-      <c r="N65" s="164" t="n">
+      <c r="N65" s="165" t="n">
         <v>20</v>
       </c>
-      <c r="O65" s="164" t="n">
+      <c r="O65" s="165" t="n">
         <v>23</v>
       </c>
-      <c r="P65" s="164" t="n">
+      <c r="P65" s="165" t="n">
         <v>25</v>
       </c>
-      <c r="Q65" s="164" t="n">
+      <c r="Q65" s="165" t="n">
         <v>27</v>
       </c>
-      <c r="R65" s="164" t="n">
+      <c r="R65" s="165" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="160" t="n">
+      <c r="L66" s="161" t="n">
         <v>0.065</v>
       </c>
-      <c r="M66" s="165">
+      <c r="M66" s="166">
         <f>(M57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N66" s="165">
+      <c r="N66" s="166">
         <f>(N57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O66" s="165">
+      <c r="O66" s="166">
         <f>(O57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P66" s="165">
+      <c r="P66" s="166">
         <f>(P57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q66" s="165">
+      <c r="Q66" s="166">
         <f>(Q57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R66" s="165">
+      <c r="R66" s="166">
         <f>(R57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="160" t="n">
+      <c r="L67" s="161" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="M67" s="165">
+      <c r="M67" s="166">
         <f>(M58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N67" s="165">
+      <c r="N67" s="166">
         <f>(N58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O67" s="165">
+      <c r="O67" s="166">
         <f>(O58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P67" s="165">
+      <c r="P67" s="166">
         <f>(P58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q67" s="165">
+      <c r="Q67" s="166">
         <f>(Q58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R67" s="165">
+      <c r="R67" s="166">
         <f>(R58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="160" t="n">
+      <c r="L68" s="161" t="n">
         <v>0.075</v>
       </c>
-      <c r="M68" s="165">
+      <c r="M68" s="166">
         <f>(M59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N68" s="165">
+      <c r="N68" s="166">
         <f>(N59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O68" s="165">
+      <c r="O68" s="166">
         <f>(O59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P68" s="165">
+      <c r="P68" s="166">
         <f>(P59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q68" s="165">
+      <c r="Q68" s="166">
         <f>(Q59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R68" s="165">
+      <c r="R68" s="166">
         <f>(R59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="160" t="n">
+      <c r="L69" s="161" t="n">
         <v>0.07679999999999999</v>
       </c>
-      <c r="M69" s="165">
+      <c r="M69" s="166">
         <f>(M60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N69" s="165">
+      <c r="N69" s="166">
         <f>(N60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O69" s="166">
+      <c r="O69" s="167">
         <f>(O60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P69" s="165">
+      <c r="P69" s="166">
         <f>(P60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q69" s="165">
+      <c r="Q69" s="166">
         <f>(Q60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R69" s="165">
+      <c r="R69" s="166">
         <f>(R60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="160" t="n">
+      <c r="L70" s="161" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="M70" s="165">
+      <c r="M70" s="166">
         <f>(M61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N70" s="165">
+      <c r="N70" s="166">
         <f>(N61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O70" s="165">
+      <c r="O70" s="166">
         <f>(O61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P70" s="165">
+      <c r="P70" s="166">
         <f>(P61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q70" s="165">
+      <c r="Q70" s="166">
         <f>(Q61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R70" s="165">
+      <c r="R70" s="166">
         <f>(R61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="L71" s="160" t="n">
+      <c r="L71" s="161" t="n">
         <v>0.095</v>
       </c>
-      <c r="M71" s="165">
+      <c r="M71" s="166">
         <f>(M62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N71" s="165">
+      <c r="N71" s="166">
         <f>(N62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O71" s="165">
+      <c r="O71" s="166">
         <f>(O62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P71" s="165">
+      <c r="P71" s="166">
         <f>(P62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q71" s="165">
+      <c r="Q71" s="166">
         <f>(Q62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R71" s="165">
+      <c r="R71" s="166">
         <f>(R62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="155" t="inlineStr">
+      <c r="L72" s="156" t="inlineStr">
         <is>
           <t>Yellow = base (Yacktman WACC=7.68%, Exit 23.0x; CAPM ref ≈9.27%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 23.0x; bull 27x; bear 17.0x.</t>
         </is>

</xml_diff>

<commit_message>
MODEL21: equity bridge subtracts forecast buyback-funded debt
Surgical fix only: D34 = D13 + stub×Y1 debt CF + Y2–Y5 debt CF (3S row 19).
Leaves 3-statement assumptions commentary unchanged from MODEL18.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FICO/templates/CFI_Template.xlsx
+++ b/FICO/templates/CFI_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22296" windowHeight="8376" tabRatio="685" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover Page" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="3 Statement Model" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DCF Model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover Page" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Statement Model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF Model" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="IS_BaseYear">'3 Statement Model'!$E$2</definedName>
@@ -95,12 +95,12 @@
     <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0.00_-;\(#,##0.00\)_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="175" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="176" formatCode="0.0"/>
-    <numFmt numFmtId="177" formatCode="#,##0.000"/>
-    <numFmt numFmtId="178" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="179" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="180" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="181" formatCode="#,##0.0"/>
+    <numFmt numFmtId="176" formatCode="#,##0.0"/>
+    <numFmt numFmtId="177" formatCode="0.0"/>
+    <numFmt numFmtId="178" formatCode="#,##0.000"/>
+    <numFmt numFmtId="179" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="180" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="181" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="48">
     <font>
@@ -541,7 +541,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -711,7 +711,7 @@
     </xf>
     <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="44" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="33" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="32" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -725,15 +725,15 @@
     <xf numFmtId="166" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="177" fontId="38" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="179" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="180" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="175" fontId="38" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="180" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="30" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -741,7 +741,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="177" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -768,9 +768,10 @@
     <xf numFmtId="164" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="44" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="181" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="174" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -789,16 +790,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="180" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="43" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="181" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="42" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="45" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="180" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="181" fontId="43" fillId="10" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="179" fontId="40" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -839,14 +840,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -869,16 +870,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -920,10 +921,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent1"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -974,10 +975,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent3"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1028,10 +1029,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent2"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1091,8 +1092,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -1104,9 +1105,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1145,16 +1146,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1183,16 +1184,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -1217,8 +1218,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1228,14 +1229,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -1263,16 +1264,16 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -1306,10 +1307,10 @@
             <v>Operating</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent2"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1352,10 +1353,10 @@
             <v>Investing</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent3"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1398,10 +1399,10 @@
             <v>FInancing</v>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:schemeClr val="accent4"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1462,8 +1463,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -1475,9 +1476,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1516,16 +1517,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1554,16 +1555,16 @@
       <legendPos val="b"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -1588,8 +1589,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1601,7 +1602,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>vengeanceaiUSCMODEL18.0</author>
+    <author>vengeanceaiUSCMODEL21.0</author>
   </authors>
   <commentList>
     <comment ref="D5" authorId="0" shapeId="0">
@@ -1652,7 +1653,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -1669,27 +1670,27 @@
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Picture 1">
-          <a:hlinkClick r:id="rId1"/>
+          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </cNvPr>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="1447799" y="762000"/>
           <a:ext cx="3359943" cy="1581150"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1700,7 +1701,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>1</col>
@@ -1720,9 +1721,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1747,9 +1748,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1771,27 +1772,27 @@
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Picture 3">
-          <a:hlinkClick r:id="rId1"/>
+          <a:hlinkClick xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </cNvPr>
         <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="647701" y="5158514"/>
           <a:ext cx="742950" cy="813659"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -6343,7 +6344,7 @@
       <c r="K1" s="94" t="n"/>
       <c r="L1" s="95" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL18.0 — Public Peer EV/EBITDA Comps</t>
+          <t>vengeanceaiUSCMODEL21.0 — Public Peer EV/EBITDA Comps</t>
         </is>
       </c>
     </row>
@@ -6754,7 +6755,7 @@
       </c>
       <c r="C13" s="109" t="inlineStr">
         <is>
-          <t>See L39 for 3S FY25 debt ref</t>
+          <t>D34 = D13 + stub×3S!J19 + K19:N19 (buyback-funded debt)</t>
         </is>
       </c>
       <c r="D13" s="121" t="n">
@@ -6907,7 +6908,7 @@
       <c r="K17" s="100" t="n"/>
       <c r="L17" s="128" t="inlineStr">
         <is>
-          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL18.0)</t>
+          <t>Terminal value &amp; scenarios (vengeanceaiUSCMODEL21.0)</t>
         </is>
       </c>
       <c r="O17" s="100" t="n"/>
@@ -7308,7 +7309,7 @@
       <c r="K26" s="100" t="n"/>
       <c r="L26" s="140" t="inlineStr">
         <is>
-          <t>vengeanceaiUSCMODEL18.0 — DCF ← 3-Statement linkage audit</t>
+          <t>vengeanceaiUSCMODEL21.0 — DCF ← 3-Statement linkage audit</t>
         </is>
       </c>
     </row>
@@ -7623,12 +7624,12 @@
       <c r="A34" s="100" t="n"/>
       <c r="B34" s="100" t="inlineStr">
         <is>
-          <t>Less: Debt</t>
+          <t>Less: Debt (today + forecast buyback-funded issuance)</t>
         </is>
       </c>
       <c r="C34" s="100" t="n"/>
-      <c r="D34" s="100">
-        <f>+D13</f>
+      <c r="D34" s="149">
+        <f>$D$13+0.646575*'3 Statement Model'!J19+'3 Statement Model'!K19+'3 Statement Model'!L19+'3 Statement Model'!M19+'3 Statement Model'!N19</f>
         <v/>
       </c>
       <c r="E34" s="100" t="n"/>
@@ -7714,7 +7715,7 @@
       <c r="E36" s="100" t="n"/>
       <c r="G36" s="100" t="n"/>
       <c r="H36" s="100" t="n"/>
-      <c r="I36" s="149" t="n"/>
+      <c r="I36" s="150" t="n"/>
       <c r="J36" s="100" t="n"/>
       <c r="L36" s="104" t="inlineStr">
         <is>
@@ -7747,7 +7748,7 @@
           <t>MODEL18: SBC add-back in FCFF; 1.4×FCF buybacks cut shares (no SBC dilution)</t>
         </is>
       </c>
-      <c r="D37" s="150">
+      <c r="D37" s="151">
         <f>$D$35/$I$16</f>
         <v/>
       </c>
@@ -7758,7 +7759,7 @@
         </is>
       </c>
       <c r="H37" s="100" t="n"/>
-      <c r="I37" s="149">
+      <c r="I37" s="150">
         <f>D11</f>
         <v/>
       </c>
@@ -7876,7 +7877,7 @@
         </is>
       </c>
       <c r="C41" s="125" t="n"/>
-      <c r="D41" s="151" t="n"/>
+      <c r="D41" s="152" t="n"/>
       <c r="E41" s="125" t="n"/>
       <c r="F41" s="125" t="n"/>
       <c r="G41" s="125" t="n"/>
@@ -7916,16 +7917,16 @@
       <c r="F42" s="100" t="n"/>
       <c r="G42" s="100" t="n"/>
       <c r="H42" s="100" t="n"/>
-      <c r="L42" s="152" t="inlineStr">
+      <c r="L42" s="153" t="inlineStr">
         <is>
           <t>EBIT link OK?</t>
         </is>
       </c>
-      <c r="M42" s="153">
+      <c r="M42" s="154">
         <f>IF(ABS(M33-M34)&lt;1,"OK","MISMATCH")</f>
         <v/>
       </c>
-      <c r="N42" s="154" t="inlineStr"/>
+      <c r="N42" s="155" t="inlineStr"/>
       <c r="O42" s="144" t="inlineStr">
         <is>
           <t>Flags if EBIT link ≠ GP−opex build</t>
@@ -7945,7 +7946,7 @@
       <c r="F43" s="100" t="n"/>
       <c r="G43" s="100" t="n"/>
       <c r="H43" s="100" t="n"/>
-      <c r="L43" s="155" t="inlineStr">
+      <c r="L43" s="156" t="inlineStr">
         <is>
           <t>Green cells are live links. FCFF = EBIT − cash tax + D&amp;A + SBC − CapEx − ΔOpNWC + ΔDeferred. D6 = Yacktman-adj CAPM 7.68% (D6←R15; raw CAPM ref 9.27%). $/share uses I16 (Y5 buyback-adjusted shares). SBC add-back does NOT dilute.</t>
         </is>
@@ -7953,7 +7954,7 @@
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="100" t="n"/>
-      <c r="B44" s="156" t="inlineStr">
+      <c r="B44" s="157" t="inlineStr">
         <is>
           <t>There are two ways to find NWC:</t>
         </is>
@@ -7969,7 +7970,7 @@
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="100" t="n"/>
-      <c r="B45" s="156" t="inlineStr">
+      <c r="B45" s="157" t="inlineStr">
         <is>
           <t>1. NWC = Current Assets (less cash) - Current Liabilities (less debt)</t>
         </is>
@@ -7985,7 +7986,7 @@
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="n"/>
-      <c r="B46" s="156" t="inlineStr">
+      <c r="B46" s="157" t="inlineStr">
         <is>
           <t>2. NWC = Accounts Receivable + Inventory - Accounts Payable</t>
         </is>
@@ -8020,7 +8021,7 @@
       <c r="F48" s="100" t="n"/>
       <c r="G48" s="100" t="n"/>
       <c r="H48" s="100" t="n"/>
-      <c r="N48" s="157" t="inlineStr">
+      <c r="N48" s="158" t="inlineStr">
         <is>
           <t xml:space="preserve">Corporate Finance Institute® </t>
         </is>
@@ -8036,7 +8037,7 @@
       <c r="F49" s="100" t="n"/>
       <c r="G49" s="100" t="n"/>
       <c r="H49" s="100" t="n"/>
-      <c r="N49" s="158" t="inlineStr">
+      <c r="N49" s="159" t="inlineStr">
         <is>
           <t>https://corporatefinanceinstitute.com/</t>
         </is>
@@ -8152,22 +8153,22 @@
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M56" s="159" t="n">
+      <c r="M56" s="160" t="n">
         <v>17</v>
       </c>
-      <c r="N56" s="159" t="n">
+      <c r="N56" s="160" t="n">
         <v>20</v>
       </c>
-      <c r="O56" s="159" t="n">
+      <c r="O56" s="160" t="n">
         <v>23</v>
       </c>
-      <c r="P56" s="159" t="n">
+      <c r="P56" s="160" t="n">
         <v>25</v>
       </c>
-      <c r="Q56" s="159" t="n">
+      <c r="Q56" s="160" t="n">
         <v>27</v>
       </c>
-      <c r="R56" s="159" t="n">
+      <c r="R56" s="160" t="n">
         <v>29</v>
       </c>
     </row>
@@ -8183,7 +8184,7 @@
       <c r="I57" s="100" t="n"/>
       <c r="J57" s="100" t="n"/>
       <c r="K57" s="100" t="n"/>
-      <c r="L57" s="160" t="n">
+      <c r="L57" s="161" t="n">
         <v>0.065</v>
       </c>
       <c r="M57" s="148">
@@ -8223,7 +8224,7 @@
       <c r="I58" s="100" t="n"/>
       <c r="J58" s="100" t="n"/>
       <c r="K58" s="100" t="n"/>
-      <c r="L58" s="160" t="n">
+      <c r="L58" s="161" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="M58" s="148">
@@ -8263,7 +8264,7 @@
       <c r="I59" s="100" t="n"/>
       <c r="J59" s="100" t="n"/>
       <c r="K59" s="100" t="n"/>
-      <c r="L59" s="160" t="n">
+      <c r="L59" s="161" t="n">
         <v>0.075</v>
       </c>
       <c r="M59" s="148">
@@ -8303,7 +8304,7 @@
       <c r="I60" s="100" t="n"/>
       <c r="J60" s="100" t="n"/>
       <c r="K60" s="100" t="n"/>
-      <c r="L60" s="160" t="n">
+      <c r="L60" s="161" t="n">
         <v>0.07679999999999999</v>
       </c>
       <c r="M60" s="148">
@@ -8314,7 +8315,7 @@
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*N$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
-      <c r="O60" s="161">
+      <c r="O60" s="162">
         <f>XNPV($L60,$D$28:$I$28,$D$18:$I$18)+($I$26+($I$21+$I$23)*O$56)/((1+$L60)^(($J$18-$D$18)/365))</f>
         <v/>
       </c>
@@ -8342,7 +8343,7 @@
       <c r="I61" s="100" t="n"/>
       <c r="J61" s="100" t="n"/>
       <c r="K61" s="100" t="n"/>
-      <c r="L61" s="160" t="n">
+      <c r="L61" s="161" t="n">
         <v>0.08500000000000001</v>
       </c>
       <c r="M61" s="148">
@@ -8371,7 +8372,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="L62" s="160" t="n">
+      <c r="L62" s="161" t="n">
         <v>0.095</v>
       </c>
       <c r="M62" s="148">
@@ -8400,213 +8401,213 @@
       </c>
     </row>
     <row r="64">
-      <c r="L64" s="162" t="inlineStr">
+      <c r="L64" s="163" t="inlineStr">
         <is>
           <t>SENSITIVITY — Equity Value / Share ($)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="L65" s="163" t="inlineStr">
+      <c r="L65" s="164" t="inlineStr">
         <is>
           <t>WACC \ Exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="M65" s="164" t="n">
+      <c r="M65" s="165" t="n">
         <v>17</v>
       </c>
-      <c r="N65" s="164" t="n">
+      <c r="N65" s="165" t="n">
         <v>20</v>
       </c>
-      <c r="O65" s="164" t="n">
+      <c r="O65" s="165" t="n">
         <v>23</v>
       </c>
-      <c r="P65" s="164" t="n">
+      <c r="P65" s="165" t="n">
         <v>25</v>
       </c>
-      <c r="Q65" s="164" t="n">
+      <c r="Q65" s="165" t="n">
         <v>27</v>
       </c>
-      <c r="R65" s="164" t="n">
+      <c r="R65" s="165" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="66">
-      <c r="L66" s="160" t="n">
+      <c r="L66" s="161" t="n">
         <v>0.065</v>
       </c>
-      <c r="M66" s="165">
+      <c r="M66" s="166">
         <f>(M57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N66" s="165">
+      <c r="N66" s="166">
         <f>(N57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O66" s="165">
+      <c r="O66" s="166">
         <f>(O57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P66" s="165">
+      <c r="P66" s="166">
         <f>(P57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q66" s="165">
+      <c r="Q66" s="166">
         <f>(Q57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R66" s="165">
+      <c r="R66" s="166">
         <f>(R57+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="L67" s="160" t="n">
+      <c r="L67" s="161" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="M67" s="165">
+      <c r="M67" s="166">
         <f>(M58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N67" s="165">
+      <c r="N67" s="166">
         <f>(N58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O67" s="165">
+      <c r="O67" s="166">
         <f>(O58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P67" s="165">
+      <c r="P67" s="166">
         <f>(P58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q67" s="165">
+      <c r="Q67" s="166">
         <f>(Q58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R67" s="165">
+      <c r="R67" s="166">
         <f>(R58+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="L68" s="160" t="n">
+      <c r="L68" s="161" t="n">
         <v>0.075</v>
       </c>
-      <c r="M68" s="165">
+      <c r="M68" s="166">
         <f>(M59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N68" s="165">
+      <c r="N68" s="166">
         <f>(N59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O68" s="165">
+      <c r="O68" s="166">
         <f>(O59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P68" s="165">
+      <c r="P68" s="166">
         <f>(P59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q68" s="165">
+      <c r="Q68" s="166">
         <f>(Q59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R68" s="165">
+      <c r="R68" s="166">
         <f>(R59+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="L69" s="160" t="n">
+      <c r="L69" s="161" t="n">
         <v>0.07679999999999999</v>
       </c>
-      <c r="M69" s="165">
+      <c r="M69" s="166">
         <f>(M60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N69" s="165">
+      <c r="N69" s="166">
         <f>(N60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O69" s="166">
+      <c r="O69" s="167">
         <f>(O60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P69" s="165">
+      <c r="P69" s="166">
         <f>(P60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q69" s="165">
+      <c r="Q69" s="166">
         <f>(Q60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R69" s="165">
+      <c r="R69" s="166">
         <f>(R60+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="L70" s="160" t="n">
+      <c r="L70" s="161" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="M70" s="165">
+      <c r="M70" s="166">
         <f>(M61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N70" s="165">
+      <c r="N70" s="166">
         <f>(N61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O70" s="165">
+      <c r="O70" s="166">
         <f>(O61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P70" s="165">
+      <c r="P70" s="166">
         <f>(P61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q70" s="165">
+      <c r="Q70" s="166">
         <f>(Q61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R70" s="165">
+      <c r="R70" s="166">
         <f>(R61+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="L71" s="160" t="n">
+      <c r="L71" s="161" t="n">
         <v>0.095</v>
       </c>
-      <c r="M71" s="165">
+      <c r="M71" s="166">
         <f>(M62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="N71" s="165">
+      <c r="N71" s="166">
         <f>(N62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="O71" s="165">
+      <c r="O71" s="166">
         <f>(O62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="P71" s="165">
+      <c r="P71" s="166">
         <f>(P62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="Q71" s="165">
+      <c r="Q71" s="166">
         <f>(Q62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
-      <c r="R71" s="165">
+      <c r="R71" s="166">
         <f>(R62+$D$33-$D$34)/$I$16</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="L72" s="155" t="inlineStr">
+      <c r="L72" s="156" t="inlineStr">
         <is>
           <t>Yellow = base (Yacktman WACC=7.68%, Exit 23.0x; CAPM ref ≈9.27%). EV formula: XNPV(explicit FCFF) + (Y5 FCFF + Exit×EBITDA) / (1+WACC)^daycount. Peer median ~18.1x → base 23.0x; bull 27x; bear 17.0x.</t>
         </is>

</xml_diff>